<commit_message>
Add high-frequency checks and enhance data validation in girls and household scripts
- Integrated high-frequency checks in `girls.py` and `household.py` to validate GPS, speed warnings, and night re-entry conditions.
- Updated `girls_columns.yaml` and `household_columns.yaml` with new parameters for speed warnings and GPS accuracy.
- Enhanced error guidance in `error-guidance.ts` to address GPS inconsistencies and speed warning issues during interviews.
- Improved data accuracy in tracking survey files by updating relevant metrics and configurations.
</commit_message>
<xml_diff>
--- a/Error_log/Enumerator_Performance.xlsx
+++ b/Error_log/Enumerator_Performance.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="performance" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="performance_pct" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="performance" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="performance_pct" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,16 +18,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -38,7 +35,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -46,21 +43,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -430,27 +418,27 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Enumerator Name</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Enumerator ID</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Total Issues</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Critical Issues</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Flag Issues</t>
         </is>
@@ -464,10 +452,10 @@
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="n">
-        <v>2437</v>
+        <v>2455</v>
       </c>
       <c r="D2" t="n">
-        <v>2435</v>
+        <v>2453</v>
       </c>
       <c r="E2" t="n">
         <v>2</v>
@@ -533,115 +521,115 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Asma Bibi</t>
+          <t>Zohra</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>373641</v>
+        <v>373692</v>
       </c>
       <c r="C6" t="n">
-        <v>134</v>
+        <v>285</v>
       </c>
       <c r="D6" t="n">
         <v>112</v>
       </c>
       <c r="E6" t="n">
-        <v>22</v>
+        <v>165</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Irum Ikram</t>
+          <t>Asma Bibi</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>373642</v>
+        <v>373641</v>
       </c>
       <c r="C7" t="n">
-        <v>109</v>
+        <v>134</v>
       </c>
       <c r="D7" t="n">
-        <v>105</v>
+        <v>112</v>
       </c>
       <c r="E7" t="n">
-        <v>4</v>
+        <v>22</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Mehran Khan</t>
+          <t>Irum Ikram</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>373684</v>
+        <v>373642</v>
       </c>
       <c r="C8" t="n">
-        <v>131</v>
+        <v>109</v>
       </c>
       <c r="D8" t="n">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="E8" t="n">
-        <v>28</v>
+        <v>4</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Sadia Rustum</t>
+          <t>Mehran Khan</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>373649</v>
+        <v>373684</v>
       </c>
       <c r="C9" t="n">
-        <v>106</v>
+        <v>131</v>
       </c>
       <c r="D9" t="n">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="E9" t="n">
-        <v>10</v>
+        <v>28</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Zohra</t>
+          <t>Samara</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>373692</v>
+        <v>373658</v>
       </c>
       <c r="C10" t="n">
-        <v>178</v>
+        <v>241</v>
       </c>
       <c r="D10" t="n">
-        <v>85</v>
+        <v>99</v>
       </c>
       <c r="E10" t="n">
-        <v>85</v>
+        <v>125</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Samara</t>
+          <t>Sadia Rustum</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>373658</v>
+        <v>373649</v>
       </c>
       <c r="C11" t="n">
-        <v>178</v>
+        <v>106</v>
       </c>
       <c r="D11" t="n">
-        <v>80</v>
+        <v>96</v>
       </c>
       <c r="E11" t="n">
-        <v>81</v>
+        <v>10</v>
       </c>
     </row>
     <row r="12">
@@ -654,162 +642,162 @@
         <v>373691</v>
       </c>
       <c r="C12" t="n">
-        <v>174</v>
+        <v>271</v>
       </c>
       <c r="D12" t="n">
-        <v>71</v>
+        <v>81</v>
       </c>
       <c r="E12" t="n">
-        <v>90</v>
+        <v>177</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Furqan Ullah Khan</t>
+          <t>Kainat</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>373683</v>
+        <v>373712</v>
       </c>
       <c r="C13" t="n">
-        <v>73</v>
+        <v>244</v>
       </c>
       <c r="D13" t="n">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="E13" t="n">
-        <v>8</v>
+        <v>160</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Khalida Bibi</t>
+          <t>Furqan Ullah Khan</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>373673</v>
+        <v>373683</v>
       </c>
       <c r="C14" t="n">
-        <v>63</v>
+        <v>76</v>
       </c>
       <c r="D14" t="n">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="E14" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Muhammad Yousaf</t>
+          <t>Khalida Bibi</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>373690</v>
+        <v>373673</v>
       </c>
       <c r="C15" t="n">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="D15" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="E15" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Javairia</t>
+          <t>Muhammad Yousaf</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>373651</v>
+        <v>373690</v>
       </c>
       <c r="C16" t="n">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="D16" t="n">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="E16" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Naureen Khan</t>
+          <t>Javairia</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>373716</v>
+        <v>373651</v>
       </c>
       <c r="C17" t="n">
-        <v>58</v>
+        <v>73</v>
       </c>
       <c r="D17" t="n">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="E17" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Jaweria</t>
+          <t>Naureen Khan</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>163495</v>
+        <v>373716</v>
       </c>
       <c r="C18" t="n">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="D18" t="n">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="E18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Bushra Ayub</t>
+          <t>Jaweria</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>373671</v>
+        <v>163495</v>
       </c>
       <c r="C19" t="n">
+        <v>56</v>
+      </c>
+      <c r="D19" t="n">
         <v>55</v>
       </c>
-      <c r="D19" t="n">
-        <v>51</v>
-      </c>
       <c r="E19" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Mahnoor</t>
+          <t>Bushra Ayub</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>373705</v>
+        <v>373671</v>
       </c>
       <c r="C20" t="n">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="D20" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="E20" t="n">
         <v>4</v>
@@ -818,17 +806,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Asma Gull</t>
+          <t>Mahnoor</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>373672</v>
+        <v>373705</v>
       </c>
       <c r="C21" t="n">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D21" t="n">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="E21" t="n">
         <v>4</v>
@@ -837,39 +825,39 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Naureen khan</t>
+          <t>Asma Gull</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>453925</v>
+        <v>373672</v>
       </c>
       <c r="C22" t="n">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="D22" t="n">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="E22" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Kainat</t>
+          <t>Naureen khan</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>373712</v>
+        <v>453925</v>
       </c>
       <c r="C23" t="n">
-        <v>155</v>
+        <v>44</v>
       </c>
       <c r="D23" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E23" t="n">
-        <v>96</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24">
@@ -882,10 +870,10 @@
         <v>564273</v>
       </c>
       <c r="C24" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D24" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E24" t="n">
         <v>4</v>
@@ -1362,47 +1350,47 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>enumerator_name</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>enumerator_id</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>total_submissions</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>total_issues</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>critical_issues</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>flag_issues</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>error_pct</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>critical_error_pct</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>flag_error_pct</t>
         </is>
@@ -1452,19 +1440,19 @@
         <v>9</v>
       </c>
       <c r="D3" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E3" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="F3" t="n">
         <v>4</v>
       </c>
       <c r="G3" t="n">
-        <v>488.89</v>
+        <v>500</v>
       </c>
       <c r="H3" t="n">
-        <v>444.44</v>
+        <v>455.56</v>
       </c>
       <c r="I3" t="n">
         <v>44.44</v>
@@ -1504,125 +1492,125 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Lati khan</t>
+          <t>Zohra</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>671211</v>
+        <v>373692</v>
       </c>
       <c r="C5" t="n">
-        <v>9</v>
+        <v>101</v>
       </c>
       <c r="D5" t="n">
-        <v>19</v>
+        <v>285</v>
       </c>
       <c r="E5" t="n">
-        <v>19</v>
+        <v>112</v>
       </c>
       <c r="F5" t="n">
-        <v>0</v>
+        <v>165</v>
       </c>
       <c r="G5" t="n">
-        <v>211.11</v>
+        <v>282.18</v>
       </c>
       <c r="H5" t="n">
-        <v>211.11</v>
+        <v>110.89</v>
       </c>
       <c r="I5" t="n">
-        <v>0</v>
+        <v>163.37</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Zohra</t>
+          <t>Rehana Bibi</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>373692</v>
+        <v>373691</v>
       </c>
       <c r="C6" t="n">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="D6" t="n">
-        <v>178</v>
+        <v>271</v>
       </c>
       <c r="E6" t="n">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="F6" t="n">
-        <v>85</v>
+        <v>177</v>
       </c>
       <c r="G6" t="n">
-        <v>176.24</v>
+        <v>244.14</v>
       </c>
       <c r="H6" t="n">
-        <v>84.16</v>
+        <v>72.97</v>
       </c>
       <c r="I6" t="n">
-        <v>84.16</v>
+        <v>159.46</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Rehana Bibi</t>
+          <t>Kainat</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>373691</v>
+        <v>373712</v>
       </c>
       <c r="C7" t="n">
-        <v>111</v>
+        <v>104</v>
       </c>
       <c r="D7" t="n">
-        <v>174</v>
+        <v>244</v>
       </c>
       <c r="E7" t="n">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="F7" t="n">
-        <v>90</v>
+        <v>160</v>
       </c>
       <c r="G7" t="n">
-        <v>156.76</v>
+        <v>234.62</v>
       </c>
       <c r="H7" t="n">
-        <v>63.96</v>
+        <v>65.38</v>
       </c>
       <c r="I7" t="n">
-        <v>81.08</v>
+        <v>153.85</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Kainat</t>
+          <t>Lati khan</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>373712</v>
+        <v>671211</v>
       </c>
       <c r="C8" t="n">
-        <v>104</v>
+        <v>9</v>
       </c>
       <c r="D8" t="n">
-        <v>155</v>
+        <v>19</v>
       </c>
       <c r="E8" t="n">
-        <v>43</v>
+        <v>19</v>
       </c>
       <c r="F8" t="n">
-        <v>96</v>
+        <v>0</v>
       </c>
       <c r="G8" t="n">
-        <v>149.04</v>
+        <v>211.11</v>
       </c>
       <c r="H8" t="n">
-        <v>41.35</v>
+        <v>211.11</v>
       </c>
       <c r="I8" t="n">
-        <v>92.31</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -1638,22 +1626,22 @@
         <v>120</v>
       </c>
       <c r="D9" t="n">
-        <v>178</v>
+        <v>241</v>
       </c>
       <c r="E9" t="n">
-        <v>80</v>
+        <v>99</v>
       </c>
       <c r="F9" t="n">
-        <v>81</v>
+        <v>125</v>
       </c>
       <c r="G9" t="n">
-        <v>148.33</v>
+        <v>200.83</v>
       </c>
       <c r="H9" t="n">
-        <v>66.67</v>
+        <v>82.5</v>
       </c>
       <c r="I9" t="n">
-        <v>67.5</v>
+        <v>104.17</v>
       </c>
     </row>
     <row r="10">
@@ -2000,94 +1988,94 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Muhammad Yousaf</t>
+          <t>Naureen</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>373690</v>
+        <v>884887</v>
       </c>
       <c r="C21" t="n">
-        <v>119</v>
+        <v>60</v>
       </c>
       <c r="D21" t="n">
-        <v>70</v>
+        <v>35</v>
       </c>
       <c r="E21" t="n">
-        <v>62</v>
+        <v>31</v>
       </c>
       <c r="F21" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="G21" t="n">
-        <v>58.82</v>
+        <v>58.33</v>
       </c>
       <c r="H21" t="n">
-        <v>52.1</v>
+        <v>51.67</v>
       </c>
       <c r="I21" t="n">
-        <v>6.72</v>
+        <v>6.67</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Naureen</t>
+          <t>Mahnoor</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>884887</v>
+        <v>373705</v>
       </c>
       <c r="C22" t="n">
-        <v>60</v>
+        <v>94</v>
       </c>
       <c r="D22" t="n">
-        <v>35</v>
+        <v>53</v>
       </c>
       <c r="E22" t="n">
-        <v>31</v>
+        <v>49</v>
       </c>
       <c r="F22" t="n">
         <v>4</v>
       </c>
       <c r="G22" t="n">
-        <v>58.33</v>
+        <v>56.38</v>
       </c>
       <c r="H22" t="n">
-        <v>51.67</v>
+        <v>52.13</v>
       </c>
       <c r="I22" t="n">
-        <v>6.67</v>
+        <v>4.26</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Mahnoor</t>
+          <t>Muhammad Yousaf</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>373705</v>
+        <v>373690</v>
       </c>
       <c r="C23" t="n">
-        <v>94</v>
+        <v>132</v>
       </c>
       <c r="D23" t="n">
-        <v>53</v>
+        <v>71</v>
       </c>
       <c r="E23" t="n">
-        <v>49</v>
+        <v>62</v>
       </c>
       <c r="F23" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="G23" t="n">
-        <v>56.38</v>
+        <v>53.79</v>
       </c>
       <c r="H23" t="n">
-        <v>52.13</v>
+        <v>46.97</v>
       </c>
       <c r="I23" t="n">
-        <v>4.26</v>
+        <v>6.82</v>
       </c>
     </row>
     <row r="24">
@@ -2186,94 +2174,94 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Munawar Khan</t>
+          <t>Bushra Ayub</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>373668</v>
+        <v>373671</v>
       </c>
       <c r="C27" t="n">
-        <v>63</v>
+        <v>138</v>
       </c>
       <c r="D27" t="n">
-        <v>26</v>
+        <v>55</v>
       </c>
       <c r="E27" t="n">
-        <v>20</v>
+        <v>51</v>
       </c>
       <c r="F27" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="G27" t="n">
-        <v>41.27</v>
+        <v>39.86</v>
       </c>
       <c r="H27" t="n">
-        <v>31.75</v>
+        <v>36.96</v>
       </c>
       <c r="I27" t="n">
-        <v>9.52</v>
+        <v>2.9</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Bushra Ayub</t>
+          <t>Furqan Ullah Khan</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>373671</v>
+        <v>373683</v>
       </c>
       <c r="C28" t="n">
-        <v>138</v>
+        <v>195</v>
       </c>
       <c r="D28" t="n">
-        <v>55</v>
+        <v>76</v>
       </c>
       <c r="E28" t="n">
-        <v>51</v>
+        <v>68</v>
       </c>
       <c r="F28" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="G28" t="n">
-        <v>39.86</v>
+        <v>38.97</v>
       </c>
       <c r="H28" t="n">
-        <v>36.96</v>
+        <v>34.87</v>
       </c>
       <c r="I28" t="n">
-        <v>2.9</v>
+        <v>4.1</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Furqan Ullah Khan</t>
+          <t>Munawar Khan</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>373683</v>
+        <v>373668</v>
       </c>
       <c r="C29" t="n">
-        <v>184</v>
+        <v>73</v>
       </c>
       <c r="D29" t="n">
-        <v>73</v>
+        <v>26</v>
       </c>
       <c r="E29" t="n">
-        <v>65</v>
+        <v>20</v>
       </c>
       <c r="F29" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G29" t="n">
-        <v>39.67</v>
+        <v>35.62</v>
       </c>
       <c r="H29" t="n">
-        <v>35.33</v>
+        <v>27.4</v>
       </c>
       <c r="I29" t="n">
-        <v>4.35</v>
+        <v>8.220000000000001</v>
       </c>
     </row>
     <row r="30">
@@ -2937,7 +2925,7 @@
         <v>564273</v>
       </c>
       <c r="C51" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D51" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Enhance data validation and integrate review checks in girls and household scripts
- Added review checks in `girls.py` and `household.py` to improve data integrity and validation processes.
- Updated error messages to provide clearer guidance for duplicate submissions and implausible interview durations.
- Integrated new GPS validation checks in `high_frequency.py` to ensure accurate location data.
- Enhanced configuration files `girls_columns.yaml` and `household_columns.yaml` with additional parameters for improved data tracking.
</commit_message>
<xml_diff>
--- a/Error_log/Enumerator_Performance.xlsx
+++ b/Error_log/Enumerator_Performance.xlsx
@@ -464,210 +464,210 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Shafaq Zahra</t>
+          <t>Zohra</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>373646</v>
+        <v>373692</v>
       </c>
       <c r="C3" t="n">
-        <v>149</v>
+        <v>334</v>
       </c>
       <c r="D3" t="n">
-        <v>133</v>
+        <v>177</v>
       </c>
       <c r="E3" t="n">
-        <v>16</v>
+        <v>153</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Shazia begum</t>
+          <t>Samara</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>373696</v>
+        <v>373658</v>
       </c>
       <c r="C4" t="n">
-        <v>139</v>
+        <v>336</v>
       </c>
       <c r="D4" t="n">
-        <v>122</v>
+        <v>173</v>
       </c>
       <c r="E4" t="n">
-        <v>17</v>
+        <v>161</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Shazia Bibi</t>
+          <t>Rehana Bibi</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>373648</v>
+        <v>373691</v>
       </c>
       <c r="C5" t="n">
-        <v>140</v>
+        <v>339</v>
       </c>
       <c r="D5" t="n">
-        <v>117</v>
+        <v>170</v>
       </c>
       <c r="E5" t="n">
-        <v>23</v>
+        <v>166</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Zohra</t>
+          <t>Kainat</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>373692</v>
+        <v>373712</v>
       </c>
       <c r="C6" t="n">
-        <v>285</v>
+        <v>331</v>
       </c>
       <c r="D6" t="n">
-        <v>112</v>
+        <v>160</v>
       </c>
       <c r="E6" t="n">
-        <v>165</v>
+        <v>171</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Asma Bibi</t>
+          <t>Shafaq Zahra</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>373641</v>
+        <v>373646</v>
       </c>
       <c r="C7" t="n">
-        <v>134</v>
+        <v>149</v>
       </c>
       <c r="D7" t="n">
-        <v>112</v>
+        <v>133</v>
       </c>
       <c r="E7" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Irum Ikram</t>
+          <t>Shazia begum</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>373642</v>
+        <v>373696</v>
       </c>
       <c r="C8" t="n">
-        <v>109</v>
+        <v>139</v>
       </c>
       <c r="D8" t="n">
-        <v>105</v>
+        <v>122</v>
       </c>
       <c r="E8" t="n">
-        <v>4</v>
+        <v>17</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Mehran Khan</t>
+          <t>Shazia Bibi</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>373684</v>
+        <v>373648</v>
       </c>
       <c r="C9" t="n">
-        <v>131</v>
+        <v>140</v>
       </c>
       <c r="D9" t="n">
-        <v>103</v>
+        <v>117</v>
       </c>
       <c r="E9" t="n">
-        <v>28</v>
+        <v>23</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Samara</t>
+          <t>Asma Bibi</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>373658</v>
+        <v>373641</v>
       </c>
       <c r="C10" t="n">
-        <v>241</v>
+        <v>134</v>
       </c>
       <c r="D10" t="n">
-        <v>99</v>
+        <v>112</v>
       </c>
       <c r="E10" t="n">
-        <v>125</v>
+        <v>22</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Sadia Rustum</t>
+          <t>Irum Ikram</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>373649</v>
+        <v>373642</v>
       </c>
       <c r="C11" t="n">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="D11" t="n">
-        <v>96</v>
+        <v>105</v>
       </c>
       <c r="E11" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Rehana Bibi</t>
+          <t>Mehran Khan</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>373691</v>
+        <v>373684</v>
       </c>
       <c r="C12" t="n">
-        <v>271</v>
+        <v>131</v>
       </c>
       <c r="D12" t="n">
-        <v>81</v>
+        <v>103</v>
       </c>
       <c r="E12" t="n">
-        <v>177</v>
+        <v>28</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Kainat</t>
+          <t>Sadia Rustum</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>373712</v>
+        <v>373649</v>
       </c>
       <c r="C13" t="n">
-        <v>244</v>
+        <v>106</v>
       </c>
       <c r="D13" t="n">
-        <v>68</v>
+        <v>96</v>
       </c>
       <c r="E13" t="n">
-        <v>160</v>
+        <v>10</v>
       </c>
     </row>
     <row r="14">
@@ -1502,146 +1502,146 @@
         <v>101</v>
       </c>
       <c r="D5" t="n">
-        <v>285</v>
+        <v>334</v>
       </c>
       <c r="E5" t="n">
-        <v>112</v>
+        <v>177</v>
       </c>
       <c r="F5" t="n">
-        <v>165</v>
+        <v>153</v>
       </c>
       <c r="G5" t="n">
-        <v>282.18</v>
+        <v>330.69</v>
       </c>
       <c r="H5" t="n">
-        <v>110.89</v>
+        <v>175.25</v>
       </c>
       <c r="I5" t="n">
-        <v>163.37</v>
+        <v>151.49</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Rehana Bibi</t>
+          <t>Kainat</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>373691</v>
+        <v>373712</v>
       </c>
       <c r="C6" t="n">
-        <v>111</v>
+        <v>104</v>
       </c>
       <c r="D6" t="n">
-        <v>271</v>
+        <v>331</v>
       </c>
       <c r="E6" t="n">
-        <v>81</v>
+        <v>160</v>
       </c>
       <c r="F6" t="n">
-        <v>177</v>
+        <v>171</v>
       </c>
       <c r="G6" t="n">
-        <v>244.14</v>
+        <v>318.27</v>
       </c>
       <c r="H6" t="n">
-        <v>72.97</v>
+        <v>153.85</v>
       </c>
       <c r="I6" t="n">
-        <v>159.46</v>
+        <v>164.42</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Kainat</t>
+          <t>Rehana Bibi</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>373712</v>
+        <v>373691</v>
       </c>
       <c r="C7" t="n">
-        <v>104</v>
+        <v>111</v>
       </c>
       <c r="D7" t="n">
-        <v>244</v>
+        <v>339</v>
       </c>
       <c r="E7" t="n">
-        <v>68</v>
+        <v>170</v>
       </c>
       <c r="F7" t="n">
-        <v>160</v>
+        <v>166</v>
       </c>
       <c r="G7" t="n">
-        <v>234.62</v>
+        <v>305.41</v>
       </c>
       <c r="H7" t="n">
-        <v>65.38</v>
+        <v>153.15</v>
       </c>
       <c r="I7" t="n">
-        <v>153.85</v>
+        <v>149.55</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Lati khan</t>
+          <t>Samara</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>671211</v>
+        <v>373658</v>
       </c>
       <c r="C8" t="n">
-        <v>9</v>
+        <v>120</v>
       </c>
       <c r="D8" t="n">
-        <v>19</v>
+        <v>336</v>
       </c>
       <c r="E8" t="n">
-        <v>19</v>
+        <v>173</v>
       </c>
       <c r="F8" t="n">
-        <v>0</v>
+        <v>161</v>
       </c>
       <c r="G8" t="n">
-        <v>211.11</v>
+        <v>280</v>
       </c>
       <c r="H8" t="n">
-        <v>211.11</v>
+        <v>144.17</v>
       </c>
       <c r="I8" t="n">
-        <v>0</v>
+        <v>134.17</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Samara</t>
+          <t>Lati khan</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>373658</v>
+        <v>671211</v>
       </c>
       <c r="C9" t="n">
-        <v>120</v>
+        <v>9</v>
       </c>
       <c r="D9" t="n">
-        <v>241</v>
+        <v>19</v>
       </c>
       <c r="E9" t="n">
-        <v>99</v>
+        <v>19</v>
       </c>
       <c r="F9" t="n">
-        <v>125</v>
+        <v>0</v>
       </c>
       <c r="G9" t="n">
-        <v>200.83</v>
+        <v>211.11</v>
       </c>
       <c r="H9" t="n">
-        <v>82.5</v>
+        <v>211.11</v>
       </c>
       <c r="I9" t="n">
-        <v>104.17</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">

</xml_diff>

<commit_message>
Refactor survey filters to include combined "HH & Girls" option and update related components for improved functionality
</commit_message>
<xml_diff>
--- a/Error_log/Enumerator_Performance.xlsx
+++ b/Error_log/Enumerator_Performance.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="performance" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="performance_pct" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="performance" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="performance_pct" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,13 +18,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -35,7 +38,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -43,12 +46,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -418,27 +430,27 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Enumerator Name</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Enumerator ID</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Total Issues</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Critical Issues</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Flag Issues</t>
         </is>
@@ -452,10 +464,10 @@
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="n">
-        <v>2455</v>
+        <v>2459</v>
       </c>
       <c r="D2" t="n">
-        <v>2453</v>
+        <v>2457</v>
       </c>
       <c r="E2" t="n">
         <v>2</v>
@@ -464,210 +476,210 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Zohra</t>
+          <t>Shafaq Zahra</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>373692</v>
+        <v>373646</v>
       </c>
       <c r="C3" t="n">
-        <v>334</v>
+        <v>149</v>
       </c>
       <c r="D3" t="n">
-        <v>177</v>
+        <v>133</v>
       </c>
       <c r="E3" t="n">
-        <v>153</v>
+        <v>16</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Samara</t>
+          <t>Shazia begum</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>373658</v>
+        <v>373696</v>
       </c>
       <c r="C4" t="n">
-        <v>336</v>
+        <v>139</v>
       </c>
       <c r="D4" t="n">
-        <v>173</v>
+        <v>122</v>
       </c>
       <c r="E4" t="n">
-        <v>161</v>
+        <v>17</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Rehana Bibi</t>
+          <t>Shazia Bibi</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>373691</v>
+        <v>373648</v>
       </c>
       <c r="C5" t="n">
-        <v>339</v>
+        <v>140</v>
       </c>
       <c r="D5" t="n">
-        <v>170</v>
+        <v>117</v>
       </c>
       <c r="E5" t="n">
-        <v>166</v>
+        <v>23</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Kainat</t>
+          <t>Asma Bibi</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>373712</v>
+        <v>373641</v>
       </c>
       <c r="C6" t="n">
-        <v>331</v>
+        <v>134</v>
       </c>
       <c r="D6" t="n">
-        <v>160</v>
+        <v>112</v>
       </c>
       <c r="E6" t="n">
-        <v>171</v>
+        <v>22</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Shafaq Zahra</t>
+          <t>Mehran Khan</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>373646</v>
+        <v>373684</v>
       </c>
       <c r="C7" t="n">
-        <v>149</v>
+        <v>134</v>
       </c>
       <c r="D7" t="n">
-        <v>133</v>
+        <v>106</v>
       </c>
       <c r="E7" t="n">
-        <v>16</v>
+        <v>28</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Shazia begum</t>
+          <t>Irum Ikram</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>373696</v>
+        <v>373642</v>
       </c>
       <c r="C8" t="n">
-        <v>139</v>
+        <v>109</v>
       </c>
       <c r="D8" t="n">
-        <v>122</v>
+        <v>105</v>
       </c>
       <c r="E8" t="n">
-        <v>17</v>
+        <v>4</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Shazia Bibi</t>
+          <t>Kainat</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>373648</v>
+        <v>373712</v>
       </c>
       <c r="C9" t="n">
-        <v>140</v>
+        <v>303</v>
       </c>
       <c r="D9" t="n">
-        <v>117</v>
+        <v>104</v>
       </c>
       <c r="E9" t="n">
-        <v>23</v>
+        <v>199</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Asma Bibi</t>
+          <t>Zohra</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>373641</v>
+        <v>373692</v>
       </c>
       <c r="C10" t="n">
-        <v>134</v>
+        <v>288</v>
       </c>
       <c r="D10" t="n">
-        <v>112</v>
+        <v>101</v>
       </c>
       <c r="E10" t="n">
-        <v>22</v>
+        <v>183</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Irum Ikram</t>
+          <t>Sadia Rustum</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>373642</v>
+        <v>373649</v>
       </c>
       <c r="C11" t="n">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="D11" t="n">
-        <v>105</v>
+        <v>96</v>
       </c>
       <c r="E11" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Mehran Khan</t>
+          <t>Rehana Bibi</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>373684</v>
+        <v>373691</v>
       </c>
       <c r="C12" t="n">
-        <v>131</v>
+        <v>287</v>
       </c>
       <c r="D12" t="n">
-        <v>103</v>
+        <v>83</v>
       </c>
       <c r="E12" t="n">
-        <v>28</v>
+        <v>201</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Sadia Rustum</t>
+          <t>Samara</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>373649</v>
+        <v>373658</v>
       </c>
       <c r="C13" t="n">
-        <v>106</v>
+        <v>274</v>
       </c>
       <c r="D13" t="n">
-        <v>96</v>
+        <v>76</v>
       </c>
       <c r="E13" t="n">
-        <v>10</v>
+        <v>196</v>
       </c>
     </row>
     <row r="14">
@@ -1350,47 +1362,47 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>enumerator_name</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>enumerator_id</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>total_submissions</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>total_issues</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>critical_issues</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>flag_issues</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>error_pct</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>critical_error_pct</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>flag_error_pct</t>
         </is>
@@ -1492,63 +1504,63 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Zohra</t>
+          <t>Kainat</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>373692</v>
+        <v>373712</v>
       </c>
       <c r="C5" t="n">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="D5" t="n">
-        <v>334</v>
+        <v>303</v>
       </c>
       <c r="E5" t="n">
-        <v>177</v>
+        <v>104</v>
       </c>
       <c r="F5" t="n">
-        <v>153</v>
+        <v>199</v>
       </c>
       <c r="G5" t="n">
-        <v>330.69</v>
+        <v>291.35</v>
       </c>
       <c r="H5" t="n">
-        <v>175.25</v>
+        <v>100</v>
       </c>
       <c r="I5" t="n">
-        <v>151.49</v>
+        <v>191.35</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Kainat</t>
+          <t>Zohra</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>373712</v>
+        <v>373692</v>
       </c>
       <c r="C6" t="n">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="D6" t="n">
-        <v>331</v>
+        <v>288</v>
       </c>
       <c r="E6" t="n">
-        <v>160</v>
+        <v>101</v>
       </c>
       <c r="F6" t="n">
-        <v>171</v>
+        <v>183</v>
       </c>
       <c r="G6" t="n">
-        <v>318.27</v>
+        <v>285.15</v>
       </c>
       <c r="H6" t="n">
-        <v>153.85</v>
+        <v>100</v>
       </c>
       <c r="I6" t="n">
-        <v>164.42</v>
+        <v>181.19</v>
       </c>
     </row>
     <row r="7">
@@ -1564,22 +1576,22 @@
         <v>111</v>
       </c>
       <c r="D7" t="n">
-        <v>339</v>
+        <v>287</v>
       </c>
       <c r="E7" t="n">
-        <v>170</v>
+        <v>83</v>
       </c>
       <c r="F7" t="n">
-        <v>166</v>
+        <v>201</v>
       </c>
       <c r="G7" t="n">
-        <v>305.41</v>
+        <v>258.56</v>
       </c>
       <c r="H7" t="n">
-        <v>153.15</v>
+        <v>74.77</v>
       </c>
       <c r="I7" t="n">
-        <v>149.55</v>
+        <v>181.08</v>
       </c>
     </row>
     <row r="8">
@@ -1595,22 +1607,22 @@
         <v>120</v>
       </c>
       <c r="D8" t="n">
-        <v>336</v>
+        <v>274</v>
       </c>
       <c r="E8" t="n">
-        <v>173</v>
+        <v>76</v>
       </c>
       <c r="F8" t="n">
-        <v>161</v>
+        <v>196</v>
       </c>
       <c r="G8" t="n">
-        <v>280</v>
+        <v>228.33</v>
       </c>
       <c r="H8" t="n">
-        <v>144.17</v>
+        <v>63.33</v>
       </c>
       <c r="I8" t="n">
-        <v>134.17</v>
+        <v>163.33</v>
       </c>
     </row>
     <row r="9">
@@ -1902,25 +1914,25 @@
         <v>373684</v>
       </c>
       <c r="C18" t="n">
-        <v>196</v>
+        <v>200</v>
       </c>
       <c r="D18" t="n">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="E18" t="n">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="F18" t="n">
         <v>28</v>
       </c>
       <c r="G18" t="n">
-        <v>66.84</v>
+        <v>67</v>
       </c>
       <c r="H18" t="n">
-        <v>52.55</v>
+        <v>53</v>
       </c>
       <c r="I18" t="n">
-        <v>14.29</v>
+        <v>14</v>
       </c>
     </row>
     <row r="19">
@@ -3352,7 +3364,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Shafaq.zahra</t>
+          <t>Shafaq Zahra</t>
         </is>
       </c>
       <c r="B65" t="inlineStr"/>

</xml_diff>

<commit_message>
Refactor error handling and reporting logic
- Removed anomaly error handling from error-loader and error-metrics, normalizing all relevant severity levels to "CRITICAL".
- Updated error metrics computation to exclude anomaly errors, focusing on critical and flag errors only.
- Adjusted error report generation to reflect changes in severity categorization, removing references to "ANOMALY".
- Cleaned up unused imports and functions related to anomaly error processing.
</commit_message>
<xml_diff>
--- a/Error_log/Enumerator_Performance.xlsx
+++ b/Error_log/Enumerator_Performance.xlsx
@@ -464,10 +464,10 @@
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="n">
-        <v>2459</v>
+        <v>2443</v>
       </c>
       <c r="D2" t="n">
-        <v>2457</v>
+        <v>2441</v>
       </c>
       <c r="E2" t="n">
         <v>2</v>
@@ -495,77 +495,77 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Shazia begum</t>
+          <t>Asma Bibi</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>373696</v>
+        <v>373641</v>
       </c>
       <c r="C4" t="n">
-        <v>139</v>
+        <v>152</v>
       </c>
       <c r="D4" t="n">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="E4" t="n">
-        <v>17</v>
+        <v>29</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Shazia Bibi</t>
+          <t>Shazia begum</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>373648</v>
+        <v>373696</v>
       </c>
       <c r="C5" t="n">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D5" t="n">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="E5" t="n">
-        <v>23</v>
+        <v>17</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Asma Bibi</t>
+          <t>Shazia Bibi</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>373641</v>
+        <v>373648</v>
       </c>
       <c r="C6" t="n">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="D6" t="n">
-        <v>112</v>
+        <v>119</v>
       </c>
       <c r="E6" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Mehran Khan</t>
+          <t>Kainat</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>373684</v>
+        <v>373712</v>
       </c>
       <c r="C7" t="n">
-        <v>134</v>
+        <v>307</v>
       </c>
       <c r="D7" t="n">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="E7" t="n">
-        <v>28</v>
+        <v>199</v>
       </c>
     </row>
     <row r="8">
@@ -578,51 +578,51 @@
         <v>373642</v>
       </c>
       <c r="C8" t="n">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="D8" t="n">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="E8" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Kainat</t>
+          <t>Zohra</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>373712</v>
+        <v>373692</v>
       </c>
       <c r="C9" t="n">
-        <v>303</v>
+        <v>289</v>
       </c>
       <c r="D9" t="n">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="E9" t="n">
-        <v>199</v>
+        <v>183</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Zohra</t>
+          <t>Mehran Khan</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>373692</v>
+        <v>373684</v>
       </c>
       <c r="C10" t="n">
-        <v>288</v>
+        <v>134</v>
       </c>
       <c r="D10" t="n">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="E10" t="n">
-        <v>183</v>
+        <v>28</v>
       </c>
     </row>
     <row r="11">
@@ -657,7 +657,7 @@
         <v>287</v>
       </c>
       <c r="D12" t="n">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="E12" t="n">
         <v>201</v>
@@ -673,10 +673,10 @@
         <v>373658</v>
       </c>
       <c r="C13" t="n">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="D13" t="n">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="E13" t="n">
         <v>196</v>
@@ -799,36 +799,36 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Bushra Ayub</t>
+          <t>Mahnoor</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>373671</v>
+        <v>373705</v>
       </c>
       <c r="C20" t="n">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="D20" t="n">
         <v>51</v>
       </c>
       <c r="E20" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Mahnoor</t>
+          <t>Bushra Ayub</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>373705</v>
+        <v>373671</v>
       </c>
       <c r="C21" t="n">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="D21" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="E21" t="n">
         <v>4</v>
@@ -1514,19 +1514,19 @@
         <v>104</v>
       </c>
       <c r="D5" t="n">
-        <v>303</v>
+        <v>307</v>
       </c>
       <c r="E5" t="n">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="F5" t="n">
         <v>199</v>
       </c>
       <c r="G5" t="n">
-        <v>291.35</v>
+        <v>295.19</v>
       </c>
       <c r="H5" t="n">
-        <v>100</v>
+        <v>103.85</v>
       </c>
       <c r="I5" t="n">
         <v>191.35</v>
@@ -1545,19 +1545,19 @@
         <v>101</v>
       </c>
       <c r="D6" t="n">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="E6" t="n">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="F6" t="n">
         <v>183</v>
       </c>
       <c r="G6" t="n">
-        <v>285.15</v>
+        <v>286.14</v>
       </c>
       <c r="H6" t="n">
-        <v>100</v>
+        <v>104.95</v>
       </c>
       <c r="I6" t="n">
         <v>181.19</v>
@@ -1579,7 +1579,7 @@
         <v>287</v>
       </c>
       <c r="E7" t="n">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="F7" t="n">
         <v>201</v>
@@ -1588,7 +1588,7 @@
         <v>258.56</v>
       </c>
       <c r="H7" t="n">
-        <v>74.77</v>
+        <v>77.48</v>
       </c>
       <c r="I7" t="n">
         <v>181.08</v>
@@ -1607,19 +1607,19 @@
         <v>120</v>
       </c>
       <c r="D8" t="n">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="E8" t="n">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="F8" t="n">
         <v>196</v>
       </c>
       <c r="G8" t="n">
-        <v>228.33</v>
+        <v>229.17</v>
       </c>
       <c r="H8" t="n">
-        <v>63.33</v>
+        <v>65.83</v>
       </c>
       <c r="I8" t="n">
         <v>163.33</v>
@@ -1721,63 +1721,63 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Shazia begum</t>
+          <t>Asma Bibi</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>373696</v>
+        <v>373641</v>
       </c>
       <c r="C12" t="n">
-        <v>179</v>
+        <v>193</v>
       </c>
       <c r="D12" t="n">
-        <v>139</v>
+        <v>152</v>
       </c>
       <c r="E12" t="n">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="F12" t="n">
-        <v>17</v>
+        <v>29</v>
       </c>
       <c r="G12" t="n">
-        <v>77.65000000000001</v>
+        <v>78.76000000000001</v>
       </c>
       <c r="H12" t="n">
-        <v>68.16</v>
+        <v>63.73</v>
       </c>
       <c r="I12" t="n">
-        <v>9.5</v>
+        <v>15.03</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Shazia Bibi</t>
+          <t>Shazia begum</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>373648</v>
+        <v>373696</v>
       </c>
       <c r="C13" t="n">
-        <v>189</v>
+        <v>179</v>
       </c>
       <c r="D13" t="n">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="E13" t="n">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="F13" t="n">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G13" t="n">
-        <v>74.06999999999999</v>
+        <v>77.65000000000001</v>
       </c>
       <c r="H13" t="n">
-        <v>61.9</v>
+        <v>68.16</v>
       </c>
       <c r="I13" t="n">
-        <v>12.17</v>
+        <v>9.5</v>
       </c>
     </row>
     <row r="14">
@@ -1790,87 +1790,87 @@
         <v>373642</v>
       </c>
       <c r="C14" t="n">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="D14" t="n">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="E14" t="n">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="F14" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="G14" t="n">
-        <v>72.67</v>
+        <v>75.66</v>
       </c>
       <c r="H14" t="n">
-        <v>70</v>
+        <v>71.05</v>
       </c>
       <c r="I14" t="n">
-        <v>2.67</v>
+        <v>4.61</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Shafaq Zahra</t>
+          <t>Shazia Bibi</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>373646</v>
+        <v>373648</v>
       </c>
       <c r="C15" t="n">
-        <v>207</v>
+        <v>191</v>
       </c>
       <c r="D15" t="n">
-        <v>149</v>
+        <v>143</v>
       </c>
       <c r="E15" t="n">
-        <v>133</v>
+        <v>119</v>
       </c>
       <c r="F15" t="n">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="G15" t="n">
-        <v>71.98</v>
+        <v>74.87</v>
       </c>
       <c r="H15" t="n">
-        <v>64.25</v>
+        <v>62.3</v>
       </c>
       <c r="I15" t="n">
-        <v>7.73</v>
+        <v>12.57</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Asma Bibi</t>
+          <t>Shafaq Zahra</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>373641</v>
+        <v>373646</v>
       </c>
       <c r="C16" t="n">
-        <v>187</v>
+        <v>207</v>
       </c>
       <c r="D16" t="n">
-        <v>134</v>
+        <v>149</v>
       </c>
       <c r="E16" t="n">
-        <v>112</v>
+        <v>133</v>
       </c>
       <c r="F16" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="G16" t="n">
-        <v>71.66</v>
+        <v>71.98</v>
       </c>
       <c r="H16" t="n">
-        <v>59.89</v>
+        <v>64.25</v>
       </c>
       <c r="I16" t="n">
-        <v>11.76</v>
+        <v>7.73</v>
       </c>
     </row>
     <row r="17">
@@ -1969,94 +1969,94 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Javairia</t>
+          <t>Mahnoor</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>373651</v>
+        <v>373705</v>
       </c>
       <c r="C20" t="n">
-        <v>120</v>
+        <v>96</v>
       </c>
       <c r="D20" t="n">
-        <v>73</v>
+        <v>61</v>
       </c>
       <c r="E20" t="n">
-        <v>60</v>
+        <v>51</v>
       </c>
       <c r="F20" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="G20" t="n">
-        <v>60.83</v>
+        <v>63.54</v>
       </c>
       <c r="H20" t="n">
-        <v>50</v>
+        <v>53.12</v>
       </c>
       <c r="I20" t="n">
-        <v>10.83</v>
+        <v>10.42</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Naureen</t>
+          <t>Javairia</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>884887</v>
+        <v>373651</v>
       </c>
       <c r="C21" t="n">
+        <v>120</v>
+      </c>
+      <c r="D21" t="n">
+        <v>73</v>
+      </c>
+      <c r="E21" t="n">
         <v>60</v>
       </c>
-      <c r="D21" t="n">
-        <v>35</v>
-      </c>
-      <c r="E21" t="n">
-        <v>31</v>
-      </c>
       <c r="F21" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="G21" t="n">
-        <v>58.33</v>
+        <v>60.83</v>
       </c>
       <c r="H21" t="n">
-        <v>51.67</v>
+        <v>50</v>
       </c>
       <c r="I21" t="n">
-        <v>6.67</v>
+        <v>10.83</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Mahnoor</t>
+          <t>Naureen</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>373705</v>
+        <v>884887</v>
       </c>
       <c r="C22" t="n">
-        <v>94</v>
+        <v>60</v>
       </c>
       <c r="D22" t="n">
-        <v>53</v>
+        <v>35</v>
       </c>
       <c r="E22" t="n">
-        <v>49</v>
+        <v>31</v>
       </c>
       <c r="F22" t="n">
         <v>4</v>
       </c>
       <c r="G22" t="n">
-        <v>56.38</v>
+        <v>58.33</v>
       </c>
       <c r="H22" t="n">
-        <v>52.13</v>
+        <v>51.67</v>
       </c>
       <c r="I22" t="n">
-        <v>4.26</v>
+        <v>6.67</v>
       </c>
     </row>
     <row r="23">

</xml_diff>

<commit_message>
chore: update error log and performance summary files
</commit_message>
<xml_diff>
--- a/Error_log/Enumerator_Performance.xlsx
+++ b/Error_log/Enumerator_Performance.xlsx
@@ -1,13 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="performance" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="performance" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="performance_pct" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,13 +18,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +38,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +46,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -417,27 +430,27 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Enumerator Name</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Enumerator ID</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Total Issues</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Critical Issues</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Flag Issues</t>
         </is>
@@ -1332,6 +1345,2173 @@
       </c>
       <c r="E48" t="n">
         <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I69"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>enumerator_name</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>enumerator_id</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>total_submissions</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>total_issues</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>critical_issues</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>flag_issues</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>error_pct</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>critical_error_pct</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>flag_error_pct</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Naureen khan</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>453925</v>
+      </c>
+      <c r="C2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D2" t="n">
+        <v>52</v>
+      </c>
+      <c r="E2" t="n">
+        <v>50</v>
+      </c>
+      <c r="F2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G2" t="n">
+        <v>2600</v>
+      </c>
+      <c r="H2" t="n">
+        <v>2500</v>
+      </c>
+      <c r="I2" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Lati Khan</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>564273</v>
+      </c>
+      <c r="C3" t="n">
+        <v>9</v>
+      </c>
+      <c r="D3" t="n">
+        <v>45</v>
+      </c>
+      <c r="E3" t="n">
+        <v>41</v>
+      </c>
+      <c r="F3" t="n">
+        <v>4</v>
+      </c>
+      <c r="G3" t="n">
+        <v>500</v>
+      </c>
+      <c r="H3" t="n">
+        <v>455.56</v>
+      </c>
+      <c r="I3" t="n">
+        <v>44.44</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Irum ikram</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>541376</v>
+      </c>
+      <c r="C4" t="n">
+        <v>8</v>
+      </c>
+      <c r="D4" t="n">
+        <v>36</v>
+      </c>
+      <c r="E4" t="n">
+        <v>31</v>
+      </c>
+      <c r="F4" t="n">
+        <v>5</v>
+      </c>
+      <c r="G4" t="n">
+        <v>450</v>
+      </c>
+      <c r="H4" t="n">
+        <v>387.5</v>
+      </c>
+      <c r="I4" t="n">
+        <v>62.5</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Kainat</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>373712</v>
+      </c>
+      <c r="C5" t="n">
+        <v>104</v>
+      </c>
+      <c r="D5" t="n">
+        <v>309</v>
+      </c>
+      <c r="E5" t="n">
+        <v>110</v>
+      </c>
+      <c r="F5" t="n">
+        <v>199</v>
+      </c>
+      <c r="G5" t="n">
+        <v>297.12</v>
+      </c>
+      <c r="H5" t="n">
+        <v>105.77</v>
+      </c>
+      <c r="I5" t="n">
+        <v>191.35</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Zohra</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>373692</v>
+      </c>
+      <c r="C6" t="n">
+        <v>101</v>
+      </c>
+      <c r="D6" t="n">
+        <v>289</v>
+      </c>
+      <c r="E6" t="n">
+        <v>106</v>
+      </c>
+      <c r="F6" t="n">
+        <v>183</v>
+      </c>
+      <c r="G6" t="n">
+        <v>286.14</v>
+      </c>
+      <c r="H6" t="n">
+        <v>104.95</v>
+      </c>
+      <c r="I6" t="n">
+        <v>181.19</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Rehana Bibi</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>373691</v>
+      </c>
+      <c r="C7" t="n">
+        <v>111</v>
+      </c>
+      <c r="D7" t="n">
+        <v>287</v>
+      </c>
+      <c r="E7" t="n">
+        <v>86</v>
+      </c>
+      <c r="F7" t="n">
+        <v>201</v>
+      </c>
+      <c r="G7" t="n">
+        <v>258.56</v>
+      </c>
+      <c r="H7" t="n">
+        <v>77.48</v>
+      </c>
+      <c r="I7" t="n">
+        <v>181.08</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Samara</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>373658</v>
+      </c>
+      <c r="C8" t="n">
+        <v>120</v>
+      </c>
+      <c r="D8" t="n">
+        <v>275</v>
+      </c>
+      <c r="E8" t="n">
+        <v>79</v>
+      </c>
+      <c r="F8" t="n">
+        <v>196</v>
+      </c>
+      <c r="G8" t="n">
+        <v>229.17</v>
+      </c>
+      <c r="H8" t="n">
+        <v>65.83</v>
+      </c>
+      <c r="I8" t="n">
+        <v>163.33</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Lati khan</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>671211</v>
+      </c>
+      <c r="C9" t="n">
+        <v>9</v>
+      </c>
+      <c r="D9" t="n">
+        <v>19</v>
+      </c>
+      <c r="E9" t="n">
+        <v>19</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" t="n">
+        <v>211.11</v>
+      </c>
+      <c r="H9" t="n">
+        <v>211.11</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Asma Bibi</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>373641</v>
+      </c>
+      <c r="C10" t="n">
+        <v>194</v>
+      </c>
+      <c r="D10" t="n">
+        <v>162</v>
+      </c>
+      <c r="E10" t="n">
+        <v>128</v>
+      </c>
+      <c r="F10" t="n">
+        <v>34</v>
+      </c>
+      <c r="G10" t="n">
+        <v>83.51000000000001</v>
+      </c>
+      <c r="H10" t="n">
+        <v>65.98</v>
+      </c>
+      <c r="I10" t="n">
+        <v>17.53</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Naureen Khan</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>373716</v>
+      </c>
+      <c r="C11" t="n">
+        <v>70</v>
+      </c>
+      <c r="D11" t="n">
+        <v>58</v>
+      </c>
+      <c r="E11" t="n">
+        <v>58</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" t="n">
+        <v>82.86</v>
+      </c>
+      <c r="H11" t="n">
+        <v>82.86</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Jaweria</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>163495</v>
+      </c>
+      <c r="C12" t="n">
+        <v>68</v>
+      </c>
+      <c r="D12" t="n">
+        <v>56</v>
+      </c>
+      <c r="E12" t="n">
+        <v>55</v>
+      </c>
+      <c r="F12" t="n">
+        <v>1</v>
+      </c>
+      <c r="G12" t="n">
+        <v>82.34999999999999</v>
+      </c>
+      <c r="H12" t="n">
+        <v>80.88</v>
+      </c>
+      <c r="I12" t="n">
+        <v>1.47</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Shazia begum</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>373696</v>
+      </c>
+      <c r="C13" t="n">
+        <v>179</v>
+      </c>
+      <c r="D13" t="n">
+        <v>139</v>
+      </c>
+      <c r="E13" t="n">
+        <v>122</v>
+      </c>
+      <c r="F13" t="n">
+        <v>17</v>
+      </c>
+      <c r="G13" t="n">
+        <v>77.65000000000001</v>
+      </c>
+      <c r="H13" t="n">
+        <v>68.16</v>
+      </c>
+      <c r="I13" t="n">
+        <v>9.5</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Irum Ikram</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>373642</v>
+      </c>
+      <c r="C14" t="n">
+        <v>152</v>
+      </c>
+      <c r="D14" t="n">
+        <v>115</v>
+      </c>
+      <c r="E14" t="n">
+        <v>108</v>
+      </c>
+      <c r="F14" t="n">
+        <v>7</v>
+      </c>
+      <c r="G14" t="n">
+        <v>75.66</v>
+      </c>
+      <c r="H14" t="n">
+        <v>71.05</v>
+      </c>
+      <c r="I14" t="n">
+        <v>4.61</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Shazia Bibi</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>373648</v>
+      </c>
+      <c r="C15" t="n">
+        <v>191</v>
+      </c>
+      <c r="D15" t="n">
+        <v>143</v>
+      </c>
+      <c r="E15" t="n">
+        <v>119</v>
+      </c>
+      <c r="F15" t="n">
+        <v>24</v>
+      </c>
+      <c r="G15" t="n">
+        <v>74.87</v>
+      </c>
+      <c r="H15" t="n">
+        <v>62.3</v>
+      </c>
+      <c r="I15" t="n">
+        <v>12.57</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Shafaq Zahra</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>373646</v>
+      </c>
+      <c r="C16" t="n">
+        <v>207</v>
+      </c>
+      <c r="D16" t="n">
+        <v>149</v>
+      </c>
+      <c r="E16" t="n">
+        <v>133</v>
+      </c>
+      <c r="F16" t="n">
+        <v>16</v>
+      </c>
+      <c r="G16" t="n">
+        <v>71.98</v>
+      </c>
+      <c r="H16" t="n">
+        <v>64.25</v>
+      </c>
+      <c r="I16" t="n">
+        <v>7.73</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Sadia Rustum</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>373649</v>
+      </c>
+      <c r="C17" t="n">
+        <v>152</v>
+      </c>
+      <c r="D17" t="n">
+        <v>106</v>
+      </c>
+      <c r="E17" t="n">
+        <v>96</v>
+      </c>
+      <c r="F17" t="n">
+        <v>10</v>
+      </c>
+      <c r="G17" t="n">
+        <v>69.73999999999999</v>
+      </c>
+      <c r="H17" t="n">
+        <v>63.16</v>
+      </c>
+      <c r="I17" t="n">
+        <v>6.58</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Mehran Khan</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>373684</v>
+      </c>
+      <c r="C18" t="n">
+        <v>200</v>
+      </c>
+      <c r="D18" t="n">
+        <v>134</v>
+      </c>
+      <c r="E18" t="n">
+        <v>106</v>
+      </c>
+      <c r="F18" t="n">
+        <v>28</v>
+      </c>
+      <c r="G18" t="n">
+        <v>67</v>
+      </c>
+      <c r="H18" t="n">
+        <v>53</v>
+      </c>
+      <c r="I18" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Lati Khan</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>373665</v>
+      </c>
+      <c r="C19" t="n">
+        <v>60</v>
+      </c>
+      <c r="D19" t="n">
+        <v>40</v>
+      </c>
+      <c r="E19" t="n">
+        <v>37</v>
+      </c>
+      <c r="F19" t="n">
+        <v>3</v>
+      </c>
+      <c r="G19" t="n">
+        <v>66.67</v>
+      </c>
+      <c r="H19" t="n">
+        <v>61.67</v>
+      </c>
+      <c r="I19" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Mahnoor</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>373705</v>
+      </c>
+      <c r="C20" t="n">
+        <v>96</v>
+      </c>
+      <c r="D20" t="n">
+        <v>61</v>
+      </c>
+      <c r="E20" t="n">
+        <v>51</v>
+      </c>
+      <c r="F20" t="n">
+        <v>10</v>
+      </c>
+      <c r="G20" t="n">
+        <v>63.54</v>
+      </c>
+      <c r="H20" t="n">
+        <v>53.12</v>
+      </c>
+      <c r="I20" t="n">
+        <v>10.42</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Javairia</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>373651</v>
+      </c>
+      <c r="C21" t="n">
+        <v>120</v>
+      </c>
+      <c r="D21" t="n">
+        <v>73</v>
+      </c>
+      <c r="E21" t="n">
+        <v>60</v>
+      </c>
+      <c r="F21" t="n">
+        <v>13</v>
+      </c>
+      <c r="G21" t="n">
+        <v>60.83</v>
+      </c>
+      <c r="H21" t="n">
+        <v>50</v>
+      </c>
+      <c r="I21" t="n">
+        <v>10.83</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Naureen</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>884887</v>
+      </c>
+      <c r="C22" t="n">
+        <v>60</v>
+      </c>
+      <c r="D22" t="n">
+        <v>35</v>
+      </c>
+      <c r="E22" t="n">
+        <v>31</v>
+      </c>
+      <c r="F22" t="n">
+        <v>4</v>
+      </c>
+      <c r="G22" t="n">
+        <v>58.33</v>
+      </c>
+      <c r="H22" t="n">
+        <v>51.67</v>
+      </c>
+      <c r="I22" t="n">
+        <v>6.67</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Muhammad Yousaf</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>373690</v>
+      </c>
+      <c r="C23" t="n">
+        <v>132</v>
+      </c>
+      <c r="D23" t="n">
+        <v>71</v>
+      </c>
+      <c r="E23" t="n">
+        <v>62</v>
+      </c>
+      <c r="F23" t="n">
+        <v>9</v>
+      </c>
+      <c r="G23" t="n">
+        <v>53.79</v>
+      </c>
+      <c r="H23" t="n">
+        <v>46.97</v>
+      </c>
+      <c r="I23" t="n">
+        <v>6.82</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Summiya Hayat</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>373710</v>
+      </c>
+      <c r="C24" t="n">
+        <v>81</v>
+      </c>
+      <c r="D24" t="n">
+        <v>40</v>
+      </c>
+      <c r="E24" t="n">
+        <v>27</v>
+      </c>
+      <c r="F24" t="n">
+        <v>13</v>
+      </c>
+      <c r="G24" t="n">
+        <v>49.38</v>
+      </c>
+      <c r="H24" t="n">
+        <v>33.33</v>
+      </c>
+      <c r="I24" t="n">
+        <v>16.05</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Muniba Shamim</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>373659</v>
+      </c>
+      <c r="C25" t="n">
+        <v>72</v>
+      </c>
+      <c r="D25" t="n">
+        <v>32</v>
+      </c>
+      <c r="E25" t="n">
+        <v>23</v>
+      </c>
+      <c r="F25" t="n">
+        <v>9</v>
+      </c>
+      <c r="G25" t="n">
+        <v>44.44</v>
+      </c>
+      <c r="H25" t="n">
+        <v>31.94</v>
+      </c>
+      <c r="I25" t="n">
+        <v>12.5</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Laiba Shams</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>373706</v>
+      </c>
+      <c r="C26" t="n">
+        <v>93</v>
+      </c>
+      <c r="D26" t="n">
+        <v>41</v>
+      </c>
+      <c r="E26" t="n">
+        <v>35</v>
+      </c>
+      <c r="F26" t="n">
+        <v>6</v>
+      </c>
+      <c r="G26" t="n">
+        <v>44.09</v>
+      </c>
+      <c r="H26" t="n">
+        <v>37.63</v>
+      </c>
+      <c r="I26" t="n">
+        <v>6.45</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Bushra Ayub</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>373671</v>
+      </c>
+      <c r="C27" t="n">
+        <v>138</v>
+      </c>
+      <c r="D27" t="n">
+        <v>55</v>
+      </c>
+      <c r="E27" t="n">
+        <v>51</v>
+      </c>
+      <c r="F27" t="n">
+        <v>4</v>
+      </c>
+      <c r="G27" t="n">
+        <v>39.86</v>
+      </c>
+      <c r="H27" t="n">
+        <v>36.96</v>
+      </c>
+      <c r="I27" t="n">
+        <v>2.9</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Furqan Ullah Khan</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>373683</v>
+      </c>
+      <c r="C28" t="n">
+        <v>195</v>
+      </c>
+      <c r="D28" t="n">
+        <v>76</v>
+      </c>
+      <c r="E28" t="n">
+        <v>68</v>
+      </c>
+      <c r="F28" t="n">
+        <v>8</v>
+      </c>
+      <c r="G28" t="n">
+        <v>38.97</v>
+      </c>
+      <c r="H28" t="n">
+        <v>34.87</v>
+      </c>
+      <c r="I28" t="n">
+        <v>4.1</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Munawar Khan</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>373668</v>
+      </c>
+      <c r="C29" t="n">
+        <v>73</v>
+      </c>
+      <c r="D29" t="n">
+        <v>26</v>
+      </c>
+      <c r="E29" t="n">
+        <v>20</v>
+      </c>
+      <c r="F29" t="n">
+        <v>6</v>
+      </c>
+      <c r="G29" t="n">
+        <v>35.62</v>
+      </c>
+      <c r="H29" t="n">
+        <v>27.4</v>
+      </c>
+      <c r="I29" t="n">
+        <v>8.220000000000001</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Khalida Bibi</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>373673</v>
+      </c>
+      <c r="C30" t="n">
+        <v>177</v>
+      </c>
+      <c r="D30" t="n">
+        <v>63</v>
+      </c>
+      <c r="E30" t="n">
+        <v>63</v>
+      </c>
+      <c r="F30" t="n">
+        <v>0</v>
+      </c>
+      <c r="G30" t="n">
+        <v>35.59</v>
+      </c>
+      <c r="H30" t="n">
+        <v>35.59</v>
+      </c>
+      <c r="I30" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Asma Gull</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>373672</v>
+      </c>
+      <c r="C31" t="n">
+        <v>144</v>
+      </c>
+      <c r="D31" t="n">
+        <v>51</v>
+      </c>
+      <c r="E31" t="n">
+        <v>47</v>
+      </c>
+      <c r="F31" t="n">
+        <v>4</v>
+      </c>
+      <c r="G31" t="n">
+        <v>35.42</v>
+      </c>
+      <c r="H31" t="n">
+        <v>32.64</v>
+      </c>
+      <c r="I31" t="n">
+        <v>2.78</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Muhammad Shahid Khan</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>373662</v>
+      </c>
+      <c r="C32" t="n">
+        <v>6</v>
+      </c>
+      <c r="D32" t="n">
+        <v>2</v>
+      </c>
+      <c r="E32" t="n">
+        <v>2</v>
+      </c>
+      <c r="F32" t="n">
+        <v>0</v>
+      </c>
+      <c r="G32" t="n">
+        <v>33.33</v>
+      </c>
+      <c r="H32" t="n">
+        <v>33.33</v>
+      </c>
+      <c r="I32" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Chashm Gul</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>373695</v>
+      </c>
+      <c r="C33" t="n">
+        <v>31</v>
+      </c>
+      <c r="D33" t="n">
+        <v>9</v>
+      </c>
+      <c r="E33" t="n">
+        <v>0</v>
+      </c>
+      <c r="F33" t="n">
+        <v>9</v>
+      </c>
+      <c r="G33" t="n">
+        <v>29.03</v>
+      </c>
+      <c r="H33" t="n">
+        <v>0</v>
+      </c>
+      <c r="I33" t="n">
+        <v>29.03</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Rahila Naaz</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>373715</v>
+      </c>
+      <c r="C34" t="n">
+        <v>4</v>
+      </c>
+      <c r="D34" t="n">
+        <v>1</v>
+      </c>
+      <c r="E34" t="n">
+        <v>0</v>
+      </c>
+      <c r="F34" t="n">
+        <v>1</v>
+      </c>
+      <c r="G34" t="n">
+        <v>25</v>
+      </c>
+      <c r="H34" t="n">
+        <v>0</v>
+      </c>
+      <c r="I34" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Zain Ul Abideen</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>373667</v>
+      </c>
+      <c r="C35" t="n">
+        <v>13</v>
+      </c>
+      <c r="D35" t="n">
+        <v>3</v>
+      </c>
+      <c r="E35" t="n">
+        <v>3</v>
+      </c>
+      <c r="F35" t="n">
+        <v>0</v>
+      </c>
+      <c r="G35" t="n">
+        <v>23.08</v>
+      </c>
+      <c r="H35" t="n">
+        <v>23.08</v>
+      </c>
+      <c r="I35" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Shehla Noor</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>373650</v>
+      </c>
+      <c r="C36" t="n">
+        <v>14</v>
+      </c>
+      <c r="D36" t="n">
+        <v>3</v>
+      </c>
+      <c r="E36" t="n">
+        <v>3</v>
+      </c>
+      <c r="F36" t="n">
+        <v>0</v>
+      </c>
+      <c r="G36" t="n">
+        <v>21.43</v>
+      </c>
+      <c r="H36" t="n">
+        <v>21.43</v>
+      </c>
+      <c r="I36" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Anum Gul</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>373656</v>
+      </c>
+      <c r="C37" t="n">
+        <v>103</v>
+      </c>
+      <c r="D37" t="n">
+        <v>18</v>
+      </c>
+      <c r="E37" t="n">
+        <v>14</v>
+      </c>
+      <c r="F37" t="n">
+        <v>4</v>
+      </c>
+      <c r="G37" t="n">
+        <v>17.48</v>
+      </c>
+      <c r="H37" t="n">
+        <v>13.59</v>
+      </c>
+      <c r="I37" t="n">
+        <v>3.88</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Muhammad Noor</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>373701</v>
+      </c>
+      <c r="C38" t="n">
+        <v>8</v>
+      </c>
+      <c r="D38" t="n">
+        <v>1</v>
+      </c>
+      <c r="E38" t="n">
+        <v>0</v>
+      </c>
+      <c r="F38" t="n">
+        <v>1</v>
+      </c>
+      <c r="G38" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="H38" t="n">
+        <v>0</v>
+      </c>
+      <c r="I38" t="n">
+        <v>12.5</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Robina Shaheen</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>373639</v>
+      </c>
+      <c r="C39" t="n">
+        <v>8</v>
+      </c>
+      <c r="D39" t="n">
+        <v>1</v>
+      </c>
+      <c r="E39" t="n">
+        <v>0</v>
+      </c>
+      <c r="F39" t="n">
+        <v>1</v>
+      </c>
+      <c r="G39" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="H39" t="n">
+        <v>0</v>
+      </c>
+      <c r="I39" t="n">
+        <v>12.5</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Alia Khan</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>373681</v>
+      </c>
+      <c r="C40" t="n">
+        <v>129</v>
+      </c>
+      <c r="D40" t="n">
+        <v>13</v>
+      </c>
+      <c r="E40" t="n">
+        <v>9</v>
+      </c>
+      <c r="F40" t="n">
+        <v>4</v>
+      </c>
+      <c r="G40" t="n">
+        <v>10.08</v>
+      </c>
+      <c r="H40" t="n">
+        <v>6.98</v>
+      </c>
+      <c r="I40" t="n">
+        <v>3.1</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Aisha Aman</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>373704</v>
+      </c>
+      <c r="C41" t="n">
+        <v>11</v>
+      </c>
+      <c r="D41" t="n">
+        <v>1</v>
+      </c>
+      <c r="E41" t="n">
+        <v>0</v>
+      </c>
+      <c r="F41" t="n">
+        <v>1</v>
+      </c>
+      <c r="G41" t="n">
+        <v>9.09</v>
+      </c>
+      <c r="H41" t="n">
+        <v>0</v>
+      </c>
+      <c r="I41" t="n">
+        <v>9.09</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Mahnoorr</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>373670</v>
+      </c>
+      <c r="C42" t="n">
+        <v>13</v>
+      </c>
+      <c r="D42" t="n">
+        <v>1</v>
+      </c>
+      <c r="E42" t="n">
+        <v>0</v>
+      </c>
+      <c r="F42" t="n">
+        <v>1</v>
+      </c>
+      <c r="G42" t="n">
+        <v>7.69</v>
+      </c>
+      <c r="H42" t="n">
+        <v>0</v>
+      </c>
+      <c r="I42" t="n">
+        <v>7.69</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Laiba Khan</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>373653</v>
+      </c>
+      <c r="C43" t="n">
+        <v>121</v>
+      </c>
+      <c r="D43" t="n">
+        <v>8</v>
+      </c>
+      <c r="E43" t="n">
+        <v>4</v>
+      </c>
+      <c r="F43" t="n">
+        <v>4</v>
+      </c>
+      <c r="G43" t="n">
+        <v>6.61</v>
+      </c>
+      <c r="H43" t="n">
+        <v>3.31</v>
+      </c>
+      <c r="I43" t="n">
+        <v>3.31</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Nillum Bibi</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>373652</v>
+      </c>
+      <c r="C44" t="n">
+        <v>169</v>
+      </c>
+      <c r="D44" t="n">
+        <v>10</v>
+      </c>
+      <c r="E44" t="n">
+        <v>7</v>
+      </c>
+      <c r="F44" t="n">
+        <v>3</v>
+      </c>
+      <c r="G44" t="n">
+        <v>5.92</v>
+      </c>
+      <c r="H44" t="n">
+        <v>4.14</v>
+      </c>
+      <c r="I44" t="n">
+        <v>1.78</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Nazia</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>373657</v>
+      </c>
+      <c r="C45" t="n">
+        <v>144</v>
+      </c>
+      <c r="D45" t="n">
+        <v>8</v>
+      </c>
+      <c r="E45" t="n">
+        <v>6</v>
+      </c>
+      <c r="F45" t="n">
+        <v>2</v>
+      </c>
+      <c r="G45" t="n">
+        <v>5.56</v>
+      </c>
+      <c r="H45" t="n">
+        <v>4.17</v>
+      </c>
+      <c r="I45" t="n">
+        <v>1.39</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Ishaq Khan</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>373699</v>
+      </c>
+      <c r="C46" t="n">
+        <v>170</v>
+      </c>
+      <c r="D46" t="n">
+        <v>6</v>
+      </c>
+      <c r="E46" t="n">
+        <v>5</v>
+      </c>
+      <c r="F46" t="n">
+        <v>1</v>
+      </c>
+      <c r="G46" t="n">
+        <v>3.53</v>
+      </c>
+      <c r="H46" t="n">
+        <v>2.94</v>
+      </c>
+      <c r="I46" t="n">
+        <v>0.59</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Gul Rukh</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>373644</v>
+      </c>
+      <c r="C47" t="n">
+        <v>6</v>
+      </c>
+      <c r="D47" t="n">
+        <v>0</v>
+      </c>
+      <c r="E47" t="n">
+        <v>0</v>
+      </c>
+      <c r="F47" t="n">
+        <v>0</v>
+      </c>
+      <c r="G47" t="n">
+        <v>0</v>
+      </c>
+      <c r="H47" t="n">
+        <v>0</v>
+      </c>
+      <c r="I47" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Hijab Zahra</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>373637</v>
+      </c>
+      <c r="C48" t="n">
+        <v>4</v>
+      </c>
+      <c r="D48" t="n">
+        <v>0</v>
+      </c>
+      <c r="E48" t="n">
+        <v>0</v>
+      </c>
+      <c r="F48" t="n">
+        <v>0</v>
+      </c>
+      <c r="G48" t="n">
+        <v>0</v>
+      </c>
+      <c r="H48" t="n">
+        <v>0</v>
+      </c>
+      <c r="I48" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Iqra Bibi</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>373708</v>
+      </c>
+      <c r="C49" t="n">
+        <v>8</v>
+      </c>
+      <c r="D49" t="n">
+        <v>0</v>
+      </c>
+      <c r="E49" t="n">
+        <v>0</v>
+      </c>
+      <c r="F49" t="n">
+        <v>0</v>
+      </c>
+      <c r="G49" t="n">
+        <v>0</v>
+      </c>
+      <c r="H49" t="n">
+        <v>0</v>
+      </c>
+      <c r="I49" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Irum ikram (duplicate name received from listed_girl_tracking_survey on June 29, 2026 12:08 UTC+00:00; submission key: uuid:b700a976-75ee-467c-87e9-1d5163ec238d)</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>541376</v>
+      </c>
+      <c r="C50" t="n">
+        <v>64</v>
+      </c>
+      <c r="D50" t="n">
+        <v>0</v>
+      </c>
+      <c r="E50" t="n">
+        <v>0</v>
+      </c>
+      <c r="F50" t="n">
+        <v>0</v>
+      </c>
+      <c r="G50" t="n">
+        <v>0</v>
+      </c>
+      <c r="H50" t="n">
+        <v>0</v>
+      </c>
+      <c r="I50" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Lati Khan (duplicate name received from listed_girl_tracking_survey on June 28, 2026 10:43 UTC+00:00; submission key: uuid:e4e89d53-e5be-40ff-bb2c-fa94c0d50011)</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>564273</v>
+      </c>
+      <c r="C51" t="n">
+        <v>56</v>
+      </c>
+      <c r="D51" t="n">
+        <v>0</v>
+      </c>
+      <c r="E51" t="n">
+        <v>0</v>
+      </c>
+      <c r="F51" t="n">
+        <v>0</v>
+      </c>
+      <c r="G51" t="n">
+        <v>0</v>
+      </c>
+      <c r="H51" t="n">
+        <v>0</v>
+      </c>
+      <c r="I51" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Lati khan</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>652938</v>
+      </c>
+      <c r="C52" t="n">
+        <v>11</v>
+      </c>
+      <c r="D52" t="n">
+        <v>0</v>
+      </c>
+      <c r="E52" t="n">
+        <v>0</v>
+      </c>
+      <c r="F52" t="n">
+        <v>0</v>
+      </c>
+      <c r="G52" t="n">
+        <v>0</v>
+      </c>
+      <c r="H52" t="n">
+        <v>0</v>
+      </c>
+      <c r="I52" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Lati khan (duplicate name received from listed_girl_tracking_survey_new_sample on July 4, 2026 14:31 UTC+00:00; submission key: uuid:6316d214-c458-4786-937a-bd81b08c15c5)</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>671211</v>
+      </c>
+      <c r="C53" t="n">
+        <v>14</v>
+      </c>
+      <c r="D53" t="n">
+        <v>0</v>
+      </c>
+      <c r="E53" t="n">
+        <v>0</v>
+      </c>
+      <c r="F53" t="n">
+        <v>0</v>
+      </c>
+      <c r="G53" t="n">
+        <v>0</v>
+      </c>
+      <c r="H53" t="n">
+        <v>0</v>
+      </c>
+      <c r="I53" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Muhammad Naeem</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>373694</v>
+      </c>
+      <c r="C54" t="n">
+        <v>6</v>
+      </c>
+      <c r="D54" t="n">
+        <v>0</v>
+      </c>
+      <c r="E54" t="n">
+        <v>0</v>
+      </c>
+      <c r="F54" t="n">
+        <v>0</v>
+      </c>
+      <c r="G54" t="n">
+        <v>0</v>
+      </c>
+      <c r="H54" t="n">
+        <v>0</v>
+      </c>
+      <c r="I54" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Muhammad Usman</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>373666</v>
+      </c>
+      <c r="C55" t="n">
+        <v>14</v>
+      </c>
+      <c r="D55" t="n">
+        <v>0</v>
+      </c>
+      <c r="E55" t="n">
+        <v>0</v>
+      </c>
+      <c r="F55" t="n">
+        <v>0</v>
+      </c>
+      <c r="G55" t="n">
+        <v>0</v>
+      </c>
+      <c r="H55" t="n">
+        <v>0</v>
+      </c>
+      <c r="I55" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Muhammad Waseem</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>373689</v>
+      </c>
+      <c r="C56" t="n">
+        <v>3</v>
+      </c>
+      <c r="D56" t="n">
+        <v>0</v>
+      </c>
+      <c r="E56" t="n">
+        <v>0</v>
+      </c>
+      <c r="F56" t="n">
+        <v>0</v>
+      </c>
+      <c r="G56" t="n">
+        <v>0</v>
+      </c>
+      <c r="H56" t="n">
+        <v>0</v>
+      </c>
+      <c r="I56" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Muhammad naeem (duplicate name received from primary_school_listing_survey on February 14, 2026 14:38 UTC+00:00; submission key: uuid:5f0e427e-5fd2-4474-be64-ae5f2c4617a2)</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>571571</v>
+      </c>
+      <c r="C57" t="n">
+        <v>8</v>
+      </c>
+      <c r="D57" t="n">
+        <v>0</v>
+      </c>
+      <c r="E57" t="n">
+        <v>0</v>
+      </c>
+      <c r="F57" t="n">
+        <v>0</v>
+      </c>
+      <c r="G57" t="n">
+        <v>0</v>
+      </c>
+      <c r="H57" t="n">
+        <v>0</v>
+      </c>
+      <c r="I57" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Nadia bibi</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>373669</v>
+      </c>
+      <c r="C58" t="n">
+        <v>10</v>
+      </c>
+      <c r="D58" t="n">
+        <v>0</v>
+      </c>
+      <c r="E58" t="n">
+        <v>0</v>
+      </c>
+      <c r="F58" t="n">
+        <v>0</v>
+      </c>
+      <c r="G58" t="n">
+        <v>0</v>
+      </c>
+      <c r="H58" t="n">
+        <v>0</v>
+      </c>
+      <c r="I58" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Naureen khan (duplicate name received from listed_girl_tracking_survey_new_sample on July 7, 2026 14:41 UTC+00:00; submission key: uuid:bbf56e1f-36f5-4ebf-9e0f-df83015a0871)</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>453925</v>
+      </c>
+      <c r="C59" t="n">
+        <v>57</v>
+      </c>
+      <c r="D59" t="n">
+        <v>0</v>
+      </c>
+      <c r="E59" t="n">
+        <v>0</v>
+      </c>
+      <c r="F59" t="n">
+        <v>0</v>
+      </c>
+      <c r="G59" t="n">
+        <v>0</v>
+      </c>
+      <c r="H59" t="n">
+        <v>0</v>
+      </c>
+      <c r="I59" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Saba Ramzan</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>373703</v>
+      </c>
+      <c r="C60" t="n">
+        <v>13</v>
+      </c>
+      <c r="D60" t="n">
+        <v>0</v>
+      </c>
+      <c r="E60" t="n">
+        <v>0</v>
+      </c>
+      <c r="F60" t="n">
+        <v>0</v>
+      </c>
+      <c r="G60" t="n">
+        <v>0</v>
+      </c>
+      <c r="H60" t="n">
+        <v>0</v>
+      </c>
+      <c r="I60" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Sadia rustum</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>852541</v>
+      </c>
+      <c r="C61" t="n">
+        <v>7</v>
+      </c>
+      <c r="D61" t="n">
+        <v>0</v>
+      </c>
+      <c r="E61" t="n">
+        <v>0</v>
+      </c>
+      <c r="F61" t="n">
+        <v>0</v>
+      </c>
+      <c r="G61" t="n">
+        <v>0</v>
+      </c>
+      <c r="H61" t="n">
+        <v>0</v>
+      </c>
+      <c r="I61" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Sajjad Khan</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
+        <v>373700</v>
+      </c>
+      <c r="C62" t="n">
+        <v>8</v>
+      </c>
+      <c r="D62" t="n">
+        <v>0</v>
+      </c>
+      <c r="E62" t="n">
+        <v>0</v>
+      </c>
+      <c r="F62" t="n">
+        <v>0</v>
+      </c>
+      <c r="G62" t="n">
+        <v>0</v>
+      </c>
+      <c r="H62" t="n">
+        <v>0</v>
+      </c>
+      <c r="I62" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Samreen</t>
+        </is>
+      </c>
+      <c r="B63" t="n">
+        <v>373711</v>
+      </c>
+      <c r="C63" t="n">
+        <v>3</v>
+      </c>
+      <c r="D63" t="n">
+        <v>0</v>
+      </c>
+      <c r="E63" t="n">
+        <v>0</v>
+      </c>
+      <c r="F63" t="n">
+        <v>0</v>
+      </c>
+      <c r="G63" t="n">
+        <v>0</v>
+      </c>
+      <c r="H63" t="n">
+        <v>0</v>
+      </c>
+      <c r="I63" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Samreen</t>
+        </is>
+      </c>
+      <c r="B64" t="n">
+        <v>639258</v>
+      </c>
+      <c r="C64" t="n">
+        <v>1</v>
+      </c>
+      <c r="D64" t="n">
+        <v>0</v>
+      </c>
+      <c r="E64" t="n">
+        <v>0</v>
+      </c>
+      <c r="F64" t="n">
+        <v>0</v>
+      </c>
+      <c r="G64" t="n">
+        <v>0</v>
+      </c>
+      <c r="H64" t="n">
+        <v>0</v>
+      </c>
+      <c r="I64" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Shafaq Zahra</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr"/>
+      <c r="C65" t="n">
+        <v>1</v>
+      </c>
+      <c r="D65" t="n">
+        <v>0</v>
+      </c>
+      <c r="E65" t="n">
+        <v>0</v>
+      </c>
+      <c r="F65" t="n">
+        <v>0</v>
+      </c>
+      <c r="G65" t="n">
+        <v>0</v>
+      </c>
+      <c r="H65" t="n">
+        <v>0</v>
+      </c>
+      <c r="I65" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Shakeel Ahmed</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>373686</v>
+      </c>
+      <c r="C66" t="n">
+        <v>3</v>
+      </c>
+      <c r="D66" t="n">
+        <v>0</v>
+      </c>
+      <c r="E66" t="n">
+        <v>0</v>
+      </c>
+      <c r="F66" t="n">
+        <v>0</v>
+      </c>
+      <c r="G66" t="n">
+        <v>0</v>
+      </c>
+      <c r="H66" t="n">
+        <v>0</v>
+      </c>
+      <c r="I66" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Sidra Khan</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
+        <v>373645</v>
+      </c>
+      <c r="C67" t="n">
+        <v>7</v>
+      </c>
+      <c r="D67" t="n">
+        <v>0</v>
+      </c>
+      <c r="E67" t="n">
+        <v>0</v>
+      </c>
+      <c r="F67" t="n">
+        <v>0</v>
+      </c>
+      <c r="G67" t="n">
+        <v>0</v>
+      </c>
+      <c r="H67" t="n">
+        <v>0</v>
+      </c>
+      <c r="I67" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Syed Haider Abbas</t>
+        </is>
+      </c>
+      <c r="B68" t="n">
+        <v>373713</v>
+      </c>
+      <c r="C68" t="n">
+        <v>2</v>
+      </c>
+      <c r="D68" t="n">
+        <v>0</v>
+      </c>
+      <c r="E68" t="n">
+        <v>0</v>
+      </c>
+      <c r="F68" t="n">
+        <v>0</v>
+      </c>
+      <c r="G68" t="n">
+        <v>0</v>
+      </c>
+      <c r="H68" t="n">
+        <v>0</v>
+      </c>
+      <c r="I68" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Usman Ali</t>
+        </is>
+      </c>
+      <c r="B69" t="n">
+        <v>373687</v>
+      </c>
+      <c r="C69" t="n">
+        <v>8</v>
+      </c>
+      <c r="D69" t="n">
+        <v>0</v>
+      </c>
+      <c r="E69" t="n">
+        <v>0</v>
+      </c>
+      <c r="F69" t="n">
+        <v>0</v>
+      </c>
+      <c r="G69" t="n">
+        <v>0</v>
+      </c>
+      <c r="H69" t="n">
+        <v>0</v>
+      </c>
+      <c r="I69" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: update age validation range for target girls in run function chore: update error log and performance summary files
</commit_message>
<xml_diff>
--- a/Error_log/Enumerator_Performance.xlsx
+++ b/Error_log/Enumerator_Performance.xlsx
@@ -590,39 +590,39 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Zohra</t>
+          <t>Mehran Khan</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>373692</v>
+        <v>373684</v>
       </c>
       <c r="C9" t="n">
-        <v>289</v>
+        <v>134</v>
       </c>
       <c r="D9" t="n">
         <v>106</v>
       </c>
       <c r="E9" t="n">
-        <v>183</v>
+        <v>28</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Mehran Khan</t>
+          <t>Zohra</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>373684</v>
+        <v>373692</v>
       </c>
       <c r="C10" t="n">
-        <v>134</v>
+        <v>287</v>
       </c>
       <c r="D10" t="n">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="E10" t="n">
-        <v>28</v>
+        <v>183</v>
       </c>
     </row>
     <row r="11">
@@ -844,10 +844,10 @@
         <v>453925</v>
       </c>
       <c r="C22" t="n">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D22" t="n">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E22" t="n">
         <v>2</v>
@@ -1421,19 +1421,19 @@
         <v>2</v>
       </c>
       <c r="D2" t="n">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E2" t="n">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="F2" t="n">
         <v>2</v>
       </c>
       <c r="G2" t="n">
-        <v>2600</v>
+        <v>2550</v>
       </c>
       <c r="H2" t="n">
-        <v>2500</v>
+        <v>2450</v>
       </c>
       <c r="I2" t="n">
         <v>100</v>
@@ -1545,19 +1545,19 @@
         <v>101</v>
       </c>
       <c r="D6" t="n">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="E6" t="n">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="F6" t="n">
         <v>183</v>
       </c>
       <c r="G6" t="n">
-        <v>286.14</v>
+        <v>284.16</v>
       </c>
       <c r="H6" t="n">
-        <v>104.95</v>
+        <v>102.97</v>
       </c>
       <c r="I6" t="n">
         <v>181.19</v>

</xml_diff>

<commit_message>
chore: update binary files for Daily Error Log and Weekly QA Summary
</commit_message>
<xml_diff>
--- a/Error_log/Enumerator_Performance.xlsx
+++ b/Error_log/Enumerator_Performance.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="performance" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="performance_pct" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="performance" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="performance_pct" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,16 +18,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -38,7 +35,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -46,21 +43,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -426,31 +414,31 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Enumerator Name</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Enumerator ID</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Total Issues</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Critical Issues</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Flag Issues</t>
         </is>
@@ -459,305 +447,1101 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Kainat</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>373712</v>
-      </c>
+          <t>UNASSIGNED (Tracking vs Household)</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr"/>
       <c r="C2" t="n">
-        <v>304</v>
+        <v>2238</v>
       </c>
       <c r="D2" t="n">
-        <v>103</v>
+        <v>2229</v>
       </c>
       <c r="E2" t="n">
-        <v>201</v>
+        <v>9</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Zohra</t>
+          <t>Asma Bibi</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>373692</v>
+        <v>373641</v>
       </c>
       <c r="C3" t="n">
-        <v>283</v>
+        <v>358</v>
       </c>
       <c r="D3" t="n">
-        <v>101</v>
+        <v>299</v>
       </c>
       <c r="E3" t="n">
-        <v>182</v>
+        <v>59</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Rehana Bibi</t>
+          <t>Mehran Khan</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>373691</v>
+        <v>373684</v>
       </c>
       <c r="C4" t="n">
-        <v>282</v>
+        <v>293</v>
       </c>
       <c r="D4" t="n">
-        <v>82</v>
+        <v>265</v>
       </c>
       <c r="E4" t="n">
-        <v>200</v>
+        <v>28</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Samara</t>
+          <t>Shazia Bibi</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>373658</v>
+        <v>373648</v>
       </c>
       <c r="C5" t="n">
-        <v>270</v>
+        <v>330</v>
       </c>
       <c r="D5" t="n">
-        <v>76</v>
+        <v>260</v>
       </c>
       <c r="E5" t="n">
-        <v>194</v>
+        <v>70</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Asma Bibi</t>
+          <t>Shazia begum</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>373641</v>
+        <v>373696</v>
       </c>
       <c r="C6" t="n">
-        <v>84</v>
+        <v>249</v>
       </c>
       <c r="D6" t="n">
-        <v>47</v>
+        <v>224</v>
       </c>
       <c r="E6" t="n">
-        <v>37</v>
+        <v>25</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Shazia Bibi</t>
+          <t>Shafaq Zahra</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>373648</v>
+        <v>373646</v>
       </c>
       <c r="C7" t="n">
-        <v>76</v>
+        <v>251</v>
       </c>
       <c r="D7" t="n">
-        <v>29</v>
+        <v>215</v>
       </c>
       <c r="E7" t="n">
-        <v>47</v>
+        <v>36</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Javairia</t>
+          <t>Irum Ikram</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>373651</v>
+        <v>373642</v>
       </c>
       <c r="C8" t="n">
-        <v>92</v>
+        <v>240</v>
       </c>
       <c r="D8" t="n">
-        <v>25</v>
+        <v>211</v>
       </c>
       <c r="E8" t="n">
-        <v>67</v>
+        <v>29</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Irum Ikram</t>
+          <t>Sadia Rustum</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>373642</v>
+        <v>373649</v>
       </c>
       <c r="C9" t="n">
-        <v>48</v>
+        <v>195</v>
       </c>
       <c r="D9" t="n">
-        <v>23</v>
+        <v>185</v>
       </c>
       <c r="E9" t="n">
-        <v>25</v>
+        <v>10</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Mahnoor</t>
+          <t>Khalida Bibi</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>373705</v>
+        <v>373673</v>
       </c>
       <c r="C10" t="n">
-        <v>52</v>
+        <v>140</v>
       </c>
       <c r="D10" t="n">
-        <v>20</v>
+        <v>140</v>
       </c>
       <c r="E10" t="n">
-        <v>32</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Nadia bibi</t>
+          <t>Mahnoor</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>373669</v>
+        <v>373705</v>
       </c>
       <c r="C11" t="n">
-        <v>41</v>
+        <v>172</v>
       </c>
       <c r="D11" t="n">
-        <v>15</v>
+        <v>136</v>
       </c>
       <c r="E11" t="n">
-        <v>26</v>
+        <v>36</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Shafaq Zahra</t>
+          <t>Javairia</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>373646</v>
+        <v>373651</v>
       </c>
       <c r="C12" t="n">
-        <v>33</v>
+        <v>215</v>
       </c>
       <c r="D12" t="n">
-        <v>13</v>
+        <v>135</v>
       </c>
       <c r="E12" t="n">
-        <v>20</v>
+        <v>80</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Naureen Khan</t>
+          <t>Kainat</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>373716</v>
+        <v>373712</v>
       </c>
       <c r="C13" t="n">
-        <v>22</v>
+        <v>333</v>
       </c>
       <c r="D13" t="n">
-        <v>13</v>
+        <v>131</v>
       </c>
       <c r="E13" t="n">
-        <v>9</v>
+        <v>202</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Laiba Shams</t>
+          <t>Naureen Khan</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>373706</v>
+        <v>373716</v>
       </c>
       <c r="C14" t="n">
-        <v>33</v>
+        <v>133</v>
       </c>
       <c r="D14" t="n">
-        <v>11</v>
+        <v>124</v>
       </c>
       <c r="E14" t="n">
-        <v>22</v>
+        <v>9</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Shazia begum</t>
+          <t>Bushra Ayub</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>373696</v>
+        <v>373671</v>
       </c>
       <c r="C15" t="n">
-        <v>13</v>
+        <v>126</v>
       </c>
       <c r="D15" t="n">
-        <v>5</v>
+        <v>122</v>
       </c>
       <c r="E15" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Naureen khan</t>
+          <t>Furqan Ullah Khan</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>453925</v>
+        <v>373683</v>
       </c>
       <c r="C16" t="n">
-        <v>7</v>
+        <v>124</v>
       </c>
       <c r="D16" t="n">
-        <v>5</v>
+        <v>116</v>
       </c>
       <c r="E16" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
+          <t>Zohra</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>373692</v>
+      </c>
+      <c r="C17" t="n">
+        <v>298</v>
+      </c>
+      <c r="D17" t="n">
+        <v>115</v>
+      </c>
+      <c r="E17" t="n">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Asma Gull</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>373672</v>
+      </c>
+      <c r="C18" t="n">
+        <v>109</v>
+      </c>
+      <c r="D18" t="n">
+        <v>105</v>
+      </c>
+      <c r="E18" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Samara</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>373658</v>
+      </c>
+      <c r="C19" t="n">
+        <v>298</v>
+      </c>
+      <c r="D19" t="n">
+        <v>102</v>
+      </c>
+      <c r="E19" t="n">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Ishaq Khan</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>373699</v>
+      </c>
+      <c r="C20" t="n">
+        <v>101</v>
+      </c>
+      <c r="D20" t="n">
+        <v>100</v>
+      </c>
+      <c r="E20" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Muhammad Yousaf</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>373690</v>
+      </c>
+      <c r="C21" t="n">
+        <v>105</v>
+      </c>
+      <c r="D21" t="n">
+        <v>96</v>
+      </c>
+      <c r="E21" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Rehana Bibi</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>373691</v>
+      </c>
+      <c r="C22" t="n">
+        <v>295</v>
+      </c>
+      <c r="D22" t="n">
+        <v>94</v>
+      </c>
+      <c r="E22" t="n">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Lati Khan</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>564273</v>
+      </c>
+      <c r="C23" t="n">
+        <v>98</v>
+      </c>
+      <c r="D23" t="n">
+        <v>94</v>
+      </c>
+      <c r="E23" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Naureen khan</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>453925</v>
+      </c>
+      <c r="C24" t="n">
+        <v>92</v>
+      </c>
+      <c r="D24" t="n">
+        <v>90</v>
+      </c>
+      <c r="E24" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Laiba Shams</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>373706</v>
+      </c>
+      <c r="C25" t="n">
+        <v>115</v>
+      </c>
+      <c r="D25" t="n">
+        <v>87</v>
+      </c>
+      <c r="E25" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Irum ikram</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>541376</v>
+      </c>
+      <c r="C26" t="n">
+        <v>88</v>
+      </c>
+      <c r="D26" t="n">
+        <v>83</v>
+      </c>
+      <c r="E26" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Lati Khan</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>373665</v>
+      </c>
+      <c r="C27" t="n">
+        <v>86</v>
+      </c>
+      <c r="D27" t="n">
+        <v>83</v>
+      </c>
+      <c r="E27" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Naureen</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>884887</v>
+      </c>
+      <c r="C28" t="n">
+        <v>86</v>
+      </c>
+      <c r="D28" t="n">
+        <v>82</v>
+      </c>
+      <c r="E28" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Jaweria</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>163495</v>
+      </c>
+      <c r="C29" t="n">
+        <v>83</v>
+      </c>
+      <c r="D29" t="n">
+        <v>82</v>
+      </c>
+      <c r="E29" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Nillum Bibi</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>373652</v>
+      </c>
+      <c r="C30" t="n">
+        <v>64</v>
+      </c>
+      <c r="D30" t="n">
+        <v>61</v>
+      </c>
+      <c r="E30" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Anum Gul</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>373656</v>
+      </c>
+      <c r="C31" t="n">
+        <v>55</v>
+      </c>
+      <c r="D31" t="n">
+        <v>51</v>
+      </c>
+      <c r="E31" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Muniba Shamim</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>373659</v>
+      </c>
+      <c r="C32" t="n">
+        <v>58</v>
+      </c>
+      <c r="D32" t="n">
+        <v>49</v>
+      </c>
+      <c r="E32" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Nazia</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>373657</v>
+      </c>
+      <c r="C33" t="n">
+        <v>51</v>
+      </c>
+      <c r="D33" t="n">
+        <v>49</v>
+      </c>
+      <c r="E33" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Alia Khan</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>373681</v>
+      </c>
+      <c r="C34" t="n">
+        <v>44</v>
+      </c>
+      <c r="D34" t="n">
+        <v>40</v>
+      </c>
+      <c r="E34" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Lati khan</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>671211</v>
+      </c>
+      <c r="C35" t="n">
+        <v>38</v>
+      </c>
+      <c r="D35" t="n">
+        <v>38</v>
+      </c>
+      <c r="E35" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
           <t>Summiya Hayat</t>
         </is>
       </c>
-      <c r="B17" t="n">
+      <c r="B36" t="n">
         <v>373710</v>
       </c>
-      <c r="C17" t="n">
-        <v>17</v>
-      </c>
-      <c r="D17" t="n">
+      <c r="C36" t="n">
+        <v>60</v>
+      </c>
+      <c r="D36" t="n">
+        <v>33</v>
+      </c>
+      <c r="E36" t="n">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Munawar Khan</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>373668</v>
+      </c>
+      <c r="C37" t="n">
+        <v>39</v>
+      </c>
+      <c r="D37" t="n">
+        <v>33</v>
+      </c>
+      <c r="E37" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Laiba Khan</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>373653</v>
+      </c>
+      <c r="C38" t="n">
+        <v>26</v>
+      </c>
+      <c r="D38" t="n">
+        <v>22</v>
+      </c>
+      <c r="E38" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Chashm Gul</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>373695</v>
+      </c>
+      <c r="C39" t="n">
+        <v>27</v>
+      </c>
+      <c r="D39" t="n">
+        <v>18</v>
+      </c>
+      <c r="E39" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Nadia bibi</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>373669</v>
+      </c>
+      <c r="C40" t="n">
+        <v>41</v>
+      </c>
+      <c r="D40" t="n">
+        <v>15</v>
+      </c>
+      <c r="E40" t="n">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Zain Ul Abideen</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>373667</v>
+      </c>
+      <c r="C41" t="n">
+        <v>12</v>
+      </c>
+      <c r="D41" t="n">
+        <v>12</v>
+      </c>
+      <c r="E41" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Lati khan</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>652938</v>
+      </c>
+      <c r="C42" t="n">
+        <v>10</v>
+      </c>
+      <c r="D42" t="n">
+        <v>10</v>
+      </c>
+      <c r="E42" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Saba Ramzan</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>373703</v>
+      </c>
+      <c r="C43" t="n">
+        <v>9</v>
+      </c>
+      <c r="D43" t="n">
+        <v>9</v>
+      </c>
+      <c r="E43" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Shehla Noor</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>373650</v>
+      </c>
+      <c r="C44" t="n">
+        <v>9</v>
+      </c>
+      <c r="D44" t="n">
+        <v>9</v>
+      </c>
+      <c r="E44" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Muhammad naeem</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>571571</v>
+      </c>
+      <c r="C45" t="n">
+        <v>10</v>
+      </c>
+      <c r="D45" t="n">
+        <v>8</v>
+      </c>
+      <c r="E45" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Sadia rustum</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>852541</v>
+      </c>
+      <c r="C46" t="n">
+        <v>5</v>
+      </c>
+      <c r="D46" t="n">
+        <v>5</v>
+      </c>
+      <c r="E46" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Usman Ali</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>373687</v>
+      </c>
+      <c r="C47" t="n">
+        <v>5</v>
+      </c>
+      <c r="D47" t="n">
+        <v>5</v>
+      </c>
+      <c r="E47" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Muhammad Noor</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>373701</v>
+      </c>
+      <c r="C48" t="n">
+        <v>4</v>
+      </c>
+      <c r="D48" t="n">
         <v>3</v>
       </c>
-      <c r="E17" t="n">
-        <v>14</v>
+      <c r="E48" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Muhammad Naeem</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>373694</v>
+      </c>
+      <c r="C49" t="n">
+        <v>3</v>
+      </c>
+      <c r="D49" t="n">
+        <v>3</v>
+      </c>
+      <c r="E49" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Muhammad Shahid Khan</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>373662</v>
+      </c>
+      <c r="C50" t="n">
+        <v>3</v>
+      </c>
+      <c r="D50" t="n">
+        <v>3</v>
+      </c>
+      <c r="E50" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Sajjad Khan</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>373700</v>
+      </c>
+      <c r="C51" t="n">
+        <v>3</v>
+      </c>
+      <c r="D51" t="n">
+        <v>3</v>
+      </c>
+      <c r="E51" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Aisha Aman</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>373704</v>
+      </c>
+      <c r="C52" t="n">
+        <v>3</v>
+      </c>
+      <c r="D52" t="n">
+        <v>2</v>
+      </c>
+      <c r="E52" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Rahila Naaz</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>373715</v>
+      </c>
+      <c r="C53" t="n">
+        <v>3</v>
+      </c>
+      <c r="D53" t="n">
+        <v>2</v>
+      </c>
+      <c r="E53" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Robina Shaheen</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>373639</v>
+      </c>
+      <c r="C54" t="n">
+        <v>3</v>
+      </c>
+      <c r="D54" t="n">
+        <v>2</v>
+      </c>
+      <c r="E54" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Iqra Bibi</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>373708</v>
+      </c>
+      <c r="C55" t="n">
+        <v>2</v>
+      </c>
+      <c r="D55" t="n">
+        <v>2</v>
+      </c>
+      <c r="E55" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Mahnoorr</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>373670</v>
+      </c>
+      <c r="C56" t="n">
+        <v>2</v>
+      </c>
+      <c r="D56" t="n">
+        <v>1</v>
+      </c>
+      <c r="E56" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Gul Rukh</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>373644</v>
+      </c>
+      <c r="C57" t="n">
+        <v>1</v>
+      </c>
+      <c r="D57" t="n">
+        <v>1</v>
+      </c>
+      <c r="E57" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Hijab Zahra</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>373637</v>
+      </c>
+      <c r="C58" t="n">
+        <v>1</v>
+      </c>
+      <c r="D58" t="n">
+        <v>1</v>
+      </c>
+      <c r="E58" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Sidra Khan</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>373645</v>
+      </c>
+      <c r="C59" t="n">
+        <v>1</v>
+      </c>
+      <c r="D59" t="n">
+        <v>1</v>
+      </c>
+      <c r="E59" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -771,51 +1555,51 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:I70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>enumerator_name</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>enumerator_id</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>total_submissions</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>total_issues</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>critical_issues</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>flag_issues</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>error_pct</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>critical_error_pct</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>flag_error_pct</t>
         </is>
@@ -824,496 +1608,2131 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Javairia</t>
+          <t>Naureen khan</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>373651</v>
+        <v>453925</v>
       </c>
       <c r="C2" t="n">
-        <v>21</v>
+        <v>2</v>
       </c>
       <c r="D2" t="n">
         <v>92</v>
       </c>
       <c r="E2" t="n">
-        <v>25</v>
+        <v>90</v>
       </c>
       <c r="F2" t="n">
-        <v>67</v>
+        <v>2</v>
       </c>
       <c r="G2" t="n">
-        <v>438.1</v>
+        <v>4600</v>
       </c>
       <c r="H2" t="n">
-        <v>119.05</v>
+        <v>4500</v>
       </c>
       <c r="I2" t="n">
-        <v>319.05</v>
+        <v>100</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Kainat</t>
+          <t>Irum ikram</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>373712</v>
+        <v>541376</v>
       </c>
       <c r="C3" t="n">
-        <v>73</v>
+        <v>8</v>
       </c>
       <c r="D3" t="n">
-        <v>304</v>
+        <v>88</v>
       </c>
       <c r="E3" t="n">
-        <v>103</v>
+        <v>83</v>
       </c>
       <c r="F3" t="n">
-        <v>201</v>
+        <v>5</v>
       </c>
       <c r="G3" t="n">
-        <v>416.44</v>
+        <v>1100</v>
       </c>
       <c r="H3" t="n">
-        <v>141.1</v>
+        <v>1037.5</v>
       </c>
       <c r="I3" t="n">
-        <v>275.34</v>
+        <v>62.5</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Zohra</t>
+          <t>Lati Khan</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>373692</v>
+        <v>564273</v>
       </c>
       <c r="C4" t="n">
-        <v>70</v>
+        <v>9</v>
       </c>
       <c r="D4" t="n">
-        <v>283</v>
+        <v>98</v>
       </c>
       <c r="E4" t="n">
-        <v>101</v>
+        <v>94</v>
       </c>
       <c r="F4" t="n">
-        <v>182</v>
+        <v>4</v>
       </c>
       <c r="G4" t="n">
-        <v>404.29</v>
+        <v>1088.89</v>
       </c>
       <c r="H4" t="n">
-        <v>144.29</v>
+        <v>1044.44</v>
       </c>
       <c r="I4" t="n">
-        <v>260</v>
+        <v>44.44</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Rehana Bibi</t>
+          <t>Lati khan</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>373691</v>
+        <v>671211</v>
       </c>
       <c r="C5" t="n">
-        <v>79</v>
+        <v>9</v>
       </c>
       <c r="D5" t="n">
-        <v>282</v>
+        <v>38</v>
       </c>
       <c r="E5" t="n">
-        <v>82</v>
+        <v>38</v>
       </c>
       <c r="F5" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="G5" t="n">
-        <v>356.96</v>
+        <v>422.22</v>
       </c>
       <c r="H5" t="n">
-        <v>103.8</v>
+        <v>422.22</v>
       </c>
       <c r="I5" t="n">
-        <v>253.16</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Samara</t>
+          <t>Kainat</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>373658</v>
+        <v>373712</v>
       </c>
       <c r="C6" t="n">
-        <v>79</v>
+        <v>104</v>
       </c>
       <c r="D6" t="n">
-        <v>270</v>
+        <v>333</v>
       </c>
       <c r="E6" t="n">
-        <v>76</v>
+        <v>131</v>
       </c>
       <c r="F6" t="n">
-        <v>194</v>
+        <v>202</v>
       </c>
       <c r="G6" t="n">
-        <v>341.77</v>
+        <v>320.19</v>
       </c>
       <c r="H6" t="n">
-        <v>96.2</v>
+        <v>125.96</v>
       </c>
       <c r="I6" t="n">
-        <v>245.57</v>
+        <v>194.23</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Asma Bibi</t>
+          <t>Zohra</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>373641</v>
+        <v>373692</v>
       </c>
       <c r="C7" t="n">
-        <v>31</v>
+        <v>101</v>
       </c>
       <c r="D7" t="n">
-        <v>84</v>
+        <v>298</v>
       </c>
       <c r="E7" t="n">
-        <v>47</v>
+        <v>115</v>
       </c>
       <c r="F7" t="n">
-        <v>37</v>
+        <v>183</v>
       </c>
       <c r="G7" t="n">
-        <v>270.97</v>
+        <v>295.05</v>
       </c>
       <c r="H7" t="n">
-        <v>151.61</v>
+        <v>113.86</v>
       </c>
       <c r="I7" t="n">
-        <v>119.35</v>
+        <v>181.19</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Shazia Bibi</t>
+          <t>Rehana Bibi</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>373648</v>
+        <v>373691</v>
       </c>
       <c r="C8" t="n">
-        <v>34</v>
+        <v>111</v>
       </c>
       <c r="D8" t="n">
-        <v>76</v>
+        <v>295</v>
       </c>
       <c r="E8" t="n">
-        <v>29</v>
+        <v>94</v>
       </c>
       <c r="F8" t="n">
-        <v>47</v>
+        <v>201</v>
       </c>
       <c r="G8" t="n">
-        <v>223.53</v>
+        <v>265.77</v>
       </c>
       <c r="H8" t="n">
-        <v>85.29000000000001</v>
+        <v>84.68000000000001</v>
       </c>
       <c r="I8" t="n">
-        <v>138.24</v>
+        <v>181.08</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Irum Ikram</t>
+          <t>Samara</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>373642</v>
+        <v>373658</v>
       </c>
       <c r="C9" t="n">
-        <v>22</v>
+        <v>120</v>
       </c>
       <c r="D9" t="n">
-        <v>48</v>
+        <v>298</v>
       </c>
       <c r="E9" t="n">
-        <v>23</v>
+        <v>102</v>
       </c>
       <c r="F9" t="n">
-        <v>25</v>
+        <v>196</v>
       </c>
       <c r="G9" t="n">
-        <v>218.18</v>
+        <v>248.33</v>
       </c>
       <c r="H9" t="n">
-        <v>104.55</v>
+        <v>85</v>
       </c>
       <c r="I9" t="n">
-        <v>113.64</v>
+        <v>163.33</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Shazia begum</t>
+          <t>Asma Bibi</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>373696</v>
+        <v>373641</v>
       </c>
       <c r="C10" t="n">
-        <v>6</v>
+        <v>218</v>
       </c>
       <c r="D10" t="n">
-        <v>13</v>
+        <v>358</v>
       </c>
       <c r="E10" t="n">
-        <v>5</v>
+        <v>299</v>
       </c>
       <c r="F10" t="n">
-        <v>8</v>
+        <v>59</v>
       </c>
       <c r="G10" t="n">
-        <v>216.67</v>
+        <v>164.22</v>
       </c>
       <c r="H10" t="n">
-        <v>83.33</v>
+        <v>137.16</v>
       </c>
       <c r="I10" t="n">
-        <v>133.33</v>
+        <v>27.06</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Nadia bibi</t>
+          <t>Naureen Khan</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>373669</v>
+        <v>373716</v>
       </c>
       <c r="C11" t="n">
-        <v>19</v>
+        <v>81</v>
       </c>
       <c r="D11" t="n">
-        <v>41</v>
+        <v>133</v>
       </c>
       <c r="E11" t="n">
-        <v>15</v>
+        <v>124</v>
       </c>
       <c r="F11" t="n">
-        <v>26</v>
+        <v>9</v>
       </c>
       <c r="G11" t="n">
-        <v>215.79</v>
+        <v>164.2</v>
       </c>
       <c r="H11" t="n">
-        <v>78.95</v>
+        <v>153.09</v>
       </c>
       <c r="I11" t="n">
-        <v>136.84</v>
+        <v>11.11</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Mahnoor</t>
+          <t>Javairia</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>373705</v>
+        <v>373651</v>
       </c>
       <c r="C12" t="n">
-        <v>25</v>
+        <v>141</v>
       </c>
       <c r="D12" t="n">
-        <v>52</v>
+        <v>215</v>
       </c>
       <c r="E12" t="n">
-        <v>20</v>
+        <v>135</v>
       </c>
       <c r="F12" t="n">
-        <v>32</v>
+        <v>80</v>
       </c>
       <c r="G12" t="n">
-        <v>208</v>
+        <v>152.48</v>
       </c>
       <c r="H12" t="n">
-        <v>80</v>
+        <v>95.73999999999999</v>
       </c>
       <c r="I12" t="n">
-        <v>128</v>
+        <v>56.74</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Shafaq Zahra</t>
+          <t>Shazia Bibi</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>373646</v>
+        <v>373648</v>
       </c>
       <c r="C13" t="n">
-        <v>16</v>
+        <v>223</v>
       </c>
       <c r="D13" t="n">
-        <v>33</v>
+        <v>330</v>
       </c>
       <c r="E13" t="n">
-        <v>13</v>
+        <v>260</v>
       </c>
       <c r="F13" t="n">
-        <v>20</v>
+        <v>70</v>
       </c>
       <c r="G13" t="n">
-        <v>206.25</v>
+        <v>147.98</v>
       </c>
       <c r="H13" t="n">
-        <v>81.25</v>
+        <v>116.59</v>
       </c>
       <c r="I13" t="n">
-        <v>125</v>
+        <v>31.39</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Naureen Khan</t>
+          <t>Mehran Khan</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>373716</v>
+        <v>373684</v>
       </c>
       <c r="C14" t="n">
-        <v>11</v>
+        <v>200</v>
       </c>
       <c r="D14" t="n">
-        <v>22</v>
+        <v>293</v>
       </c>
       <c r="E14" t="n">
-        <v>13</v>
+        <v>265</v>
       </c>
       <c r="F14" t="n">
-        <v>9</v>
+        <v>28</v>
       </c>
       <c r="G14" t="n">
-        <v>200</v>
+        <v>146.5</v>
       </c>
       <c r="H14" t="n">
-        <v>118.18</v>
+        <v>132.5</v>
       </c>
       <c r="I14" t="n">
-        <v>81.81999999999999</v>
+        <v>14</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Laiba Shams</t>
+          <t>Mahnoor</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>373706</v>
+        <v>373705</v>
       </c>
       <c r="C15" t="n">
-        <v>21</v>
+        <v>119</v>
       </c>
       <c r="D15" t="n">
-        <v>33</v>
+        <v>172</v>
       </c>
       <c r="E15" t="n">
-        <v>11</v>
+        <v>136</v>
       </c>
       <c r="F15" t="n">
-        <v>22</v>
+        <v>36</v>
       </c>
       <c r="G15" t="n">
-        <v>157.14</v>
+        <v>144.54</v>
       </c>
       <c r="H15" t="n">
-        <v>52.38</v>
+        <v>114.29</v>
       </c>
       <c r="I15" t="n">
-        <v>104.76</v>
+        <v>30.25</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Summiya Hayat</t>
+          <t>Lati Khan</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>373710</v>
+        <v>373665</v>
       </c>
       <c r="C16" t="n">
-        <v>13</v>
+        <v>60</v>
       </c>
       <c r="D16" t="n">
-        <v>17</v>
+        <v>86</v>
       </c>
       <c r="E16" t="n">
+        <v>83</v>
+      </c>
+      <c r="F16" t="n">
         <v>3</v>
       </c>
-      <c r="F16" t="n">
-        <v>14</v>
-      </c>
       <c r="G16" t="n">
-        <v>130.77</v>
+        <v>143.33</v>
       </c>
       <c r="H16" t="n">
-        <v>23.08</v>
+        <v>138.33</v>
       </c>
       <c r="I16" t="n">
-        <v>107.69</v>
+        <v>5</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
+          <t>Naureen</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>884887</v>
+      </c>
+      <c r="C17" t="n">
+        <v>60</v>
+      </c>
+      <c r="D17" t="n">
+        <v>86</v>
+      </c>
+      <c r="E17" t="n">
+        <v>82</v>
+      </c>
+      <c r="F17" t="n">
+        <v>4</v>
+      </c>
+      <c r="G17" t="n">
+        <v>143.33</v>
+      </c>
+      <c r="H17" t="n">
+        <v>136.67</v>
+      </c>
+      <c r="I17" t="n">
+        <v>6.67</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Nadia bibi</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>373669</v>
+      </c>
+      <c r="C18" t="n">
+        <v>29</v>
+      </c>
+      <c r="D18" t="n">
+        <v>41</v>
+      </c>
+      <c r="E18" t="n">
+        <v>15</v>
+      </c>
+      <c r="F18" t="n">
+        <v>26</v>
+      </c>
+      <c r="G18" t="n">
+        <v>141.38</v>
+      </c>
+      <c r="H18" t="n">
+        <v>51.72</v>
+      </c>
+      <c r="I18" t="n">
+        <v>89.66</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Irum Ikram</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>373642</v>
+      </c>
+      <c r="C19" t="n">
+        <v>172</v>
+      </c>
+      <c r="D19" t="n">
+        <v>240</v>
+      </c>
+      <c r="E19" t="n">
+        <v>211</v>
+      </c>
+      <c r="F19" t="n">
+        <v>29</v>
+      </c>
+      <c r="G19" t="n">
+        <v>139.53</v>
+      </c>
+      <c r="H19" t="n">
+        <v>122.67</v>
+      </c>
+      <c r="I19" t="n">
+        <v>16.86</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Shazia begum</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>373696</v>
+      </c>
+      <c r="C20" t="n">
+        <v>185</v>
+      </c>
+      <c r="D20" t="n">
+        <v>249</v>
+      </c>
+      <c r="E20" t="n">
+        <v>224</v>
+      </c>
+      <c r="F20" t="n">
+        <v>25</v>
+      </c>
+      <c r="G20" t="n">
+        <v>134.59</v>
+      </c>
+      <c r="H20" t="n">
+        <v>121.08</v>
+      </c>
+      <c r="I20" t="n">
+        <v>13.51</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Sadia Rustum</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>373649</v>
+      </c>
+      <c r="C21" t="n">
+        <v>152</v>
+      </c>
+      <c r="D21" t="n">
+        <v>195</v>
+      </c>
+      <c r="E21" t="n">
+        <v>185</v>
+      </c>
+      <c r="F21" t="n">
+        <v>10</v>
+      </c>
+      <c r="G21" t="n">
+        <v>128.29</v>
+      </c>
+      <c r="H21" t="n">
+        <v>121.71</v>
+      </c>
+      <c r="I21" t="n">
+        <v>6.58</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Jaweria</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>163495</v>
+      </c>
+      <c r="C22" t="n">
+        <v>68</v>
+      </c>
+      <c r="D22" t="n">
+        <v>83</v>
+      </c>
+      <c r="E22" t="n">
+        <v>82</v>
+      </c>
+      <c r="F22" t="n">
+        <v>1</v>
+      </c>
+      <c r="G22" t="n">
+        <v>122.06</v>
+      </c>
+      <c r="H22" t="n">
+        <v>120.59</v>
+      </c>
+      <c r="I22" t="n">
+        <v>1.47</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Shafaq Zahra</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>373646</v>
+      </c>
+      <c r="C23" t="n">
+        <v>223</v>
+      </c>
+      <c r="D23" t="n">
+        <v>251</v>
+      </c>
+      <c r="E23" t="n">
+        <v>215</v>
+      </c>
+      <c r="F23" t="n">
+        <v>36</v>
+      </c>
+      <c r="G23" t="n">
+        <v>112.56</v>
+      </c>
+      <c r="H23" t="n">
+        <v>96.41</v>
+      </c>
+      <c r="I23" t="n">
+        <v>16.14</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Laiba Shams</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>373706</v>
+      </c>
+      <c r="C24" t="n">
+        <v>114</v>
+      </c>
+      <c r="D24" t="n">
+        <v>115</v>
+      </c>
+      <c r="E24" t="n">
+        <v>87</v>
+      </c>
+      <c r="F24" t="n">
+        <v>28</v>
+      </c>
+      <c r="G24" t="n">
+        <v>100.88</v>
+      </c>
+      <c r="H24" t="n">
+        <v>76.31999999999999</v>
+      </c>
+      <c r="I24" t="n">
+        <v>24.56</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Zain Ul Abideen</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>373667</v>
+      </c>
+      <c r="C25" t="n">
+        <v>13</v>
+      </c>
+      <c r="D25" t="n">
+        <v>12</v>
+      </c>
+      <c r="E25" t="n">
+        <v>12</v>
+      </c>
+      <c r="F25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G25" t="n">
+        <v>92.31</v>
+      </c>
+      <c r="H25" t="n">
+        <v>92.31</v>
+      </c>
+      <c r="I25" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Bushra Ayub</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>373671</v>
+      </c>
+      <c r="C26" t="n">
+        <v>138</v>
+      </c>
+      <c r="D26" t="n">
+        <v>126</v>
+      </c>
+      <c r="E26" t="n">
+        <v>122</v>
+      </c>
+      <c r="F26" t="n">
+        <v>4</v>
+      </c>
+      <c r="G26" t="n">
+        <v>91.3</v>
+      </c>
+      <c r="H26" t="n">
+        <v>88.41</v>
+      </c>
+      <c r="I26" t="n">
+        <v>2.9</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Lati khan</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>652938</v>
+      </c>
+      <c r="C27" t="n">
+        <v>11</v>
+      </c>
+      <c r="D27" t="n">
+        <v>10</v>
+      </c>
+      <c r="E27" t="n">
+        <v>10</v>
+      </c>
+      <c r="F27" t="n">
+        <v>0</v>
+      </c>
+      <c r="G27" t="n">
+        <v>90.91</v>
+      </c>
+      <c r="H27" t="n">
+        <v>90.91</v>
+      </c>
+      <c r="I27" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Chashm Gul</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>373695</v>
+      </c>
+      <c r="C28" t="n">
+        <v>31</v>
+      </c>
+      <c r="D28" t="n">
+        <v>27</v>
+      </c>
+      <c r="E28" t="n">
+        <v>18</v>
+      </c>
+      <c r="F28" t="n">
+        <v>9</v>
+      </c>
+      <c r="G28" t="n">
+        <v>87.09999999999999</v>
+      </c>
+      <c r="H28" t="n">
+        <v>58.06</v>
+      </c>
+      <c r="I28" t="n">
+        <v>29.03</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Muniba Shamim</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>373659</v>
+      </c>
+      <c r="C29" t="n">
+        <v>72</v>
+      </c>
+      <c r="D29" t="n">
+        <v>58</v>
+      </c>
+      <c r="E29" t="n">
+        <v>49</v>
+      </c>
+      <c r="F29" t="n">
+        <v>9</v>
+      </c>
+      <c r="G29" t="n">
+        <v>80.56</v>
+      </c>
+      <c r="H29" t="n">
+        <v>68.06</v>
+      </c>
+      <c r="I29" t="n">
+        <v>12.5</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Muhammad Yousaf</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>373690</v>
+      </c>
+      <c r="C30" t="n">
+        <v>132</v>
+      </c>
+      <c r="D30" t="n">
+        <v>105</v>
+      </c>
+      <c r="E30" t="n">
+        <v>96</v>
+      </c>
+      <c r="F30" t="n">
+        <v>9</v>
+      </c>
+      <c r="G30" t="n">
+        <v>79.55</v>
+      </c>
+      <c r="H30" t="n">
+        <v>72.73</v>
+      </c>
+      <c r="I30" t="n">
+        <v>6.82</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Khalida Bibi</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>373673</v>
+      </c>
+      <c r="C31" t="n">
+        <v>177</v>
+      </c>
+      <c r="D31" t="n">
+        <v>140</v>
+      </c>
+      <c r="E31" t="n">
+        <v>140</v>
+      </c>
+      <c r="F31" t="n">
+        <v>0</v>
+      </c>
+      <c r="G31" t="n">
+        <v>79.09999999999999</v>
+      </c>
+      <c r="H31" t="n">
+        <v>79.09999999999999</v>
+      </c>
+      <c r="I31" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Asma Gull</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>373672</v>
+      </c>
+      <c r="C32" t="n">
+        <v>144</v>
+      </c>
+      <c r="D32" t="n">
+        <v>109</v>
+      </c>
+      <c r="E32" t="n">
+        <v>105</v>
+      </c>
+      <c r="F32" t="n">
+        <v>4</v>
+      </c>
+      <c r="G32" t="n">
+        <v>75.69</v>
+      </c>
+      <c r="H32" t="n">
+        <v>72.92</v>
+      </c>
+      <c r="I32" t="n">
+        <v>2.78</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Rahila Naaz</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>373715</v>
+      </c>
+      <c r="C33" t="n">
+        <v>4</v>
+      </c>
+      <c r="D33" t="n">
+        <v>3</v>
+      </c>
+      <c r="E33" t="n">
+        <v>2</v>
+      </c>
+      <c r="F33" t="n">
+        <v>1</v>
+      </c>
+      <c r="G33" t="n">
+        <v>75</v>
+      </c>
+      <c r="H33" t="n">
+        <v>50</v>
+      </c>
+      <c r="I33" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Sadia rustum</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>852541</v>
+      </c>
+      <c r="C34" t="n">
+        <v>7</v>
+      </c>
+      <c r="D34" t="n">
+        <v>5</v>
+      </c>
+      <c r="E34" t="n">
+        <v>5</v>
+      </c>
+      <c r="F34" t="n">
+        <v>0</v>
+      </c>
+      <c r="G34" t="n">
+        <v>71.43000000000001</v>
+      </c>
+      <c r="H34" t="n">
+        <v>71.43000000000001</v>
+      </c>
+      <c r="I34" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Saba Ramzan</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>373703</v>
+      </c>
+      <c r="C35" t="n">
+        <v>13</v>
+      </c>
+      <c r="D35" t="n">
+        <v>9</v>
+      </c>
+      <c r="E35" t="n">
+        <v>9</v>
+      </c>
+      <c r="F35" t="n">
+        <v>0</v>
+      </c>
+      <c r="G35" t="n">
+        <v>69.23</v>
+      </c>
+      <c r="H35" t="n">
+        <v>69.23</v>
+      </c>
+      <c r="I35" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Shehla Noor</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>373650</v>
+      </c>
+      <c r="C36" t="n">
+        <v>14</v>
+      </c>
+      <c r="D36" t="n">
+        <v>9</v>
+      </c>
+      <c r="E36" t="n">
+        <v>9</v>
+      </c>
+      <c r="F36" t="n">
+        <v>0</v>
+      </c>
+      <c r="G36" t="n">
+        <v>64.29000000000001</v>
+      </c>
+      <c r="H36" t="n">
+        <v>64.29000000000001</v>
+      </c>
+      <c r="I36" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Summiya Hayat</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>373710</v>
+      </c>
+      <c r="C37" t="n">
+        <v>94</v>
+      </c>
+      <c r="D37" t="n">
+        <v>60</v>
+      </c>
+      <c r="E37" t="n">
+        <v>33</v>
+      </c>
+      <c r="F37" t="n">
+        <v>27</v>
+      </c>
+      <c r="G37" t="n">
+        <v>63.83</v>
+      </c>
+      <c r="H37" t="n">
+        <v>35.11</v>
+      </c>
+      <c r="I37" t="n">
+        <v>28.72</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Furqan Ullah Khan</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>373683</v>
+      </c>
+      <c r="C38" t="n">
+        <v>195</v>
+      </c>
+      <c r="D38" t="n">
+        <v>124</v>
+      </c>
+      <c r="E38" t="n">
+        <v>116</v>
+      </c>
+      <c r="F38" t="n">
+        <v>8</v>
+      </c>
+      <c r="G38" t="n">
+        <v>63.59</v>
+      </c>
+      <c r="H38" t="n">
+        <v>59.49</v>
+      </c>
+      <c r="I38" t="n">
+        <v>4.1</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Usman Ali</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>373687</v>
+      </c>
+      <c r="C39" t="n">
+        <v>8</v>
+      </c>
+      <c r="D39" t="n">
+        <v>5</v>
+      </c>
+      <c r="E39" t="n">
+        <v>5</v>
+      </c>
+      <c r="F39" t="n">
+        <v>0</v>
+      </c>
+      <c r="G39" t="n">
+        <v>62.5</v>
+      </c>
+      <c r="H39" t="n">
+        <v>62.5</v>
+      </c>
+      <c r="I39" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Ishaq Khan</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>373699</v>
+      </c>
+      <c r="C40" t="n">
+        <v>170</v>
+      </c>
+      <c r="D40" t="n">
+        <v>101</v>
+      </c>
+      <c r="E40" t="n">
+        <v>100</v>
+      </c>
+      <c r="F40" t="n">
+        <v>1</v>
+      </c>
+      <c r="G40" t="n">
+        <v>59.41</v>
+      </c>
+      <c r="H40" t="n">
+        <v>58.82</v>
+      </c>
+      <c r="I40" t="n">
+        <v>0.59</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Munawar Khan</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>373668</v>
+      </c>
+      <c r="C41" t="n">
+        <v>73</v>
+      </c>
+      <c r="D41" t="n">
+        <v>39</v>
+      </c>
+      <c r="E41" t="n">
+        <v>33</v>
+      </c>
+      <c r="F41" t="n">
+        <v>6</v>
+      </c>
+      <c r="G41" t="n">
+        <v>53.42</v>
+      </c>
+      <c r="H41" t="n">
+        <v>45.21</v>
+      </c>
+      <c r="I41" t="n">
+        <v>8.220000000000001</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Anum Gul</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>373656</v>
+      </c>
+      <c r="C42" t="n">
+        <v>103</v>
+      </c>
+      <c r="D42" t="n">
+        <v>55</v>
+      </c>
+      <c r="E42" t="n">
+        <v>51</v>
+      </c>
+      <c r="F42" t="n">
+        <v>4</v>
+      </c>
+      <c r="G42" t="n">
+        <v>53.4</v>
+      </c>
+      <c r="H42" t="n">
+        <v>49.51</v>
+      </c>
+      <c r="I42" t="n">
+        <v>3.88</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Muhammad Noor</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>373701</v>
+      </c>
+      <c r="C43" t="n">
+        <v>8</v>
+      </c>
+      <c r="D43" t="n">
+        <v>4</v>
+      </c>
+      <c r="E43" t="n">
+        <v>3</v>
+      </c>
+      <c r="F43" t="n">
+        <v>1</v>
+      </c>
+      <c r="G43" t="n">
+        <v>50</v>
+      </c>
+      <c r="H43" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="I43" t="n">
+        <v>12.5</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Muhammad Naeem</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>373694</v>
+      </c>
+      <c r="C44" t="n">
+        <v>6</v>
+      </c>
+      <c r="D44" t="n">
+        <v>3</v>
+      </c>
+      <c r="E44" t="n">
+        <v>3</v>
+      </c>
+      <c r="F44" t="n">
+        <v>0</v>
+      </c>
+      <c r="G44" t="n">
+        <v>50</v>
+      </c>
+      <c r="H44" t="n">
+        <v>50</v>
+      </c>
+      <c r="I44" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Muhammad Shahid Khan</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>373662</v>
+      </c>
+      <c r="C45" t="n">
+        <v>6</v>
+      </c>
+      <c r="D45" t="n">
+        <v>3</v>
+      </c>
+      <c r="E45" t="n">
+        <v>3</v>
+      </c>
+      <c r="F45" t="n">
+        <v>0</v>
+      </c>
+      <c r="G45" t="n">
+        <v>50</v>
+      </c>
+      <c r="H45" t="n">
+        <v>50</v>
+      </c>
+      <c r="I45" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Nillum Bibi</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>373652</v>
+      </c>
+      <c r="C46" t="n">
+        <v>169</v>
+      </c>
+      <c r="D46" t="n">
+        <v>64</v>
+      </c>
+      <c r="E46" t="n">
+        <v>61</v>
+      </c>
+      <c r="F46" t="n">
+        <v>3</v>
+      </c>
+      <c r="G46" t="n">
+        <v>37.87</v>
+      </c>
+      <c r="H46" t="n">
+        <v>36.09</v>
+      </c>
+      <c r="I46" t="n">
+        <v>1.78</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Robina Shaheen</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>373639</v>
+      </c>
+      <c r="C47" t="n">
+        <v>8</v>
+      </c>
+      <c r="D47" t="n">
+        <v>3</v>
+      </c>
+      <c r="E47" t="n">
+        <v>2</v>
+      </c>
+      <c r="F47" t="n">
+        <v>1</v>
+      </c>
+      <c r="G47" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="H47" t="n">
+        <v>25</v>
+      </c>
+      <c r="I47" t="n">
+        <v>12.5</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Sajjad Khan</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>373700</v>
+      </c>
+      <c r="C48" t="n">
+        <v>8</v>
+      </c>
+      <c r="D48" t="n">
+        <v>3</v>
+      </c>
+      <c r="E48" t="n">
+        <v>3</v>
+      </c>
+      <c r="F48" t="n">
+        <v>0</v>
+      </c>
+      <c r="G48" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="H48" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="I48" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Nazia</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>373657</v>
+      </c>
+      <c r="C49" t="n">
+        <v>144</v>
+      </c>
+      <c r="D49" t="n">
+        <v>51</v>
+      </c>
+      <c r="E49" t="n">
+        <v>49</v>
+      </c>
+      <c r="F49" t="n">
+        <v>2</v>
+      </c>
+      <c r="G49" t="n">
+        <v>35.42</v>
+      </c>
+      <c r="H49" t="n">
+        <v>34.03</v>
+      </c>
+      <c r="I49" t="n">
+        <v>1.39</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Alia Khan</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>373681</v>
+      </c>
+      <c r="C50" t="n">
+        <v>129</v>
+      </c>
+      <c r="D50" t="n">
+        <v>44</v>
+      </c>
+      <c r="E50" t="n">
+        <v>40</v>
+      </c>
+      <c r="F50" t="n">
+        <v>4</v>
+      </c>
+      <c r="G50" t="n">
+        <v>34.11</v>
+      </c>
+      <c r="H50" t="n">
+        <v>31.01</v>
+      </c>
+      <c r="I50" t="n">
+        <v>3.1</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Aisha Aman</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>373704</v>
+      </c>
+      <c r="C51" t="n">
+        <v>11</v>
+      </c>
+      <c r="D51" t="n">
+        <v>3</v>
+      </c>
+      <c r="E51" t="n">
+        <v>2</v>
+      </c>
+      <c r="F51" t="n">
+        <v>1</v>
+      </c>
+      <c r="G51" t="n">
+        <v>27.27</v>
+      </c>
+      <c r="H51" t="n">
+        <v>18.18</v>
+      </c>
+      <c r="I51" t="n">
+        <v>9.09</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Iqra Bibi</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>373708</v>
+      </c>
+      <c r="C52" t="n">
+        <v>8</v>
+      </c>
+      <c r="D52" t="n">
+        <v>2</v>
+      </c>
+      <c r="E52" t="n">
+        <v>2</v>
+      </c>
+      <c r="F52" t="n">
+        <v>0</v>
+      </c>
+      <c r="G52" t="n">
+        <v>25</v>
+      </c>
+      <c r="H52" t="n">
+        <v>25</v>
+      </c>
+      <c r="I52" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Hijab Zahra</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>373637</v>
+      </c>
+      <c r="C53" t="n">
+        <v>4</v>
+      </c>
+      <c r="D53" t="n">
+        <v>1</v>
+      </c>
+      <c r="E53" t="n">
+        <v>1</v>
+      </c>
+      <c r="F53" t="n">
+        <v>0</v>
+      </c>
+      <c r="G53" t="n">
+        <v>25</v>
+      </c>
+      <c r="H53" t="n">
+        <v>25</v>
+      </c>
+      <c r="I53" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Laiba Khan</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>373653</v>
+      </c>
+      <c r="C54" t="n">
+        <v>121</v>
+      </c>
+      <c r="D54" t="n">
+        <v>26</v>
+      </c>
+      <c r="E54" t="n">
+        <v>22</v>
+      </c>
+      <c r="F54" t="n">
+        <v>4</v>
+      </c>
+      <c r="G54" t="n">
+        <v>21.49</v>
+      </c>
+      <c r="H54" t="n">
+        <v>18.18</v>
+      </c>
+      <c r="I54" t="n">
+        <v>3.31</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Gul Rukh</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>373644</v>
+      </c>
+      <c r="C55" t="n">
+        <v>6</v>
+      </c>
+      <c r="D55" t="n">
+        <v>1</v>
+      </c>
+      <c r="E55" t="n">
+        <v>1</v>
+      </c>
+      <c r="F55" t="n">
+        <v>0</v>
+      </c>
+      <c r="G55" t="n">
+        <v>16.67</v>
+      </c>
+      <c r="H55" t="n">
+        <v>16.67</v>
+      </c>
+      <c r="I55" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Mahnoorr</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>373670</v>
+      </c>
+      <c r="C56" t="n">
+        <v>13</v>
+      </c>
+      <c r="D56" t="n">
+        <v>2</v>
+      </c>
+      <c r="E56" t="n">
+        <v>1</v>
+      </c>
+      <c r="F56" t="n">
+        <v>1</v>
+      </c>
+      <c r="G56" t="n">
+        <v>15.38</v>
+      </c>
+      <c r="H56" t="n">
+        <v>7.69</v>
+      </c>
+      <c r="I56" t="n">
+        <v>7.69</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Sidra Khan</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>373645</v>
+      </c>
+      <c r="C57" t="n">
+        <v>7</v>
+      </c>
+      <c r="D57" t="n">
+        <v>1</v>
+      </c>
+      <c r="E57" t="n">
+        <v>1</v>
+      </c>
+      <c r="F57" t="n">
+        <v>0</v>
+      </c>
+      <c r="G57" t="n">
+        <v>14.29</v>
+      </c>
+      <c r="H57" t="n">
+        <v>14.29</v>
+      </c>
+      <c r="I57" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Irum ikram (duplicate name received from listed_girl_tracking_survey on June 29, 2026 12:08 UTC+00:00; submission key: uuid:b700a976-75ee-467c-87e9-1d5163ec238d)</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>541376</v>
+      </c>
+      <c r="C58" t="n">
+        <v>64</v>
+      </c>
+      <c r="D58" t="n">
+        <v>0</v>
+      </c>
+      <c r="E58" t="n">
+        <v>0</v>
+      </c>
+      <c r="F58" t="n">
+        <v>0</v>
+      </c>
+      <c r="G58" t="n">
+        <v>0</v>
+      </c>
+      <c r="H58" t="n">
+        <v>0</v>
+      </c>
+      <c r="I58" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Lati Khan (duplicate name received from listed_girl_tracking_survey on June 28, 2026 10:43 UTC+00:00; submission key: uuid:e4e89d53-e5be-40ff-bb2c-fa94c0d50011)</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>564273</v>
+      </c>
+      <c r="C59" t="n">
+        <v>56</v>
+      </c>
+      <c r="D59" t="n">
+        <v>0</v>
+      </c>
+      <c r="E59" t="n">
+        <v>0</v>
+      </c>
+      <c r="F59" t="n">
+        <v>0</v>
+      </c>
+      <c r="G59" t="n">
+        <v>0</v>
+      </c>
+      <c r="H59" t="n">
+        <v>0</v>
+      </c>
+      <c r="I59" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Lati khan (duplicate name received from listed_girl_tracking_survey_new_sample on July 4, 2026 14:31 UTC+00:00; submission key: uuid:6316d214-c458-4786-937a-bd81b08c15c5)</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>671211</v>
+      </c>
+      <c r="C60" t="n">
+        <v>14</v>
+      </c>
+      <c r="D60" t="n">
+        <v>0</v>
+      </c>
+      <c r="E60" t="n">
+        <v>0</v>
+      </c>
+      <c r="F60" t="n">
+        <v>0</v>
+      </c>
+      <c r="G60" t="n">
+        <v>0</v>
+      </c>
+      <c r="H60" t="n">
+        <v>0</v>
+      </c>
+      <c r="I60" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Muhammad Usman</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>373666</v>
+      </c>
+      <c r="C61" t="n">
+        <v>14</v>
+      </c>
+      <c r="D61" t="n">
+        <v>0</v>
+      </c>
+      <c r="E61" t="n">
+        <v>0</v>
+      </c>
+      <c r="F61" t="n">
+        <v>0</v>
+      </c>
+      <c r="G61" t="n">
+        <v>0</v>
+      </c>
+      <c r="H61" t="n">
+        <v>0</v>
+      </c>
+      <c r="I61" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Muhammad Waseem</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
+        <v>373689</v>
+      </c>
+      <c r="C62" t="n">
+        <v>3</v>
+      </c>
+      <c r="D62" t="n">
+        <v>0</v>
+      </c>
+      <c r="E62" t="n">
+        <v>0</v>
+      </c>
+      <c r="F62" t="n">
+        <v>0</v>
+      </c>
+      <c r="G62" t="n">
+        <v>0</v>
+      </c>
+      <c r="H62" t="n">
+        <v>0</v>
+      </c>
+      <c r="I62" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Muhammad naeem (duplicate name received from primary_school_listing_survey on February 14, 2026 14:38 UTC+00:00; submission key: uuid:5f0e427e-5fd2-4474-be64-ae5f2c4617a2)</t>
+        </is>
+      </c>
+      <c r="B63" t="n">
+        <v>571571</v>
+      </c>
+      <c r="C63" t="n">
+        <v>8</v>
+      </c>
+      <c r="D63" t="n">
+        <v>0</v>
+      </c>
+      <c r="E63" t="n">
+        <v>0</v>
+      </c>
+      <c r="F63" t="n">
+        <v>0</v>
+      </c>
+      <c r="G63" t="n">
+        <v>0</v>
+      </c>
+      <c r="H63" t="n">
+        <v>0</v>
+      </c>
+      <c r="I63" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
           <t>Naureen khan (duplicate name received from listed_girl_tracking_survey_new_sample on July 7, 2026 14:41 UTC+00:00; submission key: uuid:bbf56e1f-36f5-4ebf-9e0f-df83015a0871)</t>
         </is>
       </c>
-      <c r="B17" t="n">
+      <c r="B64" t="n">
         <v>453925</v>
       </c>
-      <c r="C17" t="n">
-        <v>4</v>
-      </c>
-      <c r="D17" t="n">
-        <v>0</v>
-      </c>
-      <c r="E17" t="n">
-        <v>0</v>
-      </c>
-      <c r="F17" t="n">
-        <v>0</v>
-      </c>
-      <c r="G17" t="n">
-        <v>0</v>
-      </c>
-      <c r="H17" t="n">
-        <v>0</v>
-      </c>
-      <c r="I17" t="n">
+      <c r="C64" t="n">
+        <v>57</v>
+      </c>
+      <c r="D64" t="n">
+        <v>0</v>
+      </c>
+      <c r="E64" t="n">
+        <v>0</v>
+      </c>
+      <c r="F64" t="n">
+        <v>0</v>
+      </c>
+      <c r="G64" t="n">
+        <v>0</v>
+      </c>
+      <c r="H64" t="n">
+        <v>0</v>
+      </c>
+      <c r="I64" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Samreen</t>
+        </is>
+      </c>
+      <c r="B65" t="n">
+        <v>373711</v>
+      </c>
+      <c r="C65" t="n">
+        <v>3</v>
+      </c>
+      <c r="D65" t="n">
+        <v>0</v>
+      </c>
+      <c r="E65" t="n">
+        <v>0</v>
+      </c>
+      <c r="F65" t="n">
+        <v>0</v>
+      </c>
+      <c r="G65" t="n">
+        <v>0</v>
+      </c>
+      <c r="H65" t="n">
+        <v>0</v>
+      </c>
+      <c r="I65" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Samreen</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>639258</v>
+      </c>
+      <c r="C66" t="n">
+        <v>1</v>
+      </c>
+      <c r="D66" t="n">
+        <v>0</v>
+      </c>
+      <c r="E66" t="n">
+        <v>0</v>
+      </c>
+      <c r="F66" t="n">
+        <v>0</v>
+      </c>
+      <c r="G66" t="n">
+        <v>0</v>
+      </c>
+      <c r="H66" t="n">
+        <v>0</v>
+      </c>
+      <c r="I66" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Shafaq Zahra</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr"/>
+      <c r="C67" t="n">
+        <v>1</v>
+      </c>
+      <c r="D67" t="n">
+        <v>0</v>
+      </c>
+      <c r="E67" t="n">
+        <v>0</v>
+      </c>
+      <c r="F67" t="n">
+        <v>0</v>
+      </c>
+      <c r="G67" t="n">
+        <v>0</v>
+      </c>
+      <c r="H67" t="n">
+        <v>0</v>
+      </c>
+      <c r="I67" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Shakeel Ahmed</t>
+        </is>
+      </c>
+      <c r="B68" t="n">
+        <v>373686</v>
+      </c>
+      <c r="C68" t="n">
+        <v>3</v>
+      </c>
+      <c r="D68" t="n">
+        <v>0</v>
+      </c>
+      <c r="E68" t="n">
+        <v>0</v>
+      </c>
+      <c r="F68" t="n">
+        <v>0</v>
+      </c>
+      <c r="G68" t="n">
+        <v>0</v>
+      </c>
+      <c r="H68" t="n">
+        <v>0</v>
+      </c>
+      <c r="I68" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Syed Haider Abbas</t>
+        </is>
+      </c>
+      <c r="B69" t="n">
+        <v>373713</v>
+      </c>
+      <c r="C69" t="n">
+        <v>2</v>
+      </c>
+      <c r="D69" t="n">
+        <v>0</v>
+      </c>
+      <c r="E69" t="n">
+        <v>0</v>
+      </c>
+      <c r="F69" t="n">
+        <v>0</v>
+      </c>
+      <c r="G69" t="n">
+        <v>0</v>
+      </c>
+      <c r="H69" t="n">
+        <v>0</v>
+      </c>
+      <c r="I69" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr"/>
+      <c r="B70" t="inlineStr"/>
+      <c r="C70" t="n">
+        <v>0</v>
+      </c>
+      <c r="D70" t="n">
+        <v>0</v>
+      </c>
+      <c r="E70" t="n">
+        <v>0</v>
+      </c>
+      <c r="F70" t="n">
+        <v>0</v>
+      </c>
+      <c r="G70" t="n">
+        <v>0</v>
+      </c>
+      <c r="H70" t="n">
+        <v>0</v>
+      </c>
+      <c r="I70" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add error generation script for testing and logging
</commit_message>
<xml_diff>
--- a/Error_log/Enumerator_Performance.xlsx
+++ b/Error_log/Enumerator_Performance.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="performance" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="performance_pct" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="performance" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="performance_pct" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,16 +18,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -38,7 +35,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -46,21 +43,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -430,27 +418,27 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Enumerator Name</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Enumerator ID</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Total Issues</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Critical Issues</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Flag Issues</t>
         </is>
@@ -1567,51 +1555,51 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I69"/>
+  <dimension ref="A1:I70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>enumerator_name</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>enumerator_id</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>total_submissions</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>total_issues</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>critical_issues</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>flag_issues</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>error_pct</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>critical_error_pct</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>flag_error_pct</t>
         </is>
@@ -3720,6 +3708,31 @@
         <v>0</v>
       </c>
       <c r="I69" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr"/>
+      <c r="B70" t="inlineStr"/>
+      <c r="C70" t="n">
+        <v>0</v>
+      </c>
+      <c r="D70" t="n">
+        <v>0</v>
+      </c>
+      <c r="E70" t="n">
+        <v>0</v>
+      </c>
+      <c r="F70" t="n">
+        <v>0</v>
+      </c>
+      <c r="G70" t="n">
+        <v>0</v>
+      </c>
+      <c r="H70" t="n">
+        <v>0</v>
+      </c>
+      <c r="I70" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: update Daily_Error_Log.xlsx and Weekly_QA_Summary.xlsx with latest data
</commit_message>
<xml_diff>
--- a/Error_log/Enumerator_Performance.xlsx
+++ b/Error_log/Enumerator_Performance.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="performance" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="performance_pct" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="performance" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="performance_pct" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,16 +18,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -38,7 +35,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -46,21 +43,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -426,31 +414,31 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Enumerator Name</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Enumerator ID</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Total Issues</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Critical Issues</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Flag Issues</t>
         </is>
@@ -459,304 +447,1100 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Kainat</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>373712</v>
-      </c>
+          <t>UNASSIGNED (Tracking vs Household)</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr"/>
       <c r="C2" t="n">
-        <v>129</v>
+        <v>2238</v>
       </c>
       <c r="D2" t="n">
-        <v>69</v>
+        <v>2229</v>
       </c>
       <c r="E2" t="n">
-        <v>60</v>
+        <v>9</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Zohra</t>
+          <t>Asma Bibi</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>373692</v>
+        <v>373641</v>
       </c>
       <c r="C3" t="n">
-        <v>106</v>
+        <v>356</v>
       </c>
       <c r="D3" t="n">
-        <v>55</v>
+        <v>297</v>
       </c>
       <c r="E3" t="n">
-        <v>51</v>
+        <v>59</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Samara</t>
+          <t>Mehran Khan</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>373658</v>
+        <v>373684</v>
       </c>
       <c r="C4" t="n">
-        <v>100</v>
+        <v>293</v>
       </c>
       <c r="D4" t="n">
-        <v>48</v>
+        <v>265</v>
       </c>
       <c r="E4" t="n">
-        <v>52</v>
+        <v>28</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Rehana Bibi</t>
+          <t>Shazia Bibi</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>373691</v>
+        <v>373648</v>
       </c>
       <c r="C5" t="n">
-        <v>106</v>
+        <v>330</v>
       </c>
       <c r="D5" t="n">
-        <v>47</v>
+        <v>260</v>
       </c>
       <c r="E5" t="n">
-        <v>59</v>
+        <v>70</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Asma Bibi</t>
+          <t>Shazia begum</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>373641</v>
+        <v>373696</v>
       </c>
       <c r="C6" t="n">
-        <v>17</v>
+        <v>249</v>
       </c>
       <c r="D6" t="n">
-        <v>14</v>
+        <v>224</v>
       </c>
       <c r="E6" t="n">
-        <v>3</v>
+        <v>25</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Shazia Bibi</t>
+          <t>Shafaq Zahra</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>373648</v>
+        <v>373646</v>
       </c>
       <c r="C7" t="n">
-        <v>22</v>
+        <v>250</v>
       </c>
       <c r="D7" t="n">
-        <v>11</v>
+        <v>214</v>
       </c>
       <c r="E7" t="n">
-        <v>11</v>
+        <v>36</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Mahnoor</t>
+          <t>Irum Ikram</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>373705</v>
+        <v>373642</v>
       </c>
       <c r="C8" t="n">
-        <v>17</v>
+        <v>240</v>
       </c>
       <c r="D8" t="n">
-        <v>11</v>
+        <v>211</v>
       </c>
       <c r="E8" t="n">
-        <v>6</v>
+        <v>29</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Javairia</t>
+          <t>Sadia Rustum</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>373651</v>
+        <v>373649</v>
       </c>
       <c r="C9" t="n">
-        <v>23</v>
+        <v>192</v>
       </c>
       <c r="D9" t="n">
+        <v>182</v>
+      </c>
+      <c r="E9" t="n">
         <v>10</v>
-      </c>
-      <c r="E9" t="n">
-        <v>13</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Nadia bibi</t>
+          <t>Khalida Bibi</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>373669</v>
+        <v>373673</v>
       </c>
       <c r="C10" t="n">
-        <v>19</v>
+        <v>140</v>
       </c>
       <c r="D10" t="n">
-        <v>10</v>
+        <v>140</v>
       </c>
       <c r="E10" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Irum Ikram</t>
+          <t>Javairia</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>373642</v>
+        <v>373651</v>
       </c>
       <c r="C11" t="n">
-        <v>16</v>
+        <v>214</v>
       </c>
       <c r="D11" t="n">
-        <v>10</v>
+        <v>134</v>
       </c>
       <c r="E11" t="n">
-        <v>6</v>
+        <v>80</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Shafaq Zahra</t>
+          <t>Mahnoor</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>373646</v>
+        <v>373705</v>
       </c>
       <c r="C12" t="n">
-        <v>10</v>
+        <v>168</v>
       </c>
       <c r="D12" t="n">
-        <v>7</v>
+        <v>132</v>
       </c>
       <c r="E12" t="n">
-        <v>3</v>
+        <v>36</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Naureen Khan</t>
+          <t>Kainat</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>373716</v>
+        <v>373712</v>
       </c>
       <c r="C13" t="n">
-        <v>7</v>
+        <v>333</v>
       </c>
       <c r="D13" t="n">
-        <v>5</v>
+        <v>131</v>
       </c>
       <c r="E13" t="n">
-        <v>2</v>
+        <v>202</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Laiba Shams</t>
+          <t>Naureen Khan</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>373706</v>
+        <v>373716</v>
       </c>
       <c r="C14" t="n">
-        <v>8</v>
+        <v>133</v>
       </c>
       <c r="D14" t="n">
-        <v>4</v>
+        <v>124</v>
       </c>
       <c r="E14" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Naureen khan</t>
+          <t>Bushra Ayub</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>453925</v>
+        <v>373671</v>
       </c>
       <c r="C15" t="n">
-        <v>5</v>
+        <v>126</v>
       </c>
       <c r="D15" t="n">
+        <v>122</v>
+      </c>
+      <c r="E15" t="n">
         <v>4</v>
-      </c>
-      <c r="E15" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Shazia begum</t>
+          <t>Furqan Ullah Khan</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>373696</v>
+        <v>373683</v>
       </c>
       <c r="C16" t="n">
-        <v>3</v>
+        <v>124</v>
       </c>
       <c r="D16" t="n">
-        <v>2</v>
+        <v>116</v>
       </c>
       <c r="E16" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
+          <t>Zohra</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>373692</v>
+      </c>
+      <c r="C17" t="n">
+        <v>298</v>
+      </c>
+      <c r="D17" t="n">
+        <v>115</v>
+      </c>
+      <c r="E17" t="n">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Asma Gull</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>373672</v>
+      </c>
+      <c r="C18" t="n">
+        <v>109</v>
+      </c>
+      <c r="D18" t="n">
+        <v>105</v>
+      </c>
+      <c r="E18" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Samara</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>373658</v>
+      </c>
+      <c r="C19" t="n">
+        <v>298</v>
+      </c>
+      <c r="D19" t="n">
+        <v>102</v>
+      </c>
+      <c r="E19" t="n">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Ishaq Khan</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>373699</v>
+      </c>
+      <c r="C20" t="n">
+        <v>101</v>
+      </c>
+      <c r="D20" t="n">
+        <v>100</v>
+      </c>
+      <c r="E20" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Muhammad Yousaf</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>373690</v>
+      </c>
+      <c r="C21" t="n">
+        <v>105</v>
+      </c>
+      <c r="D21" t="n">
+        <v>96</v>
+      </c>
+      <c r="E21" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Rehana Bibi</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>373691</v>
+      </c>
+      <c r="C22" t="n">
+        <v>295</v>
+      </c>
+      <c r="D22" t="n">
+        <v>94</v>
+      </c>
+      <c r="E22" t="n">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Lati Khan</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>564273</v>
+      </c>
+      <c r="C23" t="n">
+        <v>97</v>
+      </c>
+      <c r="D23" t="n">
+        <v>93</v>
+      </c>
+      <c r="E23" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Naureen khan</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>453925</v>
+      </c>
+      <c r="C24" t="n">
+        <v>91</v>
+      </c>
+      <c r="D24" t="n">
+        <v>89</v>
+      </c>
+      <c r="E24" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Laiba Shams</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>373706</v>
+      </c>
+      <c r="C25" t="n">
+        <v>114</v>
+      </c>
+      <c r="D25" t="n">
+        <v>86</v>
+      </c>
+      <c r="E25" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Irum ikram</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>541376</v>
+      </c>
+      <c r="C26" t="n">
+        <v>88</v>
+      </c>
+      <c r="D26" t="n">
+        <v>83</v>
+      </c>
+      <c r="E26" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Lati Khan</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>373665</v>
+      </c>
+      <c r="C27" t="n">
+        <v>86</v>
+      </c>
+      <c r="D27" t="n">
+        <v>83</v>
+      </c>
+      <c r="E27" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Naureen</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>884887</v>
+      </c>
+      <c r="C28" t="n">
+        <v>86</v>
+      </c>
+      <c r="D28" t="n">
+        <v>82</v>
+      </c>
+      <c r="E28" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Jaweria</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>163495</v>
+      </c>
+      <c r="C29" t="n">
+        <v>83</v>
+      </c>
+      <c r="D29" t="n">
+        <v>82</v>
+      </c>
+      <c r="E29" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Nillum Bibi</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>373652</v>
+      </c>
+      <c r="C30" t="n">
+        <v>64</v>
+      </c>
+      <c r="D30" t="n">
+        <v>61</v>
+      </c>
+      <c r="E30" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Anum Gul</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>373656</v>
+      </c>
+      <c r="C31" t="n">
+        <v>55</v>
+      </c>
+      <c r="D31" t="n">
+        <v>51</v>
+      </c>
+      <c r="E31" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Muniba Shamim</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>373659</v>
+      </c>
+      <c r="C32" t="n">
+        <v>58</v>
+      </c>
+      <c r="D32" t="n">
+        <v>49</v>
+      </c>
+      <c r="E32" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Nazia</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>373657</v>
+      </c>
+      <c r="C33" t="n">
+        <v>51</v>
+      </c>
+      <c r="D33" t="n">
+        <v>49</v>
+      </c>
+      <c r="E33" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Alia Khan</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>373681</v>
+      </c>
+      <c r="C34" t="n">
+        <v>44</v>
+      </c>
+      <c r="D34" t="n">
+        <v>40</v>
+      </c>
+      <c r="E34" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Lati khan</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>671211</v>
+      </c>
+      <c r="C35" t="n">
+        <v>38</v>
+      </c>
+      <c r="D35" t="n">
+        <v>38</v>
+      </c>
+      <c r="E35" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
           <t>Summiya Hayat</t>
         </is>
       </c>
-      <c r="B17" t="n">
+      <c r="B36" t="n">
         <v>373710</v>
       </c>
-      <c r="C17" t="n">
+      <c r="C36" t="n">
+        <v>60</v>
+      </c>
+      <c r="D36" t="n">
+        <v>33</v>
+      </c>
+      <c r="E36" t="n">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Munawar Khan</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>373668</v>
+      </c>
+      <c r="C37" t="n">
+        <v>38</v>
+      </c>
+      <c r="D37" t="n">
+        <v>32</v>
+      </c>
+      <c r="E37" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Laiba Khan</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>373653</v>
+      </c>
+      <c r="C38" t="n">
+        <v>26</v>
+      </c>
+      <c r="D38" t="n">
+        <v>22</v>
+      </c>
+      <c r="E38" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Chashm Gul</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>373695</v>
+      </c>
+      <c r="C39" t="n">
+        <v>27</v>
+      </c>
+      <c r="D39" t="n">
+        <v>18</v>
+      </c>
+      <c r="E39" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Nadia bibi</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>373669</v>
+      </c>
+      <c r="C40" t="n">
+        <v>41</v>
+      </c>
+      <c r="D40" t="n">
+        <v>15</v>
+      </c>
+      <c r="E40" t="n">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Zain Ul Abideen</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>373667</v>
+      </c>
+      <c r="C41" t="n">
+        <v>12</v>
+      </c>
+      <c r="D41" t="n">
+        <v>12</v>
+      </c>
+      <c r="E41" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Lati khan</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>652938</v>
+      </c>
+      <c r="C42" t="n">
+        <v>10</v>
+      </c>
+      <c r="D42" t="n">
+        <v>10</v>
+      </c>
+      <c r="E42" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Saba Ramzan</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>373703</v>
+      </c>
+      <c r="C43" t="n">
+        <v>9</v>
+      </c>
+      <c r="D43" t="n">
+        <v>9</v>
+      </c>
+      <c r="E43" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Shehla Noor</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>373650</v>
+      </c>
+      <c r="C44" t="n">
+        <v>9</v>
+      </c>
+      <c r="D44" t="n">
+        <v>9</v>
+      </c>
+      <c r="E44" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Muhammad naeem</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>571571</v>
+      </c>
+      <c r="C45" t="n">
+        <v>10</v>
+      </c>
+      <c r="D45" t="n">
+        <v>8</v>
+      </c>
+      <c r="E45" t="n">
         <v>2</v>
       </c>
-      <c r="D17" t="n">
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Sadia rustum</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>852541</v>
+      </c>
+      <c r="C46" t="n">
+        <v>5</v>
+      </c>
+      <c r="D46" t="n">
+        <v>5</v>
+      </c>
+      <c r="E46" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Usman Ali</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>373687</v>
+      </c>
+      <c r="C47" t="n">
+        <v>5</v>
+      </c>
+      <c r="D47" t="n">
+        <v>5</v>
+      </c>
+      <c r="E47" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Muhammad Noor</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>373701</v>
+      </c>
+      <c r="C48" t="n">
+        <v>4</v>
+      </c>
+      <c r="D48" t="n">
+        <v>3</v>
+      </c>
+      <c r="E48" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Muhammad Naeem</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>373694</v>
+      </c>
+      <c r="C49" t="n">
+        <v>3</v>
+      </c>
+      <c r="D49" t="n">
+        <v>3</v>
+      </c>
+      <c r="E49" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Muhammad Shahid Khan</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>373662</v>
+      </c>
+      <c r="C50" t="n">
+        <v>3</v>
+      </c>
+      <c r="D50" t="n">
+        <v>3</v>
+      </c>
+      <c r="E50" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Sajjad Khan</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>373700</v>
+      </c>
+      <c r="C51" t="n">
+        <v>3</v>
+      </c>
+      <c r="D51" t="n">
+        <v>3</v>
+      </c>
+      <c r="E51" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Aisha Aman</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>373704</v>
+      </c>
+      <c r="C52" t="n">
+        <v>3</v>
+      </c>
+      <c r="D52" t="n">
         <v>2</v>
       </c>
-      <c r="E17" t="n">
+      <c r="E52" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Rahila Naaz</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>373715</v>
+      </c>
+      <c r="C53" t="n">
+        <v>3</v>
+      </c>
+      <c r="D53" t="n">
+        <v>2</v>
+      </c>
+      <c r="E53" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Robina Shaheen</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>373639</v>
+      </c>
+      <c r="C54" t="n">
+        <v>3</v>
+      </c>
+      <c r="D54" t="n">
+        <v>2</v>
+      </c>
+      <c r="E54" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Iqra Bibi</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>373708</v>
+      </c>
+      <c r="C55" t="n">
+        <v>2</v>
+      </c>
+      <c r="D55" t="n">
+        <v>2</v>
+      </c>
+      <c r="E55" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Mahnoorr</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>373670</v>
+      </c>
+      <c r="C56" t="n">
+        <v>2</v>
+      </c>
+      <c r="D56" t="n">
+        <v>1</v>
+      </c>
+      <c r="E56" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Gul Rukh</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>373644</v>
+      </c>
+      <c r="C57" t="n">
+        <v>1</v>
+      </c>
+      <c r="D57" t="n">
+        <v>1</v>
+      </c>
+      <c r="E57" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Hijab Zahra</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>373637</v>
+      </c>
+      <c r="C58" t="n">
+        <v>1</v>
+      </c>
+      <c r="D58" t="n">
+        <v>1</v>
+      </c>
+      <c r="E58" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Sidra Khan</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>373645</v>
+      </c>
+      <c r="C59" t="n">
+        <v>1</v>
+      </c>
+      <c r="D59" t="n">
+        <v>1</v>
+      </c>
+      <c r="E59" t="n">
         <v>0</v>
       </c>
     </row>
@@ -771,51 +1555,51 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:I70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>enumerator_name</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>enumerator_id</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>total_submissions</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>total_issues</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>critical_issues</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>flag_issues</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>error_pct</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>critical_error_pct</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>flag_error_pct</t>
         </is>
@@ -824,496 +1608,2131 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Kainat</t>
+          <t>Naureen khan</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>373712</v>
+        <v>453925</v>
       </c>
       <c r="C2" t="n">
-        <v>33</v>
+        <v>2</v>
       </c>
       <c r="D2" t="n">
-        <v>129</v>
+        <v>91</v>
       </c>
       <c r="E2" t="n">
-        <v>69</v>
+        <v>89</v>
       </c>
       <c r="F2" t="n">
-        <v>60</v>
+        <v>2</v>
       </c>
       <c r="G2" t="n">
-        <v>390.91</v>
+        <v>4550</v>
       </c>
       <c r="H2" t="n">
-        <v>209.09</v>
+        <v>4450</v>
       </c>
       <c r="I2" t="n">
-        <v>181.82</v>
+        <v>100</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Zohra</t>
+          <t>Irum ikram</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>373692</v>
+        <v>541376</v>
       </c>
       <c r="C3" t="n">
-        <v>29</v>
+        <v>8</v>
       </c>
       <c r="D3" t="n">
-        <v>106</v>
+        <v>88</v>
       </c>
       <c r="E3" t="n">
-        <v>55</v>
+        <v>83</v>
       </c>
       <c r="F3" t="n">
-        <v>51</v>
+        <v>5</v>
       </c>
       <c r="G3" t="n">
-        <v>365.52</v>
+        <v>1100</v>
       </c>
       <c r="H3" t="n">
-        <v>189.66</v>
+        <v>1037.5</v>
       </c>
       <c r="I3" t="n">
-        <v>175.86</v>
+        <v>62.5</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Samara</t>
+          <t>Lati Khan</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>373658</v>
+        <v>564273</v>
       </c>
       <c r="C4" t="n">
-        <v>31</v>
+        <v>9</v>
       </c>
       <c r="D4" t="n">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="E4" t="n">
-        <v>48</v>
+        <v>93</v>
       </c>
       <c r="F4" t="n">
-        <v>52</v>
+        <v>4</v>
       </c>
       <c r="G4" t="n">
-        <v>322.58</v>
+        <v>1077.78</v>
       </c>
       <c r="H4" t="n">
-        <v>154.84</v>
+        <v>1033.33</v>
       </c>
       <c r="I4" t="n">
-        <v>167.74</v>
+        <v>44.44</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Rehana Bibi</t>
+          <t>Lati khan</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>373691</v>
+        <v>671211</v>
       </c>
       <c r="C5" t="n">
-        <v>33</v>
+        <v>9</v>
       </c>
       <c r="D5" t="n">
-        <v>106</v>
+        <v>38</v>
       </c>
       <c r="E5" t="n">
-        <v>47</v>
+        <v>38</v>
       </c>
       <c r="F5" t="n">
-        <v>59</v>
+        <v>0</v>
       </c>
       <c r="G5" t="n">
-        <v>321.21</v>
+        <v>422.22</v>
       </c>
       <c r="H5" t="n">
-        <v>142.42</v>
+        <v>422.22</v>
       </c>
       <c r="I5" t="n">
-        <v>178.79</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Javairia</t>
+          <t>Kainat</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>373651</v>
+        <v>373712</v>
       </c>
       <c r="C6" t="n">
-        <v>8</v>
+        <v>104</v>
       </c>
       <c r="D6" t="n">
-        <v>23</v>
+        <v>333</v>
       </c>
       <c r="E6" t="n">
-        <v>10</v>
+        <v>131</v>
       </c>
       <c r="F6" t="n">
-        <v>13</v>
+        <v>202</v>
       </c>
       <c r="G6" t="n">
-        <v>287.5</v>
+        <v>320.19</v>
       </c>
       <c r="H6" t="n">
-        <v>125</v>
+        <v>125.96</v>
       </c>
       <c r="I6" t="n">
-        <v>162.5</v>
+        <v>194.23</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Nadia bibi</t>
+          <t>Zohra</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>373669</v>
+        <v>373692</v>
       </c>
       <c r="C7" t="n">
-        <v>8</v>
+        <v>101</v>
       </c>
       <c r="D7" t="n">
-        <v>19</v>
+        <v>298</v>
       </c>
       <c r="E7" t="n">
-        <v>10</v>
+        <v>115</v>
       </c>
       <c r="F7" t="n">
-        <v>9</v>
+        <v>183</v>
       </c>
       <c r="G7" t="n">
-        <v>237.5</v>
+        <v>295.05</v>
       </c>
       <c r="H7" t="n">
-        <v>125</v>
+        <v>113.86</v>
       </c>
       <c r="I7" t="n">
-        <v>112.5</v>
+        <v>181.19</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Irum Ikram</t>
+          <t>Rehana Bibi</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>373642</v>
+        <v>373691</v>
       </c>
       <c r="C8" t="n">
-        <v>8</v>
+        <v>111</v>
       </c>
       <c r="D8" t="n">
-        <v>16</v>
+        <v>295</v>
       </c>
       <c r="E8" t="n">
-        <v>10</v>
+        <v>94</v>
       </c>
       <c r="F8" t="n">
-        <v>6</v>
+        <v>201</v>
       </c>
       <c r="G8" t="n">
-        <v>200</v>
+        <v>265.77</v>
       </c>
       <c r="H8" t="n">
-        <v>125</v>
+        <v>84.68000000000001</v>
       </c>
       <c r="I8" t="n">
-        <v>75</v>
+        <v>181.08</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Naureen Khan</t>
+          <t>Samara</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>373716</v>
+        <v>373658</v>
       </c>
       <c r="C9" t="n">
-        <v>4</v>
+        <v>120</v>
       </c>
       <c r="D9" t="n">
-        <v>7</v>
+        <v>298</v>
       </c>
       <c r="E9" t="n">
-        <v>5</v>
+        <v>102</v>
       </c>
       <c r="F9" t="n">
-        <v>2</v>
+        <v>196</v>
       </c>
       <c r="G9" t="n">
-        <v>175</v>
+        <v>248.33</v>
       </c>
       <c r="H9" t="n">
-        <v>125</v>
+        <v>85</v>
       </c>
       <c r="I9" t="n">
-        <v>50</v>
+        <v>163.33</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Asma Bibi</t>
+          <t>Naureen Khan</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>373641</v>
+        <v>373716</v>
       </c>
       <c r="C10" t="n">
-        <v>10</v>
+        <v>81</v>
       </c>
       <c r="D10" t="n">
-        <v>17</v>
+        <v>133</v>
       </c>
       <c r="E10" t="n">
-        <v>14</v>
+        <v>124</v>
       </c>
       <c r="F10" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="G10" t="n">
-        <v>170</v>
+        <v>164.2</v>
       </c>
       <c r="H10" t="n">
-        <v>140</v>
+        <v>153.09</v>
       </c>
       <c r="I10" t="n">
-        <v>30</v>
+        <v>11.11</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Mahnoor</t>
+          <t>Asma Bibi</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>373705</v>
+        <v>373641</v>
       </c>
       <c r="C11" t="n">
-        <v>10</v>
+        <v>218</v>
       </c>
       <c r="D11" t="n">
-        <v>17</v>
+        <v>356</v>
       </c>
       <c r="E11" t="n">
-        <v>11</v>
+        <v>297</v>
       </c>
       <c r="F11" t="n">
-        <v>6</v>
+        <v>59</v>
       </c>
       <c r="G11" t="n">
-        <v>170</v>
+        <v>163.3</v>
       </c>
       <c r="H11" t="n">
-        <v>110</v>
+        <v>136.24</v>
       </c>
       <c r="I11" t="n">
-        <v>60</v>
+        <v>27.06</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Shazia Bibi</t>
+          <t>Javairia</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>373648</v>
+        <v>373651</v>
       </c>
       <c r="C12" t="n">
-        <v>13</v>
+        <v>141</v>
       </c>
       <c r="D12" t="n">
-        <v>22</v>
+        <v>214</v>
       </c>
       <c r="E12" t="n">
-        <v>11</v>
+        <v>134</v>
       </c>
       <c r="F12" t="n">
-        <v>11</v>
+        <v>80</v>
       </c>
       <c r="G12" t="n">
-        <v>169.23</v>
+        <v>151.77</v>
       </c>
       <c r="H12" t="n">
-        <v>84.62</v>
+        <v>95.04000000000001</v>
       </c>
       <c r="I12" t="n">
-        <v>84.62</v>
+        <v>56.74</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Shafaq Zahra</t>
+          <t>Shazia Bibi</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>373646</v>
+        <v>373648</v>
       </c>
       <c r="C13" t="n">
-        <v>6</v>
+        <v>223</v>
       </c>
       <c r="D13" t="n">
-        <v>10</v>
+        <v>330</v>
       </c>
       <c r="E13" t="n">
-        <v>7</v>
+        <v>260</v>
       </c>
       <c r="F13" t="n">
-        <v>3</v>
+        <v>70</v>
       </c>
       <c r="G13" t="n">
-        <v>166.67</v>
+        <v>147.98</v>
       </c>
       <c r="H13" t="n">
-        <v>116.67</v>
+        <v>116.59</v>
       </c>
       <c r="I13" t="n">
-        <v>50</v>
+        <v>31.39</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Shazia begum</t>
+          <t>Mehran Khan</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>373696</v>
+        <v>373684</v>
       </c>
       <c r="C14" t="n">
-        <v>2</v>
+        <v>200</v>
       </c>
       <c r="D14" t="n">
-        <v>3</v>
+        <v>293</v>
       </c>
       <c r="E14" t="n">
-        <v>2</v>
+        <v>265</v>
       </c>
       <c r="F14" t="n">
-        <v>1</v>
+        <v>28</v>
       </c>
       <c r="G14" t="n">
-        <v>150</v>
+        <v>146.5</v>
       </c>
       <c r="H14" t="n">
-        <v>100</v>
+        <v>132.5</v>
       </c>
       <c r="I14" t="n">
-        <v>50</v>
+        <v>14</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Laiba Shams</t>
+          <t>Lati Khan</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>373706</v>
+        <v>373665</v>
       </c>
       <c r="C15" t="n">
-        <v>8</v>
+        <v>60</v>
       </c>
       <c r="D15" t="n">
-        <v>8</v>
+        <v>86</v>
       </c>
       <c r="E15" t="n">
-        <v>4</v>
+        <v>83</v>
       </c>
       <c r="F15" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G15" t="n">
-        <v>100</v>
+        <v>143.33</v>
       </c>
       <c r="H15" t="n">
-        <v>50</v>
+        <v>138.33</v>
       </c>
       <c r="I15" t="n">
-        <v>50</v>
+        <v>5</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Summiya Hayat</t>
+          <t>Naureen</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>373710</v>
+        <v>884887</v>
       </c>
       <c r="C16" t="n">
-        <v>5</v>
+        <v>60</v>
       </c>
       <c r="D16" t="n">
-        <v>2</v>
+        <v>86</v>
       </c>
       <c r="E16" t="n">
-        <v>2</v>
+        <v>82</v>
       </c>
       <c r="F16" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G16" t="n">
-        <v>40</v>
+        <v>143.33</v>
       </c>
       <c r="H16" t="n">
-        <v>40</v>
+        <v>136.67</v>
       </c>
       <c r="I16" t="n">
-        <v>0</v>
+        <v>6.67</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
+          <t>Nadia bibi</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>373669</v>
+      </c>
+      <c r="C17" t="n">
+        <v>29</v>
+      </c>
+      <c r="D17" t="n">
+        <v>41</v>
+      </c>
+      <c r="E17" t="n">
+        <v>15</v>
+      </c>
+      <c r="F17" t="n">
+        <v>26</v>
+      </c>
+      <c r="G17" t="n">
+        <v>141.38</v>
+      </c>
+      <c r="H17" t="n">
+        <v>51.72</v>
+      </c>
+      <c r="I17" t="n">
+        <v>89.66</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Mahnoor</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>373705</v>
+      </c>
+      <c r="C18" t="n">
+        <v>119</v>
+      </c>
+      <c r="D18" t="n">
+        <v>168</v>
+      </c>
+      <c r="E18" t="n">
+        <v>132</v>
+      </c>
+      <c r="F18" t="n">
+        <v>36</v>
+      </c>
+      <c r="G18" t="n">
+        <v>141.18</v>
+      </c>
+      <c r="H18" t="n">
+        <v>110.92</v>
+      </c>
+      <c r="I18" t="n">
+        <v>30.25</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Irum Ikram</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>373642</v>
+      </c>
+      <c r="C19" t="n">
+        <v>172</v>
+      </c>
+      <c r="D19" t="n">
+        <v>240</v>
+      </c>
+      <c r="E19" t="n">
+        <v>211</v>
+      </c>
+      <c r="F19" t="n">
+        <v>29</v>
+      </c>
+      <c r="G19" t="n">
+        <v>139.53</v>
+      </c>
+      <c r="H19" t="n">
+        <v>122.67</v>
+      </c>
+      <c r="I19" t="n">
+        <v>16.86</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Shazia begum</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>373696</v>
+      </c>
+      <c r="C20" t="n">
+        <v>185</v>
+      </c>
+      <c r="D20" t="n">
+        <v>249</v>
+      </c>
+      <c r="E20" t="n">
+        <v>224</v>
+      </c>
+      <c r="F20" t="n">
+        <v>25</v>
+      </c>
+      <c r="G20" t="n">
+        <v>134.59</v>
+      </c>
+      <c r="H20" t="n">
+        <v>121.08</v>
+      </c>
+      <c r="I20" t="n">
+        <v>13.51</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Sadia Rustum</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>373649</v>
+      </c>
+      <c r="C21" t="n">
+        <v>152</v>
+      </c>
+      <c r="D21" t="n">
+        <v>192</v>
+      </c>
+      <c r="E21" t="n">
+        <v>182</v>
+      </c>
+      <c r="F21" t="n">
+        <v>10</v>
+      </c>
+      <c r="G21" t="n">
+        <v>126.32</v>
+      </c>
+      <c r="H21" t="n">
+        <v>119.74</v>
+      </c>
+      <c r="I21" t="n">
+        <v>6.58</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Jaweria</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>163495</v>
+      </c>
+      <c r="C22" t="n">
+        <v>68</v>
+      </c>
+      <c r="D22" t="n">
+        <v>83</v>
+      </c>
+      <c r="E22" t="n">
+        <v>82</v>
+      </c>
+      <c r="F22" t="n">
+        <v>1</v>
+      </c>
+      <c r="G22" t="n">
+        <v>122.06</v>
+      </c>
+      <c r="H22" t="n">
+        <v>120.59</v>
+      </c>
+      <c r="I22" t="n">
+        <v>1.47</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Shafaq Zahra</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>373646</v>
+      </c>
+      <c r="C23" t="n">
+        <v>223</v>
+      </c>
+      <c r="D23" t="n">
+        <v>250</v>
+      </c>
+      <c r="E23" t="n">
+        <v>214</v>
+      </c>
+      <c r="F23" t="n">
+        <v>36</v>
+      </c>
+      <c r="G23" t="n">
+        <v>112.11</v>
+      </c>
+      <c r="H23" t="n">
+        <v>95.95999999999999</v>
+      </c>
+      <c r="I23" t="n">
+        <v>16.14</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Laiba Shams</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>373706</v>
+      </c>
+      <c r="C24" t="n">
+        <v>114</v>
+      </c>
+      <c r="D24" t="n">
+        <v>114</v>
+      </c>
+      <c r="E24" t="n">
+        <v>86</v>
+      </c>
+      <c r="F24" t="n">
+        <v>28</v>
+      </c>
+      <c r="G24" t="n">
+        <v>100</v>
+      </c>
+      <c r="H24" t="n">
+        <v>75.44</v>
+      </c>
+      <c r="I24" t="n">
+        <v>24.56</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Zain Ul Abideen</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>373667</v>
+      </c>
+      <c r="C25" t="n">
+        <v>13</v>
+      </c>
+      <c r="D25" t="n">
+        <v>12</v>
+      </c>
+      <c r="E25" t="n">
+        <v>12</v>
+      </c>
+      <c r="F25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G25" t="n">
+        <v>92.31</v>
+      </c>
+      <c r="H25" t="n">
+        <v>92.31</v>
+      </c>
+      <c r="I25" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Bushra Ayub</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>373671</v>
+      </c>
+      <c r="C26" t="n">
+        <v>138</v>
+      </c>
+      <c r="D26" t="n">
+        <v>126</v>
+      </c>
+      <c r="E26" t="n">
+        <v>122</v>
+      </c>
+      <c r="F26" t="n">
+        <v>4</v>
+      </c>
+      <c r="G26" t="n">
+        <v>91.3</v>
+      </c>
+      <c r="H26" t="n">
+        <v>88.41</v>
+      </c>
+      <c r="I26" t="n">
+        <v>2.9</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Lati khan</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>652938</v>
+      </c>
+      <c r="C27" t="n">
+        <v>11</v>
+      </c>
+      <c r="D27" t="n">
+        <v>10</v>
+      </c>
+      <c r="E27" t="n">
+        <v>10</v>
+      </c>
+      <c r="F27" t="n">
+        <v>0</v>
+      </c>
+      <c r="G27" t="n">
+        <v>90.91</v>
+      </c>
+      <c r="H27" t="n">
+        <v>90.91</v>
+      </c>
+      <c r="I27" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Chashm Gul</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>373695</v>
+      </c>
+      <c r="C28" t="n">
+        <v>31</v>
+      </c>
+      <c r="D28" t="n">
+        <v>27</v>
+      </c>
+      <c r="E28" t="n">
+        <v>18</v>
+      </c>
+      <c r="F28" t="n">
+        <v>9</v>
+      </c>
+      <c r="G28" t="n">
+        <v>87.09999999999999</v>
+      </c>
+      <c r="H28" t="n">
+        <v>58.06</v>
+      </c>
+      <c r="I28" t="n">
+        <v>29.03</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Muniba Shamim</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>373659</v>
+      </c>
+      <c r="C29" t="n">
+        <v>72</v>
+      </c>
+      <c r="D29" t="n">
+        <v>58</v>
+      </c>
+      <c r="E29" t="n">
+        <v>49</v>
+      </c>
+      <c r="F29" t="n">
+        <v>9</v>
+      </c>
+      <c r="G29" t="n">
+        <v>80.56</v>
+      </c>
+      <c r="H29" t="n">
+        <v>68.06</v>
+      </c>
+      <c r="I29" t="n">
+        <v>12.5</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Muhammad Yousaf</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>373690</v>
+      </c>
+      <c r="C30" t="n">
+        <v>132</v>
+      </c>
+      <c r="D30" t="n">
+        <v>105</v>
+      </c>
+      <c r="E30" t="n">
+        <v>96</v>
+      </c>
+      <c r="F30" t="n">
+        <v>9</v>
+      </c>
+      <c r="G30" t="n">
+        <v>79.55</v>
+      </c>
+      <c r="H30" t="n">
+        <v>72.73</v>
+      </c>
+      <c r="I30" t="n">
+        <v>6.82</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Khalida Bibi</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>373673</v>
+      </c>
+      <c r="C31" t="n">
+        <v>177</v>
+      </c>
+      <c r="D31" t="n">
+        <v>140</v>
+      </c>
+      <c r="E31" t="n">
+        <v>140</v>
+      </c>
+      <c r="F31" t="n">
+        <v>0</v>
+      </c>
+      <c r="G31" t="n">
+        <v>79.09999999999999</v>
+      </c>
+      <c r="H31" t="n">
+        <v>79.09999999999999</v>
+      </c>
+      <c r="I31" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Asma Gull</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>373672</v>
+      </c>
+      <c r="C32" t="n">
+        <v>144</v>
+      </c>
+      <c r="D32" t="n">
+        <v>109</v>
+      </c>
+      <c r="E32" t="n">
+        <v>105</v>
+      </c>
+      <c r="F32" t="n">
+        <v>4</v>
+      </c>
+      <c r="G32" t="n">
+        <v>75.69</v>
+      </c>
+      <c r="H32" t="n">
+        <v>72.92</v>
+      </c>
+      <c r="I32" t="n">
+        <v>2.78</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Rahila Naaz</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>373715</v>
+      </c>
+      <c r="C33" t="n">
+        <v>4</v>
+      </c>
+      <c r="D33" t="n">
+        <v>3</v>
+      </c>
+      <c r="E33" t="n">
+        <v>2</v>
+      </c>
+      <c r="F33" t="n">
+        <v>1</v>
+      </c>
+      <c r="G33" t="n">
+        <v>75</v>
+      </c>
+      <c r="H33" t="n">
+        <v>50</v>
+      </c>
+      <c r="I33" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Sadia rustum</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>852541</v>
+      </c>
+      <c r="C34" t="n">
+        <v>7</v>
+      </c>
+      <c r="D34" t="n">
+        <v>5</v>
+      </c>
+      <c r="E34" t="n">
+        <v>5</v>
+      </c>
+      <c r="F34" t="n">
+        <v>0</v>
+      </c>
+      <c r="G34" t="n">
+        <v>71.43000000000001</v>
+      </c>
+      <c r="H34" t="n">
+        <v>71.43000000000001</v>
+      </c>
+      <c r="I34" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Saba Ramzan</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>373703</v>
+      </c>
+      <c r="C35" t="n">
+        <v>13</v>
+      </c>
+      <c r="D35" t="n">
+        <v>9</v>
+      </c>
+      <c r="E35" t="n">
+        <v>9</v>
+      </c>
+      <c r="F35" t="n">
+        <v>0</v>
+      </c>
+      <c r="G35" t="n">
+        <v>69.23</v>
+      </c>
+      <c r="H35" t="n">
+        <v>69.23</v>
+      </c>
+      <c r="I35" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Shehla Noor</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>373650</v>
+      </c>
+      <c r="C36" t="n">
+        <v>14</v>
+      </c>
+      <c r="D36" t="n">
+        <v>9</v>
+      </c>
+      <c r="E36" t="n">
+        <v>9</v>
+      </c>
+      <c r="F36" t="n">
+        <v>0</v>
+      </c>
+      <c r="G36" t="n">
+        <v>64.29000000000001</v>
+      </c>
+      <c r="H36" t="n">
+        <v>64.29000000000001</v>
+      </c>
+      <c r="I36" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Summiya Hayat</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>373710</v>
+      </c>
+      <c r="C37" t="n">
+        <v>94</v>
+      </c>
+      <c r="D37" t="n">
+        <v>60</v>
+      </c>
+      <c r="E37" t="n">
+        <v>33</v>
+      </c>
+      <c r="F37" t="n">
+        <v>27</v>
+      </c>
+      <c r="G37" t="n">
+        <v>63.83</v>
+      </c>
+      <c r="H37" t="n">
+        <v>35.11</v>
+      </c>
+      <c r="I37" t="n">
+        <v>28.72</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Furqan Ullah Khan</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>373683</v>
+      </c>
+      <c r="C38" t="n">
+        <v>195</v>
+      </c>
+      <c r="D38" t="n">
+        <v>124</v>
+      </c>
+      <c r="E38" t="n">
+        <v>116</v>
+      </c>
+      <c r="F38" t="n">
+        <v>8</v>
+      </c>
+      <c r="G38" t="n">
+        <v>63.59</v>
+      </c>
+      <c r="H38" t="n">
+        <v>59.49</v>
+      </c>
+      <c r="I38" t="n">
+        <v>4.1</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Usman Ali</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>373687</v>
+      </c>
+      <c r="C39" t="n">
+        <v>8</v>
+      </c>
+      <c r="D39" t="n">
+        <v>5</v>
+      </c>
+      <c r="E39" t="n">
+        <v>5</v>
+      </c>
+      <c r="F39" t="n">
+        <v>0</v>
+      </c>
+      <c r="G39" t="n">
+        <v>62.5</v>
+      </c>
+      <c r="H39" t="n">
+        <v>62.5</v>
+      </c>
+      <c r="I39" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Ishaq Khan</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>373699</v>
+      </c>
+      <c r="C40" t="n">
+        <v>170</v>
+      </c>
+      <c r="D40" t="n">
+        <v>101</v>
+      </c>
+      <c r="E40" t="n">
+        <v>100</v>
+      </c>
+      <c r="F40" t="n">
+        <v>1</v>
+      </c>
+      <c r="G40" t="n">
+        <v>59.41</v>
+      </c>
+      <c r="H40" t="n">
+        <v>58.82</v>
+      </c>
+      <c r="I40" t="n">
+        <v>0.59</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Anum Gul</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>373656</v>
+      </c>
+      <c r="C41" t="n">
+        <v>103</v>
+      </c>
+      <c r="D41" t="n">
+        <v>55</v>
+      </c>
+      <c r="E41" t="n">
+        <v>51</v>
+      </c>
+      <c r="F41" t="n">
+        <v>4</v>
+      </c>
+      <c r="G41" t="n">
+        <v>53.4</v>
+      </c>
+      <c r="H41" t="n">
+        <v>49.51</v>
+      </c>
+      <c r="I41" t="n">
+        <v>3.88</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Munawar Khan</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>373668</v>
+      </c>
+      <c r="C42" t="n">
+        <v>73</v>
+      </c>
+      <c r="D42" t="n">
+        <v>38</v>
+      </c>
+      <c r="E42" t="n">
+        <v>32</v>
+      </c>
+      <c r="F42" t="n">
+        <v>6</v>
+      </c>
+      <c r="G42" t="n">
+        <v>52.05</v>
+      </c>
+      <c r="H42" t="n">
+        <v>43.84</v>
+      </c>
+      <c r="I42" t="n">
+        <v>8.220000000000001</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Muhammad Noor</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>373701</v>
+      </c>
+      <c r="C43" t="n">
+        <v>8</v>
+      </c>
+      <c r="D43" t="n">
+        <v>4</v>
+      </c>
+      <c r="E43" t="n">
+        <v>3</v>
+      </c>
+      <c r="F43" t="n">
+        <v>1</v>
+      </c>
+      <c r="G43" t="n">
+        <v>50</v>
+      </c>
+      <c r="H43" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="I43" t="n">
+        <v>12.5</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Muhammad Naeem</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>373694</v>
+      </c>
+      <c r="C44" t="n">
+        <v>6</v>
+      </c>
+      <c r="D44" t="n">
+        <v>3</v>
+      </c>
+      <c r="E44" t="n">
+        <v>3</v>
+      </c>
+      <c r="F44" t="n">
+        <v>0</v>
+      </c>
+      <c r="G44" t="n">
+        <v>50</v>
+      </c>
+      <c r="H44" t="n">
+        <v>50</v>
+      </c>
+      <c r="I44" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Muhammad Shahid Khan</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>373662</v>
+      </c>
+      <c r="C45" t="n">
+        <v>6</v>
+      </c>
+      <c r="D45" t="n">
+        <v>3</v>
+      </c>
+      <c r="E45" t="n">
+        <v>3</v>
+      </c>
+      <c r="F45" t="n">
+        <v>0</v>
+      </c>
+      <c r="G45" t="n">
+        <v>50</v>
+      </c>
+      <c r="H45" t="n">
+        <v>50</v>
+      </c>
+      <c r="I45" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Nillum Bibi</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>373652</v>
+      </c>
+      <c r="C46" t="n">
+        <v>169</v>
+      </c>
+      <c r="D46" t="n">
+        <v>64</v>
+      </c>
+      <c r="E46" t="n">
+        <v>61</v>
+      </c>
+      <c r="F46" t="n">
+        <v>3</v>
+      </c>
+      <c r="G46" t="n">
+        <v>37.87</v>
+      </c>
+      <c r="H46" t="n">
+        <v>36.09</v>
+      </c>
+      <c r="I46" t="n">
+        <v>1.78</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Robina Shaheen</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>373639</v>
+      </c>
+      <c r="C47" t="n">
+        <v>8</v>
+      </c>
+      <c r="D47" t="n">
+        <v>3</v>
+      </c>
+      <c r="E47" t="n">
+        <v>2</v>
+      </c>
+      <c r="F47" t="n">
+        <v>1</v>
+      </c>
+      <c r="G47" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="H47" t="n">
+        <v>25</v>
+      </c>
+      <c r="I47" t="n">
+        <v>12.5</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Sajjad Khan</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>373700</v>
+      </c>
+      <c r="C48" t="n">
+        <v>8</v>
+      </c>
+      <c r="D48" t="n">
+        <v>3</v>
+      </c>
+      <c r="E48" t="n">
+        <v>3</v>
+      </c>
+      <c r="F48" t="n">
+        <v>0</v>
+      </c>
+      <c r="G48" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="H48" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="I48" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Nazia</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>373657</v>
+      </c>
+      <c r="C49" t="n">
+        <v>144</v>
+      </c>
+      <c r="D49" t="n">
+        <v>51</v>
+      </c>
+      <c r="E49" t="n">
+        <v>49</v>
+      </c>
+      <c r="F49" t="n">
+        <v>2</v>
+      </c>
+      <c r="G49" t="n">
+        <v>35.42</v>
+      </c>
+      <c r="H49" t="n">
+        <v>34.03</v>
+      </c>
+      <c r="I49" t="n">
+        <v>1.39</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Alia Khan</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>373681</v>
+      </c>
+      <c r="C50" t="n">
+        <v>129</v>
+      </c>
+      <c r="D50" t="n">
+        <v>44</v>
+      </c>
+      <c r="E50" t="n">
+        <v>40</v>
+      </c>
+      <c r="F50" t="n">
+        <v>4</v>
+      </c>
+      <c r="G50" t="n">
+        <v>34.11</v>
+      </c>
+      <c r="H50" t="n">
+        <v>31.01</v>
+      </c>
+      <c r="I50" t="n">
+        <v>3.1</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Aisha Aman</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>373704</v>
+      </c>
+      <c r="C51" t="n">
+        <v>11</v>
+      </c>
+      <c r="D51" t="n">
+        <v>3</v>
+      </c>
+      <c r="E51" t="n">
+        <v>2</v>
+      </c>
+      <c r="F51" t="n">
+        <v>1</v>
+      </c>
+      <c r="G51" t="n">
+        <v>27.27</v>
+      </c>
+      <c r="H51" t="n">
+        <v>18.18</v>
+      </c>
+      <c r="I51" t="n">
+        <v>9.09</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Iqra Bibi</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>373708</v>
+      </c>
+      <c r="C52" t="n">
+        <v>8</v>
+      </c>
+      <c r="D52" t="n">
+        <v>2</v>
+      </c>
+      <c r="E52" t="n">
+        <v>2</v>
+      </c>
+      <c r="F52" t="n">
+        <v>0</v>
+      </c>
+      <c r="G52" t="n">
+        <v>25</v>
+      </c>
+      <c r="H52" t="n">
+        <v>25</v>
+      </c>
+      <c r="I52" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Hijab Zahra</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>373637</v>
+      </c>
+      <c r="C53" t="n">
+        <v>4</v>
+      </c>
+      <c r="D53" t="n">
+        <v>1</v>
+      </c>
+      <c r="E53" t="n">
+        <v>1</v>
+      </c>
+      <c r="F53" t="n">
+        <v>0</v>
+      </c>
+      <c r="G53" t="n">
+        <v>25</v>
+      </c>
+      <c r="H53" t="n">
+        <v>25</v>
+      </c>
+      <c r="I53" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Laiba Khan</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>373653</v>
+      </c>
+      <c r="C54" t="n">
+        <v>121</v>
+      </c>
+      <c r="D54" t="n">
+        <v>26</v>
+      </c>
+      <c r="E54" t="n">
+        <v>22</v>
+      </c>
+      <c r="F54" t="n">
+        <v>4</v>
+      </c>
+      <c r="G54" t="n">
+        <v>21.49</v>
+      </c>
+      <c r="H54" t="n">
+        <v>18.18</v>
+      </c>
+      <c r="I54" t="n">
+        <v>3.31</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Gul Rukh</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>373644</v>
+      </c>
+      <c r="C55" t="n">
+        <v>6</v>
+      </c>
+      <c r="D55" t="n">
+        <v>1</v>
+      </c>
+      <c r="E55" t="n">
+        <v>1</v>
+      </c>
+      <c r="F55" t="n">
+        <v>0</v>
+      </c>
+      <c r="G55" t="n">
+        <v>16.67</v>
+      </c>
+      <c r="H55" t="n">
+        <v>16.67</v>
+      </c>
+      <c r="I55" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Mahnoorr</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>373670</v>
+      </c>
+      <c r="C56" t="n">
+        <v>13</v>
+      </c>
+      <c r="D56" t="n">
+        <v>2</v>
+      </c>
+      <c r="E56" t="n">
+        <v>1</v>
+      </c>
+      <c r="F56" t="n">
+        <v>1</v>
+      </c>
+      <c r="G56" t="n">
+        <v>15.38</v>
+      </c>
+      <c r="H56" t="n">
+        <v>7.69</v>
+      </c>
+      <c r="I56" t="n">
+        <v>7.69</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Sidra Khan</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>373645</v>
+      </c>
+      <c r="C57" t="n">
+        <v>7</v>
+      </c>
+      <c r="D57" t="n">
+        <v>1</v>
+      </c>
+      <c r="E57" t="n">
+        <v>1</v>
+      </c>
+      <c r="F57" t="n">
+        <v>0</v>
+      </c>
+      <c r="G57" t="n">
+        <v>14.29</v>
+      </c>
+      <c r="H57" t="n">
+        <v>14.29</v>
+      </c>
+      <c r="I57" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Irum ikram (duplicate name received from listed_girl_tracking_survey on June 29, 2026 12:08 UTC+00:00; submission key: uuid:b700a976-75ee-467c-87e9-1d5163ec238d)</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>541376</v>
+      </c>
+      <c r="C58" t="n">
+        <v>64</v>
+      </c>
+      <c r="D58" t="n">
+        <v>0</v>
+      </c>
+      <c r="E58" t="n">
+        <v>0</v>
+      </c>
+      <c r="F58" t="n">
+        <v>0</v>
+      </c>
+      <c r="G58" t="n">
+        <v>0</v>
+      </c>
+      <c r="H58" t="n">
+        <v>0</v>
+      </c>
+      <c r="I58" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Lati Khan (duplicate name received from listed_girl_tracking_survey on June 28, 2026 10:43 UTC+00:00; submission key: uuid:e4e89d53-e5be-40ff-bb2c-fa94c0d50011)</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>564273</v>
+      </c>
+      <c r="C59" t="n">
+        <v>56</v>
+      </c>
+      <c r="D59" t="n">
+        <v>0</v>
+      </c>
+      <c r="E59" t="n">
+        <v>0</v>
+      </c>
+      <c r="F59" t="n">
+        <v>0</v>
+      </c>
+      <c r="G59" t="n">
+        <v>0</v>
+      </c>
+      <c r="H59" t="n">
+        <v>0</v>
+      </c>
+      <c r="I59" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Lati khan (duplicate name received from listed_girl_tracking_survey_new_sample on July 4, 2026 14:31 UTC+00:00; submission key: uuid:6316d214-c458-4786-937a-bd81b08c15c5)</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>671211</v>
+      </c>
+      <c r="C60" t="n">
+        <v>14</v>
+      </c>
+      <c r="D60" t="n">
+        <v>0</v>
+      </c>
+      <c r="E60" t="n">
+        <v>0</v>
+      </c>
+      <c r="F60" t="n">
+        <v>0</v>
+      </c>
+      <c r="G60" t="n">
+        <v>0</v>
+      </c>
+      <c r="H60" t="n">
+        <v>0</v>
+      </c>
+      <c r="I60" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Muhammad Usman</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>373666</v>
+      </c>
+      <c r="C61" t="n">
+        <v>14</v>
+      </c>
+      <c r="D61" t="n">
+        <v>0</v>
+      </c>
+      <c r="E61" t="n">
+        <v>0</v>
+      </c>
+      <c r="F61" t="n">
+        <v>0</v>
+      </c>
+      <c r="G61" t="n">
+        <v>0</v>
+      </c>
+      <c r="H61" t="n">
+        <v>0</v>
+      </c>
+      <c r="I61" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Muhammad Waseem</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
+        <v>373689</v>
+      </c>
+      <c r="C62" t="n">
+        <v>3</v>
+      </c>
+      <c r="D62" t="n">
+        <v>0</v>
+      </c>
+      <c r="E62" t="n">
+        <v>0</v>
+      </c>
+      <c r="F62" t="n">
+        <v>0</v>
+      </c>
+      <c r="G62" t="n">
+        <v>0</v>
+      </c>
+      <c r="H62" t="n">
+        <v>0</v>
+      </c>
+      <c r="I62" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Muhammad naeem (duplicate name received from primary_school_listing_survey on February 14, 2026 14:38 UTC+00:00; submission key: uuid:5f0e427e-5fd2-4474-be64-ae5f2c4617a2)</t>
+        </is>
+      </c>
+      <c r="B63" t="n">
+        <v>571571</v>
+      </c>
+      <c r="C63" t="n">
+        <v>8</v>
+      </c>
+      <c r="D63" t="n">
+        <v>0</v>
+      </c>
+      <c r="E63" t="n">
+        <v>0</v>
+      </c>
+      <c r="F63" t="n">
+        <v>0</v>
+      </c>
+      <c r="G63" t="n">
+        <v>0</v>
+      </c>
+      <c r="H63" t="n">
+        <v>0</v>
+      </c>
+      <c r="I63" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
           <t>Naureen khan (duplicate name received from listed_girl_tracking_survey_new_sample on July 7, 2026 14:41 UTC+00:00; submission key: uuid:bbf56e1f-36f5-4ebf-9e0f-df83015a0871)</t>
         </is>
       </c>
-      <c r="B17" t="n">
+      <c r="B64" t="n">
         <v>453925</v>
       </c>
-      <c r="C17" t="n">
+      <c r="C64" t="n">
+        <v>57</v>
+      </c>
+      <c r="D64" t="n">
+        <v>0</v>
+      </c>
+      <c r="E64" t="n">
+        <v>0</v>
+      </c>
+      <c r="F64" t="n">
+        <v>0</v>
+      </c>
+      <c r="G64" t="n">
+        <v>0</v>
+      </c>
+      <c r="H64" t="n">
+        <v>0</v>
+      </c>
+      <c r="I64" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Samreen</t>
+        </is>
+      </c>
+      <c r="B65" t="n">
+        <v>373711</v>
+      </c>
+      <c r="C65" t="n">
+        <v>3</v>
+      </c>
+      <c r="D65" t="n">
+        <v>0</v>
+      </c>
+      <c r="E65" t="n">
+        <v>0</v>
+      </c>
+      <c r="F65" t="n">
+        <v>0</v>
+      </c>
+      <c r="G65" t="n">
+        <v>0</v>
+      </c>
+      <c r="H65" t="n">
+        <v>0</v>
+      </c>
+      <c r="I65" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Samreen</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>639258</v>
+      </c>
+      <c r="C66" t="n">
+        <v>1</v>
+      </c>
+      <c r="D66" t="n">
+        <v>0</v>
+      </c>
+      <c r="E66" t="n">
+        <v>0</v>
+      </c>
+      <c r="F66" t="n">
+        <v>0</v>
+      </c>
+      <c r="G66" t="n">
+        <v>0</v>
+      </c>
+      <c r="H66" t="n">
+        <v>0</v>
+      </c>
+      <c r="I66" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Shafaq Zahra</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr"/>
+      <c r="C67" t="n">
+        <v>1</v>
+      </c>
+      <c r="D67" t="n">
+        <v>0</v>
+      </c>
+      <c r="E67" t="n">
+        <v>0</v>
+      </c>
+      <c r="F67" t="n">
+        <v>0</v>
+      </c>
+      <c r="G67" t="n">
+        <v>0</v>
+      </c>
+      <c r="H67" t="n">
+        <v>0</v>
+      </c>
+      <c r="I67" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Shakeel Ahmed</t>
+        </is>
+      </c>
+      <c r="B68" t="n">
+        <v>373686</v>
+      </c>
+      <c r="C68" t="n">
+        <v>3</v>
+      </c>
+      <c r="D68" t="n">
+        <v>0</v>
+      </c>
+      <c r="E68" t="n">
+        <v>0</v>
+      </c>
+      <c r="F68" t="n">
+        <v>0</v>
+      </c>
+      <c r="G68" t="n">
+        <v>0</v>
+      </c>
+      <c r="H68" t="n">
+        <v>0</v>
+      </c>
+      <c r="I68" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Syed Haider Abbas</t>
+        </is>
+      </c>
+      <c r="B69" t="n">
+        <v>373713</v>
+      </c>
+      <c r="C69" t="n">
         <v>2</v>
       </c>
-      <c r="D17" t="n">
-        <v>0</v>
-      </c>
-      <c r="E17" t="n">
-        <v>0</v>
-      </c>
-      <c r="F17" t="n">
-        <v>0</v>
-      </c>
-      <c r="G17" t="n">
-        <v>0</v>
-      </c>
-      <c r="H17" t="n">
-        <v>0</v>
-      </c>
-      <c r="I17" t="n">
+      <c r="D69" t="n">
+        <v>0</v>
+      </c>
+      <c r="E69" t="n">
+        <v>0</v>
+      </c>
+      <c r="F69" t="n">
+        <v>0</v>
+      </c>
+      <c r="G69" t="n">
+        <v>0</v>
+      </c>
+      <c r="H69" t="n">
+        <v>0</v>
+      </c>
+      <c r="I69" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr"/>
+      <c r="B70" t="inlineStr"/>
+      <c r="C70" t="n">
+        <v>0</v>
+      </c>
+      <c r="D70" t="n">
+        <v>0</v>
+      </c>
+      <c r="E70" t="n">
+        <v>0</v>
+      </c>
+      <c r="F70" t="n">
+        <v>0</v>
+      </c>
+      <c r="G70" t="n">
+        <v>0</v>
+      </c>
+      <c r="H70" t="n">
+        <v>0</v>
+      </c>
+      <c r="I70" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: enhance duplicate handling in data quality checks and update related documentation
</commit_message>
<xml_diff>
--- a/Error_log/Enumerator_Performance.xlsx
+++ b/Error_log/Enumerator_Performance.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="performance" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="performance_pct" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="performance" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="performance_pct" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,16 +18,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -38,7 +35,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -46,21 +43,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -430,27 +418,27 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Enumerator Name</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Enumerator ID</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Total Issues</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Critical Issues</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Flag Issues</t>
         </is>
@@ -483,10 +471,10 @@
         <v>373641</v>
       </c>
       <c r="C3" t="n">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="D3" t="n">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="E3" t="n">
         <v>59</v>
@@ -521,10 +509,10 @@
         <v>373648</v>
       </c>
       <c r="C5" t="n">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="D5" t="n">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="E5" t="n">
         <v>70</v>
@@ -578,10 +566,10 @@
         <v>373642</v>
       </c>
       <c r="C8" t="n">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="D8" t="n">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="E8" t="n">
         <v>29</v>
@@ -749,10 +737,10 @@
         <v>373692</v>
       </c>
       <c r="C17" t="n">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="D17" t="n">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="E17" t="n">
         <v>183</v>
@@ -837,39 +825,39 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Rehana Bibi</t>
+          <t>Lati Khan</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>373691</v>
+        <v>564273</v>
       </c>
       <c r="C22" t="n">
-        <v>295</v>
+        <v>97</v>
       </c>
       <c r="D22" t="n">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E22" t="n">
-        <v>201</v>
+        <v>4</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Lati Khan</t>
+          <t>Rehana Bibi</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>564273</v>
+        <v>373691</v>
       </c>
       <c r="C23" t="n">
-        <v>97</v>
+        <v>293</v>
       </c>
       <c r="D23" t="n">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E23" t="n">
-        <v>4</v>
+        <v>201</v>
       </c>
     </row>
     <row r="24">
@@ -1567,51 +1555,51 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I69"/>
+  <dimension ref="A1:I70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>enumerator_name</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>enumerator_id</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>total_submissions</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>total_issues</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>critical_issues</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>flag_issues</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>error_pct</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>critical_error_pct</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>flag_error_pct</t>
         </is>
@@ -1785,19 +1773,19 @@
         <v>101</v>
       </c>
       <c r="D7" t="n">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="E7" t="n">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="F7" t="n">
         <v>183</v>
       </c>
       <c r="G7" t="n">
-        <v>295.05</v>
+        <v>292.08</v>
       </c>
       <c r="H7" t="n">
-        <v>113.86</v>
+        <v>110.89</v>
       </c>
       <c r="I7" t="n">
         <v>181.19</v>
@@ -1816,19 +1804,19 @@
         <v>111</v>
       </c>
       <c r="D8" t="n">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="E8" t="n">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="F8" t="n">
         <v>201</v>
       </c>
       <c r="G8" t="n">
-        <v>265.77</v>
+        <v>263.96</v>
       </c>
       <c r="H8" t="n">
-        <v>84.68000000000001</v>
+        <v>82.88</v>
       </c>
       <c r="I8" t="n">
         <v>181.08</v>
@@ -1909,19 +1897,19 @@
         <v>218</v>
       </c>
       <c r="D11" t="n">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="E11" t="n">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="F11" t="n">
         <v>59</v>
       </c>
       <c r="G11" t="n">
-        <v>163.3</v>
+        <v>162.39</v>
       </c>
       <c r="H11" t="n">
-        <v>136.24</v>
+        <v>135.32</v>
       </c>
       <c r="I11" t="n">
         <v>27.06</v>
@@ -1971,19 +1959,19 @@
         <v>223</v>
       </c>
       <c r="D13" t="n">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="E13" t="n">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="F13" t="n">
         <v>70</v>
       </c>
       <c r="G13" t="n">
-        <v>147.98</v>
+        <v>147.09</v>
       </c>
       <c r="H13" t="n">
-        <v>116.59</v>
+        <v>115.7</v>
       </c>
       <c r="I13" t="n">
         <v>31.39</v>
@@ -2157,19 +2145,19 @@
         <v>172</v>
       </c>
       <c r="D19" t="n">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="E19" t="n">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="F19" t="n">
         <v>29</v>
       </c>
       <c r="G19" t="n">
-        <v>139.53</v>
+        <v>137.79</v>
       </c>
       <c r="H19" t="n">
-        <v>122.67</v>
+        <v>120.93</v>
       </c>
       <c r="I19" t="n">
         <v>16.86</v>
@@ -3720,6 +3708,31 @@
         <v>0</v>
       </c>
       <c r="I69" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr"/>
+      <c r="B70" t="inlineStr"/>
+      <c r="C70" t="n">
+        <v>0</v>
+      </c>
+      <c r="D70" t="n">
+        <v>0</v>
+      </c>
+      <c r="E70" t="n">
+        <v>0</v>
+      </c>
+      <c r="F70" t="n">
+        <v>0</v>
+      </c>
+      <c r="G70" t="n">
+        <v>0</v>
+      </c>
+      <c r="H70" t="n">
+        <v>0</v>
+      </c>
+      <c r="I70" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: update high frequency checks and refresh Daily_Error_Log.xlsx, Enumerator_Performance.xlsx, and Weekly_QA_Summary.xlsx with latest data
</commit_message>
<xml_diff>
--- a/Error_log/Enumerator_Performance.xlsx
+++ b/Error_log/Enumerator_Performance.xlsx
@@ -471,10 +471,10 @@
         <v>373641</v>
       </c>
       <c r="C3" t="n">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="D3" t="n">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="E3" t="n">
         <v>59</v>
@@ -509,10 +509,10 @@
         <v>373648</v>
       </c>
       <c r="C5" t="n">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="D5" t="n">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="E5" t="n">
         <v>70</v>
@@ -566,10 +566,10 @@
         <v>373642</v>
       </c>
       <c r="C8" t="n">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="D8" t="n">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="E8" t="n">
         <v>29</v>
@@ -851,10 +851,10 @@
         <v>373691</v>
       </c>
       <c r="C23" t="n">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="D23" t="n">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="E23" t="n">
         <v>201</v>
@@ -1804,19 +1804,19 @@
         <v>111</v>
       </c>
       <c r="D8" t="n">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="E8" t="n">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="F8" t="n">
         <v>201</v>
       </c>
       <c r="G8" t="n">
-        <v>263.96</v>
+        <v>262.16</v>
       </c>
       <c r="H8" t="n">
-        <v>82.88</v>
+        <v>81.08</v>
       </c>
       <c r="I8" t="n">
         <v>181.08</v>
@@ -1897,19 +1897,19 @@
         <v>218</v>
       </c>
       <c r="D11" t="n">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="E11" t="n">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="F11" t="n">
         <v>59</v>
       </c>
       <c r="G11" t="n">
-        <v>162.39</v>
+        <v>161.47</v>
       </c>
       <c r="H11" t="n">
-        <v>135.32</v>
+        <v>134.4</v>
       </c>
       <c r="I11" t="n">
         <v>27.06</v>
@@ -1949,63 +1949,63 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Shazia Bibi</t>
+          <t>Mehran Khan</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>373648</v>
+        <v>373684</v>
       </c>
       <c r="C13" t="n">
-        <v>223</v>
+        <v>200</v>
       </c>
       <c r="D13" t="n">
-        <v>328</v>
+        <v>293</v>
       </c>
       <c r="E13" t="n">
-        <v>258</v>
+        <v>265</v>
       </c>
       <c r="F13" t="n">
-        <v>70</v>
+        <v>28</v>
       </c>
       <c r="G13" t="n">
-        <v>147.09</v>
+        <v>146.5</v>
       </c>
       <c r="H13" t="n">
-        <v>115.7</v>
+        <v>132.5</v>
       </c>
       <c r="I13" t="n">
-        <v>31.39</v>
+        <v>14</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Mehran Khan</t>
+          <t>Shazia Bibi</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>373684</v>
+        <v>373648</v>
       </c>
       <c r="C14" t="n">
-        <v>200</v>
+        <v>223</v>
       </c>
       <c r="D14" t="n">
-        <v>293</v>
+        <v>326</v>
       </c>
       <c r="E14" t="n">
-        <v>265</v>
+        <v>256</v>
       </c>
       <c r="F14" t="n">
-        <v>28</v>
+        <v>70</v>
       </c>
       <c r="G14" t="n">
-        <v>146.5</v>
+        <v>146.19</v>
       </c>
       <c r="H14" t="n">
-        <v>132.5</v>
+        <v>114.8</v>
       </c>
       <c r="I14" t="n">
-        <v>14</v>
+        <v>31.39</v>
       </c>
     </row>
     <row r="15">
@@ -2145,19 +2145,19 @@
         <v>172</v>
       </c>
       <c r="D19" t="n">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="E19" t="n">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="F19" t="n">
         <v>29</v>
       </c>
       <c r="G19" t="n">
-        <v>137.79</v>
+        <v>136.05</v>
       </c>
       <c r="H19" t="n">
-        <v>120.93</v>
+        <v>119.19</v>
       </c>
       <c r="I19" t="n">
         <v>16.86</v>

</xml_diff>

<commit_message>
feat: update Daily_Error_Log.xlsx, Enumerator_Performance.xlsx, and Weekly_QA_Summary.xlsx with latest data
</commit_message>
<xml_diff>
--- a/Error_log/Enumerator_Performance.xlsx
+++ b/Error_log/Enumerator_Performance.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -447,305 +447,1101 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Kainat</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>373712</v>
-      </c>
+          <t>UNASSIGNED (Tracking vs Household)</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr"/>
       <c r="C2" t="n">
-        <v>305</v>
+        <v>2133</v>
       </c>
       <c r="D2" t="n">
-        <v>104</v>
+        <v>2120</v>
       </c>
       <c r="E2" t="n">
-        <v>201</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Zohra</t>
+          <t>Asma Bibi</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>373692</v>
+        <v>373641</v>
       </c>
       <c r="C3" t="n">
-        <v>280</v>
+        <v>396</v>
       </c>
       <c r="D3" t="n">
-        <v>98</v>
+        <v>323</v>
       </c>
       <c r="E3" t="n">
-        <v>182</v>
+        <v>73</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Rehana Bibi</t>
+          <t>Mehran Khan</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>373691</v>
+        <v>373684</v>
       </c>
       <c r="C4" t="n">
-        <v>278</v>
+        <v>293</v>
       </c>
       <c r="D4" t="n">
-        <v>78</v>
+        <v>265</v>
       </c>
       <c r="E4" t="n">
-        <v>200</v>
+        <v>28</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Samara</t>
+          <t>Shazia Bibi</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>373658</v>
+        <v>373648</v>
       </c>
       <c r="C5" t="n">
-        <v>270</v>
+        <v>343</v>
       </c>
       <c r="D5" t="n">
-        <v>76</v>
+        <v>258</v>
       </c>
       <c r="E5" t="n">
-        <v>194</v>
+        <v>85</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Asma Bibi</t>
+          <t>Shafaq Zahra</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>373641</v>
+        <v>373646</v>
       </c>
       <c r="C6" t="n">
-        <v>80</v>
+        <v>299</v>
       </c>
       <c r="D6" t="n">
-        <v>43</v>
+        <v>236</v>
       </c>
       <c r="E6" t="n">
-        <v>37</v>
+        <v>63</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Javairia</t>
+          <t>Shazia begum</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>373651</v>
+        <v>373696</v>
       </c>
       <c r="C7" t="n">
-        <v>92</v>
+        <v>280</v>
       </c>
       <c r="D7" t="n">
-        <v>25</v>
+        <v>235</v>
       </c>
       <c r="E7" t="n">
-        <v>67</v>
+        <v>45</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Shazia Bibi</t>
+          <t>Irum Ikram</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>373648</v>
+        <v>373642</v>
       </c>
       <c r="C8" t="n">
-        <v>72</v>
+        <v>258</v>
       </c>
       <c r="D8" t="n">
-        <v>25</v>
+        <v>218</v>
       </c>
       <c r="E8" t="n">
-        <v>47</v>
+        <v>40</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Mahnoor</t>
+          <t>Sadia Rustum</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>373705</v>
+        <v>373649</v>
       </c>
       <c r="C9" t="n">
-        <v>51</v>
+        <v>192</v>
       </c>
       <c r="D9" t="n">
-        <v>19</v>
+        <v>182</v>
       </c>
       <c r="E9" t="n">
-        <v>32</v>
+        <v>10</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Irum Ikram</t>
+          <t>Javairia</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>373642</v>
+        <v>373651</v>
       </c>
       <c r="C10" t="n">
-        <v>42</v>
+        <v>247</v>
       </c>
       <c r="D10" t="n">
-        <v>17</v>
+        <v>151</v>
       </c>
       <c r="E10" t="n">
-        <v>25</v>
+        <v>96</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Nadia bibi</t>
+          <t>Mahnoor</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>373669</v>
+        <v>373705</v>
       </c>
       <c r="C11" t="n">
-        <v>41</v>
+        <v>196</v>
       </c>
       <c r="D11" t="n">
-        <v>15</v>
+        <v>148</v>
       </c>
       <c r="E11" t="n">
-        <v>26</v>
+        <v>48</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Naureen Khan</t>
+          <t>Khalida Bibi</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>373716</v>
+        <v>373673</v>
       </c>
       <c r="C12" t="n">
-        <v>22</v>
+        <v>140</v>
       </c>
       <c r="D12" t="n">
-        <v>13</v>
+        <v>140</v>
       </c>
       <c r="E12" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Shafaq Zahra</t>
+          <t>Naureen Khan</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>373646</v>
+        <v>373716</v>
       </c>
       <c r="C13" t="n">
-        <v>32</v>
+        <v>161</v>
       </c>
       <c r="D13" t="n">
-        <v>12</v>
+        <v>133</v>
       </c>
       <c r="E13" t="n">
-        <v>20</v>
+        <v>28</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Laiba Shams</t>
+          <t>Kainat</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>373706</v>
+        <v>373712</v>
       </c>
       <c r="C14" t="n">
-        <v>32</v>
+        <v>333</v>
       </c>
       <c r="D14" t="n">
-        <v>10</v>
+        <v>131</v>
       </c>
       <c r="E14" t="n">
-        <v>22</v>
+        <v>202</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Shazia begum</t>
+          <t>Bushra Ayub</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>373696</v>
+        <v>373671</v>
       </c>
       <c r="C15" t="n">
-        <v>13</v>
+        <v>126</v>
       </c>
       <c r="D15" t="n">
-        <v>5</v>
+        <v>122</v>
       </c>
       <c r="E15" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Naureen khan</t>
+          <t>Furqan Ullah Khan</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>453925</v>
+        <v>373683</v>
       </c>
       <c r="C16" t="n">
-        <v>6</v>
+        <v>124</v>
       </c>
       <c r="D16" t="n">
-        <v>4</v>
+        <v>116</v>
       </c>
       <c r="E16" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
+          <t>Zohra</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>373692</v>
+      </c>
+      <c r="C17" t="n">
+        <v>295</v>
+      </c>
+      <c r="D17" t="n">
+        <v>112</v>
+      </c>
+      <c r="E17" t="n">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Asma Gull</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>373672</v>
+      </c>
+      <c r="C18" t="n">
+        <v>109</v>
+      </c>
+      <c r="D18" t="n">
+        <v>105</v>
+      </c>
+      <c r="E18" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Samara</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>373658</v>
+      </c>
+      <c r="C19" t="n">
+        <v>298</v>
+      </c>
+      <c r="D19" t="n">
+        <v>102</v>
+      </c>
+      <c r="E19" t="n">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Ishaq Khan</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>373699</v>
+      </c>
+      <c r="C20" t="n">
+        <v>101</v>
+      </c>
+      <c r="D20" t="n">
+        <v>100</v>
+      </c>
+      <c r="E20" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Muhammad Yousaf</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>373690</v>
+      </c>
+      <c r="C21" t="n">
+        <v>105</v>
+      </c>
+      <c r="D21" t="n">
+        <v>96</v>
+      </c>
+      <c r="E21" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Laiba Shams</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>373706</v>
+      </c>
+      <c r="C22" t="n">
+        <v>131</v>
+      </c>
+      <c r="D22" t="n">
+        <v>95</v>
+      </c>
+      <c r="E22" t="n">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Lati Khan</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>564273</v>
+      </c>
+      <c r="C23" t="n">
+        <v>97</v>
+      </c>
+      <c r="D23" t="n">
+        <v>93</v>
+      </c>
+      <c r="E23" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Rehana Bibi</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>373691</v>
+      </c>
+      <c r="C24" t="n">
+        <v>291</v>
+      </c>
+      <c r="D24" t="n">
+        <v>90</v>
+      </c>
+      <c r="E24" t="n">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Naureen khan</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>453925</v>
+      </c>
+      <c r="C25" t="n">
+        <v>91</v>
+      </c>
+      <c r="D25" t="n">
+        <v>89</v>
+      </c>
+      <c r="E25" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Irum ikram</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>541376</v>
+      </c>
+      <c r="C26" t="n">
+        <v>88</v>
+      </c>
+      <c r="D26" t="n">
+        <v>83</v>
+      </c>
+      <c r="E26" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Lati Khan</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>373665</v>
+      </c>
+      <c r="C27" t="n">
+        <v>86</v>
+      </c>
+      <c r="D27" t="n">
+        <v>83</v>
+      </c>
+      <c r="E27" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Naureen</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>884887</v>
+      </c>
+      <c r="C28" t="n">
+        <v>86</v>
+      </c>
+      <c r="D28" t="n">
+        <v>82</v>
+      </c>
+      <c r="E28" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Jaweria</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>163495</v>
+      </c>
+      <c r="C29" t="n">
+        <v>83</v>
+      </c>
+      <c r="D29" t="n">
+        <v>82</v>
+      </c>
+      <c r="E29" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Nillum Bibi</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>373652</v>
+      </c>
+      <c r="C30" t="n">
+        <v>64</v>
+      </c>
+      <c r="D30" t="n">
+        <v>61</v>
+      </c>
+      <c r="E30" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Anum Gul</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>373656</v>
+      </c>
+      <c r="C31" t="n">
+        <v>55</v>
+      </c>
+      <c r="D31" t="n">
+        <v>51</v>
+      </c>
+      <c r="E31" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Muniba Shamim</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>373659</v>
+      </c>
+      <c r="C32" t="n">
+        <v>58</v>
+      </c>
+      <c r="D32" t="n">
+        <v>49</v>
+      </c>
+      <c r="E32" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Nazia</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>373657</v>
+      </c>
+      <c r="C33" t="n">
+        <v>51</v>
+      </c>
+      <c r="D33" t="n">
+        <v>49</v>
+      </c>
+      <c r="E33" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
           <t>Summiya Hayat</t>
         </is>
       </c>
-      <c r="B17" t="n">
+      <c r="B34" t="n">
         <v>373710</v>
       </c>
-      <c r="C17" t="n">
-        <v>17</v>
-      </c>
-      <c r="D17" t="n">
+      <c r="C34" t="n">
+        <v>71</v>
+      </c>
+      <c r="D34" t="n">
+        <v>40</v>
+      </c>
+      <c r="E34" t="n">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Alia Khan</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>373681</v>
+      </c>
+      <c r="C35" t="n">
+        <v>44</v>
+      </c>
+      <c r="D35" t="n">
+        <v>40</v>
+      </c>
+      <c r="E35" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Lati khan</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>671211</v>
+      </c>
+      <c r="C36" t="n">
+        <v>38</v>
+      </c>
+      <c r="D36" t="n">
+        <v>38</v>
+      </c>
+      <c r="E36" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Munawar Khan</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>373668</v>
+      </c>
+      <c r="C37" t="n">
+        <v>38</v>
+      </c>
+      <c r="D37" t="n">
+        <v>32</v>
+      </c>
+      <c r="E37" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Laiba Khan</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>373653</v>
+      </c>
+      <c r="C38" t="n">
+        <v>26</v>
+      </c>
+      <c r="D38" t="n">
+        <v>22</v>
+      </c>
+      <c r="E38" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Nadia bibi</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>373669</v>
+      </c>
+      <c r="C39" t="n">
+        <v>54</v>
+      </c>
+      <c r="D39" t="n">
+        <v>21</v>
+      </c>
+      <c r="E39" t="n">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Chashm Gul</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>373695</v>
+      </c>
+      <c r="C40" t="n">
+        <v>27</v>
+      </c>
+      <c r="D40" t="n">
+        <v>18</v>
+      </c>
+      <c r="E40" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Zain Ul Abideen</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>373667</v>
+      </c>
+      <c r="C41" t="n">
+        <v>12</v>
+      </c>
+      <c r="D41" t="n">
+        <v>12</v>
+      </c>
+      <c r="E41" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Lati khan</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>652938</v>
+      </c>
+      <c r="C42" t="n">
+        <v>10</v>
+      </c>
+      <c r="D42" t="n">
+        <v>10</v>
+      </c>
+      <c r="E42" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Saba Ramzan</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>373703</v>
+      </c>
+      <c r="C43" t="n">
+        <v>9</v>
+      </c>
+      <c r="D43" t="n">
+        <v>9</v>
+      </c>
+      <c r="E43" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Shehla Noor</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>373650</v>
+      </c>
+      <c r="C44" t="n">
+        <v>9</v>
+      </c>
+      <c r="D44" t="n">
+        <v>9</v>
+      </c>
+      <c r="E44" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Muhammad naeem</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>571571</v>
+      </c>
+      <c r="C45" t="n">
+        <v>10</v>
+      </c>
+      <c r="D45" t="n">
+        <v>8</v>
+      </c>
+      <c r="E45" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Sadia rustum</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>852541</v>
+      </c>
+      <c r="C46" t="n">
+        <v>5</v>
+      </c>
+      <c r="D46" t="n">
+        <v>5</v>
+      </c>
+      <c r="E46" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Usman Ali</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>373687</v>
+      </c>
+      <c r="C47" t="n">
+        <v>5</v>
+      </c>
+      <c r="D47" t="n">
+        <v>5</v>
+      </c>
+      <c r="E47" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Muhammad Noor</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>373701</v>
+      </c>
+      <c r="C48" t="n">
+        <v>4</v>
+      </c>
+      <c r="D48" t="n">
         <v>3</v>
       </c>
-      <c r="E17" t="n">
-        <v>14</v>
+      <c r="E48" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Muhammad Naeem</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>373694</v>
+      </c>
+      <c r="C49" t="n">
+        <v>3</v>
+      </c>
+      <c r="D49" t="n">
+        <v>3</v>
+      </c>
+      <c r="E49" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Muhammad Shahid Khan</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>373662</v>
+      </c>
+      <c r="C50" t="n">
+        <v>3</v>
+      </c>
+      <c r="D50" t="n">
+        <v>3</v>
+      </c>
+      <c r="E50" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Sajjad Khan</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>373700</v>
+      </c>
+      <c r="C51" t="n">
+        <v>3</v>
+      </c>
+      <c r="D51" t="n">
+        <v>3</v>
+      </c>
+      <c r="E51" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Aisha Aman</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>373704</v>
+      </c>
+      <c r="C52" t="n">
+        <v>3</v>
+      </c>
+      <c r="D52" t="n">
+        <v>2</v>
+      </c>
+      <c r="E52" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Rahila Naaz</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>373715</v>
+      </c>
+      <c r="C53" t="n">
+        <v>3</v>
+      </c>
+      <c r="D53" t="n">
+        <v>2</v>
+      </c>
+      <c r="E53" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Robina Shaheen</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>373639</v>
+      </c>
+      <c r="C54" t="n">
+        <v>3</v>
+      </c>
+      <c r="D54" t="n">
+        <v>2</v>
+      </c>
+      <c r="E54" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Iqra Bibi</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>373708</v>
+      </c>
+      <c r="C55" t="n">
+        <v>2</v>
+      </c>
+      <c r="D55" t="n">
+        <v>2</v>
+      </c>
+      <c r="E55" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Mahnoorr</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>373670</v>
+      </c>
+      <c r="C56" t="n">
+        <v>2</v>
+      </c>
+      <c r="D56" t="n">
+        <v>1</v>
+      </c>
+      <c r="E56" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Gul Rukh</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>373644</v>
+      </c>
+      <c r="C57" t="n">
+        <v>1</v>
+      </c>
+      <c r="D57" t="n">
+        <v>1</v>
+      </c>
+      <c r="E57" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Hijab Zahra</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>373637</v>
+      </c>
+      <c r="C58" t="n">
+        <v>1</v>
+      </c>
+      <c r="D58" t="n">
+        <v>1</v>
+      </c>
+      <c r="E58" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Sidra Khan</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>373645</v>
+      </c>
+      <c r="C59" t="n">
+        <v>1</v>
+      </c>
+      <c r="D59" t="n">
+        <v>1</v>
+      </c>
+      <c r="E59" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -759,7 +1555,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:I70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -812,496 +1608,2131 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Javairia</t>
+          <t>Naureen khan</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>373651</v>
+        <v>453925</v>
       </c>
       <c r="C2" t="n">
-        <v>21</v>
+        <v>2</v>
       </c>
       <c r="D2" t="n">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="E2" t="n">
-        <v>25</v>
+        <v>89</v>
       </c>
       <c r="F2" t="n">
-        <v>67</v>
+        <v>2</v>
       </c>
       <c r="G2" t="n">
-        <v>438.1</v>
+        <v>4550</v>
       </c>
       <c r="H2" t="n">
-        <v>119.05</v>
+        <v>4450</v>
       </c>
       <c r="I2" t="n">
-        <v>319.05</v>
+        <v>100</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Kainat</t>
+          <t>Irum ikram</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>373712</v>
+        <v>541376</v>
       </c>
       <c r="C3" t="n">
-        <v>73</v>
+        <v>8</v>
       </c>
       <c r="D3" t="n">
-        <v>305</v>
+        <v>88</v>
       </c>
       <c r="E3" t="n">
-        <v>104</v>
+        <v>83</v>
       </c>
       <c r="F3" t="n">
-        <v>201</v>
+        <v>5</v>
       </c>
       <c r="G3" t="n">
-        <v>417.81</v>
+        <v>1100</v>
       </c>
       <c r="H3" t="n">
-        <v>142.47</v>
+        <v>1037.5</v>
       </c>
       <c r="I3" t="n">
-        <v>275.34</v>
+        <v>62.5</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Zohra</t>
+          <t>Lati Khan</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>373692</v>
+        <v>564273</v>
       </c>
       <c r="C4" t="n">
-        <v>70</v>
+        <v>9</v>
       </c>
       <c r="D4" t="n">
-        <v>280</v>
+        <v>97</v>
       </c>
       <c r="E4" t="n">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="F4" t="n">
-        <v>182</v>
+        <v>4</v>
       </c>
       <c r="G4" t="n">
-        <v>400</v>
+        <v>1077.78</v>
       </c>
       <c r="H4" t="n">
-        <v>140</v>
+        <v>1033.33</v>
       </c>
       <c r="I4" t="n">
-        <v>260</v>
+        <v>44.44</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Rehana Bibi</t>
+          <t>Lati khan</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>373691</v>
+        <v>671211</v>
       </c>
       <c r="C5" t="n">
-        <v>79</v>
+        <v>9</v>
       </c>
       <c r="D5" t="n">
-        <v>278</v>
+        <v>38</v>
       </c>
       <c r="E5" t="n">
-        <v>78</v>
+        <v>38</v>
       </c>
       <c r="F5" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="G5" t="n">
-        <v>351.9</v>
+        <v>422.22</v>
       </c>
       <c r="H5" t="n">
-        <v>98.73</v>
+        <v>422.22</v>
       </c>
       <c r="I5" t="n">
-        <v>253.16</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Samara</t>
+          <t>Kainat</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>373658</v>
+        <v>373712</v>
       </c>
       <c r="C6" t="n">
-        <v>79</v>
+        <v>104</v>
       </c>
       <c r="D6" t="n">
-        <v>270</v>
+        <v>333</v>
       </c>
       <c r="E6" t="n">
-        <v>76</v>
+        <v>131</v>
       </c>
       <c r="F6" t="n">
-        <v>194</v>
+        <v>202</v>
       </c>
       <c r="G6" t="n">
-        <v>341.77</v>
+        <v>320.19</v>
       </c>
       <c r="H6" t="n">
-        <v>96.2</v>
+        <v>125.96</v>
       </c>
       <c r="I6" t="n">
-        <v>245.57</v>
+        <v>194.23</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Asma Bibi</t>
+          <t>Zohra</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>373641</v>
+        <v>373692</v>
       </c>
       <c r="C7" t="n">
-        <v>31</v>
+        <v>101</v>
       </c>
       <c r="D7" t="n">
-        <v>80</v>
+        <v>295</v>
       </c>
       <c r="E7" t="n">
-        <v>43</v>
+        <v>112</v>
       </c>
       <c r="F7" t="n">
-        <v>37</v>
+        <v>183</v>
       </c>
       <c r="G7" t="n">
-        <v>258.06</v>
+        <v>292.08</v>
       </c>
       <c r="H7" t="n">
-        <v>138.71</v>
+        <v>110.89</v>
       </c>
       <c r="I7" t="n">
-        <v>119.35</v>
+        <v>181.19</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Shazia begum</t>
+          <t>Rehana Bibi</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>373696</v>
+        <v>373691</v>
       </c>
       <c r="C8" t="n">
-        <v>6</v>
+        <v>111</v>
       </c>
       <c r="D8" t="n">
-        <v>13</v>
+        <v>291</v>
       </c>
       <c r="E8" t="n">
-        <v>5</v>
+        <v>90</v>
       </c>
       <c r="F8" t="n">
-        <v>8</v>
+        <v>201</v>
       </c>
       <c r="G8" t="n">
-        <v>216.67</v>
+        <v>262.16</v>
       </c>
       <c r="H8" t="n">
-        <v>83.33</v>
+        <v>81.08</v>
       </c>
       <c r="I8" t="n">
-        <v>133.33</v>
+        <v>181.08</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Nadia bibi</t>
+          <t>Samara</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>373669</v>
+        <v>373658</v>
       </c>
       <c r="C9" t="n">
-        <v>19</v>
+        <v>120</v>
       </c>
       <c r="D9" t="n">
-        <v>41</v>
+        <v>298</v>
       </c>
       <c r="E9" t="n">
-        <v>15</v>
+        <v>102</v>
       </c>
       <c r="F9" t="n">
-        <v>26</v>
+        <v>196</v>
       </c>
       <c r="G9" t="n">
-        <v>215.79</v>
+        <v>248.33</v>
       </c>
       <c r="H9" t="n">
-        <v>78.95</v>
+        <v>85</v>
       </c>
       <c r="I9" t="n">
-        <v>136.84</v>
+        <v>163.33</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Shazia Bibi</t>
+          <t>Naureen Khan</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>373648</v>
+        <v>373716</v>
       </c>
       <c r="C10" t="n">
-        <v>34</v>
+        <v>94</v>
       </c>
       <c r="D10" t="n">
-        <v>72</v>
+        <v>161</v>
       </c>
       <c r="E10" t="n">
-        <v>25</v>
+        <v>133</v>
       </c>
       <c r="F10" t="n">
-        <v>47</v>
+        <v>28</v>
       </c>
       <c r="G10" t="n">
-        <v>211.76</v>
+        <v>171.28</v>
       </c>
       <c r="H10" t="n">
-        <v>73.53</v>
+        <v>141.49</v>
       </c>
       <c r="I10" t="n">
-        <v>138.24</v>
+        <v>29.79</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Mahnoor</t>
+          <t>Asma Bibi</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>373705</v>
+        <v>373641</v>
       </c>
       <c r="C11" t="n">
-        <v>25</v>
+        <v>235</v>
       </c>
       <c r="D11" t="n">
-        <v>51</v>
+        <v>396</v>
       </c>
       <c r="E11" t="n">
-        <v>19</v>
+        <v>323</v>
       </c>
       <c r="F11" t="n">
-        <v>32</v>
+        <v>73</v>
       </c>
       <c r="G11" t="n">
-        <v>204</v>
+        <v>168.51</v>
       </c>
       <c r="H11" t="n">
-        <v>76</v>
+        <v>137.45</v>
       </c>
       <c r="I11" t="n">
-        <v>128</v>
+        <v>31.06</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Shafaq Zahra</t>
+          <t>Javairia</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>373646</v>
+        <v>373651</v>
       </c>
       <c r="C12" t="n">
-        <v>16</v>
+        <v>152</v>
       </c>
       <c r="D12" t="n">
-        <v>32</v>
+        <v>247</v>
       </c>
       <c r="E12" t="n">
-        <v>12</v>
+        <v>151</v>
       </c>
       <c r="F12" t="n">
-        <v>20</v>
+        <v>96</v>
       </c>
       <c r="G12" t="n">
-        <v>200</v>
+        <v>162.5</v>
       </c>
       <c r="H12" t="n">
-        <v>75</v>
+        <v>99.34</v>
       </c>
       <c r="I12" t="n">
-        <v>125</v>
+        <v>63.16</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Naureen Khan</t>
+          <t>Nadia bibi</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>373716</v>
+        <v>373669</v>
       </c>
       <c r="C13" t="n">
-        <v>11</v>
+        <v>35</v>
       </c>
       <c r="D13" t="n">
-        <v>22</v>
+        <v>54</v>
       </c>
       <c r="E13" t="n">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="F13" t="n">
-        <v>9</v>
+        <v>33</v>
       </c>
       <c r="G13" t="n">
-        <v>200</v>
+        <v>154.29</v>
       </c>
       <c r="H13" t="n">
-        <v>118.18</v>
+        <v>60</v>
       </c>
       <c r="I13" t="n">
-        <v>81.81999999999999</v>
+        <v>94.29000000000001</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Irum Ikram</t>
+          <t>Mahnoor</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>373642</v>
+        <v>373705</v>
       </c>
       <c r="C14" t="n">
-        <v>22</v>
+        <v>133</v>
       </c>
       <c r="D14" t="n">
-        <v>42</v>
+        <v>196</v>
       </c>
       <c r="E14" t="n">
-        <v>17</v>
+        <v>148</v>
       </c>
       <c r="F14" t="n">
-        <v>25</v>
+        <v>48</v>
       </c>
       <c r="G14" t="n">
-        <v>190.91</v>
+        <v>147.37</v>
       </c>
       <c r="H14" t="n">
-        <v>77.27</v>
+        <v>111.28</v>
       </c>
       <c r="I14" t="n">
-        <v>113.64</v>
+        <v>36.09</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Laiba Shams</t>
+          <t>Shazia Bibi</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>373706</v>
+        <v>373648</v>
       </c>
       <c r="C15" t="n">
-        <v>21</v>
+        <v>234</v>
       </c>
       <c r="D15" t="n">
-        <v>32</v>
+        <v>343</v>
       </c>
       <c r="E15" t="n">
-        <v>10</v>
+        <v>258</v>
       </c>
       <c r="F15" t="n">
-        <v>22</v>
+        <v>85</v>
       </c>
       <c r="G15" t="n">
-        <v>152.38</v>
+        <v>146.58</v>
       </c>
       <c r="H15" t="n">
-        <v>47.62</v>
+        <v>110.26</v>
       </c>
       <c r="I15" t="n">
-        <v>104.76</v>
+        <v>36.32</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Summiya Hayat</t>
+          <t>Mehran Khan</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>373710</v>
+        <v>373684</v>
       </c>
       <c r="C16" t="n">
-        <v>13</v>
+        <v>200</v>
       </c>
       <c r="D16" t="n">
-        <v>17</v>
+        <v>293</v>
       </c>
       <c r="E16" t="n">
-        <v>3</v>
+        <v>265</v>
       </c>
       <c r="F16" t="n">
+        <v>28</v>
+      </c>
+      <c r="G16" t="n">
+        <v>146.5</v>
+      </c>
+      <c r="H16" t="n">
+        <v>132.5</v>
+      </c>
+      <c r="I16" t="n">
         <v>14</v>
-      </c>
-      <c r="G16" t="n">
-        <v>130.77</v>
-      </c>
-      <c r="H16" t="n">
-        <v>23.08</v>
-      </c>
-      <c r="I16" t="n">
-        <v>107.69</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
+          <t>Lati Khan</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>373665</v>
+      </c>
+      <c r="C17" t="n">
+        <v>60</v>
+      </c>
+      <c r="D17" t="n">
+        <v>86</v>
+      </c>
+      <c r="E17" t="n">
+        <v>83</v>
+      </c>
+      <c r="F17" t="n">
+        <v>3</v>
+      </c>
+      <c r="G17" t="n">
+        <v>143.33</v>
+      </c>
+      <c r="H17" t="n">
+        <v>138.33</v>
+      </c>
+      <c r="I17" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Naureen</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>884887</v>
+      </c>
+      <c r="C18" t="n">
+        <v>60</v>
+      </c>
+      <c r="D18" t="n">
+        <v>86</v>
+      </c>
+      <c r="E18" t="n">
+        <v>82</v>
+      </c>
+      <c r="F18" t="n">
+        <v>4</v>
+      </c>
+      <c r="G18" t="n">
+        <v>143.33</v>
+      </c>
+      <c r="H18" t="n">
+        <v>136.67</v>
+      </c>
+      <c r="I18" t="n">
+        <v>6.67</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Shazia begum</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>373696</v>
+      </c>
+      <c r="C19" t="n">
+        <v>197</v>
+      </c>
+      <c r="D19" t="n">
+        <v>280</v>
+      </c>
+      <c r="E19" t="n">
+        <v>235</v>
+      </c>
+      <c r="F19" t="n">
+        <v>45</v>
+      </c>
+      <c r="G19" t="n">
+        <v>142.13</v>
+      </c>
+      <c r="H19" t="n">
+        <v>119.29</v>
+      </c>
+      <c r="I19" t="n">
+        <v>22.84</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Irum Ikram</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>373642</v>
+      </c>
+      <c r="C20" t="n">
+        <v>183</v>
+      </c>
+      <c r="D20" t="n">
+        <v>258</v>
+      </c>
+      <c r="E20" t="n">
+        <v>218</v>
+      </c>
+      <c r="F20" t="n">
+        <v>40</v>
+      </c>
+      <c r="G20" t="n">
+        <v>140.98</v>
+      </c>
+      <c r="H20" t="n">
+        <v>119.13</v>
+      </c>
+      <c r="I20" t="n">
+        <v>21.86</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Sadia Rustum</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>373649</v>
+      </c>
+      <c r="C21" t="n">
+        <v>152</v>
+      </c>
+      <c r="D21" t="n">
+        <v>192</v>
+      </c>
+      <c r="E21" t="n">
+        <v>182</v>
+      </c>
+      <c r="F21" t="n">
+        <v>10</v>
+      </c>
+      <c r="G21" t="n">
+        <v>126.32</v>
+      </c>
+      <c r="H21" t="n">
+        <v>119.74</v>
+      </c>
+      <c r="I21" t="n">
+        <v>6.58</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Shafaq Zahra</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>373646</v>
+      </c>
+      <c r="C22" t="n">
+        <v>239</v>
+      </c>
+      <c r="D22" t="n">
+        <v>299</v>
+      </c>
+      <c r="E22" t="n">
+        <v>236</v>
+      </c>
+      <c r="F22" t="n">
+        <v>63</v>
+      </c>
+      <c r="G22" t="n">
+        <v>125.1</v>
+      </c>
+      <c r="H22" t="n">
+        <v>98.73999999999999</v>
+      </c>
+      <c r="I22" t="n">
+        <v>26.36</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Jaweria</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>163495</v>
+      </c>
+      <c r="C23" t="n">
+        <v>68</v>
+      </c>
+      <c r="D23" t="n">
+        <v>83</v>
+      </c>
+      <c r="E23" t="n">
+        <v>82</v>
+      </c>
+      <c r="F23" t="n">
+        <v>1</v>
+      </c>
+      <c r="G23" t="n">
+        <v>122.06</v>
+      </c>
+      <c r="H23" t="n">
+        <v>120.59</v>
+      </c>
+      <c r="I23" t="n">
+        <v>1.47</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Laiba Shams</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>373706</v>
+      </c>
+      <c r="C24" t="n">
+        <v>127</v>
+      </c>
+      <c r="D24" t="n">
+        <v>131</v>
+      </c>
+      <c r="E24" t="n">
+        <v>95</v>
+      </c>
+      <c r="F24" t="n">
+        <v>36</v>
+      </c>
+      <c r="G24" t="n">
+        <v>103.15</v>
+      </c>
+      <c r="H24" t="n">
+        <v>74.8</v>
+      </c>
+      <c r="I24" t="n">
+        <v>28.35</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Zain Ul Abideen</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>373667</v>
+      </c>
+      <c r="C25" t="n">
+        <v>13</v>
+      </c>
+      <c r="D25" t="n">
+        <v>12</v>
+      </c>
+      <c r="E25" t="n">
+        <v>12</v>
+      </c>
+      <c r="F25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G25" t="n">
+        <v>92.31</v>
+      </c>
+      <c r="H25" t="n">
+        <v>92.31</v>
+      </c>
+      <c r="I25" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Bushra Ayub</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>373671</v>
+      </c>
+      <c r="C26" t="n">
+        <v>138</v>
+      </c>
+      <c r="D26" t="n">
+        <v>126</v>
+      </c>
+      <c r="E26" t="n">
+        <v>122</v>
+      </c>
+      <c r="F26" t="n">
+        <v>4</v>
+      </c>
+      <c r="G26" t="n">
+        <v>91.3</v>
+      </c>
+      <c r="H26" t="n">
+        <v>88.41</v>
+      </c>
+      <c r="I26" t="n">
+        <v>2.9</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Lati khan</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>652938</v>
+      </c>
+      <c r="C27" t="n">
+        <v>11</v>
+      </c>
+      <c r="D27" t="n">
+        <v>10</v>
+      </c>
+      <c r="E27" t="n">
+        <v>10</v>
+      </c>
+      <c r="F27" t="n">
+        <v>0</v>
+      </c>
+      <c r="G27" t="n">
+        <v>90.91</v>
+      </c>
+      <c r="H27" t="n">
+        <v>90.91</v>
+      </c>
+      <c r="I27" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Chashm Gul</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>373695</v>
+      </c>
+      <c r="C28" t="n">
+        <v>31</v>
+      </c>
+      <c r="D28" t="n">
+        <v>27</v>
+      </c>
+      <c r="E28" t="n">
+        <v>18</v>
+      </c>
+      <c r="F28" t="n">
+        <v>9</v>
+      </c>
+      <c r="G28" t="n">
+        <v>87.09999999999999</v>
+      </c>
+      <c r="H28" t="n">
+        <v>58.06</v>
+      </c>
+      <c r="I28" t="n">
+        <v>29.03</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Muniba Shamim</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>373659</v>
+      </c>
+      <c r="C29" t="n">
+        <v>72</v>
+      </c>
+      <c r="D29" t="n">
+        <v>58</v>
+      </c>
+      <c r="E29" t="n">
+        <v>49</v>
+      </c>
+      <c r="F29" t="n">
+        <v>9</v>
+      </c>
+      <c r="G29" t="n">
+        <v>80.56</v>
+      </c>
+      <c r="H29" t="n">
+        <v>68.06</v>
+      </c>
+      <c r="I29" t="n">
+        <v>12.5</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Muhammad Yousaf</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>373690</v>
+      </c>
+      <c r="C30" t="n">
+        <v>132</v>
+      </c>
+      <c r="D30" t="n">
+        <v>105</v>
+      </c>
+      <c r="E30" t="n">
+        <v>96</v>
+      </c>
+      <c r="F30" t="n">
+        <v>9</v>
+      </c>
+      <c r="G30" t="n">
+        <v>79.55</v>
+      </c>
+      <c r="H30" t="n">
+        <v>72.73</v>
+      </c>
+      <c r="I30" t="n">
+        <v>6.82</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Khalida Bibi</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>373673</v>
+      </c>
+      <c r="C31" t="n">
+        <v>177</v>
+      </c>
+      <c r="D31" t="n">
+        <v>140</v>
+      </c>
+      <c r="E31" t="n">
+        <v>140</v>
+      </c>
+      <c r="F31" t="n">
+        <v>0</v>
+      </c>
+      <c r="G31" t="n">
+        <v>79.09999999999999</v>
+      </c>
+      <c r="H31" t="n">
+        <v>79.09999999999999</v>
+      </c>
+      <c r="I31" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Asma Gull</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>373672</v>
+      </c>
+      <c r="C32" t="n">
+        <v>144</v>
+      </c>
+      <c r="D32" t="n">
+        <v>109</v>
+      </c>
+      <c r="E32" t="n">
+        <v>105</v>
+      </c>
+      <c r="F32" t="n">
+        <v>4</v>
+      </c>
+      <c r="G32" t="n">
+        <v>75.69</v>
+      </c>
+      <c r="H32" t="n">
+        <v>72.92</v>
+      </c>
+      <c r="I32" t="n">
+        <v>2.78</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Rahila Naaz</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>373715</v>
+      </c>
+      <c r="C33" t="n">
+        <v>4</v>
+      </c>
+      <c r="D33" t="n">
+        <v>3</v>
+      </c>
+      <c r="E33" t="n">
+        <v>2</v>
+      </c>
+      <c r="F33" t="n">
+        <v>1</v>
+      </c>
+      <c r="G33" t="n">
+        <v>75</v>
+      </c>
+      <c r="H33" t="n">
+        <v>50</v>
+      </c>
+      <c r="I33" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Sadia rustum</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>852541</v>
+      </c>
+      <c r="C34" t="n">
+        <v>7</v>
+      </c>
+      <c r="D34" t="n">
+        <v>5</v>
+      </c>
+      <c r="E34" t="n">
+        <v>5</v>
+      </c>
+      <c r="F34" t="n">
+        <v>0</v>
+      </c>
+      <c r="G34" t="n">
+        <v>71.43000000000001</v>
+      </c>
+      <c r="H34" t="n">
+        <v>71.43000000000001</v>
+      </c>
+      <c r="I34" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Saba Ramzan</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>373703</v>
+      </c>
+      <c r="C35" t="n">
+        <v>13</v>
+      </c>
+      <c r="D35" t="n">
+        <v>9</v>
+      </c>
+      <c r="E35" t="n">
+        <v>9</v>
+      </c>
+      <c r="F35" t="n">
+        <v>0</v>
+      </c>
+      <c r="G35" t="n">
+        <v>69.23</v>
+      </c>
+      <c r="H35" t="n">
+        <v>69.23</v>
+      </c>
+      <c r="I35" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Summiya Hayat</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>373710</v>
+      </c>
+      <c r="C36" t="n">
+        <v>103</v>
+      </c>
+      <c r="D36" t="n">
+        <v>71</v>
+      </c>
+      <c r="E36" t="n">
+        <v>40</v>
+      </c>
+      <c r="F36" t="n">
+        <v>31</v>
+      </c>
+      <c r="G36" t="n">
+        <v>68.93000000000001</v>
+      </c>
+      <c r="H36" t="n">
+        <v>38.83</v>
+      </c>
+      <c r="I36" t="n">
+        <v>30.1</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Shehla Noor</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>373650</v>
+      </c>
+      <c r="C37" t="n">
+        <v>14</v>
+      </c>
+      <c r="D37" t="n">
+        <v>9</v>
+      </c>
+      <c r="E37" t="n">
+        <v>9</v>
+      </c>
+      <c r="F37" t="n">
+        <v>0</v>
+      </c>
+      <c r="G37" t="n">
+        <v>64.29000000000001</v>
+      </c>
+      <c r="H37" t="n">
+        <v>64.29000000000001</v>
+      </c>
+      <c r="I37" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Furqan Ullah Khan</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>373683</v>
+      </c>
+      <c r="C38" t="n">
+        <v>195</v>
+      </c>
+      <c r="D38" t="n">
+        <v>124</v>
+      </c>
+      <c r="E38" t="n">
+        <v>116</v>
+      </c>
+      <c r="F38" t="n">
+        <v>8</v>
+      </c>
+      <c r="G38" t="n">
+        <v>63.59</v>
+      </c>
+      <c r="H38" t="n">
+        <v>59.49</v>
+      </c>
+      <c r="I38" t="n">
+        <v>4.1</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Usman Ali</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>373687</v>
+      </c>
+      <c r="C39" t="n">
+        <v>8</v>
+      </c>
+      <c r="D39" t="n">
+        <v>5</v>
+      </c>
+      <c r="E39" t="n">
+        <v>5</v>
+      </c>
+      <c r="F39" t="n">
+        <v>0</v>
+      </c>
+      <c r="G39" t="n">
+        <v>62.5</v>
+      </c>
+      <c r="H39" t="n">
+        <v>62.5</v>
+      </c>
+      <c r="I39" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Ishaq Khan</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>373699</v>
+      </c>
+      <c r="C40" t="n">
+        <v>170</v>
+      </c>
+      <c r="D40" t="n">
+        <v>101</v>
+      </c>
+      <c r="E40" t="n">
+        <v>100</v>
+      </c>
+      <c r="F40" t="n">
+        <v>1</v>
+      </c>
+      <c r="G40" t="n">
+        <v>59.41</v>
+      </c>
+      <c r="H40" t="n">
+        <v>58.82</v>
+      </c>
+      <c r="I40" t="n">
+        <v>0.59</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Anum Gul</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>373656</v>
+      </c>
+      <c r="C41" t="n">
+        <v>103</v>
+      </c>
+      <c r="D41" t="n">
+        <v>55</v>
+      </c>
+      <c r="E41" t="n">
+        <v>51</v>
+      </c>
+      <c r="F41" t="n">
+        <v>4</v>
+      </c>
+      <c r="G41" t="n">
+        <v>53.4</v>
+      </c>
+      <c r="H41" t="n">
+        <v>49.51</v>
+      </c>
+      <c r="I41" t="n">
+        <v>3.88</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Munawar Khan</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>373668</v>
+      </c>
+      <c r="C42" t="n">
+        <v>73</v>
+      </c>
+      <c r="D42" t="n">
+        <v>38</v>
+      </c>
+      <c r="E42" t="n">
+        <v>32</v>
+      </c>
+      <c r="F42" t="n">
+        <v>6</v>
+      </c>
+      <c r="G42" t="n">
+        <v>52.05</v>
+      </c>
+      <c r="H42" t="n">
+        <v>43.84</v>
+      </c>
+      <c r="I42" t="n">
+        <v>8.220000000000001</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Muhammad Noor</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>373701</v>
+      </c>
+      <c r="C43" t="n">
+        <v>8</v>
+      </c>
+      <c r="D43" t="n">
+        <v>4</v>
+      </c>
+      <c r="E43" t="n">
+        <v>3</v>
+      </c>
+      <c r="F43" t="n">
+        <v>1</v>
+      </c>
+      <c r="G43" t="n">
+        <v>50</v>
+      </c>
+      <c r="H43" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="I43" t="n">
+        <v>12.5</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Muhammad Naeem</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>373694</v>
+      </c>
+      <c r="C44" t="n">
+        <v>6</v>
+      </c>
+      <c r="D44" t="n">
+        <v>3</v>
+      </c>
+      <c r="E44" t="n">
+        <v>3</v>
+      </c>
+      <c r="F44" t="n">
+        <v>0</v>
+      </c>
+      <c r="G44" t="n">
+        <v>50</v>
+      </c>
+      <c r="H44" t="n">
+        <v>50</v>
+      </c>
+      <c r="I44" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Muhammad Shahid Khan</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>373662</v>
+      </c>
+      <c r="C45" t="n">
+        <v>6</v>
+      </c>
+      <c r="D45" t="n">
+        <v>3</v>
+      </c>
+      <c r="E45" t="n">
+        <v>3</v>
+      </c>
+      <c r="F45" t="n">
+        <v>0</v>
+      </c>
+      <c r="G45" t="n">
+        <v>50</v>
+      </c>
+      <c r="H45" t="n">
+        <v>50</v>
+      </c>
+      <c r="I45" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Nillum Bibi</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>373652</v>
+      </c>
+      <c r="C46" t="n">
+        <v>169</v>
+      </c>
+      <c r="D46" t="n">
+        <v>64</v>
+      </c>
+      <c r="E46" t="n">
+        <v>61</v>
+      </c>
+      <c r="F46" t="n">
+        <v>3</v>
+      </c>
+      <c r="G46" t="n">
+        <v>37.87</v>
+      </c>
+      <c r="H46" t="n">
+        <v>36.09</v>
+      </c>
+      <c r="I46" t="n">
+        <v>1.78</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Robina Shaheen</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>373639</v>
+      </c>
+      <c r="C47" t="n">
+        <v>8</v>
+      </c>
+      <c r="D47" t="n">
+        <v>3</v>
+      </c>
+      <c r="E47" t="n">
+        <v>2</v>
+      </c>
+      <c r="F47" t="n">
+        <v>1</v>
+      </c>
+      <c r="G47" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="H47" t="n">
+        <v>25</v>
+      </c>
+      <c r="I47" t="n">
+        <v>12.5</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Sajjad Khan</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>373700</v>
+      </c>
+      <c r="C48" t="n">
+        <v>8</v>
+      </c>
+      <c r="D48" t="n">
+        <v>3</v>
+      </c>
+      <c r="E48" t="n">
+        <v>3</v>
+      </c>
+      <c r="F48" t="n">
+        <v>0</v>
+      </c>
+      <c r="G48" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="H48" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="I48" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Nazia</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>373657</v>
+      </c>
+      <c r="C49" t="n">
+        <v>144</v>
+      </c>
+      <c r="D49" t="n">
+        <v>51</v>
+      </c>
+      <c r="E49" t="n">
+        <v>49</v>
+      </c>
+      <c r="F49" t="n">
+        <v>2</v>
+      </c>
+      <c r="G49" t="n">
+        <v>35.42</v>
+      </c>
+      <c r="H49" t="n">
+        <v>34.03</v>
+      </c>
+      <c r="I49" t="n">
+        <v>1.39</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Alia Khan</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>373681</v>
+      </c>
+      <c r="C50" t="n">
+        <v>129</v>
+      </c>
+      <c r="D50" t="n">
+        <v>44</v>
+      </c>
+      <c r="E50" t="n">
+        <v>40</v>
+      </c>
+      <c r="F50" t="n">
+        <v>4</v>
+      </c>
+      <c r="G50" t="n">
+        <v>34.11</v>
+      </c>
+      <c r="H50" t="n">
+        <v>31.01</v>
+      </c>
+      <c r="I50" t="n">
+        <v>3.1</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Aisha Aman</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>373704</v>
+      </c>
+      <c r="C51" t="n">
+        <v>11</v>
+      </c>
+      <c r="D51" t="n">
+        <v>3</v>
+      </c>
+      <c r="E51" t="n">
+        <v>2</v>
+      </c>
+      <c r="F51" t="n">
+        <v>1</v>
+      </c>
+      <c r="G51" t="n">
+        <v>27.27</v>
+      </c>
+      <c r="H51" t="n">
+        <v>18.18</v>
+      </c>
+      <c r="I51" t="n">
+        <v>9.09</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Iqra Bibi</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>373708</v>
+      </c>
+      <c r="C52" t="n">
+        <v>8</v>
+      </c>
+      <c r="D52" t="n">
+        <v>2</v>
+      </c>
+      <c r="E52" t="n">
+        <v>2</v>
+      </c>
+      <c r="F52" t="n">
+        <v>0</v>
+      </c>
+      <c r="G52" t="n">
+        <v>25</v>
+      </c>
+      <c r="H52" t="n">
+        <v>25</v>
+      </c>
+      <c r="I52" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Hijab Zahra</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>373637</v>
+      </c>
+      <c r="C53" t="n">
+        <v>4</v>
+      </c>
+      <c r="D53" t="n">
+        <v>1</v>
+      </c>
+      <c r="E53" t="n">
+        <v>1</v>
+      </c>
+      <c r="F53" t="n">
+        <v>0</v>
+      </c>
+      <c r="G53" t="n">
+        <v>25</v>
+      </c>
+      <c r="H53" t="n">
+        <v>25</v>
+      </c>
+      <c r="I53" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Laiba Khan</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>373653</v>
+      </c>
+      <c r="C54" t="n">
+        <v>121</v>
+      </c>
+      <c r="D54" t="n">
+        <v>26</v>
+      </c>
+      <c r="E54" t="n">
+        <v>22</v>
+      </c>
+      <c r="F54" t="n">
+        <v>4</v>
+      </c>
+      <c r="G54" t="n">
+        <v>21.49</v>
+      </c>
+      <c r="H54" t="n">
+        <v>18.18</v>
+      </c>
+      <c r="I54" t="n">
+        <v>3.31</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Gul Rukh</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>373644</v>
+      </c>
+      <c r="C55" t="n">
+        <v>6</v>
+      </c>
+      <c r="D55" t="n">
+        <v>1</v>
+      </c>
+      <c r="E55" t="n">
+        <v>1</v>
+      </c>
+      <c r="F55" t="n">
+        <v>0</v>
+      </c>
+      <c r="G55" t="n">
+        <v>16.67</v>
+      </c>
+      <c r="H55" t="n">
+        <v>16.67</v>
+      </c>
+      <c r="I55" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Mahnoorr</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>373670</v>
+      </c>
+      <c r="C56" t="n">
+        <v>13</v>
+      </c>
+      <c r="D56" t="n">
+        <v>2</v>
+      </c>
+      <c r="E56" t="n">
+        <v>1</v>
+      </c>
+      <c r="F56" t="n">
+        <v>1</v>
+      </c>
+      <c r="G56" t="n">
+        <v>15.38</v>
+      </c>
+      <c r="H56" t="n">
+        <v>7.69</v>
+      </c>
+      <c r="I56" t="n">
+        <v>7.69</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Sidra Khan</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>373645</v>
+      </c>
+      <c r="C57" t="n">
+        <v>7</v>
+      </c>
+      <c r="D57" t="n">
+        <v>1</v>
+      </c>
+      <c r="E57" t="n">
+        <v>1</v>
+      </c>
+      <c r="F57" t="n">
+        <v>0</v>
+      </c>
+      <c r="G57" t="n">
+        <v>14.29</v>
+      </c>
+      <c r="H57" t="n">
+        <v>14.29</v>
+      </c>
+      <c r="I57" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Irum ikram (duplicate name received from listed_girl_tracking_survey on June 29, 2026 12:08 UTC+00:00; submission key: uuid:b700a976-75ee-467c-87e9-1d5163ec238d)</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>541376</v>
+      </c>
+      <c r="C58" t="n">
+        <v>64</v>
+      </c>
+      <c r="D58" t="n">
+        <v>0</v>
+      </c>
+      <c r="E58" t="n">
+        <v>0</v>
+      </c>
+      <c r="F58" t="n">
+        <v>0</v>
+      </c>
+      <c r="G58" t="n">
+        <v>0</v>
+      </c>
+      <c r="H58" t="n">
+        <v>0</v>
+      </c>
+      <c r="I58" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Lati Khan (duplicate name received from listed_girl_tracking_survey on June 28, 2026 10:43 UTC+00:00; submission key: uuid:e4e89d53-e5be-40ff-bb2c-fa94c0d50011)</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>564273</v>
+      </c>
+      <c r="C59" t="n">
+        <v>56</v>
+      </c>
+      <c r="D59" t="n">
+        <v>0</v>
+      </c>
+      <c r="E59" t="n">
+        <v>0</v>
+      </c>
+      <c r="F59" t="n">
+        <v>0</v>
+      </c>
+      <c r="G59" t="n">
+        <v>0</v>
+      </c>
+      <c r="H59" t="n">
+        <v>0</v>
+      </c>
+      <c r="I59" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Lati khan (duplicate name received from listed_girl_tracking_survey_new_sample on July 4, 2026 14:31 UTC+00:00; submission key: uuid:6316d214-c458-4786-937a-bd81b08c15c5)</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>671211</v>
+      </c>
+      <c r="C60" t="n">
+        <v>14</v>
+      </c>
+      <c r="D60" t="n">
+        <v>0</v>
+      </c>
+      <c r="E60" t="n">
+        <v>0</v>
+      </c>
+      <c r="F60" t="n">
+        <v>0</v>
+      </c>
+      <c r="G60" t="n">
+        <v>0</v>
+      </c>
+      <c r="H60" t="n">
+        <v>0</v>
+      </c>
+      <c r="I60" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Muhammad Usman</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>373666</v>
+      </c>
+      <c r="C61" t="n">
+        <v>14</v>
+      </c>
+      <c r="D61" t="n">
+        <v>0</v>
+      </c>
+      <c r="E61" t="n">
+        <v>0</v>
+      </c>
+      <c r="F61" t="n">
+        <v>0</v>
+      </c>
+      <c r="G61" t="n">
+        <v>0</v>
+      </c>
+      <c r="H61" t="n">
+        <v>0</v>
+      </c>
+      <c r="I61" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Muhammad Waseem</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
+        <v>373689</v>
+      </c>
+      <c r="C62" t="n">
+        <v>3</v>
+      </c>
+      <c r="D62" t="n">
+        <v>0</v>
+      </c>
+      <c r="E62" t="n">
+        <v>0</v>
+      </c>
+      <c r="F62" t="n">
+        <v>0</v>
+      </c>
+      <c r="G62" t="n">
+        <v>0</v>
+      </c>
+      <c r="H62" t="n">
+        <v>0</v>
+      </c>
+      <c r="I62" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Muhammad naeem (duplicate name received from primary_school_listing_survey on February 14, 2026 14:38 UTC+00:00; submission key: uuid:5f0e427e-5fd2-4474-be64-ae5f2c4617a2)</t>
+        </is>
+      </c>
+      <c r="B63" t="n">
+        <v>571571</v>
+      </c>
+      <c r="C63" t="n">
+        <v>8</v>
+      </c>
+      <c r="D63" t="n">
+        <v>0</v>
+      </c>
+      <c r="E63" t="n">
+        <v>0</v>
+      </c>
+      <c r="F63" t="n">
+        <v>0</v>
+      </c>
+      <c r="G63" t="n">
+        <v>0</v>
+      </c>
+      <c r="H63" t="n">
+        <v>0</v>
+      </c>
+      <c r="I63" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
           <t>Naureen khan (duplicate name received from listed_girl_tracking_survey_new_sample on July 7, 2026 14:41 UTC+00:00; submission key: uuid:bbf56e1f-36f5-4ebf-9e0f-df83015a0871)</t>
         </is>
       </c>
-      <c r="B17" t="n">
+      <c r="B64" t="n">
         <v>453925</v>
       </c>
-      <c r="C17" t="n">
-        <v>4</v>
-      </c>
-      <c r="D17" t="n">
-        <v>0</v>
-      </c>
-      <c r="E17" t="n">
-        <v>0</v>
-      </c>
-      <c r="F17" t="n">
-        <v>0</v>
-      </c>
-      <c r="G17" t="n">
-        <v>0</v>
-      </c>
-      <c r="H17" t="n">
-        <v>0</v>
-      </c>
-      <c r="I17" t="n">
+      <c r="C64" t="n">
+        <v>57</v>
+      </c>
+      <c r="D64" t="n">
+        <v>0</v>
+      </c>
+      <c r="E64" t="n">
+        <v>0</v>
+      </c>
+      <c r="F64" t="n">
+        <v>0</v>
+      </c>
+      <c r="G64" t="n">
+        <v>0</v>
+      </c>
+      <c r="H64" t="n">
+        <v>0</v>
+      </c>
+      <c r="I64" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Samreen</t>
+        </is>
+      </c>
+      <c r="B65" t="n">
+        <v>373711</v>
+      </c>
+      <c r="C65" t="n">
+        <v>3</v>
+      </c>
+      <c r="D65" t="n">
+        <v>0</v>
+      </c>
+      <c r="E65" t="n">
+        <v>0</v>
+      </c>
+      <c r="F65" t="n">
+        <v>0</v>
+      </c>
+      <c r="G65" t="n">
+        <v>0</v>
+      </c>
+      <c r="H65" t="n">
+        <v>0</v>
+      </c>
+      <c r="I65" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Samreen</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>639258</v>
+      </c>
+      <c r="C66" t="n">
+        <v>1</v>
+      </c>
+      <c r="D66" t="n">
+        <v>0</v>
+      </c>
+      <c r="E66" t="n">
+        <v>0</v>
+      </c>
+      <c r="F66" t="n">
+        <v>0</v>
+      </c>
+      <c r="G66" t="n">
+        <v>0</v>
+      </c>
+      <c r="H66" t="n">
+        <v>0</v>
+      </c>
+      <c r="I66" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Shafaq Zahra</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr"/>
+      <c r="C67" t="n">
+        <v>1</v>
+      </c>
+      <c r="D67" t="n">
+        <v>0</v>
+      </c>
+      <c r="E67" t="n">
+        <v>0</v>
+      </c>
+      <c r="F67" t="n">
+        <v>0</v>
+      </c>
+      <c r="G67" t="n">
+        <v>0</v>
+      </c>
+      <c r="H67" t="n">
+        <v>0</v>
+      </c>
+      <c r="I67" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Shakeel Ahmed</t>
+        </is>
+      </c>
+      <c r="B68" t="n">
+        <v>373686</v>
+      </c>
+      <c r="C68" t="n">
+        <v>3</v>
+      </c>
+      <c r="D68" t="n">
+        <v>0</v>
+      </c>
+      <c r="E68" t="n">
+        <v>0</v>
+      </c>
+      <c r="F68" t="n">
+        <v>0</v>
+      </c>
+      <c r="G68" t="n">
+        <v>0</v>
+      </c>
+      <c r="H68" t="n">
+        <v>0</v>
+      </c>
+      <c r="I68" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Syed Haider Abbas</t>
+        </is>
+      </c>
+      <c r="B69" t="n">
+        <v>373713</v>
+      </c>
+      <c r="C69" t="n">
+        <v>2</v>
+      </c>
+      <c r="D69" t="n">
+        <v>0</v>
+      </c>
+      <c r="E69" t="n">
+        <v>0</v>
+      </c>
+      <c r="F69" t="n">
+        <v>0</v>
+      </c>
+      <c r="G69" t="n">
+        <v>0</v>
+      </c>
+      <c r="H69" t="n">
+        <v>0</v>
+      </c>
+      <c r="I69" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr"/>
+      <c r="B70" t="inlineStr"/>
+      <c r="C70" t="n">
+        <v>0</v>
+      </c>
+      <c r="D70" t="n">
+        <v>0</v>
+      </c>
+      <c r="E70" t="n">
+        <v>0</v>
+      </c>
+      <c r="F70" t="n">
+        <v>0</v>
+      </c>
+      <c r="G70" t="n">
+        <v>0</v>
+      </c>
+      <c r="H70" t="n">
+        <v>0</v>
+      </c>
+      <c r="I70" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: implement deduplication for duplicate-family issues and update related logic
</commit_message>
<xml_diff>
--- a/Error_log/Enumerator_Performance.xlsx
+++ b/Error_log/Enumerator_Performance.xlsx
@@ -509,10 +509,10 @@
         <v>373648</v>
       </c>
       <c r="C5" t="n">
-        <v>343</v>
+        <v>340</v>
       </c>
       <c r="D5" t="n">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="E5" t="n">
         <v>85</v>
@@ -547,10 +547,10 @@
         <v>373696</v>
       </c>
       <c r="C7" t="n">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="D7" t="n">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="E7" t="n">
         <v>45</v>
@@ -604,10 +604,10 @@
         <v>373651</v>
       </c>
       <c r="C10" t="n">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="D10" t="n">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="E10" t="n">
         <v>96</v>
@@ -680,10 +680,10 @@
         <v>373712</v>
       </c>
       <c r="C14" t="n">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="D14" t="n">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="E14" t="n">
         <v>202</v>
@@ -737,10 +737,10 @@
         <v>373692</v>
       </c>
       <c r="C17" t="n">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="D17" t="n">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E17" t="n">
         <v>183</v>
@@ -1742,19 +1742,19 @@
         <v>104</v>
       </c>
       <c r="D6" t="n">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="E6" t="n">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="F6" t="n">
         <v>202</v>
       </c>
       <c r="G6" t="n">
-        <v>320.19</v>
+        <v>318.27</v>
       </c>
       <c r="H6" t="n">
-        <v>125.96</v>
+        <v>124.04</v>
       </c>
       <c r="I6" t="n">
         <v>194.23</v>
@@ -1773,19 +1773,19 @@
         <v>101</v>
       </c>
       <c r="D7" t="n">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="E7" t="n">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="F7" t="n">
         <v>183</v>
       </c>
       <c r="G7" t="n">
-        <v>292.08</v>
+        <v>290.1</v>
       </c>
       <c r="H7" t="n">
-        <v>110.89</v>
+        <v>108.91</v>
       </c>
       <c r="I7" t="n">
         <v>181.19</v>
@@ -1928,19 +1928,19 @@
         <v>152</v>
       </c>
       <c r="D12" t="n">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="E12" t="n">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="F12" t="n">
         <v>96</v>
       </c>
       <c r="G12" t="n">
-        <v>162.5</v>
+        <v>161.18</v>
       </c>
       <c r="H12" t="n">
-        <v>99.34</v>
+        <v>98.03</v>
       </c>
       <c r="I12" t="n">
         <v>63.16</v>
@@ -2011,63 +2011,63 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Shazia Bibi</t>
+          <t>Mehran Khan</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>373648</v>
+        <v>373684</v>
       </c>
       <c r="C15" t="n">
-        <v>234</v>
+        <v>200</v>
       </c>
       <c r="D15" t="n">
-        <v>343</v>
+        <v>293</v>
       </c>
       <c r="E15" t="n">
-        <v>258</v>
+        <v>265</v>
       </c>
       <c r="F15" t="n">
-        <v>85</v>
+        <v>28</v>
       </c>
       <c r="G15" t="n">
-        <v>146.58</v>
+        <v>146.5</v>
       </c>
       <c r="H15" t="n">
-        <v>110.26</v>
+        <v>132.5</v>
       </c>
       <c r="I15" t="n">
-        <v>36.32</v>
+        <v>14</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Mehran Khan</t>
+          <t>Shazia Bibi</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>373684</v>
+        <v>373648</v>
       </c>
       <c r="C16" t="n">
-        <v>200</v>
+        <v>234</v>
       </c>
       <c r="D16" t="n">
-        <v>293</v>
+        <v>340</v>
       </c>
       <c r="E16" t="n">
-        <v>265</v>
+        <v>255</v>
       </c>
       <c r="F16" t="n">
-        <v>28</v>
+        <v>85</v>
       </c>
       <c r="G16" t="n">
-        <v>146.5</v>
+        <v>145.3</v>
       </c>
       <c r="H16" t="n">
-        <v>132.5</v>
+        <v>108.97</v>
       </c>
       <c r="I16" t="n">
-        <v>14</v>
+        <v>36.32</v>
       </c>
     </row>
     <row r="17">
@@ -2145,19 +2145,19 @@
         <v>197</v>
       </c>
       <c r="D19" t="n">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="E19" t="n">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="F19" t="n">
         <v>45</v>
       </c>
       <c r="G19" t="n">
-        <v>142.13</v>
+        <v>141.12</v>
       </c>
       <c r="H19" t="n">
-        <v>119.29</v>
+        <v>118.27</v>
       </c>
       <c r="I19" t="n">
         <v>22.84</v>

</xml_diff>

<commit_message>
feat: update recategorization logic for household duplicates and refresh related Excel files
</commit_message>
<xml_diff>
--- a/Error_log/Enumerator_Performance.xlsx
+++ b/Error_log/Enumerator_Performance.xlsx
@@ -509,10 +509,10 @@
         <v>373648</v>
       </c>
       <c r="C5" t="n">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="D5" t="n">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="E5" t="n">
         <v>85</v>
@@ -737,10 +737,10 @@
         <v>373692</v>
       </c>
       <c r="C17" t="n">
-        <v>293</v>
+        <v>290</v>
       </c>
       <c r="D17" t="n">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="E17" t="n">
         <v>183</v>
@@ -1773,19 +1773,19 @@
         <v>101</v>
       </c>
       <c r="D7" t="n">
-        <v>293</v>
+        <v>290</v>
       </c>
       <c r="E7" t="n">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="F7" t="n">
         <v>183</v>
       </c>
       <c r="G7" t="n">
-        <v>290.1</v>
+        <v>287.13</v>
       </c>
       <c r="H7" t="n">
-        <v>108.91</v>
+        <v>105.94</v>
       </c>
       <c r="I7" t="n">
         <v>181.19</v>
@@ -2052,19 +2052,19 @@
         <v>234</v>
       </c>
       <c r="D16" t="n">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="E16" t="n">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="F16" t="n">
         <v>85</v>
       </c>
       <c r="G16" t="n">
-        <v>145.3</v>
+        <v>144.87</v>
       </c>
       <c r="H16" t="n">
-        <v>108.97</v>
+        <v>108.55</v>
       </c>
       <c r="I16" t="n">
         <v>36.32</v>

</xml_diff>

<commit_message>
feat: add guidance for incomplete respondent records and enhance household submission checks
</commit_message>
<xml_diff>
--- a/Error_log/Enumerator_Performance.xlsx
+++ b/Error_log/Enumerator_Performance.xlsx
@@ -509,10 +509,10 @@
         <v>373648</v>
       </c>
       <c r="C5" t="n">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="D5" t="n">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="E5" t="n">
         <v>98</v>
@@ -528,10 +528,10 @@
         <v>373646</v>
       </c>
       <c r="C6" t="n">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="D6" t="n">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="E6" t="n">
         <v>67</v>
@@ -547,10 +547,10 @@
         <v>373696</v>
       </c>
       <c r="C7" t="n">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="D7" t="n">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="E7" t="n">
         <v>62</v>
@@ -566,10 +566,10 @@
         <v>373642</v>
       </c>
       <c r="C8" t="n">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="D8" t="n">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="E8" t="n">
         <v>48</v>
@@ -661,10 +661,10 @@
         <v>373716</v>
       </c>
       <c r="C13" t="n">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D13" t="n">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="E13" t="n">
         <v>31</v>
@@ -737,10 +737,10 @@
         <v>373692</v>
       </c>
       <c r="C17" t="n">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="D17" t="n">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="E17" t="n">
         <v>183</v>
@@ -775,10 +775,10 @@
         <v>373658</v>
       </c>
       <c r="C19" t="n">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="D19" t="n">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="E19" t="n">
         <v>196</v>
@@ -1091,39 +1091,39 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Lati khan</t>
+          <t>Nadia bibi</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>671211</v>
+        <v>373669</v>
       </c>
       <c r="C36" t="n">
-        <v>38</v>
+        <v>91</v>
       </c>
       <c r="D36" t="n">
         <v>38</v>
       </c>
       <c r="E36" t="n">
-        <v>0</v>
+        <v>53</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Nadia bibi</t>
+          <t>Lati khan</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>373669</v>
+        <v>671211</v>
       </c>
       <c r="C37" t="n">
-        <v>90</v>
+        <v>38</v>
       </c>
       <c r="D37" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="E37" t="n">
-        <v>53</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38">
@@ -1773,19 +1773,19 @@
         <v>101</v>
       </c>
       <c r="D7" t="n">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="E7" t="n">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F7" t="n">
         <v>183</v>
       </c>
       <c r="G7" t="n">
-        <v>287.13</v>
+        <v>288.12</v>
       </c>
       <c r="H7" t="n">
-        <v>105.94</v>
+        <v>106.93</v>
       </c>
       <c r="I7" t="n">
         <v>181.19</v>
@@ -1835,19 +1835,19 @@
         <v>120</v>
       </c>
       <c r="D9" t="n">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="E9" t="n">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="F9" t="n">
         <v>196</v>
       </c>
       <c r="G9" t="n">
-        <v>248.33</v>
+        <v>249.17</v>
       </c>
       <c r="H9" t="n">
-        <v>85</v>
+        <v>85.83</v>
       </c>
       <c r="I9" t="n">
         <v>163.33</v>
@@ -1866,19 +1866,19 @@
         <v>49</v>
       </c>
       <c r="D10" t="n">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="E10" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F10" t="n">
         <v>53</v>
       </c>
       <c r="G10" t="n">
-        <v>183.67</v>
+        <v>185.71</v>
       </c>
       <c r="H10" t="n">
-        <v>75.51000000000001</v>
+        <v>77.55</v>
       </c>
       <c r="I10" t="n">
         <v>108.16</v>
@@ -1928,19 +1928,19 @@
         <v>100</v>
       </c>
       <c r="D12" t="n">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="E12" t="n">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F12" t="n">
         <v>31</v>
       </c>
       <c r="G12" t="n">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="H12" t="n">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="I12" t="n">
         <v>31</v>
@@ -1980,63 +1980,63 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Mahnoor</t>
+          <t>Shazia Bibi</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>373705</v>
+        <v>373648</v>
       </c>
       <c r="C14" t="n">
-        <v>140</v>
+        <v>240</v>
       </c>
       <c r="D14" t="n">
-        <v>207</v>
+        <v>355</v>
       </c>
       <c r="E14" t="n">
-        <v>155</v>
+        <v>257</v>
       </c>
       <c r="F14" t="n">
-        <v>52</v>
+        <v>98</v>
       </c>
       <c r="G14" t="n">
-        <v>147.86</v>
+        <v>147.92</v>
       </c>
       <c r="H14" t="n">
-        <v>110.71</v>
+        <v>107.08</v>
       </c>
       <c r="I14" t="n">
-        <v>37.14</v>
+        <v>40.83</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Shazia Bibi</t>
+          <t>Mahnoor</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>373648</v>
+        <v>373705</v>
       </c>
       <c r="C15" t="n">
-        <v>240</v>
+        <v>140</v>
       </c>
       <c r="D15" t="n">
-        <v>354</v>
+        <v>207</v>
       </c>
       <c r="E15" t="n">
-        <v>256</v>
+        <v>155</v>
       </c>
       <c r="F15" t="n">
-        <v>98</v>
+        <v>52</v>
       </c>
       <c r="G15" t="n">
-        <v>147.5</v>
+        <v>147.86</v>
       </c>
       <c r="H15" t="n">
-        <v>106.67</v>
+        <v>110.71</v>
       </c>
       <c r="I15" t="n">
-        <v>40.83</v>
+        <v>37.14</v>
       </c>
     </row>
     <row r="16">
@@ -2083,19 +2083,19 @@
         <v>203</v>
       </c>
       <c r="D17" t="n">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="E17" t="n">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="F17" t="n">
         <v>62</v>
       </c>
       <c r="G17" t="n">
-        <v>145.32</v>
+        <v>145.81</v>
       </c>
       <c r="H17" t="n">
-        <v>114.78</v>
+        <v>115.27</v>
       </c>
       <c r="I17" t="n">
         <v>30.54</v>
@@ -2114,19 +2114,19 @@
         <v>189</v>
       </c>
       <c r="D18" t="n">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="E18" t="n">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="F18" t="n">
         <v>48</v>
       </c>
       <c r="G18" t="n">
-        <v>143.39</v>
+        <v>143.92</v>
       </c>
       <c r="H18" t="n">
-        <v>117.99</v>
+        <v>118.52</v>
       </c>
       <c r="I18" t="n">
         <v>25.4</v>
@@ -2238,19 +2238,19 @@
         <v>245</v>
       </c>
       <c r="D22" t="n">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="E22" t="n">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="F22" t="n">
         <v>67</v>
       </c>
       <c r="G22" t="n">
-        <v>124.49</v>
+        <v>124.9</v>
       </c>
       <c r="H22" t="n">
-        <v>97.14</v>
+        <v>97.55</v>
       </c>
       <c r="I22" t="n">
         <v>27.35</v>

</xml_diff>

<commit_message>
feat: optimize data processing and enhance performance across multiple scripts
</commit_message>
<xml_diff>
--- a/Error_log/Enumerator_Performance.xlsx
+++ b/Error_log/Enumerator_Performance.xlsx
@@ -464,10 +464,10 @@
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="n">
-        <v>1917</v>
+        <v>1863</v>
       </c>
       <c r="D2" t="n">
-        <v>1898</v>
+        <v>1844</v>
       </c>
       <c r="E2" t="n">
         <v>19</v>

</xml_diff>

<commit_message>
feat: update error guidance and refine parental consent checks in girls.py
</commit_message>
<xml_diff>
--- a/Error_log/Enumerator_Performance.xlsx
+++ b/Error_log/Enumerator_Performance.xlsx
@@ -483,13 +483,13 @@
         <v>373641</v>
       </c>
       <c r="C3" t="n">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="D3" t="n">
         <v>353</v>
       </c>
       <c r="E3" t="n">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="4">
@@ -540,13 +540,13 @@
         <v>373646</v>
       </c>
       <c r="C6" t="n">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="D6" t="n">
         <v>250</v>
       </c>
       <c r="E6" t="n">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="7">
@@ -578,13 +578,13 @@
         <v>373642</v>
       </c>
       <c r="C8" t="n">
-        <v>288</v>
+        <v>284</v>
       </c>
       <c r="D8" t="n">
         <v>232</v>
       </c>
       <c r="E8" t="n">
-        <v>56</v>
+        <v>52</v>
       </c>
     </row>
     <row r="9">
@@ -616,13 +616,13 @@
         <v>373651</v>
       </c>
       <c r="C10" t="n">
-        <v>309</v>
+        <v>290</v>
       </c>
       <c r="D10" t="n">
         <v>166</v>
       </c>
       <c r="E10" t="n">
-        <v>143</v>
+        <v>124</v>
       </c>
     </row>
     <row r="11">
@@ -635,13 +635,13 @@
         <v>373705</v>
       </c>
       <c r="C11" t="n">
-        <v>224</v>
+        <v>216</v>
       </c>
       <c r="D11" t="n">
         <v>164</v>
       </c>
       <c r="E11" t="n">
-        <v>60</v>
+        <v>52</v>
       </c>
     </row>
     <row r="12">
@@ -749,13 +749,13 @@
         <v>373706</v>
       </c>
       <c r="C17" t="n">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="D17" t="n">
         <v>111</v>
       </c>
       <c r="E17" t="n">
-        <v>46</v>
+        <v>42</v>
       </c>
     </row>
     <row r="18">
@@ -768,13 +768,13 @@
         <v>373692</v>
       </c>
       <c r="C18" t="n">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="D18" t="n">
         <v>108</v>
       </c>
       <c r="E18" t="n">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="19">
@@ -996,13 +996,13 @@
         <v>373710</v>
       </c>
       <c r="C30" t="n">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="D30" t="n">
         <v>62</v>
       </c>
       <c r="E30" t="n">
-        <v>40</v>
+        <v>35</v>
       </c>
     </row>
     <row r="31">
@@ -1091,13 +1091,13 @@
         <v>373669</v>
       </c>
       <c r="C35" t="n">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="D35" t="n">
         <v>45</v>
       </c>
       <c r="E35" t="n">
-        <v>73</v>
+        <v>69</v>
       </c>
     </row>
     <row r="36">
@@ -1785,22 +1785,22 @@
         <v>101</v>
       </c>
       <c r="D7" t="n">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="E7" t="n">
         <v>108</v>
       </c>
       <c r="F7" t="n">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="G7" t="n">
-        <v>288.12</v>
+        <v>287.13</v>
       </c>
       <c r="H7" t="n">
         <v>106.93</v>
       </c>
       <c r="I7" t="n">
-        <v>181.19</v>
+        <v>180.2</v>
       </c>
     </row>
     <row r="8">
@@ -1868,125 +1868,125 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Nadia bibi</t>
+          <t>Asma Bibi</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>373669</v>
+        <v>373641</v>
       </c>
       <c r="C10" t="n">
-        <v>65</v>
+        <v>261</v>
       </c>
       <c r="D10" t="n">
-        <v>118</v>
+        <v>463</v>
       </c>
       <c r="E10" t="n">
-        <v>45</v>
+        <v>353</v>
       </c>
       <c r="F10" t="n">
-        <v>73</v>
+        <v>110</v>
       </c>
       <c r="G10" t="n">
-        <v>181.54</v>
+        <v>177.39</v>
       </c>
       <c r="H10" t="n">
-        <v>69.23</v>
+        <v>135.25</v>
       </c>
       <c r="I10" t="n">
-        <v>112.31</v>
+        <v>42.15</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Asma Bibi</t>
+          <t>Nadia bibi</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>373641</v>
+        <v>373669</v>
       </c>
       <c r="C11" t="n">
-        <v>261</v>
+        <v>65</v>
       </c>
       <c r="D11" t="n">
-        <v>464</v>
+        <v>114</v>
       </c>
       <c r="E11" t="n">
-        <v>353</v>
+        <v>45</v>
       </c>
       <c r="F11" t="n">
-        <v>111</v>
+        <v>69</v>
       </c>
       <c r="G11" t="n">
-        <v>177.78</v>
+        <v>175.38</v>
       </c>
       <c r="H11" t="n">
-        <v>135.25</v>
+        <v>69.23</v>
       </c>
       <c r="I11" t="n">
-        <v>42.53</v>
+        <v>106.15</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Javairia</t>
+          <t>Naureen Khan</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>373651</v>
+        <v>373716</v>
       </c>
       <c r="C12" t="n">
-        <v>174</v>
+        <v>105</v>
       </c>
       <c r="D12" t="n">
-        <v>309</v>
+        <v>176</v>
       </c>
       <c r="E12" t="n">
-        <v>166</v>
+        <v>138</v>
       </c>
       <c r="F12" t="n">
-        <v>143</v>
+        <v>38</v>
       </c>
       <c r="G12" t="n">
-        <v>177.59</v>
+        <v>167.62</v>
       </c>
       <c r="H12" t="n">
-        <v>95.40000000000001</v>
+        <v>131.43</v>
       </c>
       <c r="I12" t="n">
-        <v>82.18000000000001</v>
+        <v>36.19</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Naureen Khan</t>
+          <t>Javairia</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>373716</v>
+        <v>373651</v>
       </c>
       <c r="C13" t="n">
-        <v>105</v>
+        <v>174</v>
       </c>
       <c r="D13" t="n">
-        <v>176</v>
+        <v>290</v>
       </c>
       <c r="E13" t="n">
-        <v>138</v>
+        <v>166</v>
       </c>
       <c r="F13" t="n">
-        <v>38</v>
+        <v>124</v>
       </c>
       <c r="G13" t="n">
-        <v>167.62</v>
+        <v>166.67</v>
       </c>
       <c r="H13" t="n">
-        <v>131.43</v>
+        <v>95.40000000000001</v>
       </c>
       <c r="I13" t="n">
-        <v>36.19</v>
+        <v>71.26000000000001</v>
       </c>
     </row>
     <row r="14">
@@ -2054,63 +2054,63 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Irum Ikram</t>
+          <t>Shazia Bibi</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>373642</v>
+        <v>373648</v>
       </c>
       <c r="C16" t="n">
-        <v>198</v>
+        <v>259</v>
       </c>
       <c r="D16" t="n">
-        <v>288</v>
+        <v>375</v>
       </c>
       <c r="E16" t="n">
-        <v>232</v>
+        <v>266</v>
       </c>
       <c r="F16" t="n">
-        <v>56</v>
+        <v>109</v>
       </c>
       <c r="G16" t="n">
-        <v>145.45</v>
+        <v>144.79</v>
       </c>
       <c r="H16" t="n">
-        <v>117.17</v>
+        <v>102.7</v>
       </c>
       <c r="I16" t="n">
-        <v>28.28</v>
+        <v>42.08</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Shazia Bibi</t>
+          <t>Irum Ikram</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>373648</v>
+        <v>373642</v>
       </c>
       <c r="C17" t="n">
-        <v>259</v>
+        <v>198</v>
       </c>
       <c r="D17" t="n">
-        <v>375</v>
+        <v>284</v>
       </c>
       <c r="E17" t="n">
-        <v>266</v>
+        <v>232</v>
       </c>
       <c r="F17" t="n">
-        <v>109</v>
+        <v>52</v>
       </c>
       <c r="G17" t="n">
-        <v>144.79</v>
+        <v>143.43</v>
       </c>
       <c r="H17" t="n">
-        <v>102.7</v>
+        <v>117.17</v>
       </c>
       <c r="I17" t="n">
-        <v>42.08</v>
+        <v>26.26</v>
       </c>
     </row>
     <row r="18">
@@ -2188,22 +2188,22 @@
         <v>158</v>
       </c>
       <c r="D20" t="n">
-        <v>224</v>
+        <v>216</v>
       </c>
       <c r="E20" t="n">
         <v>164</v>
       </c>
       <c r="F20" t="n">
-        <v>60</v>
+        <v>52</v>
       </c>
       <c r="G20" t="n">
-        <v>141.77</v>
+        <v>136.71</v>
       </c>
       <c r="H20" t="n">
         <v>103.8</v>
       </c>
       <c r="I20" t="n">
-        <v>37.97</v>
+        <v>32.91</v>
       </c>
     </row>
     <row r="21">
@@ -2250,22 +2250,22 @@
         <v>266</v>
       </c>
       <c r="D22" t="n">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="E22" t="n">
         <v>250</v>
       </c>
       <c r="F22" t="n">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="G22" t="n">
-        <v>125.94</v>
+        <v>125.56</v>
       </c>
       <c r="H22" t="n">
         <v>93.98</v>
       </c>
       <c r="I22" t="n">
-        <v>31.95</v>
+        <v>31.58</v>
       </c>
     </row>
     <row r="23">
@@ -2312,22 +2312,22 @@
         <v>155</v>
       </c>
       <c r="D24" t="n">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="E24" t="n">
         <v>111</v>
       </c>
       <c r="F24" t="n">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="G24" t="n">
-        <v>101.29</v>
+        <v>98.70999999999999</v>
       </c>
       <c r="H24" t="n">
         <v>71.61</v>
       </c>
       <c r="I24" t="n">
-        <v>29.68</v>
+        <v>27.1</v>
       </c>
     </row>
     <row r="25">
@@ -2457,125 +2457,125 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Summiya Hayat</t>
+          <t>Muniba Shamim</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>373710</v>
+        <v>373659</v>
       </c>
       <c r="C29" t="n">
-        <v>124</v>
+        <v>72</v>
       </c>
       <c r="D29" t="n">
-        <v>102</v>
+        <v>58</v>
       </c>
       <c r="E29" t="n">
-        <v>62</v>
+        <v>49</v>
       </c>
       <c r="F29" t="n">
-        <v>40</v>
+        <v>9</v>
       </c>
       <c r="G29" t="n">
-        <v>82.26000000000001</v>
+        <v>80.56</v>
       </c>
       <c r="H29" t="n">
-        <v>50</v>
+        <v>68.06</v>
       </c>
       <c r="I29" t="n">
-        <v>32.26</v>
+        <v>12.5</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Muniba Shamim</t>
+          <t>Muhammad Yousaf</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>373659</v>
+        <v>373690</v>
       </c>
       <c r="C30" t="n">
-        <v>72</v>
+        <v>132</v>
       </c>
       <c r="D30" t="n">
-        <v>58</v>
+        <v>105</v>
       </c>
       <c r="E30" t="n">
-        <v>49</v>
+        <v>96</v>
       </c>
       <c r="F30" t="n">
         <v>9</v>
       </c>
       <c r="G30" t="n">
-        <v>80.56</v>
+        <v>79.55</v>
       </c>
       <c r="H30" t="n">
-        <v>68.06</v>
+        <v>72.73</v>
       </c>
       <c r="I30" t="n">
-        <v>12.5</v>
+        <v>6.82</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Muhammad Yousaf</t>
+          <t>Khalida Bibi</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>373690</v>
+        <v>373673</v>
       </c>
       <c r="C31" t="n">
-        <v>132</v>
+        <v>177</v>
       </c>
       <c r="D31" t="n">
-        <v>105</v>
+        <v>140</v>
       </c>
       <c r="E31" t="n">
-        <v>96</v>
+        <v>140</v>
       </c>
       <c r="F31" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="G31" t="n">
-        <v>79.55</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="H31" t="n">
-        <v>72.73</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="I31" t="n">
-        <v>6.82</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Khalida Bibi</t>
+          <t>Summiya Hayat</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>373673</v>
+        <v>373710</v>
       </c>
       <c r="C32" t="n">
-        <v>177</v>
+        <v>124</v>
       </c>
       <c r="D32" t="n">
-        <v>140</v>
+        <v>97</v>
       </c>
       <c r="E32" t="n">
-        <v>140</v>
+        <v>62</v>
       </c>
       <c r="F32" t="n">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="G32" t="n">
-        <v>79.09999999999999</v>
+        <v>78.23</v>
       </c>
       <c r="H32" t="n">
-        <v>79.09999999999999</v>
+        <v>50</v>
       </c>
       <c r="I32" t="n">
-        <v>0</v>
+        <v>28.23</v>
       </c>
     </row>
     <row r="33">

</xml_diff>

<commit_message>
feat: enhance household review logic to include family roster in size calculations
</commit_message>
<xml_diff>
--- a/Error_log/Enumerator_Performance.xlsx
+++ b/Error_log/Enumerator_Performance.xlsx
@@ -540,13 +540,13 @@
         <v>373646</v>
       </c>
       <c r="C6" t="n">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="D6" t="n">
         <v>250</v>
       </c>
       <c r="E6" t="n">
-        <v>84</v>
+        <v>82</v>
       </c>
     </row>
     <row r="7">
@@ -578,13 +578,13 @@
         <v>373642</v>
       </c>
       <c r="C8" t="n">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="D8" t="n">
         <v>232</v>
       </c>
       <c r="E8" t="n">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="9">
@@ -616,13 +616,13 @@
         <v>373651</v>
       </c>
       <c r="C10" t="n">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="D10" t="n">
         <v>166</v>
       </c>
       <c r="E10" t="n">
-        <v>124</v>
+        <v>122</v>
       </c>
     </row>
     <row r="11">
@@ -692,13 +692,13 @@
         <v>373712</v>
       </c>
       <c r="C14" t="n">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="D14" t="n">
         <v>129</v>
       </c>
       <c r="E14" t="n">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="15">
@@ -768,13 +768,13 @@
         <v>373692</v>
       </c>
       <c r="C18" t="n">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="D18" t="n">
         <v>108</v>
       </c>
       <c r="E18" t="n">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
     <row r="19">
@@ -806,13 +806,13 @@
         <v>373658</v>
       </c>
       <c r="C20" t="n">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="D20" t="n">
         <v>103</v>
       </c>
       <c r="E20" t="n">
-        <v>196</v>
+        <v>194</v>
       </c>
     </row>
     <row r="21">
@@ -882,13 +882,13 @@
         <v>373691</v>
       </c>
       <c r="C24" t="n">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="D24" t="n">
         <v>90</v>
       </c>
       <c r="E24" t="n">
-        <v>201</v>
+        <v>199</v>
       </c>
     </row>
     <row r="25">
@@ -1754,22 +1754,22 @@
         <v>104</v>
       </c>
       <c r="D6" t="n">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="E6" t="n">
         <v>129</v>
       </c>
       <c r="F6" t="n">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="G6" t="n">
-        <v>318.27</v>
+        <v>317.31</v>
       </c>
       <c r="H6" t="n">
         <v>124.04</v>
       </c>
       <c r="I6" t="n">
-        <v>194.23</v>
+        <v>193.27</v>
       </c>
     </row>
     <row r="7">
@@ -1785,22 +1785,22 @@
         <v>101</v>
       </c>
       <c r="D7" t="n">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="E7" t="n">
         <v>108</v>
       </c>
       <c r="F7" t="n">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="G7" t="n">
-        <v>287.13</v>
+        <v>286.14</v>
       </c>
       <c r="H7" t="n">
         <v>106.93</v>
       </c>
       <c r="I7" t="n">
-        <v>180.2</v>
+        <v>179.21</v>
       </c>
     </row>
     <row r="8">
@@ -1816,22 +1816,22 @@
         <v>111</v>
       </c>
       <c r="D8" t="n">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="E8" t="n">
         <v>90</v>
       </c>
       <c r="F8" t="n">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="G8" t="n">
-        <v>262.16</v>
+        <v>260.36</v>
       </c>
       <c r="H8" t="n">
         <v>81.08</v>
       </c>
       <c r="I8" t="n">
-        <v>181.08</v>
+        <v>179.28</v>
       </c>
     </row>
     <row r="9">
@@ -1847,22 +1847,22 @@
         <v>120</v>
       </c>
       <c r="D9" t="n">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="E9" t="n">
         <v>103</v>
       </c>
       <c r="F9" t="n">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="G9" t="n">
-        <v>249.17</v>
+        <v>247.5</v>
       </c>
       <c r="H9" t="n">
         <v>85.83</v>
       </c>
       <c r="I9" t="n">
-        <v>163.33</v>
+        <v>161.67</v>
       </c>
     </row>
     <row r="10">
@@ -1971,22 +1971,22 @@
         <v>174</v>
       </c>
       <c r="D13" t="n">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="E13" t="n">
         <v>166</v>
       </c>
       <c r="F13" t="n">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="G13" t="n">
-        <v>166.67</v>
+        <v>165.52</v>
       </c>
       <c r="H13" t="n">
         <v>95.40000000000001</v>
       </c>
       <c r="I13" t="n">
-        <v>71.26000000000001</v>
+        <v>70.11</v>
       </c>
     </row>
     <row r="14">
@@ -2085,42 +2085,42 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Irum Ikram</t>
+          <t>Lati Khan</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>373642</v>
+        <v>373665</v>
       </c>
       <c r="C17" t="n">
-        <v>198</v>
+        <v>60</v>
       </c>
       <c r="D17" t="n">
-        <v>284</v>
+        <v>86</v>
       </c>
       <c r="E17" t="n">
-        <v>232</v>
+        <v>83</v>
       </c>
       <c r="F17" t="n">
-        <v>52</v>
+        <v>3</v>
       </c>
       <c r="G17" t="n">
-        <v>143.43</v>
+        <v>143.33</v>
       </c>
       <c r="H17" t="n">
-        <v>117.17</v>
+        <v>138.33</v>
       </c>
       <c r="I17" t="n">
-        <v>26.26</v>
+        <v>5</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Lati Khan</t>
+          <t>Naureen</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>373665</v>
+        <v>884887</v>
       </c>
       <c r="C18" t="n">
         <v>60</v>
@@ -2129,50 +2129,50 @@
         <v>86</v>
       </c>
       <c r="E18" t="n">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="F18" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G18" t="n">
         <v>143.33</v>
       </c>
       <c r="H18" t="n">
-        <v>138.33</v>
+        <v>136.67</v>
       </c>
       <c r="I18" t="n">
-        <v>5</v>
+        <v>6.67</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Naureen</t>
+          <t>Irum Ikram</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>884887</v>
+        <v>373642</v>
       </c>
       <c r="C19" t="n">
-        <v>60</v>
+        <v>198</v>
       </c>
       <c r="D19" t="n">
-        <v>86</v>
+        <v>283</v>
       </c>
       <c r="E19" t="n">
-        <v>82</v>
+        <v>232</v>
       </c>
       <c r="F19" t="n">
-        <v>4</v>
+        <v>51</v>
       </c>
       <c r="G19" t="n">
-        <v>143.33</v>
+        <v>142.93</v>
       </c>
       <c r="H19" t="n">
-        <v>136.67</v>
+        <v>117.17</v>
       </c>
       <c r="I19" t="n">
-        <v>6.67</v>
+        <v>25.76</v>
       </c>
     </row>
     <row r="20">
@@ -2250,22 +2250,22 @@
         <v>266</v>
       </c>
       <c r="D22" t="n">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="E22" t="n">
         <v>250</v>
       </c>
       <c r="F22" t="n">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="G22" t="n">
-        <v>125.56</v>
+        <v>124.81</v>
       </c>
       <c r="H22" t="n">
         <v>93.98</v>
       </c>
       <c r="I22" t="n">
-        <v>31.58</v>
+        <v>30.83</v>
       </c>
     </row>
     <row r="23">

</xml_diff>

<commit_message>
feat: implement consent validation logic and enhance speed check integrity
</commit_message>
<xml_diff>
--- a/Error_log/Enumerator_Performance.xlsx
+++ b/Error_log/Enumerator_Performance.xlsx
@@ -483,10 +483,10 @@
         <v>373641</v>
       </c>
       <c r="C3" t="n">
-        <v>463</v>
+        <v>461</v>
       </c>
       <c r="D3" t="n">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="E3" t="n">
         <v>110</v>
@@ -495,39 +495,39 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Shazia Bibi</t>
+          <t>Mehran Khan</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>373648</v>
+        <v>373684</v>
       </c>
       <c r="C4" t="n">
-        <v>375</v>
+        <v>293</v>
       </c>
       <c r="D4" t="n">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="E4" t="n">
-        <v>109</v>
+        <v>28</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Mehran Khan</t>
+          <t>Shazia Bibi</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>373684</v>
+        <v>373648</v>
       </c>
       <c r="C5" t="n">
-        <v>293</v>
+        <v>372</v>
       </c>
       <c r="D5" t="n">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="E5" t="n">
-        <v>28</v>
+        <v>109</v>
       </c>
     </row>
     <row r="6">
@@ -540,10 +540,10 @@
         <v>373646</v>
       </c>
       <c r="C6" t="n">
-        <v>332</v>
+        <v>328</v>
       </c>
       <c r="D6" t="n">
-        <v>250</v>
+        <v>246</v>
       </c>
       <c r="E6" t="n">
         <v>82</v>
@@ -559,10 +559,10 @@
         <v>373696</v>
       </c>
       <c r="C7" t="n">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="D7" t="n">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="E7" t="n">
         <v>94</v>
@@ -578,10 +578,10 @@
         <v>373642</v>
       </c>
       <c r="C8" t="n">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="D8" t="n">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="E8" t="n">
         <v>51</v>
@@ -616,10 +616,10 @@
         <v>373651</v>
       </c>
       <c r="C10" t="n">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="D10" t="n">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="E10" t="n">
         <v>122</v>
@@ -635,10 +635,10 @@
         <v>373705</v>
       </c>
       <c r="C11" t="n">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="D11" t="n">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="E11" t="n">
         <v>52</v>
@@ -749,10 +749,10 @@
         <v>373706</v>
       </c>
       <c r="C17" t="n">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="D17" t="n">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="E17" t="n">
         <v>42</v>
@@ -761,77 +761,77 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Zohra</t>
+          <t>Asma Gull</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>373692</v>
+        <v>373672</v>
       </c>
       <c r="C18" t="n">
-        <v>289</v>
+        <v>109</v>
       </c>
       <c r="D18" t="n">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="E18" t="n">
-        <v>181</v>
+        <v>4</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Asma Gull</t>
+          <t>Zohra</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>373672</v>
+        <v>373692</v>
       </c>
       <c r="C19" t="n">
-        <v>109</v>
+        <v>283</v>
       </c>
       <c r="D19" t="n">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="E19" t="n">
-        <v>4</v>
+        <v>181</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Samara</t>
+          <t>Ishaq Khan</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>373658</v>
+        <v>373699</v>
       </c>
       <c r="C20" t="n">
-        <v>297</v>
+        <v>101</v>
       </c>
       <c r="D20" t="n">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="E20" t="n">
-        <v>194</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Ishaq Khan</t>
+          <t>Samara</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>373699</v>
+        <v>373658</v>
       </c>
       <c r="C21" t="n">
-        <v>101</v>
+        <v>293</v>
       </c>
       <c r="D21" t="n">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E21" t="n">
-        <v>1</v>
+        <v>194</v>
       </c>
     </row>
     <row r="22">
@@ -875,39 +875,39 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Rehana Bibi</t>
+          <t>Naureen khan</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>373691</v>
+        <v>453925</v>
       </c>
       <c r="C24" t="n">
-        <v>289</v>
+        <v>91</v>
       </c>
       <c r="D24" t="n">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="E24" t="n">
-        <v>199</v>
+        <v>2</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Naureen khan</t>
+          <t>Rehana Bibi</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>453925</v>
+        <v>373691</v>
       </c>
       <c r="C25" t="n">
-        <v>91</v>
+        <v>288</v>
       </c>
       <c r="D25" t="n">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="E25" t="n">
-        <v>2</v>
+        <v>200</v>
       </c>
     </row>
     <row r="26">
@@ -996,10 +996,10 @@
         <v>373710</v>
       </c>
       <c r="C30" t="n">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D30" t="n">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E30" t="n">
         <v>35</v>
@@ -1091,10 +1091,10 @@
         <v>373669</v>
       </c>
       <c r="C35" t="n">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D35" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E35" t="n">
         <v>69</v>
@@ -1785,19 +1785,19 @@
         <v>101</v>
       </c>
       <c r="D7" t="n">
-        <v>289</v>
+        <v>283</v>
       </c>
       <c r="E7" t="n">
-        <v>108</v>
+        <v>102</v>
       </c>
       <c r="F7" t="n">
         <v>181</v>
       </c>
       <c r="G7" t="n">
-        <v>286.14</v>
+        <v>280.2</v>
       </c>
       <c r="H7" t="n">
-        <v>106.93</v>
+        <v>100.99</v>
       </c>
       <c r="I7" t="n">
         <v>179.21</v>
@@ -1816,22 +1816,22 @@
         <v>111</v>
       </c>
       <c r="D8" t="n">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="E8" t="n">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="F8" t="n">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="G8" t="n">
-        <v>260.36</v>
+        <v>259.46</v>
       </c>
       <c r="H8" t="n">
-        <v>81.08</v>
+        <v>79.28</v>
       </c>
       <c r="I8" t="n">
-        <v>179.28</v>
+        <v>180.18</v>
       </c>
     </row>
     <row r="9">
@@ -1847,19 +1847,19 @@
         <v>120</v>
       </c>
       <c r="D9" t="n">
-        <v>297</v>
+        <v>293</v>
       </c>
       <c r="E9" t="n">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="F9" t="n">
         <v>194</v>
       </c>
       <c r="G9" t="n">
-        <v>247.5</v>
+        <v>244.17</v>
       </c>
       <c r="H9" t="n">
-        <v>85.83</v>
+        <v>82.5</v>
       </c>
       <c r="I9" t="n">
         <v>161.67</v>
@@ -1878,19 +1878,19 @@
         <v>261</v>
       </c>
       <c r="D10" t="n">
-        <v>463</v>
+        <v>461</v>
       </c>
       <c r="E10" t="n">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="F10" t="n">
         <v>110</v>
       </c>
       <c r="G10" t="n">
-        <v>177.39</v>
+        <v>176.63</v>
       </c>
       <c r="H10" t="n">
-        <v>135.25</v>
+        <v>134.48</v>
       </c>
       <c r="I10" t="n">
         <v>42.15</v>
@@ -1909,19 +1909,19 @@
         <v>65</v>
       </c>
       <c r="D11" t="n">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E11" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F11" t="n">
         <v>69</v>
       </c>
       <c r="G11" t="n">
-        <v>175.38</v>
+        <v>173.85</v>
       </c>
       <c r="H11" t="n">
-        <v>69.23</v>
+        <v>67.69</v>
       </c>
       <c r="I11" t="n">
         <v>106.15</v>
@@ -1971,19 +1971,19 @@
         <v>174</v>
       </c>
       <c r="D13" t="n">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="E13" t="n">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="F13" t="n">
         <v>122</v>
       </c>
       <c r="G13" t="n">
-        <v>165.52</v>
+        <v>164.37</v>
       </c>
       <c r="H13" t="n">
-        <v>95.40000000000001</v>
+        <v>94.25</v>
       </c>
       <c r="I13" t="n">
         <v>70.11</v>
@@ -1992,63 +1992,63 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Shazia begum</t>
+          <t>Mehran Khan</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>373696</v>
+        <v>373684</v>
       </c>
       <c r="C14" t="n">
-        <v>225</v>
+        <v>200</v>
       </c>
       <c r="D14" t="n">
-        <v>330</v>
+        <v>293</v>
       </c>
       <c r="E14" t="n">
-        <v>236</v>
+        <v>265</v>
       </c>
       <c r="F14" t="n">
-        <v>94</v>
+        <v>28</v>
       </c>
       <c r="G14" t="n">
-        <v>146.67</v>
+        <v>146.5</v>
       </c>
       <c r="H14" t="n">
-        <v>104.89</v>
+        <v>132.5</v>
       </c>
       <c r="I14" t="n">
-        <v>41.78</v>
+        <v>14</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Mehran Khan</t>
+          <t>Shazia begum</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>373684</v>
+        <v>373696</v>
       </c>
       <c r="C15" t="n">
-        <v>200</v>
+        <v>225</v>
       </c>
       <c r="D15" t="n">
-        <v>293</v>
+        <v>328</v>
       </c>
       <c r="E15" t="n">
-        <v>265</v>
+        <v>234</v>
       </c>
       <c r="F15" t="n">
-        <v>28</v>
+        <v>94</v>
       </c>
       <c r="G15" t="n">
-        <v>146.5</v>
+        <v>145.78</v>
       </c>
       <c r="H15" t="n">
-        <v>132.5</v>
+        <v>104</v>
       </c>
       <c r="I15" t="n">
-        <v>14</v>
+        <v>41.78</v>
       </c>
     </row>
     <row r="16">
@@ -2064,19 +2064,19 @@
         <v>259</v>
       </c>
       <c r="D16" t="n">
-        <v>375</v>
+        <v>372</v>
       </c>
       <c r="E16" t="n">
-        <v>266</v>
+        <v>263</v>
       </c>
       <c r="F16" t="n">
         <v>109</v>
       </c>
       <c r="G16" t="n">
-        <v>144.79</v>
+        <v>143.63</v>
       </c>
       <c r="H16" t="n">
-        <v>102.7</v>
+        <v>101.54</v>
       </c>
       <c r="I16" t="n">
         <v>42.08</v>
@@ -2157,19 +2157,19 @@
         <v>198</v>
       </c>
       <c r="D19" t="n">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="E19" t="n">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="F19" t="n">
         <v>51</v>
       </c>
       <c r="G19" t="n">
-        <v>142.93</v>
+        <v>142.42</v>
       </c>
       <c r="H19" t="n">
-        <v>117.17</v>
+        <v>116.67</v>
       </c>
       <c r="I19" t="n">
         <v>25.76</v>
@@ -2188,19 +2188,19 @@
         <v>158</v>
       </c>
       <c r="D20" t="n">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="E20" t="n">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="F20" t="n">
         <v>52</v>
       </c>
       <c r="G20" t="n">
-        <v>136.71</v>
+        <v>134.81</v>
       </c>
       <c r="H20" t="n">
-        <v>103.8</v>
+        <v>101.9</v>
       </c>
       <c r="I20" t="n">
         <v>32.91</v>
@@ -2250,19 +2250,19 @@
         <v>266</v>
       </c>
       <c r="D22" t="n">
-        <v>332</v>
+        <v>328</v>
       </c>
       <c r="E22" t="n">
-        <v>250</v>
+        <v>246</v>
       </c>
       <c r="F22" t="n">
         <v>82</v>
       </c>
       <c r="G22" t="n">
-        <v>124.81</v>
+        <v>123.31</v>
       </c>
       <c r="H22" t="n">
-        <v>93.98</v>
+        <v>92.48</v>
       </c>
       <c r="I22" t="n">
         <v>30.83</v>
@@ -2312,19 +2312,19 @@
         <v>155</v>
       </c>
       <c r="D24" t="n">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="E24" t="n">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="F24" t="n">
         <v>42</v>
       </c>
       <c r="G24" t="n">
-        <v>98.70999999999999</v>
+        <v>96.13</v>
       </c>
       <c r="H24" t="n">
-        <v>71.61</v>
+        <v>69.03</v>
       </c>
       <c r="I24" t="n">
         <v>27.1</v>
@@ -2560,19 +2560,19 @@
         <v>124</v>
       </c>
       <c r="D32" t="n">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E32" t="n">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F32" t="n">
         <v>35</v>
       </c>
       <c r="G32" t="n">
-        <v>78.23</v>
+        <v>77.42</v>
       </c>
       <c r="H32" t="n">
-        <v>50</v>
+        <v>49.19</v>
       </c>
       <c r="I32" t="n">
         <v>28.23</v>

</xml_diff>

<commit_message>
feat: update guidance for GPS mismatch to specify Mother's Household GPS
</commit_message>
<xml_diff>
--- a/Error_log/Enumerator_Performance.xlsx
+++ b/Error_log/Enumerator_Performance.xlsx
@@ -483,10 +483,10 @@
         <v>373641</v>
       </c>
       <c r="C3" t="n">
-        <v>461</v>
+        <v>457</v>
       </c>
       <c r="D3" t="n">
-        <v>351</v>
+        <v>347</v>
       </c>
       <c r="E3" t="n">
         <v>110</v>
@@ -521,10 +521,10 @@
         <v>373648</v>
       </c>
       <c r="C5" t="n">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="D5" t="n">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="E5" t="n">
         <v>109</v>
@@ -540,10 +540,10 @@
         <v>373646</v>
       </c>
       <c r="C6" t="n">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="D6" t="n">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="E6" t="n">
         <v>82</v>
@@ -578,10 +578,10 @@
         <v>373642</v>
       </c>
       <c r="C8" t="n">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="D8" t="n">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="E8" t="n">
         <v>51</v>
@@ -635,10 +635,10 @@
         <v>373705</v>
       </c>
       <c r="C11" t="n">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="D11" t="n">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="E11" t="n">
         <v>52</v>
@@ -749,10 +749,10 @@
         <v>373706</v>
       </c>
       <c r="C17" t="n">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D17" t="n">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="E17" t="n">
         <v>42</v>
@@ -989,39 +989,39 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Summiya Hayat</t>
+          <t>Nillum Bibi</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>373710</v>
+        <v>373652</v>
       </c>
       <c r="C30" t="n">
-        <v>96</v>
+        <v>64</v>
       </c>
       <c r="D30" t="n">
         <v>61</v>
       </c>
       <c r="E30" t="n">
-        <v>35</v>
+        <v>3</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Nillum Bibi</t>
+          <t>Summiya Hayat</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>373652</v>
+        <v>373710</v>
       </c>
       <c r="C31" t="n">
-        <v>64</v>
+        <v>95</v>
       </c>
       <c r="D31" t="n">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E31" t="n">
-        <v>3</v>
+        <v>35</v>
       </c>
     </row>
     <row r="32">
@@ -1878,19 +1878,19 @@
         <v>261</v>
       </c>
       <c r="D10" t="n">
-        <v>461</v>
+        <v>457</v>
       </c>
       <c r="E10" t="n">
-        <v>351</v>
+        <v>347</v>
       </c>
       <c r="F10" t="n">
         <v>110</v>
       </c>
       <c r="G10" t="n">
-        <v>176.63</v>
+        <v>175.1</v>
       </c>
       <c r="H10" t="n">
-        <v>134.48</v>
+        <v>132.95</v>
       </c>
       <c r="I10" t="n">
         <v>42.15</v>
@@ -2054,42 +2054,42 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Shazia Bibi</t>
+          <t>Lati Khan</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>373648</v>
+        <v>373665</v>
       </c>
       <c r="C16" t="n">
-        <v>259</v>
+        <v>60</v>
       </c>
       <c r="D16" t="n">
-        <v>372</v>
+        <v>86</v>
       </c>
       <c r="E16" t="n">
-        <v>263</v>
+        <v>83</v>
       </c>
       <c r="F16" t="n">
-        <v>109</v>
+        <v>3</v>
       </c>
       <c r="G16" t="n">
-        <v>143.63</v>
+        <v>143.33</v>
       </c>
       <c r="H16" t="n">
-        <v>101.54</v>
+        <v>138.33</v>
       </c>
       <c r="I16" t="n">
-        <v>42.08</v>
+        <v>5</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Lati Khan</t>
+          <t>Naureen</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>373665</v>
+        <v>884887</v>
       </c>
       <c r="C17" t="n">
         <v>60</v>
@@ -2098,50 +2098,50 @@
         <v>86</v>
       </c>
       <c r="E17" t="n">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="F17" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G17" t="n">
         <v>143.33</v>
       </c>
       <c r="H17" t="n">
-        <v>138.33</v>
+        <v>136.67</v>
       </c>
       <c r="I17" t="n">
-        <v>5</v>
+        <v>6.67</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Naureen</t>
+          <t>Shazia Bibi</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>884887</v>
+        <v>373648</v>
       </c>
       <c r="C18" t="n">
-        <v>60</v>
+        <v>259</v>
       </c>
       <c r="D18" t="n">
-        <v>86</v>
+        <v>371</v>
       </c>
       <c r="E18" t="n">
-        <v>82</v>
+        <v>262</v>
       </c>
       <c r="F18" t="n">
-        <v>4</v>
+        <v>109</v>
       </c>
       <c r="G18" t="n">
-        <v>143.33</v>
+        <v>143.24</v>
       </c>
       <c r="H18" t="n">
-        <v>136.67</v>
+        <v>101.16</v>
       </c>
       <c r="I18" t="n">
-        <v>6.67</v>
+        <v>42.08</v>
       </c>
     </row>
     <row r="19">
@@ -2157,19 +2157,19 @@
         <v>198</v>
       </c>
       <c r="D19" t="n">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="E19" t="n">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="F19" t="n">
         <v>51</v>
       </c>
       <c r="G19" t="n">
-        <v>142.42</v>
+        <v>141.92</v>
       </c>
       <c r="H19" t="n">
-        <v>116.67</v>
+        <v>116.16</v>
       </c>
       <c r="I19" t="n">
         <v>25.76</v>
@@ -2188,19 +2188,19 @@
         <v>158</v>
       </c>
       <c r="D20" t="n">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="E20" t="n">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="F20" t="n">
         <v>52</v>
       </c>
       <c r="G20" t="n">
-        <v>134.81</v>
+        <v>134.18</v>
       </c>
       <c r="H20" t="n">
-        <v>101.9</v>
+        <v>101.27</v>
       </c>
       <c r="I20" t="n">
         <v>32.91</v>
@@ -2250,19 +2250,19 @@
         <v>266</v>
       </c>
       <c r="D22" t="n">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="E22" t="n">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="F22" t="n">
         <v>82</v>
       </c>
       <c r="G22" t="n">
-        <v>123.31</v>
+        <v>122.93</v>
       </c>
       <c r="H22" t="n">
-        <v>92.48</v>
+        <v>92.11</v>
       </c>
       <c r="I22" t="n">
         <v>30.83</v>
@@ -2312,19 +2312,19 @@
         <v>155</v>
       </c>
       <c r="D24" t="n">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="E24" t="n">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F24" t="n">
         <v>42</v>
       </c>
       <c r="G24" t="n">
-        <v>96.13</v>
+        <v>95.48</v>
       </c>
       <c r="H24" t="n">
-        <v>69.03</v>
+        <v>68.39</v>
       </c>
       <c r="I24" t="n">
         <v>27.1</v>
@@ -2560,19 +2560,19 @@
         <v>124</v>
       </c>
       <c r="D32" t="n">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E32" t="n">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F32" t="n">
         <v>35</v>
       </c>
       <c r="G32" t="n">
-        <v>77.42</v>
+        <v>76.61</v>
       </c>
       <c r="H32" t="n">
-        <v>49.19</v>
+        <v>48.39</v>
       </c>
       <c r="I32" t="n">
         <v>28.23</v>

</xml_diff>

<commit_message>
feat: update error log and performance summary files
</commit_message>
<xml_diff>
--- a/Error_log/Enumerator_Performance.xlsx
+++ b/Error_log/Enumerator_Performance.xlsx
@@ -464,13 +464,13 @@
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="n">
-        <v>1863</v>
+        <v>1822</v>
       </c>
       <c r="D2" t="n">
-        <v>1844</v>
+        <v>1800</v>
       </c>
       <c r="E2" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
     </row>
     <row r="3">
@@ -521,10 +521,10 @@
         <v>373648</v>
       </c>
       <c r="C5" t="n">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="D5" t="n">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="E5" t="n">
         <v>109</v>
@@ -540,13 +540,13 @@
         <v>373646</v>
       </c>
       <c r="C6" t="n">
-        <v>327</v>
+        <v>336</v>
       </c>
       <c r="D6" t="n">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="E6" t="n">
-        <v>82</v>
+        <v>88</v>
       </c>
     </row>
     <row r="7">
@@ -559,13 +559,13 @@
         <v>373696</v>
       </c>
       <c r="C7" t="n">
-        <v>328</v>
+        <v>331</v>
       </c>
       <c r="D7" t="n">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="E7" t="n">
-        <v>94</v>
+        <v>96</v>
       </c>
     </row>
     <row r="8">
@@ -578,13 +578,13 @@
         <v>373642</v>
       </c>
       <c r="C8" t="n">
-        <v>281</v>
+        <v>286</v>
       </c>
       <c r="D8" t="n">
         <v>230</v>
       </c>
       <c r="E8" t="n">
-        <v>51</v>
+        <v>56</v>
       </c>
     </row>
     <row r="9">
@@ -616,13 +616,13 @@
         <v>373651</v>
       </c>
       <c r="C10" t="n">
-        <v>286</v>
+        <v>295</v>
       </c>
       <c r="D10" t="n">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="E10" t="n">
-        <v>122</v>
+        <v>128</v>
       </c>
     </row>
     <row r="11">
@@ -635,51 +635,51 @@
         <v>373705</v>
       </c>
       <c r="C11" t="n">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="D11" t="n">
         <v>160</v>
       </c>
       <c r="E11" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Khalida Bibi</t>
+          <t>Naureen Khan</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>373673</v>
+        <v>373716</v>
       </c>
       <c r="C12" t="n">
-        <v>140</v>
+        <v>194</v>
       </c>
       <c r="D12" t="n">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="E12" t="n">
-        <v>0</v>
+        <v>49</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Naureen Khan</t>
+          <t>Khalida Bibi</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>373716</v>
+        <v>373673</v>
       </c>
       <c r="C13" t="n">
-        <v>176</v>
+        <v>140</v>
       </c>
       <c r="D13" t="n">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="E13" t="n">
-        <v>38</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -749,13 +749,13 @@
         <v>373706</v>
       </c>
       <c r="C17" t="n">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="D17" t="n">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="E17" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="18">
@@ -989,39 +989,39 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Nillum Bibi</t>
+          <t>Summiya Hayat</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>373652</v>
+        <v>373710</v>
       </c>
       <c r="C30" t="n">
-        <v>64</v>
+        <v>102</v>
       </c>
       <c r="D30" t="n">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="E30" t="n">
-        <v>3</v>
+        <v>36</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Summiya Hayat</t>
+          <t>Nillum Bibi</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>373710</v>
+        <v>373652</v>
       </c>
       <c r="C31" t="n">
-        <v>95</v>
+        <v>64</v>
       </c>
       <c r="D31" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E31" t="n">
-        <v>35</v>
+        <v>3</v>
       </c>
     </row>
     <row r="32">
@@ -1091,13 +1091,13 @@
         <v>373669</v>
       </c>
       <c r="C35" t="n">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="D35" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="E35" t="n">
-        <v>69</v>
+        <v>73</v>
       </c>
     </row>
     <row r="36">
@@ -1906,87 +1906,87 @@
         <v>373669</v>
       </c>
       <c r="C11" t="n">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="D11" t="n">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="E11" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="F11" t="n">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="G11" t="n">
-        <v>173.85</v>
+        <v>167.61</v>
       </c>
       <c r="H11" t="n">
-        <v>67.69</v>
+        <v>64.79000000000001</v>
       </c>
       <c r="I11" t="n">
-        <v>106.15</v>
+        <v>102.82</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Naureen Khan</t>
+          <t>Javairia</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>373716</v>
+        <v>373651</v>
       </c>
       <c r="C12" t="n">
-        <v>105</v>
+        <v>179</v>
       </c>
       <c r="D12" t="n">
-        <v>176</v>
+        <v>295</v>
       </c>
       <c r="E12" t="n">
-        <v>138</v>
+        <v>167</v>
       </c>
       <c r="F12" t="n">
-        <v>38</v>
+        <v>128</v>
       </c>
       <c r="G12" t="n">
-        <v>167.62</v>
+        <v>164.8</v>
       </c>
       <c r="H12" t="n">
-        <v>131.43</v>
+        <v>93.3</v>
       </c>
       <c r="I12" t="n">
-        <v>36.19</v>
+        <v>71.51000000000001</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Javairia</t>
+          <t>Naureen Khan</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>373651</v>
+        <v>373716</v>
       </c>
       <c r="C13" t="n">
-        <v>174</v>
+        <v>123</v>
       </c>
       <c r="D13" t="n">
-        <v>286</v>
+        <v>194</v>
       </c>
       <c r="E13" t="n">
-        <v>164</v>
+        <v>145</v>
       </c>
       <c r="F13" t="n">
-        <v>122</v>
+        <v>49</v>
       </c>
       <c r="G13" t="n">
-        <v>164.37</v>
+        <v>157.72</v>
       </c>
       <c r="H13" t="n">
-        <v>94.25</v>
+        <v>117.89</v>
       </c>
       <c r="I13" t="n">
-        <v>70.11</v>
+        <v>39.84</v>
       </c>
     </row>
     <row r="14">
@@ -2023,32 +2023,32 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Shazia begum</t>
+          <t>Shazia Bibi</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>373696</v>
+        <v>373648</v>
       </c>
       <c r="C15" t="n">
-        <v>225</v>
+        <v>260</v>
       </c>
       <c r="D15" t="n">
-        <v>328</v>
+        <v>373</v>
       </c>
       <c r="E15" t="n">
-        <v>234</v>
+        <v>264</v>
       </c>
       <c r="F15" t="n">
-        <v>94</v>
+        <v>109</v>
       </c>
       <c r="G15" t="n">
-        <v>145.78</v>
+        <v>143.46</v>
       </c>
       <c r="H15" t="n">
-        <v>104</v>
+        <v>101.54</v>
       </c>
       <c r="I15" t="n">
-        <v>41.78</v>
+        <v>41.92</v>
       </c>
     </row>
     <row r="16">
@@ -2116,32 +2116,32 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Shazia Bibi</t>
+          <t>Shazia begum</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>373648</v>
+        <v>373696</v>
       </c>
       <c r="C18" t="n">
-        <v>259</v>
+        <v>232</v>
       </c>
       <c r="D18" t="n">
-        <v>371</v>
+        <v>331</v>
       </c>
       <c r="E18" t="n">
-        <v>262</v>
+        <v>235</v>
       </c>
       <c r="F18" t="n">
-        <v>109</v>
+        <v>96</v>
       </c>
       <c r="G18" t="n">
-        <v>143.24</v>
+        <v>142.67</v>
       </c>
       <c r="H18" t="n">
-        <v>101.16</v>
+        <v>101.29</v>
       </c>
       <c r="I18" t="n">
-        <v>42.08</v>
+        <v>41.38</v>
       </c>
     </row>
     <row r="19">
@@ -2154,25 +2154,25 @@
         <v>373642</v>
       </c>
       <c r="C19" t="n">
-        <v>198</v>
+        <v>203</v>
       </c>
       <c r="D19" t="n">
-        <v>281</v>
+        <v>286</v>
       </c>
       <c r="E19" t="n">
         <v>230</v>
       </c>
       <c r="F19" t="n">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="G19" t="n">
-        <v>141.92</v>
+        <v>140.89</v>
       </c>
       <c r="H19" t="n">
-        <v>116.16</v>
+        <v>113.3</v>
       </c>
       <c r="I19" t="n">
-        <v>25.76</v>
+        <v>27.59</v>
       </c>
     </row>
     <row r="20">
@@ -2185,25 +2185,25 @@
         <v>373705</v>
       </c>
       <c r="C20" t="n">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="D20" t="n">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="E20" t="n">
         <v>160</v>
       </c>
       <c r="F20" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="G20" t="n">
-        <v>134.18</v>
+        <v>132.1</v>
       </c>
       <c r="H20" t="n">
-        <v>101.27</v>
+        <v>98.77</v>
       </c>
       <c r="I20" t="n">
-        <v>32.91</v>
+        <v>33.33</v>
       </c>
     </row>
     <row r="21">
@@ -2247,25 +2247,25 @@
         <v>373646</v>
       </c>
       <c r="C22" t="n">
-        <v>266</v>
+        <v>273</v>
       </c>
       <c r="D22" t="n">
-        <v>327</v>
+        <v>336</v>
       </c>
       <c r="E22" t="n">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="F22" t="n">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="G22" t="n">
-        <v>122.93</v>
+        <v>123.08</v>
       </c>
       <c r="H22" t="n">
-        <v>92.11</v>
+        <v>90.84</v>
       </c>
       <c r="I22" t="n">
-        <v>30.83</v>
+        <v>32.23</v>
       </c>
     </row>
     <row r="23">
@@ -2309,25 +2309,25 @@
         <v>373706</v>
       </c>
       <c r="C24" t="n">
-        <v>155</v>
+        <v>162</v>
       </c>
       <c r="D24" t="n">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="E24" t="n">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="F24" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G24" t="n">
-        <v>95.48</v>
+        <v>93.83</v>
       </c>
       <c r="H24" t="n">
-        <v>68.39</v>
+        <v>67.28</v>
       </c>
       <c r="I24" t="n">
-        <v>27.1</v>
+        <v>26.54</v>
       </c>
     </row>
     <row r="25">
@@ -2557,25 +2557,25 @@
         <v>373710</v>
       </c>
       <c r="C32" t="n">
-        <v>124</v>
+        <v>131</v>
       </c>
       <c r="D32" t="n">
-        <v>95</v>
+        <v>102</v>
       </c>
       <c r="E32" t="n">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="F32" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="G32" t="n">
-        <v>76.61</v>
+        <v>77.86</v>
       </c>
       <c r="H32" t="n">
-        <v>48.39</v>
+        <v>50.38</v>
       </c>
       <c r="I32" t="n">
-        <v>28.23</v>
+        <v>27.48</v>
       </c>
     </row>
     <row r="33">

</xml_diff>

<commit_message>
feat: refactor household protocol logic and update error log files
</commit_message>
<xml_diff>
--- a/Error_log/Enumerator_Performance.xlsx
+++ b/Error_log/Enumerator_Performance.xlsx
@@ -483,70 +483,70 @@
         <v>373641</v>
       </c>
       <c r="C3" t="n">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="D3" t="n">
-        <v>347</v>
+        <v>368</v>
       </c>
       <c r="E3" t="n">
-        <v>110</v>
+        <v>90</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Mehran Khan</t>
+          <t>Shafaq Zahra</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>373684</v>
+        <v>373646</v>
       </c>
       <c r="C4" t="n">
-        <v>293</v>
+        <v>341</v>
       </c>
       <c r="D4" t="n">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="E4" t="n">
-        <v>28</v>
+        <v>74</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Shazia Bibi</t>
+          <t>Mehran Khan</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>373648</v>
+        <v>373684</v>
       </c>
       <c r="C5" t="n">
-        <v>373</v>
+        <v>293</v>
       </c>
       <c r="D5" t="n">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="E5" t="n">
-        <v>109</v>
+        <v>28</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Shafaq Zahra</t>
+          <t>Shazia Bibi</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>373646</v>
+        <v>373648</v>
       </c>
       <c r="C6" t="n">
-        <v>336</v>
+        <v>355</v>
       </c>
       <c r="D6" t="n">
-        <v>248</v>
+        <v>264</v>
       </c>
       <c r="E6" t="n">
-        <v>88</v>
+        <v>91</v>
       </c>
     </row>
     <row r="7">
@@ -559,13 +559,13 @@
         <v>373696</v>
       </c>
       <c r="C7" t="n">
-        <v>331</v>
+        <v>318</v>
       </c>
       <c r="D7" t="n">
         <v>235</v>
       </c>
       <c r="E7" t="n">
-        <v>96</v>
+        <v>83</v>
       </c>
     </row>
     <row r="8">
@@ -578,13 +578,13 @@
         <v>373642</v>
       </c>
       <c r="C8" t="n">
-        <v>286</v>
+        <v>272</v>
       </c>
       <c r="D8" t="n">
         <v>230</v>
       </c>
       <c r="E8" t="n">
-        <v>56</v>
+        <v>42</v>
       </c>
     </row>
     <row r="9">
@@ -616,13 +616,13 @@
         <v>373651</v>
       </c>
       <c r="C10" t="n">
-        <v>295</v>
+        <v>286</v>
       </c>
       <c r="D10" t="n">
         <v>167</v>
       </c>
       <c r="E10" t="n">
-        <v>128</v>
+        <v>119</v>
       </c>
     </row>
     <row r="11">
@@ -635,13 +635,13 @@
         <v>373705</v>
       </c>
       <c r="C11" t="n">
-        <v>214</v>
+        <v>206</v>
       </c>
       <c r="D11" t="n">
         <v>160</v>
       </c>
       <c r="E11" t="n">
-        <v>54</v>
+        <v>46</v>
       </c>
     </row>
     <row r="12">
@@ -654,13 +654,13 @@
         <v>373716</v>
       </c>
       <c r="C12" t="n">
-        <v>194</v>
+        <v>182</v>
       </c>
       <c r="D12" t="n">
         <v>145</v>
       </c>
       <c r="E12" t="n">
-        <v>49</v>
+        <v>37</v>
       </c>
     </row>
     <row r="13">
@@ -692,13 +692,13 @@
         <v>373712</v>
       </c>
       <c r="C14" t="n">
-        <v>330</v>
+        <v>324</v>
       </c>
       <c r="D14" t="n">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="E14" t="n">
-        <v>201</v>
+        <v>194</v>
       </c>
     </row>
     <row r="15">
@@ -749,13 +749,13 @@
         <v>373706</v>
       </c>
       <c r="C17" t="n">
-        <v>152</v>
+        <v>144</v>
       </c>
       <c r="D17" t="n">
         <v>109</v>
       </c>
       <c r="E17" t="n">
-        <v>43</v>
+        <v>35</v>
       </c>
     </row>
     <row r="18">
@@ -787,51 +787,51 @@
         <v>373692</v>
       </c>
       <c r="C19" t="n">
-        <v>283</v>
+        <v>274</v>
       </c>
       <c r="D19" t="n">
         <v>102</v>
       </c>
       <c r="E19" t="n">
-        <v>181</v>
+        <v>172</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Ishaq Khan</t>
+          <t>Samara</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>373699</v>
+        <v>373658</v>
       </c>
       <c r="C20" t="n">
-        <v>101</v>
+        <v>281</v>
       </c>
       <c r="D20" t="n">
         <v>100</v>
       </c>
       <c r="E20" t="n">
-        <v>1</v>
+        <v>181</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Samara</t>
+          <t>Ishaq Khan</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>373658</v>
+        <v>373699</v>
       </c>
       <c r="C21" t="n">
-        <v>293</v>
+        <v>101</v>
       </c>
       <c r="D21" t="n">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="E21" t="n">
-        <v>194</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22">
@@ -875,39 +875,39 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Naureen khan</t>
+          <t>Rehana Bibi</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>453925</v>
+        <v>373691</v>
       </c>
       <c r="C24" t="n">
-        <v>91</v>
+        <v>278</v>
       </c>
       <c r="D24" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E24" t="n">
-        <v>2</v>
+        <v>188</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Rehana Bibi</t>
+          <t>Naureen khan</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>373691</v>
+        <v>453925</v>
       </c>
       <c r="C25" t="n">
-        <v>288</v>
+        <v>91</v>
       </c>
       <c r="D25" t="n">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="E25" t="n">
-        <v>200</v>
+        <v>2</v>
       </c>
     </row>
     <row r="26">
@@ -996,13 +996,13 @@
         <v>373710</v>
       </c>
       <c r="C30" t="n">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="D30" t="n">
         <v>66</v>
       </c>
       <c r="E30" t="n">
-        <v>36</v>
+        <v>30</v>
       </c>
     </row>
     <row r="31">
@@ -1091,13 +1091,13 @@
         <v>373669</v>
       </c>
       <c r="C35" t="n">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="D35" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E35" t="n">
-        <v>73</v>
+        <v>69</v>
       </c>
     </row>
     <row r="36">
@@ -1754,22 +1754,22 @@
         <v>104</v>
       </c>
       <c r="D6" t="n">
-        <v>330</v>
+        <v>324</v>
       </c>
       <c r="E6" t="n">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="F6" t="n">
-        <v>201</v>
+        <v>194</v>
       </c>
       <c r="G6" t="n">
-        <v>317.31</v>
+        <v>311.54</v>
       </c>
       <c r="H6" t="n">
-        <v>124.04</v>
+        <v>125</v>
       </c>
       <c r="I6" t="n">
-        <v>193.27</v>
+        <v>186.54</v>
       </c>
     </row>
     <row r="7">
@@ -1785,22 +1785,22 @@
         <v>101</v>
       </c>
       <c r="D7" t="n">
-        <v>283</v>
+        <v>274</v>
       </c>
       <c r="E7" t="n">
         <v>102</v>
       </c>
       <c r="F7" t="n">
-        <v>181</v>
+        <v>172</v>
       </c>
       <c r="G7" t="n">
-        <v>280.2</v>
+        <v>271.29</v>
       </c>
       <c r="H7" t="n">
         <v>100.99</v>
       </c>
       <c r="I7" t="n">
-        <v>179.21</v>
+        <v>170.3</v>
       </c>
     </row>
     <row r="8">
@@ -1816,22 +1816,22 @@
         <v>111</v>
       </c>
       <c r="D8" t="n">
-        <v>288</v>
+        <v>278</v>
       </c>
       <c r="E8" t="n">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="F8" t="n">
-        <v>200</v>
+        <v>188</v>
       </c>
       <c r="G8" t="n">
-        <v>259.46</v>
+        <v>250.45</v>
       </c>
       <c r="H8" t="n">
-        <v>79.28</v>
+        <v>81.08</v>
       </c>
       <c r="I8" t="n">
-        <v>180.18</v>
+        <v>169.37</v>
       </c>
     </row>
     <row r="9">
@@ -1847,22 +1847,22 @@
         <v>120</v>
       </c>
       <c r="D9" t="n">
-        <v>293</v>
+        <v>281</v>
       </c>
       <c r="E9" t="n">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="F9" t="n">
-        <v>194</v>
+        <v>181</v>
       </c>
       <c r="G9" t="n">
-        <v>244.17</v>
+        <v>234.17</v>
       </c>
       <c r="H9" t="n">
-        <v>82.5</v>
+        <v>83.33</v>
       </c>
       <c r="I9" t="n">
-        <v>161.67</v>
+        <v>150.83</v>
       </c>
     </row>
     <row r="10">
@@ -1878,22 +1878,22 @@
         <v>261</v>
       </c>
       <c r="D10" t="n">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="E10" t="n">
-        <v>347</v>
+        <v>368</v>
       </c>
       <c r="F10" t="n">
-        <v>110</v>
+        <v>90</v>
       </c>
       <c r="G10" t="n">
-        <v>175.1</v>
+        <v>175.48</v>
       </c>
       <c r="H10" t="n">
-        <v>132.95</v>
+        <v>141</v>
       </c>
       <c r="I10" t="n">
-        <v>42.15</v>
+        <v>34.48</v>
       </c>
     </row>
     <row r="11">
@@ -1909,22 +1909,22 @@
         <v>71</v>
       </c>
       <c r="D11" t="n">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="E11" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="F11" t="n">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="G11" t="n">
-        <v>167.61</v>
+        <v>163.38</v>
       </c>
       <c r="H11" t="n">
-        <v>64.79000000000001</v>
+        <v>66.2</v>
       </c>
       <c r="I11" t="n">
-        <v>102.82</v>
+        <v>97.18000000000001</v>
       </c>
     </row>
     <row r="12">
@@ -1940,22 +1940,22 @@
         <v>179</v>
       </c>
       <c r="D12" t="n">
-        <v>295</v>
+        <v>286</v>
       </c>
       <c r="E12" t="n">
         <v>167</v>
       </c>
       <c r="F12" t="n">
-        <v>128</v>
+        <v>119</v>
       </c>
       <c r="G12" t="n">
-        <v>164.8</v>
+        <v>159.78</v>
       </c>
       <c r="H12" t="n">
         <v>93.3</v>
       </c>
       <c r="I12" t="n">
-        <v>71.51000000000001</v>
+        <v>66.48</v>
       </c>
     </row>
     <row r="13">
@@ -1971,22 +1971,22 @@
         <v>123</v>
       </c>
       <c r="D13" t="n">
-        <v>194</v>
+        <v>182</v>
       </c>
       <c r="E13" t="n">
         <v>145</v>
       </c>
       <c r="F13" t="n">
-        <v>49</v>
+        <v>37</v>
       </c>
       <c r="G13" t="n">
-        <v>157.72</v>
+        <v>147.97</v>
       </c>
       <c r="H13" t="n">
         <v>117.89</v>
       </c>
       <c r="I13" t="n">
-        <v>39.84</v>
+        <v>30.08</v>
       </c>
     </row>
     <row r="14">
@@ -2023,42 +2023,42 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Shazia Bibi</t>
+          <t>Lati Khan</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>373648</v>
+        <v>373665</v>
       </c>
       <c r="C15" t="n">
-        <v>260</v>
+        <v>60</v>
       </c>
       <c r="D15" t="n">
-        <v>373</v>
+        <v>86</v>
       </c>
       <c r="E15" t="n">
-        <v>264</v>
+        <v>83</v>
       </c>
       <c r="F15" t="n">
-        <v>109</v>
+        <v>3</v>
       </c>
       <c r="G15" t="n">
-        <v>143.46</v>
+        <v>143.33</v>
       </c>
       <c r="H15" t="n">
-        <v>101.54</v>
+        <v>138.33</v>
       </c>
       <c r="I15" t="n">
-        <v>41.92</v>
+        <v>5</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Lati Khan</t>
+          <t>Naureen</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>373665</v>
+        <v>884887</v>
       </c>
       <c r="C16" t="n">
         <v>60</v>
@@ -2067,81 +2067,81 @@
         <v>86</v>
       </c>
       <c r="E16" t="n">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="F16" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G16" t="n">
         <v>143.33</v>
       </c>
       <c r="H16" t="n">
-        <v>138.33</v>
+        <v>136.67</v>
       </c>
       <c r="I16" t="n">
-        <v>5</v>
+        <v>6.67</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Naureen</t>
+          <t>Shazia begum</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>884887</v>
+        <v>373696</v>
       </c>
       <c r="C17" t="n">
-        <v>60</v>
+        <v>232</v>
       </c>
       <c r="D17" t="n">
-        <v>86</v>
+        <v>318</v>
       </c>
       <c r="E17" t="n">
-        <v>82</v>
+        <v>235</v>
       </c>
       <c r="F17" t="n">
-        <v>4</v>
+        <v>83</v>
       </c>
       <c r="G17" t="n">
-        <v>143.33</v>
+        <v>137.07</v>
       </c>
       <c r="H17" t="n">
-        <v>136.67</v>
+        <v>101.29</v>
       </c>
       <c r="I17" t="n">
-        <v>6.67</v>
+        <v>35.78</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Shazia begum</t>
+          <t>Shazia Bibi</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>373696</v>
+        <v>373648</v>
       </c>
       <c r="C18" t="n">
-        <v>232</v>
+        <v>260</v>
       </c>
       <c r="D18" t="n">
-        <v>331</v>
+        <v>355</v>
       </c>
       <c r="E18" t="n">
-        <v>235</v>
+        <v>264</v>
       </c>
       <c r="F18" t="n">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="G18" t="n">
-        <v>142.67</v>
+        <v>136.54</v>
       </c>
       <c r="H18" t="n">
-        <v>101.29</v>
+        <v>101.54</v>
       </c>
       <c r="I18" t="n">
-        <v>41.38</v>
+        <v>35</v>
       </c>
     </row>
     <row r="19">
@@ -2157,22 +2157,22 @@
         <v>203</v>
       </c>
       <c r="D19" t="n">
-        <v>286</v>
+        <v>272</v>
       </c>
       <c r="E19" t="n">
         <v>230</v>
       </c>
       <c r="F19" t="n">
-        <v>56</v>
+        <v>42</v>
       </c>
       <c r="G19" t="n">
-        <v>140.89</v>
+        <v>133.99</v>
       </c>
       <c r="H19" t="n">
         <v>113.3</v>
       </c>
       <c r="I19" t="n">
-        <v>27.59</v>
+        <v>20.69</v>
       </c>
     </row>
     <row r="20">
@@ -2188,22 +2188,22 @@
         <v>162</v>
       </c>
       <c r="D20" t="n">
-        <v>214</v>
+        <v>206</v>
       </c>
       <c r="E20" t="n">
         <v>160</v>
       </c>
       <c r="F20" t="n">
-        <v>54</v>
+        <v>46</v>
       </c>
       <c r="G20" t="n">
-        <v>132.1</v>
+        <v>127.16</v>
       </c>
       <c r="H20" t="n">
         <v>98.77</v>
       </c>
       <c r="I20" t="n">
-        <v>33.33</v>
+        <v>28.4</v>
       </c>
     </row>
     <row r="21">
@@ -2250,22 +2250,22 @@
         <v>273</v>
       </c>
       <c r="D22" t="n">
-        <v>336</v>
+        <v>341</v>
       </c>
       <c r="E22" t="n">
-        <v>248</v>
+        <v>267</v>
       </c>
       <c r="F22" t="n">
-        <v>88</v>
+        <v>74</v>
       </c>
       <c r="G22" t="n">
-        <v>123.08</v>
+        <v>124.91</v>
       </c>
       <c r="H22" t="n">
-        <v>90.84</v>
+        <v>97.8</v>
       </c>
       <c r="I22" t="n">
-        <v>32.23</v>
+        <v>27.11</v>
       </c>
     </row>
     <row r="23">
@@ -2302,125 +2302,125 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Laiba Shams</t>
+          <t>Zain Ul Abideen</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>373706</v>
+        <v>373667</v>
       </c>
       <c r="C24" t="n">
-        <v>162</v>
+        <v>13</v>
       </c>
       <c r="D24" t="n">
-        <v>152</v>
+        <v>12</v>
       </c>
       <c r="E24" t="n">
-        <v>109</v>
+        <v>12</v>
       </c>
       <c r="F24" t="n">
-        <v>43</v>
+        <v>0</v>
       </c>
       <c r="G24" t="n">
-        <v>93.83</v>
+        <v>92.31</v>
       </c>
       <c r="H24" t="n">
-        <v>67.28</v>
+        <v>92.31</v>
       </c>
       <c r="I24" t="n">
-        <v>26.54</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Zain Ul Abideen</t>
+          <t>Bushra Ayub</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>373667</v>
+        <v>373671</v>
       </c>
       <c r="C25" t="n">
-        <v>13</v>
+        <v>138</v>
       </c>
       <c r="D25" t="n">
-        <v>12</v>
+        <v>126</v>
       </c>
       <c r="E25" t="n">
-        <v>12</v>
+        <v>122</v>
       </c>
       <c r="F25" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G25" t="n">
-        <v>92.31</v>
+        <v>91.3</v>
       </c>
       <c r="H25" t="n">
-        <v>92.31</v>
+        <v>88.41</v>
       </c>
       <c r="I25" t="n">
-        <v>0</v>
+        <v>2.9</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Bushra Ayub</t>
+          <t>Lati khan</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>373671</v>
+        <v>652938</v>
       </c>
       <c r="C26" t="n">
-        <v>138</v>
+        <v>11</v>
       </c>
       <c r="D26" t="n">
-        <v>126</v>
+        <v>10</v>
       </c>
       <c r="E26" t="n">
-        <v>122</v>
+        <v>10</v>
       </c>
       <c r="F26" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G26" t="n">
-        <v>91.3</v>
+        <v>90.91</v>
       </c>
       <c r="H26" t="n">
-        <v>88.41</v>
+        <v>90.91</v>
       </c>
       <c r="I26" t="n">
-        <v>2.9</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Lati khan</t>
+          <t>Laiba Shams</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>652938</v>
+        <v>373706</v>
       </c>
       <c r="C27" t="n">
-        <v>11</v>
+        <v>162</v>
       </c>
       <c r="D27" t="n">
-        <v>10</v>
+        <v>144</v>
       </c>
       <c r="E27" t="n">
-        <v>10</v>
+        <v>109</v>
       </c>
       <c r="F27" t="n">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="G27" t="n">
-        <v>90.91</v>
+        <v>88.89</v>
       </c>
       <c r="H27" t="n">
-        <v>90.91</v>
+        <v>67.28</v>
       </c>
       <c r="I27" t="n">
-        <v>0</v>
+        <v>21.6</v>
       </c>
     </row>
     <row r="28">
@@ -2550,94 +2550,94 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Summiya Hayat</t>
+          <t>Asma Gull</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>373710</v>
+        <v>373672</v>
       </c>
       <c r="C32" t="n">
-        <v>131</v>
+        <v>144</v>
       </c>
       <c r="D32" t="n">
-        <v>102</v>
+        <v>109</v>
       </c>
       <c r="E32" t="n">
-        <v>66</v>
+        <v>105</v>
       </c>
       <c r="F32" t="n">
-        <v>36</v>
+        <v>4</v>
       </c>
       <c r="G32" t="n">
-        <v>77.86</v>
+        <v>75.69</v>
       </c>
       <c r="H32" t="n">
-        <v>50.38</v>
+        <v>72.92</v>
       </c>
       <c r="I32" t="n">
-        <v>27.48</v>
+        <v>2.78</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Asma Gull</t>
+          <t>Rahila Naaz</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>373672</v>
+        <v>373715</v>
       </c>
       <c r="C33" t="n">
-        <v>144</v>
+        <v>4</v>
       </c>
       <c r="D33" t="n">
-        <v>109</v>
+        <v>3</v>
       </c>
       <c r="E33" t="n">
-        <v>105</v>
+        <v>2</v>
       </c>
       <c r="F33" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G33" t="n">
-        <v>75.69</v>
+        <v>75</v>
       </c>
       <c r="H33" t="n">
-        <v>72.92</v>
+        <v>50</v>
       </c>
       <c r="I33" t="n">
-        <v>2.78</v>
+        <v>25</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Rahila Naaz</t>
+          <t>Summiya Hayat</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>373715</v>
+        <v>373710</v>
       </c>
       <c r="C34" t="n">
-        <v>4</v>
+        <v>131</v>
       </c>
       <c r="D34" t="n">
-        <v>3</v>
+        <v>96</v>
       </c>
       <c r="E34" t="n">
-        <v>2</v>
+        <v>66</v>
       </c>
       <c r="F34" t="n">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="G34" t="n">
-        <v>75</v>
+        <v>73.28</v>
       </c>
       <c r="H34" t="n">
-        <v>50</v>
+        <v>50.38</v>
       </c>
       <c r="I34" t="n">
-        <v>25</v>
+        <v>22.9</v>
       </c>
     </row>
     <row r="35">

</xml_diff>

<commit_message>
feat: enhance duration validation logic and update error log files
</commit_message>
<xml_diff>
--- a/Error_log/Enumerator_Performance.xlsx
+++ b/Error_log/Enumerator_Performance.xlsx
@@ -483,10 +483,10 @@
         <v>373641</v>
       </c>
       <c r="C3" t="n">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="D3" t="n">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="E3" t="n">
         <v>90</v>
@@ -502,10 +502,10 @@
         <v>373646</v>
       </c>
       <c r="C4" t="n">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="D4" t="n">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="E4" t="n">
         <v>74</v>
@@ -540,10 +540,10 @@
         <v>373648</v>
       </c>
       <c r="C6" t="n">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="D6" t="n">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="E6" t="n">
         <v>91</v>
@@ -647,39 +647,39 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Naureen Khan</t>
+          <t>Khalida Bibi</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>373716</v>
+        <v>373673</v>
       </c>
       <c r="C12" t="n">
-        <v>182</v>
+        <v>140</v>
       </c>
       <c r="D12" t="n">
-        <v>145</v>
+        <v>140</v>
       </c>
       <c r="E12" t="n">
-        <v>37</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Khalida Bibi</t>
+          <t>Naureen Khan</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>373673</v>
+        <v>373716</v>
       </c>
       <c r="C13" t="n">
-        <v>140</v>
+        <v>174</v>
       </c>
       <c r="D13" t="n">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="E13" t="n">
-        <v>0</v>
+        <v>37</v>
       </c>
     </row>
     <row r="14">
@@ -749,10 +749,10 @@
         <v>373706</v>
       </c>
       <c r="C17" t="n">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="D17" t="n">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="E17" t="n">
         <v>35</v>
@@ -1878,19 +1878,19 @@
         <v>261</v>
       </c>
       <c r="D10" t="n">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="E10" t="n">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="F10" t="n">
         <v>90</v>
       </c>
       <c r="G10" t="n">
-        <v>175.48</v>
+        <v>175.1</v>
       </c>
       <c r="H10" t="n">
-        <v>141</v>
+        <v>140.61</v>
       </c>
       <c r="I10" t="n">
         <v>34.48</v>
@@ -1961,73 +1961,73 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Naureen Khan</t>
+          <t>Mehran Khan</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>373716</v>
+        <v>373684</v>
       </c>
       <c r="C13" t="n">
-        <v>123</v>
+        <v>200</v>
       </c>
       <c r="D13" t="n">
-        <v>182</v>
+        <v>293</v>
       </c>
       <c r="E13" t="n">
-        <v>145</v>
+        <v>265</v>
       </c>
       <c r="F13" t="n">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="G13" t="n">
-        <v>147.97</v>
+        <v>146.5</v>
       </c>
       <c r="H13" t="n">
-        <v>117.89</v>
+        <v>132.5</v>
       </c>
       <c r="I13" t="n">
-        <v>30.08</v>
+        <v>14</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Mehran Khan</t>
+          <t>Lati Khan</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>373684</v>
+        <v>373665</v>
       </c>
       <c r="C14" t="n">
-        <v>200</v>
+        <v>60</v>
       </c>
       <c r="D14" t="n">
-        <v>293</v>
+        <v>86</v>
       </c>
       <c r="E14" t="n">
-        <v>265</v>
+        <v>83</v>
       </c>
       <c r="F14" t="n">
-        <v>28</v>
+        <v>3</v>
       </c>
       <c r="G14" t="n">
-        <v>146.5</v>
+        <v>143.33</v>
       </c>
       <c r="H14" t="n">
-        <v>132.5</v>
+        <v>138.33</v>
       </c>
       <c r="I14" t="n">
-        <v>14</v>
+        <v>5</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Lati Khan</t>
+          <t>Naureen</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>373665</v>
+        <v>884887</v>
       </c>
       <c r="C15" t="n">
         <v>60</v>
@@ -2036,50 +2036,50 @@
         <v>86</v>
       </c>
       <c r="E15" t="n">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="F15" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G15" t="n">
         <v>143.33</v>
       </c>
       <c r="H15" t="n">
-        <v>138.33</v>
+        <v>136.67</v>
       </c>
       <c r="I15" t="n">
-        <v>5</v>
+        <v>6.67</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Naureen</t>
+          <t>Naureen Khan</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>884887</v>
+        <v>373716</v>
       </c>
       <c r="C16" t="n">
-        <v>60</v>
+        <v>123</v>
       </c>
       <c r="D16" t="n">
-        <v>86</v>
+        <v>174</v>
       </c>
       <c r="E16" t="n">
-        <v>82</v>
+        <v>137</v>
       </c>
       <c r="F16" t="n">
-        <v>4</v>
+        <v>37</v>
       </c>
       <c r="G16" t="n">
-        <v>143.33</v>
+        <v>141.46</v>
       </c>
       <c r="H16" t="n">
-        <v>136.67</v>
+        <v>111.38</v>
       </c>
       <c r="I16" t="n">
-        <v>6.67</v>
+        <v>30.08</v>
       </c>
     </row>
     <row r="17">
@@ -2126,19 +2126,19 @@
         <v>260</v>
       </c>
       <c r="D18" t="n">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="E18" t="n">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="F18" t="n">
         <v>91</v>
       </c>
       <c r="G18" t="n">
-        <v>136.54</v>
+        <v>136.15</v>
       </c>
       <c r="H18" t="n">
-        <v>101.54</v>
+        <v>101.15</v>
       </c>
       <c r="I18" t="n">
         <v>35</v>
@@ -2250,19 +2250,19 @@
         <v>273</v>
       </c>
       <c r="D22" t="n">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="E22" t="n">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="F22" t="n">
         <v>74</v>
       </c>
       <c r="G22" t="n">
-        <v>124.91</v>
+        <v>124.54</v>
       </c>
       <c r="H22" t="n">
-        <v>97.8</v>
+        <v>97.44</v>
       </c>
       <c r="I22" t="n">
         <v>27.11</v>
@@ -2405,19 +2405,19 @@
         <v>162</v>
       </c>
       <c r="D27" t="n">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E27" t="n">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="F27" t="n">
         <v>35</v>
       </c>
       <c r="G27" t="n">
-        <v>88.89</v>
+        <v>88.27</v>
       </c>
       <c r="H27" t="n">
-        <v>67.28</v>
+        <v>66.67</v>
       </c>
       <c r="I27" t="n">
         <v>21.6</v>

</xml_diff>

<commit_message>
feat: add alternative start and end time columns for improved duration validation
</commit_message>
<xml_diff>
--- a/Error_log/Enumerator_Performance.xlsx
+++ b/Error_log/Enumerator_Performance.xlsx
@@ -483,10 +483,10 @@
         <v>373641</v>
       </c>
       <c r="C3" t="n">
-        <v>457</v>
+        <v>455</v>
       </c>
       <c r="D3" t="n">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="E3" t="n">
         <v>90</v>
@@ -578,10 +578,10 @@
         <v>373642</v>
       </c>
       <c r="C8" t="n">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="D8" t="n">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="E8" t="n">
         <v>42</v>
@@ -673,10 +673,10 @@
         <v>373716</v>
       </c>
       <c r="C13" t="n">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="D13" t="n">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="E13" t="n">
         <v>37</v>
@@ -1878,19 +1878,19 @@
         <v>261</v>
       </c>
       <c r="D10" t="n">
-        <v>457</v>
+        <v>455</v>
       </c>
       <c r="E10" t="n">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="F10" t="n">
         <v>90</v>
       </c>
       <c r="G10" t="n">
-        <v>175.1</v>
+        <v>174.33</v>
       </c>
       <c r="H10" t="n">
-        <v>140.61</v>
+        <v>139.85</v>
       </c>
       <c r="I10" t="n">
         <v>34.48</v>
@@ -2064,19 +2064,19 @@
         <v>123</v>
       </c>
       <c r="D16" t="n">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="E16" t="n">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="F16" t="n">
         <v>37</v>
       </c>
       <c r="G16" t="n">
-        <v>141.46</v>
+        <v>140.65</v>
       </c>
       <c r="H16" t="n">
-        <v>111.38</v>
+        <v>110.57</v>
       </c>
       <c r="I16" t="n">
         <v>30.08</v>
@@ -2157,19 +2157,19 @@
         <v>203</v>
       </c>
       <c r="D19" t="n">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="E19" t="n">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="F19" t="n">
         <v>42</v>
       </c>
       <c r="G19" t="n">
-        <v>133.99</v>
+        <v>133.5</v>
       </c>
       <c r="H19" t="n">
-        <v>113.3</v>
+        <v>112.81</v>
       </c>
       <c r="I19" t="n">
         <v>20.69</v>

</xml_diff>

<commit_message>
feat: add 26-Sep DI Khan/Hangu data quality session and update checks
</commit_message>
<xml_diff>
--- a/Error_log/Enumerator_Performance.xlsx
+++ b/Error_log/Enumerator_Performance.xlsx
@@ -464,13 +464,13 @@
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="n">
-        <v>1822</v>
+        <v>1744</v>
       </c>
       <c r="D2" t="n">
-        <v>1800</v>
+        <v>1721</v>
       </c>
       <c r="E2" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="3">
@@ -483,32 +483,32 @@
         <v>373641</v>
       </c>
       <c r="C3" t="n">
-        <v>455</v>
+        <v>469</v>
       </c>
       <c r="D3" t="n">
-        <v>365</v>
+        <v>342</v>
       </c>
       <c r="E3" t="n">
-        <v>90</v>
+        <v>127</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Shafaq Zahra</t>
+          <t>Shazia Bibi</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>373646</v>
+        <v>373648</v>
       </c>
       <c r="C4" t="n">
-        <v>340</v>
+        <v>362</v>
       </c>
       <c r="D4" t="n">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="E4" t="n">
-        <v>74</v>
+        <v>97</v>
       </c>
     </row>
     <row r="5">
@@ -533,20 +533,20 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Shazia Bibi</t>
+          <t>Shafaq Zahra</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>373648</v>
+        <v>373646</v>
       </c>
       <c r="C6" t="n">
-        <v>354</v>
+        <v>357</v>
       </c>
       <c r="D6" t="n">
-        <v>263</v>
+        <v>244</v>
       </c>
       <c r="E6" t="n">
-        <v>91</v>
+        <v>113</v>
       </c>
     </row>
     <row r="7">
@@ -559,13 +559,13 @@
         <v>373696</v>
       </c>
       <c r="C7" t="n">
-        <v>318</v>
+        <v>322</v>
       </c>
       <c r="D7" t="n">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="E7" t="n">
-        <v>83</v>
+        <v>86</v>
       </c>
     </row>
     <row r="8">
@@ -578,13 +578,13 @@
         <v>373642</v>
       </c>
       <c r="C8" t="n">
-        <v>271</v>
+        <v>278</v>
       </c>
       <c r="D8" t="n">
         <v>229</v>
       </c>
       <c r="E8" t="n">
-        <v>42</v>
+        <v>49</v>
       </c>
     </row>
     <row r="9">
@@ -616,13 +616,13 @@
         <v>373651</v>
       </c>
       <c r="C10" t="n">
-        <v>286</v>
+        <v>302</v>
       </c>
       <c r="D10" t="n">
-        <v>167</v>
+        <v>174</v>
       </c>
       <c r="E10" t="n">
-        <v>119</v>
+        <v>128</v>
       </c>
     </row>
     <row r="11">
@@ -635,13 +635,13 @@
         <v>373705</v>
       </c>
       <c r="C11" t="n">
-        <v>206</v>
+        <v>214</v>
       </c>
       <c r="D11" t="n">
         <v>160</v>
       </c>
       <c r="E11" t="n">
-        <v>46</v>
+        <v>54</v>
       </c>
     </row>
     <row r="12">
@@ -673,13 +673,13 @@
         <v>373716</v>
       </c>
       <c r="C13" t="n">
-        <v>173</v>
+        <v>182</v>
       </c>
       <c r="D13" t="n">
         <v>136</v>
       </c>
       <c r="E13" t="n">
-        <v>37</v>
+        <v>46</v>
       </c>
     </row>
     <row r="14">
@@ -695,10 +695,10 @@
         <v>324</v>
       </c>
       <c r="D14" t="n">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="E14" t="n">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="15">
@@ -749,13 +749,13 @@
         <v>373706</v>
       </c>
       <c r="C17" t="n">
-        <v>143</v>
+        <v>157</v>
       </c>
       <c r="D17" t="n">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="E17" t="n">
-        <v>35</v>
+        <v>45</v>
       </c>
     </row>
     <row r="18">
@@ -780,20 +780,20 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Zohra</t>
+          <t>Ishaq Khan</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>373692</v>
+        <v>373699</v>
       </c>
       <c r="C19" t="n">
-        <v>274</v>
+        <v>101</v>
       </c>
       <c r="D19" t="n">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="E19" t="n">
-        <v>172</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20">
@@ -806,32 +806,32 @@
         <v>373658</v>
       </c>
       <c r="C20" t="n">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="D20" t="n">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="E20" t="n">
-        <v>181</v>
+        <v>183</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Ishaq Khan</t>
+          <t>Zohra</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>373699</v>
+        <v>373692</v>
       </c>
       <c r="C21" t="n">
-        <v>101</v>
+        <v>273</v>
       </c>
       <c r="D21" t="n">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="E21" t="n">
-        <v>1</v>
+        <v>177</v>
       </c>
     </row>
     <row r="22">
@@ -875,39 +875,39 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Rehana Bibi</t>
+          <t>Naureen khan</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>373691</v>
+        <v>453925</v>
       </c>
       <c r="C24" t="n">
-        <v>278</v>
+        <v>92</v>
       </c>
       <c r="D24" t="n">
         <v>90</v>
       </c>
       <c r="E24" t="n">
-        <v>188</v>
+        <v>2</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Naureen khan</t>
+          <t>Rehana Bibi</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>453925</v>
+        <v>373691</v>
       </c>
       <c r="C25" t="n">
-        <v>91</v>
+        <v>278</v>
       </c>
       <c r="D25" t="n">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="E25" t="n">
-        <v>2</v>
+        <v>190</v>
       </c>
     </row>
     <row r="26">
@@ -996,13 +996,13 @@
         <v>373710</v>
       </c>
       <c r="C30" t="n">
-        <v>96</v>
+        <v>106</v>
       </c>
       <c r="D30" t="n">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="E30" t="n">
-        <v>30</v>
+        <v>33</v>
       </c>
     </row>
     <row r="31">
@@ -1091,13 +1091,13 @@
         <v>373669</v>
       </c>
       <c r="C35" t="n">
-        <v>116</v>
+        <v>125</v>
       </c>
       <c r="D35" t="n">
         <v>47</v>
       </c>
       <c r="E35" t="n">
-        <v>69</v>
+        <v>78</v>
       </c>
     </row>
     <row r="36">
@@ -1630,19 +1630,19 @@
         <v>2</v>
       </c>
       <c r="D2" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="E2" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="F2" t="n">
         <v>2</v>
       </c>
       <c r="G2" t="n">
-        <v>4550</v>
+        <v>4600</v>
       </c>
       <c r="H2" t="n">
-        <v>4450</v>
+        <v>4500</v>
       </c>
       <c r="I2" t="n">
         <v>100</v>
@@ -1757,19 +1757,19 @@
         <v>324</v>
       </c>
       <c r="E6" t="n">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F6" t="n">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="G6" t="n">
         <v>311.54</v>
       </c>
       <c r="H6" t="n">
-        <v>125</v>
+        <v>124.04</v>
       </c>
       <c r="I6" t="n">
-        <v>186.54</v>
+        <v>187.5</v>
       </c>
     </row>
     <row r="7">
@@ -1785,22 +1785,22 @@
         <v>101</v>
       </c>
       <c r="D7" t="n">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="E7" t="n">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="F7" t="n">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="G7" t="n">
-        <v>271.29</v>
+        <v>270.3</v>
       </c>
       <c r="H7" t="n">
-        <v>100.99</v>
+        <v>95.05</v>
       </c>
       <c r="I7" t="n">
-        <v>170.3</v>
+        <v>175.25</v>
       </c>
     </row>
     <row r="8">
@@ -1819,19 +1819,19 @@
         <v>278</v>
       </c>
       <c r="E8" t="n">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="F8" t="n">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="G8" t="n">
         <v>250.45</v>
       </c>
       <c r="H8" t="n">
-        <v>81.08</v>
+        <v>79.28</v>
       </c>
       <c r="I8" t="n">
-        <v>169.37</v>
+        <v>171.17</v>
       </c>
     </row>
     <row r="9">
@@ -1847,22 +1847,22 @@
         <v>120</v>
       </c>
       <c r="D9" t="n">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="E9" t="n">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="F9" t="n">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="G9" t="n">
-        <v>234.17</v>
+        <v>233.33</v>
       </c>
       <c r="H9" t="n">
-        <v>83.33</v>
+        <v>80.83</v>
       </c>
       <c r="I9" t="n">
-        <v>150.83</v>
+        <v>152.5</v>
       </c>
     </row>
     <row r="10">
@@ -1878,84 +1878,84 @@
         <v>261</v>
       </c>
       <c r="D10" t="n">
-        <v>455</v>
+        <v>469</v>
       </c>
       <c r="E10" t="n">
-        <v>365</v>
+        <v>342</v>
       </c>
       <c r="F10" t="n">
-        <v>90</v>
+        <v>127</v>
       </c>
       <c r="G10" t="n">
-        <v>174.33</v>
+        <v>179.69</v>
       </c>
       <c r="H10" t="n">
-        <v>139.85</v>
+        <v>131.03</v>
       </c>
       <c r="I10" t="n">
-        <v>34.48</v>
+        <v>48.66</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Nadia bibi</t>
+          <t>Javairia</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>373669</v>
+        <v>373651</v>
       </c>
       <c r="C11" t="n">
-        <v>71</v>
+        <v>187</v>
       </c>
       <c r="D11" t="n">
-        <v>116</v>
+        <v>302</v>
       </c>
       <c r="E11" t="n">
-        <v>47</v>
+        <v>174</v>
       </c>
       <c r="F11" t="n">
-        <v>69</v>
+        <v>128</v>
       </c>
       <c r="G11" t="n">
-        <v>163.38</v>
+        <v>161.5</v>
       </c>
       <c r="H11" t="n">
-        <v>66.2</v>
+        <v>93.05</v>
       </c>
       <c r="I11" t="n">
-        <v>97.18000000000001</v>
+        <v>68.45</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Javairia</t>
+          <t>Nadia bibi</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>373651</v>
+        <v>373669</v>
       </c>
       <c r="C12" t="n">
-        <v>179</v>
+        <v>81</v>
       </c>
       <c r="D12" t="n">
-        <v>286</v>
+        <v>125</v>
       </c>
       <c r="E12" t="n">
-        <v>167</v>
+        <v>47</v>
       </c>
       <c r="F12" t="n">
-        <v>119</v>
+        <v>78</v>
       </c>
       <c r="G12" t="n">
-        <v>159.78</v>
+        <v>154.32</v>
       </c>
       <c r="H12" t="n">
-        <v>93.3</v>
+        <v>58.02</v>
       </c>
       <c r="I12" t="n">
-        <v>66.48</v>
+        <v>96.3</v>
       </c>
     </row>
     <row r="13">
@@ -2061,149 +2061,149 @@
         <v>373716</v>
       </c>
       <c r="C16" t="n">
-        <v>123</v>
+        <v>130</v>
       </c>
       <c r="D16" t="n">
-        <v>173</v>
+        <v>182</v>
       </c>
       <c r="E16" t="n">
         <v>136</v>
       </c>
       <c r="F16" t="n">
-        <v>37</v>
+        <v>46</v>
       </c>
       <c r="G16" t="n">
-        <v>140.65</v>
+        <v>140</v>
       </c>
       <c r="H16" t="n">
-        <v>110.57</v>
+        <v>104.62</v>
       </c>
       <c r="I16" t="n">
-        <v>30.08</v>
+        <v>35.38</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Shazia begum</t>
+          <t>Irum Ikram</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>373696</v>
+        <v>373642</v>
       </c>
       <c r="C17" t="n">
-        <v>232</v>
+        <v>206</v>
       </c>
       <c r="D17" t="n">
-        <v>318</v>
+        <v>278</v>
       </c>
       <c r="E17" t="n">
-        <v>235</v>
+        <v>229</v>
       </c>
       <c r="F17" t="n">
-        <v>83</v>
+        <v>49</v>
       </c>
       <c r="G17" t="n">
-        <v>137.07</v>
+        <v>134.95</v>
       </c>
       <c r="H17" t="n">
-        <v>101.29</v>
+        <v>111.17</v>
       </c>
       <c r="I17" t="n">
-        <v>35.78</v>
+        <v>23.79</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Shazia Bibi</t>
+          <t>Shazia begum</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>373648</v>
+        <v>373696</v>
       </c>
       <c r="C18" t="n">
-        <v>260</v>
+        <v>239</v>
       </c>
       <c r="D18" t="n">
-        <v>354</v>
+        <v>322</v>
       </c>
       <c r="E18" t="n">
-        <v>263</v>
+        <v>236</v>
       </c>
       <c r="F18" t="n">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="G18" t="n">
-        <v>136.15</v>
+        <v>134.73</v>
       </c>
       <c r="H18" t="n">
-        <v>101.15</v>
+        <v>98.73999999999999</v>
       </c>
       <c r="I18" t="n">
-        <v>35</v>
+        <v>35.98</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Irum Ikram</t>
+          <t>Shazia Bibi</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>373642</v>
+        <v>373648</v>
       </c>
       <c r="C19" t="n">
-        <v>203</v>
+        <v>273</v>
       </c>
       <c r="D19" t="n">
-        <v>271</v>
+        <v>362</v>
       </c>
       <c r="E19" t="n">
-        <v>229</v>
+        <v>265</v>
       </c>
       <c r="F19" t="n">
-        <v>42</v>
+        <v>97</v>
       </c>
       <c r="G19" t="n">
-        <v>133.5</v>
+        <v>132.6</v>
       </c>
       <c r="H19" t="n">
-        <v>112.81</v>
+        <v>97.06999999999999</v>
       </c>
       <c r="I19" t="n">
-        <v>20.69</v>
+        <v>35.53</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Mahnoor</t>
+          <t>Shafaq Zahra</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>373705</v>
+        <v>373646</v>
       </c>
       <c r="C20" t="n">
-        <v>162</v>
+        <v>280</v>
       </c>
       <c r="D20" t="n">
-        <v>206</v>
+        <v>357</v>
       </c>
       <c r="E20" t="n">
-        <v>160</v>
+        <v>244</v>
       </c>
       <c r="F20" t="n">
-        <v>46</v>
+        <v>113</v>
       </c>
       <c r="G20" t="n">
-        <v>127.16</v>
+        <v>127.5</v>
       </c>
       <c r="H20" t="n">
-        <v>98.77</v>
+        <v>87.14</v>
       </c>
       <c r="I20" t="n">
-        <v>28.4</v>
+        <v>40.36</v>
       </c>
     </row>
     <row r="21">
@@ -2240,63 +2240,63 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Shafaq Zahra</t>
+          <t>Jaweria</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>373646</v>
+        <v>163495</v>
       </c>
       <c r="C22" t="n">
-        <v>273</v>
+        <v>68</v>
       </c>
       <c r="D22" t="n">
-        <v>340</v>
+        <v>83</v>
       </c>
       <c r="E22" t="n">
-        <v>266</v>
+        <v>82</v>
       </c>
       <c r="F22" t="n">
-        <v>74</v>
+        <v>1</v>
       </c>
       <c r="G22" t="n">
-        <v>124.54</v>
+        <v>122.06</v>
       </c>
       <c r="H22" t="n">
-        <v>97.44</v>
+        <v>120.59</v>
       </c>
       <c r="I22" t="n">
-        <v>27.11</v>
+        <v>1.47</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Jaweria</t>
+          <t>Mahnoor</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>163495</v>
+        <v>373705</v>
       </c>
       <c r="C23" t="n">
-        <v>68</v>
+        <v>176</v>
       </c>
       <c r="D23" t="n">
-        <v>83</v>
+        <v>214</v>
       </c>
       <c r="E23" t="n">
-        <v>82</v>
+        <v>160</v>
       </c>
       <c r="F23" t="n">
-        <v>1</v>
+        <v>54</v>
       </c>
       <c r="G23" t="n">
-        <v>122.06</v>
+        <v>121.59</v>
       </c>
       <c r="H23" t="n">
-        <v>120.59</v>
+        <v>90.91</v>
       </c>
       <c r="I23" t="n">
-        <v>1.47</v>
+        <v>30.68</v>
       </c>
     </row>
     <row r="24">
@@ -2402,25 +2402,25 @@
         <v>373706</v>
       </c>
       <c r="C27" t="n">
-        <v>162</v>
+        <v>175</v>
       </c>
       <c r="D27" t="n">
-        <v>143</v>
+        <v>157</v>
       </c>
       <c r="E27" t="n">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="F27" t="n">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="G27" t="n">
-        <v>88.27</v>
+        <v>89.70999999999999</v>
       </c>
       <c r="H27" t="n">
-        <v>66.67</v>
+        <v>64</v>
       </c>
       <c r="I27" t="n">
-        <v>21.6</v>
+        <v>25.71</v>
       </c>
     </row>
     <row r="28">
@@ -2619,25 +2619,25 @@
         <v>373710</v>
       </c>
       <c r="C34" t="n">
-        <v>131</v>
+        <v>142</v>
       </c>
       <c r="D34" t="n">
-        <v>96</v>
+        <v>106</v>
       </c>
       <c r="E34" t="n">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="F34" t="n">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="G34" t="n">
-        <v>73.28</v>
+        <v>74.65000000000001</v>
       </c>
       <c r="H34" t="n">
-        <v>50.38</v>
+        <v>51.41</v>
       </c>
       <c r="I34" t="n">
-        <v>22.9</v>
+        <v>23.24</v>
       </c>
     </row>
     <row r="35">

</xml_diff>

<commit_message>
feat: enhance name matching logic and update error log files
</commit_message>
<xml_diff>
--- a/Error_log/Enumerator_Performance.xlsx
+++ b/Error_log/Enumerator_Performance.xlsx
@@ -483,13 +483,13 @@
         <v>373641</v>
       </c>
       <c r="C3" t="n">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="D3" t="n">
         <v>370</v>
       </c>
       <c r="E3" t="n">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="4">
@@ -502,13 +502,13 @@
         <v>373648</v>
       </c>
       <c r="C4" t="n">
-        <v>363</v>
+        <v>358</v>
       </c>
       <c r="D4" t="n">
         <v>268</v>
       </c>
       <c r="E4" t="n">
-        <v>95</v>
+        <v>90</v>
       </c>
     </row>
     <row r="5">
@@ -559,13 +559,13 @@
         <v>373696</v>
       </c>
       <c r="C7" t="n">
-        <v>322</v>
+        <v>317</v>
       </c>
       <c r="D7" t="n">
         <v>237</v>
       </c>
       <c r="E7" t="n">
-        <v>85</v>
+        <v>80</v>
       </c>
     </row>
     <row r="8">
@@ -578,13 +578,13 @@
         <v>373642</v>
       </c>
       <c r="C8" t="n">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="D8" t="n">
         <v>229</v>
       </c>
       <c r="E8" t="n">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="9">
@@ -616,13 +616,13 @@
         <v>373705</v>
       </c>
       <c r="C10" t="n">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="D10" t="n">
         <v>179</v>
       </c>
       <c r="E10" t="n">
-        <v>49</v>
+        <v>46</v>
       </c>
     </row>
     <row r="11">
@@ -635,13 +635,13 @@
         <v>373651</v>
       </c>
       <c r="C11" t="n">
-        <v>317</v>
+        <v>309</v>
       </c>
       <c r="D11" t="n">
         <v>178</v>
       </c>
       <c r="E11" t="n">
-        <v>139</v>
+        <v>131</v>
       </c>
     </row>
     <row r="12">
@@ -654,13 +654,13 @@
         <v>373716</v>
       </c>
       <c r="C12" t="n">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="D12" t="n">
         <v>140</v>
       </c>
       <c r="E12" t="n">
-        <v>42</v>
+        <v>38</v>
       </c>
     </row>
     <row r="13">
@@ -692,13 +692,13 @@
         <v>373712</v>
       </c>
       <c r="C14" t="n">
-        <v>324</v>
+        <v>314</v>
       </c>
       <c r="D14" t="n">
         <v>130</v>
       </c>
       <c r="E14" t="n">
-        <v>194</v>
+        <v>184</v>
       </c>
     </row>
     <row r="15">
@@ -711,13 +711,13 @@
         <v>373706</v>
       </c>
       <c r="C15" t="n">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D15" t="n">
         <v>122</v>
       </c>
       <c r="E15" t="n">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="16">
@@ -787,13 +787,13 @@
         <v>373692</v>
       </c>
       <c r="C19" t="n">
-        <v>274</v>
+        <v>267</v>
       </c>
       <c r="D19" t="n">
         <v>102</v>
       </c>
       <c r="E19" t="n">
-        <v>172</v>
+        <v>165</v>
       </c>
     </row>
     <row r="20">
@@ -806,13 +806,13 @@
         <v>373658</v>
       </c>
       <c r="C20" t="n">
-        <v>281</v>
+        <v>278</v>
       </c>
       <c r="D20" t="n">
         <v>100</v>
       </c>
       <c r="E20" t="n">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="21">
@@ -882,13 +882,13 @@
         <v>373691</v>
       </c>
       <c r="C24" t="n">
-        <v>278</v>
+        <v>273</v>
       </c>
       <c r="D24" t="n">
         <v>90</v>
       </c>
       <c r="E24" t="n">
-        <v>188</v>
+        <v>183</v>
       </c>
     </row>
     <row r="25">
@@ -920,13 +920,13 @@
         <v>373710</v>
       </c>
       <c r="C26" t="n">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D26" t="n">
         <v>84</v>
       </c>
       <c r="E26" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="27">
@@ -1034,13 +1034,13 @@
         <v>373669</v>
       </c>
       <c r="C32" t="n">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="D32" t="n">
         <v>55</v>
       </c>
       <c r="E32" t="n">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
     <row r="33">
@@ -1773,22 +1773,22 @@
         <v>104</v>
       </c>
       <c r="D6" t="n">
-        <v>324</v>
+        <v>314</v>
       </c>
       <c r="E6" t="n">
         <v>130</v>
       </c>
       <c r="F6" t="n">
-        <v>194</v>
+        <v>184</v>
       </c>
       <c r="G6" t="n">
-        <v>311.54</v>
+        <v>301.92</v>
       </c>
       <c r="H6" t="n">
         <v>125</v>
       </c>
       <c r="I6" t="n">
-        <v>186.54</v>
+        <v>176.92</v>
       </c>
     </row>
     <row r="7">
@@ -1804,22 +1804,22 @@
         <v>101</v>
       </c>
       <c r="D7" t="n">
-        <v>274</v>
+        <v>267</v>
       </c>
       <c r="E7" t="n">
         <v>102</v>
       </c>
       <c r="F7" t="n">
-        <v>172</v>
+        <v>165</v>
       </c>
       <c r="G7" t="n">
-        <v>271.29</v>
+        <v>264.36</v>
       </c>
       <c r="H7" t="n">
         <v>100.99</v>
       </c>
       <c r="I7" t="n">
-        <v>170.3</v>
+        <v>163.37</v>
       </c>
     </row>
     <row r="8">
@@ -1835,22 +1835,22 @@
         <v>111</v>
       </c>
       <c r="D8" t="n">
-        <v>278</v>
+        <v>273</v>
       </c>
       <c r="E8" t="n">
         <v>90</v>
       </c>
       <c r="F8" t="n">
-        <v>188</v>
+        <v>183</v>
       </c>
       <c r="G8" t="n">
-        <v>250.45</v>
+        <v>245.95</v>
       </c>
       <c r="H8" t="n">
         <v>81.08</v>
       </c>
       <c r="I8" t="n">
-        <v>169.37</v>
+        <v>164.86</v>
       </c>
     </row>
     <row r="9">
@@ -1866,22 +1866,22 @@
         <v>120</v>
       </c>
       <c r="D9" t="n">
-        <v>281</v>
+        <v>278</v>
       </c>
       <c r="E9" t="n">
         <v>100</v>
       </c>
       <c r="F9" t="n">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="G9" t="n">
-        <v>234.17</v>
+        <v>231.67</v>
       </c>
       <c r="H9" t="n">
         <v>83.33</v>
       </c>
       <c r="I9" t="n">
-        <v>150.83</v>
+        <v>148.33</v>
       </c>
     </row>
     <row r="10">
@@ -1897,22 +1897,22 @@
         <v>270</v>
       </c>
       <c r="D10" t="n">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="E10" t="n">
         <v>370</v>
       </c>
       <c r="F10" t="n">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="G10" t="n">
-        <v>171.48</v>
+        <v>171.11</v>
       </c>
       <c r="H10" t="n">
         <v>137.04</v>
       </c>
       <c r="I10" t="n">
-        <v>34.44</v>
+        <v>34.07</v>
       </c>
     </row>
     <row r="11">
@@ -1959,22 +1959,22 @@
         <v>195</v>
       </c>
       <c r="D12" t="n">
-        <v>317</v>
+        <v>309</v>
       </c>
       <c r="E12" t="n">
         <v>178</v>
       </c>
       <c r="F12" t="n">
-        <v>139</v>
+        <v>131</v>
       </c>
       <c r="G12" t="n">
-        <v>162.56</v>
+        <v>158.46</v>
       </c>
       <c r="H12" t="n">
         <v>91.28</v>
       </c>
       <c r="I12" t="n">
-        <v>71.28</v>
+        <v>67.18000000000001</v>
       </c>
     </row>
     <row r="13">
@@ -2083,22 +2083,22 @@
         <v>93</v>
       </c>
       <c r="D16" t="n">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="E16" t="n">
         <v>55</v>
       </c>
       <c r="F16" t="n">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="G16" t="n">
-        <v>140.86</v>
+        <v>138.71</v>
       </c>
       <c r="H16" t="n">
         <v>59.14</v>
       </c>
       <c r="I16" t="n">
-        <v>81.72</v>
+        <v>79.56999999999999</v>
       </c>
     </row>
     <row r="17">
@@ -2114,84 +2114,84 @@
         <v>239</v>
       </c>
       <c r="D17" t="n">
-        <v>322</v>
+        <v>317</v>
       </c>
       <c r="E17" t="n">
         <v>237</v>
       </c>
       <c r="F17" t="n">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="G17" t="n">
-        <v>134.73</v>
+        <v>132.64</v>
       </c>
       <c r="H17" t="n">
         <v>99.16</v>
       </c>
       <c r="I17" t="n">
-        <v>35.56</v>
+        <v>33.47</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Naureen Khan</t>
+          <t>Irum Ikram</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>373716</v>
+        <v>373642</v>
       </c>
       <c r="C18" t="n">
-        <v>139</v>
+        <v>212</v>
       </c>
       <c r="D18" t="n">
-        <v>182</v>
+        <v>274</v>
       </c>
       <c r="E18" t="n">
-        <v>140</v>
+        <v>229</v>
       </c>
       <c r="F18" t="n">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="G18" t="n">
-        <v>130.94</v>
+        <v>129.25</v>
       </c>
       <c r="H18" t="n">
-        <v>100.72</v>
+        <v>108.02</v>
       </c>
       <c r="I18" t="n">
-        <v>30.22</v>
+        <v>21.23</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Irum Ikram</t>
+          <t>Naureen Khan</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>373642</v>
+        <v>373716</v>
       </c>
       <c r="C19" t="n">
-        <v>212</v>
+        <v>139</v>
       </c>
       <c r="D19" t="n">
-        <v>276</v>
+        <v>178</v>
       </c>
       <c r="E19" t="n">
-        <v>229</v>
+        <v>140</v>
       </c>
       <c r="F19" t="n">
-        <v>47</v>
+        <v>38</v>
       </c>
       <c r="G19" t="n">
-        <v>130.19</v>
+        <v>128.06</v>
       </c>
       <c r="H19" t="n">
-        <v>108.02</v>
+        <v>100.72</v>
       </c>
       <c r="I19" t="n">
-        <v>22.17</v>
+        <v>27.34</v>
       </c>
     </row>
     <row r="20">
@@ -2207,22 +2207,22 @@
         <v>281</v>
       </c>
       <c r="D20" t="n">
-        <v>363</v>
+        <v>358</v>
       </c>
       <c r="E20" t="n">
         <v>268</v>
       </c>
       <c r="F20" t="n">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="G20" t="n">
-        <v>129.18</v>
+        <v>127.4</v>
       </c>
       <c r="H20" t="n">
         <v>95.37</v>
       </c>
       <c r="I20" t="n">
-        <v>33.81</v>
+        <v>32.03</v>
       </c>
     </row>
     <row r="21">
@@ -2290,63 +2290,63 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Mahnoor</t>
+          <t>Shafaq Zahra</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>373705</v>
+        <v>373646</v>
       </c>
       <c r="C23" t="n">
-        <v>189</v>
+        <v>288</v>
       </c>
       <c r="D23" t="n">
-        <v>228</v>
+        <v>347</v>
       </c>
       <c r="E23" t="n">
-        <v>179</v>
+        <v>268</v>
       </c>
       <c r="F23" t="n">
-        <v>49</v>
+        <v>79</v>
       </c>
       <c r="G23" t="n">
-        <v>120.63</v>
+        <v>120.49</v>
       </c>
       <c r="H23" t="n">
-        <v>94.70999999999999</v>
+        <v>93.06</v>
       </c>
       <c r="I23" t="n">
-        <v>25.93</v>
+        <v>27.43</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Shafaq Zahra</t>
+          <t>Mahnoor</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>373646</v>
+        <v>373705</v>
       </c>
       <c r="C24" t="n">
-        <v>288</v>
+        <v>189</v>
       </c>
       <c r="D24" t="n">
-        <v>347</v>
+        <v>225</v>
       </c>
       <c r="E24" t="n">
-        <v>268</v>
+        <v>179</v>
       </c>
       <c r="F24" t="n">
-        <v>79</v>
+        <v>46</v>
       </c>
       <c r="G24" t="n">
-        <v>120.49</v>
+        <v>119.05</v>
       </c>
       <c r="H24" t="n">
-        <v>93.06</v>
+        <v>94.70999999999999</v>
       </c>
       <c r="I24" t="n">
-        <v>27.43</v>
+        <v>24.34</v>
       </c>
     </row>
     <row r="25">
@@ -2455,22 +2455,22 @@
         <v>188</v>
       </c>
       <c r="D28" t="n">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="E28" t="n">
         <v>122</v>
       </c>
       <c r="F28" t="n">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G28" t="n">
-        <v>87.77</v>
+        <v>87.23</v>
       </c>
       <c r="H28" t="n">
         <v>64.89</v>
       </c>
       <c r="I28" t="n">
-        <v>22.87</v>
+        <v>22.34</v>
       </c>
     </row>
     <row r="29">
@@ -2662,63 +2662,63 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Summiya Hayat</t>
+          <t>Sadia rustum</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>373710</v>
+        <v>852541</v>
       </c>
       <c r="C35" t="n">
-        <v>159</v>
+        <v>7</v>
       </c>
       <c r="D35" t="n">
-        <v>114</v>
+        <v>5</v>
       </c>
       <c r="E35" t="n">
-        <v>84</v>
+        <v>5</v>
       </c>
       <c r="F35" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="G35" t="n">
-        <v>71.7</v>
+        <v>71.43000000000001</v>
       </c>
       <c r="H35" t="n">
-        <v>52.83</v>
+        <v>71.43000000000001</v>
       </c>
       <c r="I35" t="n">
-        <v>18.87</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Sadia rustum</t>
+          <t>Summiya Hayat</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>852541</v>
+        <v>373710</v>
       </c>
       <c r="C36" t="n">
-        <v>7</v>
+        <v>159</v>
       </c>
       <c r="D36" t="n">
-        <v>5</v>
+        <v>113</v>
       </c>
       <c r="E36" t="n">
-        <v>5</v>
+        <v>84</v>
       </c>
       <c r="F36" t="n">
-        <v>0</v>
+        <v>29</v>
       </c>
       <c r="G36" t="n">
-        <v>71.43000000000001</v>
+        <v>71.06999999999999</v>
       </c>
       <c r="H36" t="n">
-        <v>71.43000000000001</v>
+        <v>52.83</v>
       </c>
       <c r="I36" t="n">
-        <v>0</v>
+        <v>18.24</v>
       </c>
     </row>
     <row r="37">

</xml_diff>

<commit_message>
feat: add logic for identifying listed girl and update education expenditure guidance
</commit_message>
<xml_diff>
--- a/Error_log/Enumerator_Performance.xlsx
+++ b/Error_log/Enumerator_Performance.xlsx
@@ -483,13 +483,13 @@
         <v>373641</v>
       </c>
       <c r="C3" t="n">
-        <v>466</v>
+        <v>463</v>
       </c>
       <c r="D3" t="n">
         <v>372</v>
       </c>
       <c r="E3" t="n">
-        <v>94</v>
+        <v>91</v>
       </c>
     </row>
     <row r="4">
@@ -502,13 +502,13 @@
         <v>373646</v>
       </c>
       <c r="C4" t="n">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="D4" t="n">
         <v>274</v>
       </c>
       <c r="E4" t="n">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="5">
@@ -521,13 +521,13 @@
         <v>373648</v>
       </c>
       <c r="C5" t="n">
-        <v>359</v>
+        <v>355</v>
       </c>
       <c r="D5" t="n">
         <v>270</v>
       </c>
       <c r="E5" t="n">
-        <v>89</v>
+        <v>85</v>
       </c>
     </row>
     <row r="6">
@@ -597,13 +597,13 @@
         <v>373651</v>
       </c>
       <c r="C9" t="n">
-        <v>320</v>
+        <v>313</v>
       </c>
       <c r="D9" t="n">
         <v>183</v>
       </c>
       <c r="E9" t="n">
-        <v>137</v>
+        <v>130</v>
       </c>
     </row>
     <row r="10">
@@ -635,13 +635,13 @@
         <v>373705</v>
       </c>
       <c r="C11" t="n">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="D11" t="n">
         <v>180</v>
       </c>
       <c r="E11" t="n">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="12">
@@ -654,13 +654,13 @@
         <v>373716</v>
       </c>
       <c r="C12" t="n">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="D12" t="n">
         <v>145</v>
       </c>
       <c r="E12" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="13">
@@ -692,13 +692,13 @@
         <v>373712</v>
       </c>
       <c r="C14" t="n">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="D14" t="n">
         <v>126</v>
       </c>
       <c r="E14" t="n">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="15">
@@ -730,13 +730,13 @@
         <v>373706</v>
       </c>
       <c r="C16" t="n">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="D16" t="n">
         <v>121</v>
       </c>
       <c r="E16" t="n">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="17">
@@ -901,13 +901,13 @@
         <v>373691</v>
       </c>
       <c r="C25" t="n">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="D25" t="n">
         <v>84</v>
       </c>
       <c r="E25" t="n">
-        <v>183</v>
+        <v>181</v>
       </c>
     </row>
     <row r="26">
@@ -1034,13 +1034,13 @@
         <v>373669</v>
       </c>
       <c r="C32" t="n">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="D32" t="n">
         <v>51</v>
       </c>
       <c r="E32" t="n">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="33">
@@ -1300,13 +1300,13 @@
         <v>752327</v>
       </c>
       <c r="C46" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="D46" t="n">
         <v>7</v>
       </c>
       <c r="E46" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="47">
@@ -1773,22 +1773,22 @@
         <v>104</v>
       </c>
       <c r="D6" t="n">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="E6" t="n">
         <v>126</v>
       </c>
       <c r="F6" t="n">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="G6" t="n">
-        <v>297.12</v>
+        <v>296.15</v>
       </c>
       <c r="H6" t="n">
         <v>121.15</v>
       </c>
       <c r="I6" t="n">
-        <v>175.96</v>
+        <v>175</v>
       </c>
     </row>
     <row r="7">
@@ -1835,22 +1835,22 @@
         <v>111</v>
       </c>
       <c r="D8" t="n">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="E8" t="n">
         <v>84</v>
       </c>
       <c r="F8" t="n">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="G8" t="n">
-        <v>240.54</v>
+        <v>238.74</v>
       </c>
       <c r="H8" t="n">
         <v>75.68000000000001</v>
       </c>
       <c r="I8" t="n">
-        <v>164.86</v>
+        <v>163.06</v>
       </c>
     </row>
     <row r="9">
@@ -1887,63 +1887,63 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>aisha.aman</t>
+          <t>Asma Bibi</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>752327</v>
+        <v>373641</v>
       </c>
       <c r="C10" t="n">
-        <v>11</v>
+        <v>277</v>
       </c>
       <c r="D10" t="n">
-        <v>20</v>
+        <v>463</v>
       </c>
       <c r="E10" t="n">
-        <v>7</v>
+        <v>372</v>
       </c>
       <c r="F10" t="n">
-        <v>13</v>
+        <v>91</v>
       </c>
       <c r="G10" t="n">
-        <v>181.82</v>
+        <v>167.15</v>
       </c>
       <c r="H10" t="n">
-        <v>63.64</v>
+        <v>134.3</v>
       </c>
       <c r="I10" t="n">
-        <v>118.18</v>
+        <v>32.85</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Asma Bibi</t>
+          <t>aisha.aman</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>373641</v>
+        <v>752327</v>
       </c>
       <c r="C11" t="n">
-        <v>277</v>
+        <v>11</v>
       </c>
       <c r="D11" t="n">
-        <v>466</v>
+        <v>17</v>
       </c>
       <c r="E11" t="n">
-        <v>372</v>
+        <v>7</v>
       </c>
       <c r="F11" t="n">
-        <v>94</v>
+        <v>10</v>
       </c>
       <c r="G11" t="n">
-        <v>168.23</v>
+        <v>154.55</v>
       </c>
       <c r="H11" t="n">
-        <v>134.3</v>
+        <v>63.64</v>
       </c>
       <c r="I11" t="n">
-        <v>33.94</v>
+        <v>90.91</v>
       </c>
     </row>
     <row r="12">
@@ -1959,22 +1959,22 @@
         <v>203</v>
       </c>
       <c r="D12" t="n">
-        <v>320</v>
+        <v>313</v>
       </c>
       <c r="E12" t="n">
         <v>183</v>
       </c>
       <c r="F12" t="n">
-        <v>137</v>
+        <v>130</v>
       </c>
       <c r="G12" t="n">
-        <v>157.64</v>
+        <v>154.19</v>
       </c>
       <c r="H12" t="n">
         <v>90.15000000000001</v>
       </c>
       <c r="I12" t="n">
-        <v>67.48999999999999</v>
+        <v>64.04000000000001</v>
       </c>
     </row>
     <row r="13">
@@ -2073,63 +2073,63 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Nadia bibi</t>
+          <t>Shazia begum</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>373669</v>
+        <v>373696</v>
       </c>
       <c r="C16" t="n">
-        <v>93</v>
+        <v>239</v>
       </c>
       <c r="D16" t="n">
-        <v>125</v>
+        <v>318</v>
       </c>
       <c r="E16" t="n">
-        <v>51</v>
+        <v>238</v>
       </c>
       <c r="F16" t="n">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="G16" t="n">
-        <v>134.41</v>
+        <v>133.05</v>
       </c>
       <c r="H16" t="n">
-        <v>54.84</v>
+        <v>99.58</v>
       </c>
       <c r="I16" t="n">
-        <v>79.56999999999999</v>
+        <v>33.47</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Shazia begum</t>
+          <t>Nadia bibi</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>373696</v>
+        <v>373669</v>
       </c>
       <c r="C17" t="n">
-        <v>239</v>
+        <v>93</v>
       </c>
       <c r="D17" t="n">
-        <v>318</v>
+        <v>123</v>
       </c>
       <c r="E17" t="n">
-        <v>238</v>
+        <v>51</v>
       </c>
       <c r="F17" t="n">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="G17" t="n">
-        <v>133.05</v>
+        <v>132.26</v>
       </c>
       <c r="H17" t="n">
-        <v>99.58</v>
+        <v>54.84</v>
       </c>
       <c r="I17" t="n">
-        <v>33.47</v>
+        <v>77.42</v>
       </c>
     </row>
     <row r="18">
@@ -2207,22 +2207,22 @@
         <v>149</v>
       </c>
       <c r="D20" t="n">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="E20" t="n">
         <v>145</v>
       </c>
       <c r="F20" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G20" t="n">
-        <v>124.16</v>
+        <v>123.49</v>
       </c>
       <c r="H20" t="n">
         <v>97.31999999999999</v>
       </c>
       <c r="I20" t="n">
-        <v>26.85</v>
+        <v>26.17</v>
       </c>
     </row>
     <row r="21">
@@ -2238,22 +2238,22 @@
         <v>290</v>
       </c>
       <c r="D21" t="n">
-        <v>359</v>
+        <v>355</v>
       </c>
       <c r="E21" t="n">
         <v>270</v>
       </c>
       <c r="F21" t="n">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="G21" t="n">
-        <v>123.79</v>
+        <v>122.41</v>
       </c>
       <c r="H21" t="n">
         <v>93.09999999999999</v>
       </c>
       <c r="I21" t="n">
-        <v>30.69</v>
+        <v>29.31</v>
       </c>
     </row>
     <row r="22">
@@ -2300,22 +2300,22 @@
         <v>297</v>
       </c>
       <c r="D23" t="n">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="E23" t="n">
         <v>274</v>
       </c>
       <c r="F23" t="n">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="G23" t="n">
-        <v>120.88</v>
+        <v>120.54</v>
       </c>
       <c r="H23" t="n">
         <v>92.26000000000001</v>
       </c>
       <c r="I23" t="n">
-        <v>28.62</v>
+        <v>28.28</v>
       </c>
     </row>
     <row r="24">
@@ -2331,22 +2331,22 @@
         <v>199</v>
       </c>
       <c r="D24" t="n">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="E24" t="n">
         <v>180</v>
       </c>
       <c r="F24" t="n">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="G24" t="n">
-        <v>116.58</v>
+        <v>116.08</v>
       </c>
       <c r="H24" t="n">
         <v>90.45</v>
       </c>
       <c r="I24" t="n">
-        <v>26.13</v>
+        <v>25.63</v>
       </c>
     </row>
     <row r="25">
@@ -2486,22 +2486,22 @@
         <v>194</v>
       </c>
       <c r="D29" t="n">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="E29" t="n">
         <v>121</v>
       </c>
       <c r="F29" t="n">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="G29" t="n">
-        <v>84.02</v>
+        <v>82.98999999999999</v>
       </c>
       <c r="H29" t="n">
         <v>62.37</v>
       </c>
       <c r="I29" t="n">
-        <v>21.65</v>
+        <v>20.62</v>
       </c>
     </row>
     <row r="30">

</xml_diff>

<commit_message>
feat: update harassment guidance logic and refine error messages
</commit_message>
<xml_diff>
--- a/Error_log/Enumerator_Performance.xlsx
+++ b/Error_log/Enumerator_Performance.xlsx
@@ -521,13 +521,13 @@
         <v>373648</v>
       </c>
       <c r="C5" t="n">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="D5" t="n">
         <v>270</v>
       </c>
       <c r="E5" t="n">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="6">
@@ -597,13 +597,13 @@
         <v>373651</v>
       </c>
       <c r="C9" t="n">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="D9" t="n">
         <v>183</v>
       </c>
       <c r="E9" t="n">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="10">
@@ -1034,13 +1034,13 @@
         <v>373669</v>
       </c>
       <c r="C32" t="n">
-        <v>123</v>
+        <v>106</v>
       </c>
       <c r="D32" t="n">
         <v>51</v>
       </c>
       <c r="E32" t="n">
-        <v>72</v>
+        <v>55</v>
       </c>
     </row>
     <row r="33">
@@ -1959,22 +1959,22 @@
         <v>203</v>
       </c>
       <c r="D12" t="n">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="E12" t="n">
         <v>183</v>
       </c>
       <c r="F12" t="n">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="G12" t="n">
-        <v>154.19</v>
+        <v>153.69</v>
       </c>
       <c r="H12" t="n">
         <v>90.15000000000001</v>
       </c>
       <c r="I12" t="n">
-        <v>64.04000000000001</v>
+        <v>63.55</v>
       </c>
     </row>
     <row r="13">
@@ -2104,249 +2104,249 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Nadia bibi</t>
+          <t>Irum Ikram</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>373669</v>
+        <v>373642</v>
       </c>
       <c r="C17" t="n">
-        <v>93</v>
+        <v>218</v>
       </c>
       <c r="D17" t="n">
-        <v>123</v>
+        <v>285</v>
       </c>
       <c r="E17" t="n">
-        <v>51</v>
+        <v>231</v>
       </c>
       <c r="F17" t="n">
-        <v>72</v>
+        <v>54</v>
       </c>
       <c r="G17" t="n">
-        <v>132.26</v>
+        <v>130.73</v>
       </c>
       <c r="H17" t="n">
-        <v>54.84</v>
+        <v>105.96</v>
       </c>
       <c r="I17" t="n">
-        <v>77.42</v>
+        <v>24.77</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Irum Ikram</t>
+          <t>Sadia Rustum</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>373642</v>
+        <v>373649</v>
       </c>
       <c r="C18" t="n">
-        <v>218</v>
+        <v>152</v>
       </c>
       <c r="D18" t="n">
-        <v>285</v>
+        <v>192</v>
       </c>
       <c r="E18" t="n">
-        <v>231</v>
+        <v>182</v>
       </c>
       <c r="F18" t="n">
-        <v>54</v>
+        <v>10</v>
       </c>
       <c r="G18" t="n">
-        <v>130.73</v>
+        <v>126.32</v>
       </c>
       <c r="H18" t="n">
-        <v>105.96</v>
+        <v>119.74</v>
       </c>
       <c r="I18" t="n">
-        <v>24.77</v>
+        <v>6.58</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Sadia Rustum</t>
+          <t>Naureen Khan</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>373649</v>
+        <v>373716</v>
       </c>
       <c r="C19" t="n">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="D19" t="n">
-        <v>192</v>
+        <v>184</v>
       </c>
       <c r="E19" t="n">
-        <v>182</v>
+        <v>145</v>
       </c>
       <c r="F19" t="n">
-        <v>10</v>
+        <v>39</v>
       </c>
       <c r="G19" t="n">
-        <v>126.32</v>
+        <v>123.49</v>
       </c>
       <c r="H19" t="n">
-        <v>119.74</v>
+        <v>97.31999999999999</v>
       </c>
       <c r="I19" t="n">
-        <v>6.58</v>
+        <v>26.17</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Naureen Khan</t>
+          <t>Shazia Bibi</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>373716</v>
+        <v>373648</v>
       </c>
       <c r="C20" t="n">
-        <v>149</v>
+        <v>290</v>
       </c>
       <c r="D20" t="n">
-        <v>184</v>
+        <v>354</v>
       </c>
       <c r="E20" t="n">
-        <v>145</v>
+        <v>270</v>
       </c>
       <c r="F20" t="n">
-        <v>39</v>
+        <v>84</v>
       </c>
       <c r="G20" t="n">
-        <v>123.49</v>
+        <v>122.07</v>
       </c>
       <c r="H20" t="n">
-        <v>97.31999999999999</v>
+        <v>93.09999999999999</v>
       </c>
       <c r="I20" t="n">
-        <v>26.17</v>
+        <v>28.97</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Shazia Bibi</t>
+          <t>Jaweria</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>373648</v>
+        <v>163495</v>
       </c>
       <c r="C21" t="n">
-        <v>290</v>
+        <v>68</v>
       </c>
       <c r="D21" t="n">
-        <v>355</v>
+        <v>83</v>
       </c>
       <c r="E21" t="n">
-        <v>270</v>
+        <v>82</v>
       </c>
       <c r="F21" t="n">
-        <v>85</v>
+        <v>1</v>
       </c>
       <c r="G21" t="n">
-        <v>122.41</v>
+        <v>122.06</v>
       </c>
       <c r="H21" t="n">
-        <v>93.09999999999999</v>
+        <v>120.59</v>
       </c>
       <c r="I21" t="n">
-        <v>29.31</v>
+        <v>1.47</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Jaweria</t>
+          <t>Shafaq Zahra</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>163495</v>
+        <v>373646</v>
       </c>
       <c r="C22" t="n">
-        <v>68</v>
+        <v>297</v>
       </c>
       <c r="D22" t="n">
-        <v>83</v>
+        <v>358</v>
       </c>
       <c r="E22" t="n">
-        <v>82</v>
+        <v>274</v>
       </c>
       <c r="F22" t="n">
-        <v>1</v>
+        <v>84</v>
       </c>
       <c r="G22" t="n">
-        <v>122.06</v>
+        <v>120.54</v>
       </c>
       <c r="H22" t="n">
-        <v>120.59</v>
+        <v>92.26000000000001</v>
       </c>
       <c r="I22" t="n">
-        <v>1.47</v>
+        <v>28.28</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Shafaq Zahra</t>
+          <t>Mahnoor</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>373646</v>
+        <v>373705</v>
       </c>
       <c r="C23" t="n">
-        <v>297</v>
+        <v>199</v>
       </c>
       <c r="D23" t="n">
-        <v>358</v>
+        <v>231</v>
       </c>
       <c r="E23" t="n">
-        <v>274</v>
+        <v>180</v>
       </c>
       <c r="F23" t="n">
-        <v>84</v>
+        <v>51</v>
       </c>
       <c r="G23" t="n">
-        <v>120.54</v>
+        <v>116.08</v>
       </c>
       <c r="H23" t="n">
-        <v>92.26000000000001</v>
+        <v>90.45</v>
       </c>
       <c r="I23" t="n">
-        <v>28.28</v>
+        <v>25.63</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Mahnoor</t>
+          <t>Nadia bibi</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>373705</v>
+        <v>373669</v>
       </c>
       <c r="C24" t="n">
-        <v>199</v>
+        <v>93</v>
       </c>
       <c r="D24" t="n">
-        <v>231</v>
+        <v>106</v>
       </c>
       <c r="E24" t="n">
-        <v>180</v>
+        <v>51</v>
       </c>
       <c r="F24" t="n">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="G24" t="n">
-        <v>116.08</v>
+        <v>113.98</v>
       </c>
       <c r="H24" t="n">
-        <v>90.45</v>
+        <v>54.84</v>
       </c>
       <c r="I24" t="n">
-        <v>25.63</v>
+        <v>59.14</v>
       </c>
     </row>
     <row r="25">

</xml_diff>

<commit_message>
feat: enhance error guidance to include 'No attempt' in incorrect counts
</commit_message>
<xml_diff>
--- a/Error_log/Enumerator_Performance.xlsx
+++ b/Error_log/Enumerator_Performance.xlsx
@@ -502,10 +502,10 @@
         <v>373646</v>
       </c>
       <c r="C4" t="n">
-        <v>361</v>
+        <v>365</v>
       </c>
       <c r="D4" t="n">
-        <v>276</v>
+        <v>280</v>
       </c>
       <c r="E4" t="n">
         <v>85</v>
@@ -521,10 +521,10 @@
         <v>373648</v>
       </c>
       <c r="C5" t="n">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="D5" t="n">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="E5" t="n">
         <v>84</v>
@@ -635,10 +635,10 @@
         <v>373705</v>
       </c>
       <c r="C11" t="n">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="D11" t="n">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="E11" t="n">
         <v>52</v>
@@ -654,10 +654,10 @@
         <v>373716</v>
       </c>
       <c r="C12" t="n">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="D12" t="n">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="E12" t="n">
         <v>39</v>
@@ -787,10 +787,10 @@
         <v>373692</v>
       </c>
       <c r="C19" t="n">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="D19" t="n">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E19" t="n">
         <v>165</v>
@@ -799,39 +799,39 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Samara</t>
+          <t>Ishaq Khan</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>373658</v>
+        <v>373699</v>
       </c>
       <c r="C20" t="n">
-        <v>278</v>
+        <v>101</v>
       </c>
       <c r="D20" t="n">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E20" t="n">
-        <v>177</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Ishaq Khan</t>
+          <t>Samara</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>373699</v>
+        <v>373658</v>
       </c>
       <c r="C21" t="n">
-        <v>101</v>
+        <v>276</v>
       </c>
       <c r="D21" t="n">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E21" t="n">
-        <v>1</v>
+        <v>177</v>
       </c>
     </row>
     <row r="22">
@@ -1804,19 +1804,19 @@
         <v>101</v>
       </c>
       <c r="D7" t="n">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="E7" t="n">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F7" t="n">
         <v>165</v>
       </c>
       <c r="G7" t="n">
-        <v>264.36</v>
+        <v>263.37</v>
       </c>
       <c r="H7" t="n">
-        <v>100.99</v>
+        <v>100</v>
       </c>
       <c r="I7" t="n">
         <v>163.37</v>
@@ -1866,19 +1866,19 @@
         <v>120</v>
       </c>
       <c r="D9" t="n">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="E9" t="n">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="F9" t="n">
         <v>177</v>
       </c>
       <c r="G9" t="n">
-        <v>231.67</v>
+        <v>230</v>
       </c>
       <c r="H9" t="n">
-        <v>84.17</v>
+        <v>82.5</v>
       </c>
       <c r="I9" t="n">
         <v>147.5</v>
@@ -2176,19 +2176,19 @@
         <v>149</v>
       </c>
       <c r="D19" t="n">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="E19" t="n">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="F19" t="n">
         <v>39</v>
       </c>
       <c r="G19" t="n">
-        <v>123.49</v>
+        <v>122.15</v>
       </c>
       <c r="H19" t="n">
-        <v>97.31999999999999</v>
+        <v>95.97</v>
       </c>
       <c r="I19" t="n">
         <v>26.17</v>
@@ -2228,63 +2228,63 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Shazia Bibi</t>
+          <t>Shafaq Zahra</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>373648</v>
+        <v>373646</v>
       </c>
       <c r="C21" t="n">
-        <v>296</v>
+        <v>303</v>
       </c>
       <c r="D21" t="n">
-        <v>354</v>
+        <v>365</v>
       </c>
       <c r="E21" t="n">
-        <v>270</v>
+        <v>280</v>
       </c>
       <c r="F21" t="n">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="G21" t="n">
-        <v>119.59</v>
+        <v>120.46</v>
       </c>
       <c r="H21" t="n">
-        <v>91.22</v>
+        <v>92.41</v>
       </c>
       <c r="I21" t="n">
-        <v>28.38</v>
+        <v>28.05</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Shafaq Zahra</t>
+          <t>Shazia Bibi</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>373646</v>
+        <v>373648</v>
       </c>
       <c r="C22" t="n">
-        <v>303</v>
+        <v>296</v>
       </c>
       <c r="D22" t="n">
-        <v>361</v>
+        <v>353</v>
       </c>
       <c r="E22" t="n">
-        <v>276</v>
+        <v>269</v>
       </c>
       <c r="F22" t="n">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="G22" t="n">
-        <v>119.14</v>
+        <v>119.26</v>
       </c>
       <c r="H22" t="n">
-        <v>91.09</v>
+        <v>90.88</v>
       </c>
       <c r="I22" t="n">
-        <v>28.05</v>
+        <v>28.38</v>
       </c>
     </row>
     <row r="23">
@@ -2300,19 +2300,19 @@
         <v>203</v>
       </c>
       <c r="D23" t="n">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="E23" t="n">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="F23" t="n">
         <v>52</v>
       </c>
       <c r="G23" t="n">
-        <v>114.29</v>
+        <v>113.79</v>
       </c>
       <c r="H23" t="n">
-        <v>88.67</v>
+        <v>88.18000000000001</v>
       </c>
       <c r="I23" t="n">
         <v>25.62</v>

</xml_diff>

<commit_message>
chore: update binary files for error logs and performance summaries
</commit_message>
<xml_diff>
--- a/Error_log/Enumerator_Performance.xlsx
+++ b/Error_log/Enumerator_Performance.xlsx
@@ -464,10 +464,10 @@
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="n">
-        <v>1544</v>
+        <v>1534</v>
       </c>
       <c r="D2" t="n">
-        <v>1506</v>
+        <v>1496</v>
       </c>
       <c r="E2" t="n">
         <v>38</v>
@@ -578,13 +578,13 @@
         <v>373642</v>
       </c>
       <c r="C8" t="n">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="D8" t="n">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="E8" t="n">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="9">
@@ -616,13 +616,13 @@
         <v>373705</v>
       </c>
       <c r="C10" t="n">
-        <v>249</v>
+        <v>255</v>
       </c>
       <c r="D10" t="n">
         <v>186</v>
       </c>
       <c r="E10" t="n">
-        <v>63</v>
+        <v>69</v>
       </c>
     </row>
     <row r="11">
@@ -685,39 +685,39 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Kainat</t>
+          <t>Laiba Shams</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>373712</v>
+        <v>373706</v>
       </c>
       <c r="C14" t="n">
-        <v>308</v>
+        <v>172</v>
       </c>
       <c r="D14" t="n">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="E14" t="n">
-        <v>182</v>
+        <v>45</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Laiba Shams</t>
+          <t>Kainat</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>373706</v>
+        <v>373712</v>
       </c>
       <c r="C15" t="n">
-        <v>170</v>
+        <v>308</v>
       </c>
       <c r="D15" t="n">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="E15" t="n">
-        <v>45</v>
+        <v>182</v>
       </c>
     </row>
     <row r="16">
@@ -1034,13 +1034,13 @@
         <v>373669</v>
       </c>
       <c r="C32" t="n">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="D32" t="n">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="E32" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="33">
@@ -2111,25 +2111,25 @@
         <v>373642</v>
       </c>
       <c r="C17" t="n">
+        <v>239</v>
+      </c>
+      <c r="D17" t="n">
+        <v>307</v>
+      </c>
+      <c r="E17" t="n">
         <v>238</v>
       </c>
-      <c r="D17" t="n">
-        <v>306</v>
-      </c>
-      <c r="E17" t="n">
-        <v>236</v>
-      </c>
       <c r="F17" t="n">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G17" t="n">
-        <v>128.57</v>
+        <v>128.45</v>
       </c>
       <c r="H17" t="n">
-        <v>99.16</v>
+        <v>99.58</v>
       </c>
       <c r="I17" t="n">
-        <v>29.41</v>
+        <v>28.87</v>
       </c>
     </row>
     <row r="18">
@@ -2297,25 +2297,25 @@
         <v>373705</v>
       </c>
       <c r="C23" t="n">
-        <v>212</v>
+        <v>217</v>
       </c>
       <c r="D23" t="n">
-        <v>249</v>
+        <v>255</v>
       </c>
       <c r="E23" t="n">
         <v>186</v>
       </c>
       <c r="F23" t="n">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="G23" t="n">
-        <v>117.45</v>
+        <v>117.51</v>
       </c>
       <c r="H23" t="n">
-        <v>87.73999999999999</v>
+        <v>85.70999999999999</v>
       </c>
       <c r="I23" t="n">
-        <v>29.72</v>
+        <v>31.8</v>
       </c>
     </row>
     <row r="24">
@@ -2328,25 +2328,25 @@
         <v>373669</v>
       </c>
       <c r="C24" t="n">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="D24" t="n">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="E24" t="n">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="F24" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="G24" t="n">
-        <v>108.41</v>
+        <v>107.21</v>
       </c>
       <c r="H24" t="n">
-        <v>51.4</v>
+        <v>51.35</v>
       </c>
       <c r="I24" t="n">
-        <v>57.01</v>
+        <v>55.86</v>
       </c>
     </row>
     <row r="25">
@@ -2483,25 +2483,25 @@
         <v>373706</v>
       </c>
       <c r="C29" t="n">
-        <v>207</v>
+        <v>212</v>
       </c>
       <c r="D29" t="n">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="E29" t="n">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="F29" t="n">
         <v>45</v>
       </c>
       <c r="G29" t="n">
-        <v>82.13</v>
+        <v>81.13</v>
       </c>
       <c r="H29" t="n">
-        <v>60.39</v>
+        <v>59.91</v>
       </c>
       <c r="I29" t="n">
-        <v>21.74</v>
+        <v>21.23</v>
       </c>
     </row>
     <row r="30">
@@ -2731,7 +2731,7 @@
         <v>373710</v>
       </c>
       <c r="C37" t="n">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="D37" t="n">
         <v>118</v>
@@ -2743,13 +2743,13 @@
         <v>33</v>
       </c>
       <c r="G37" t="n">
-        <v>66.29000000000001</v>
+        <v>64.48</v>
       </c>
       <c r="H37" t="n">
-        <v>47.75</v>
+        <v>46.45</v>
       </c>
       <c r="I37" t="n">
-        <v>18.54</v>
+        <v>18.03</v>
       </c>
     </row>
     <row r="38">

</xml_diff>

<commit_message>
Implement structural updates and optimizations across multiple modules
</commit_message>
<xml_diff>
--- a/Error_log/Enumerator_Performance.xlsx
+++ b/Error_log/Enumerator_Performance.xlsx
@@ -464,13 +464,13 @@
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="n">
-        <v>1534</v>
+        <v>1526</v>
       </c>
       <c r="D2" t="n">
-        <v>1496</v>
+        <v>1487</v>
       </c>
       <c r="E2" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="3">
@@ -483,13 +483,13 @@
         <v>373641</v>
       </c>
       <c r="C3" t="n">
-        <v>499</v>
+        <v>495</v>
       </c>
       <c r="D3" t="n">
         <v>395</v>
       </c>
       <c r="E3" t="n">
-        <v>104</v>
+        <v>100</v>
       </c>
     </row>
     <row r="4">
@@ -502,13 +502,13 @@
         <v>373646</v>
       </c>
       <c r="C4" t="n">
-        <v>395</v>
+        <v>391</v>
       </c>
       <c r="D4" t="n">
         <v>284</v>
       </c>
       <c r="E4" t="n">
-        <v>111</v>
+        <v>107</v>
       </c>
     </row>
     <row r="5">
@@ -521,13 +521,13 @@
         <v>373648</v>
       </c>
       <c r="C5" t="n">
-        <v>369</v>
+        <v>365</v>
       </c>
       <c r="D5" t="n">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="E5" t="n">
-        <v>93</v>
+        <v>88</v>
       </c>
     </row>
     <row r="6">
@@ -559,13 +559,13 @@
         <v>373696</v>
       </c>
       <c r="C7" t="n">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="D7" t="n">
         <v>238</v>
       </c>
       <c r="E7" t="n">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="8">
@@ -578,13 +578,13 @@
         <v>373642</v>
       </c>
       <c r="C8" t="n">
-        <v>307</v>
+        <v>301</v>
       </c>
       <c r="D8" t="n">
         <v>238</v>
       </c>
       <c r="E8" t="n">
-        <v>69</v>
+        <v>63</v>
       </c>
     </row>
     <row r="9">
@@ -597,13 +597,13 @@
         <v>373651</v>
       </c>
       <c r="C9" t="n">
-        <v>353</v>
+        <v>350</v>
       </c>
       <c r="D9" t="n">
         <v>208</v>
       </c>
       <c r="E9" t="n">
-        <v>145</v>
+        <v>142</v>
       </c>
     </row>
     <row r="10">
@@ -616,13 +616,13 @@
         <v>373705</v>
       </c>
       <c r="C10" t="n">
-        <v>255</v>
+        <v>249</v>
       </c>
       <c r="D10" t="n">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="E10" t="n">
-        <v>69</v>
+        <v>61</v>
       </c>
     </row>
     <row r="11">
@@ -654,13 +654,13 @@
         <v>373716</v>
       </c>
       <c r="C12" t="n">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="D12" t="n">
         <v>149</v>
       </c>
       <c r="E12" t="n">
-        <v>52</v>
+        <v>48</v>
       </c>
     </row>
     <row r="13">
@@ -685,39 +685,39 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Laiba Shams</t>
+          <t>Kainat</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>373706</v>
+        <v>373712</v>
       </c>
       <c r="C14" t="n">
-        <v>172</v>
+        <v>308</v>
       </c>
       <c r="D14" t="n">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E14" t="n">
-        <v>45</v>
+        <v>182</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Kainat</t>
+          <t>Laiba Shams</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>373712</v>
+        <v>373706</v>
       </c>
       <c r="C15" t="n">
-        <v>308</v>
+        <v>166</v>
       </c>
       <c r="D15" t="n">
         <v>126</v>
       </c>
       <c r="E15" t="n">
-        <v>182</v>
+        <v>40</v>
       </c>
     </row>
     <row r="16">
@@ -780,58 +780,58 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Ishaq Khan</t>
+          <t>Zohra</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>373699</v>
+        <v>373692</v>
       </c>
       <c r="C19" t="n">
+        <v>266</v>
+      </c>
+      <c r="D19" t="n">
         <v>101</v>
       </c>
-      <c r="D19" t="n">
-        <v>100</v>
-      </c>
       <c r="E19" t="n">
-        <v>1</v>
+        <v>165</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Samara</t>
+          <t>Ishaq Khan</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>373658</v>
+        <v>373699</v>
       </c>
       <c r="C20" t="n">
-        <v>276</v>
+        <v>101</v>
       </c>
       <c r="D20" t="n">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="E20" t="n">
-        <v>177</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Zohra</t>
+          <t>Samara</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>373692</v>
+        <v>373658</v>
       </c>
       <c r="C21" t="n">
-        <v>265</v>
+        <v>276</v>
       </c>
       <c r="D21" t="n">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="E21" t="n">
-        <v>168</v>
+        <v>177</v>
       </c>
     </row>
     <row r="22">
@@ -901,13 +901,13 @@
         <v>373710</v>
       </c>
       <c r="C25" t="n">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="D25" t="n">
         <v>85</v>
       </c>
       <c r="E25" t="n">
-        <v>33</v>
+        <v>29</v>
       </c>
     </row>
     <row r="26">
@@ -1034,13 +1034,13 @@
         <v>373669</v>
       </c>
       <c r="C32" t="n">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="D32" t="n">
         <v>57</v>
       </c>
       <c r="E32" t="n">
-        <v>62</v>
+        <v>58</v>
       </c>
     </row>
     <row r="33">
@@ -1148,13 +1148,13 @@
         <v>752327</v>
       </c>
       <c r="C38" t="n">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D38" t="n">
         <v>33</v>
       </c>
       <c r="E38" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="39">
@@ -1804,22 +1804,22 @@
         <v>101</v>
       </c>
       <c r="D7" t="n">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="E7" t="n">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="F7" t="n">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="G7" t="n">
-        <v>262.38</v>
+        <v>263.37</v>
       </c>
       <c r="H7" t="n">
-        <v>96.04000000000001</v>
+        <v>100</v>
       </c>
       <c r="I7" t="n">
-        <v>166.34</v>
+        <v>163.37</v>
       </c>
     </row>
     <row r="8">
@@ -1897,22 +1897,22 @@
         <v>36</v>
       </c>
       <c r="D10" t="n">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E10" t="n">
         <v>33</v>
       </c>
       <c r="F10" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G10" t="n">
-        <v>166.67</v>
+        <v>163.89</v>
       </c>
       <c r="H10" t="n">
         <v>91.67</v>
       </c>
       <c r="I10" t="n">
-        <v>75</v>
+        <v>72.22</v>
       </c>
     </row>
     <row r="11">
@@ -1928,22 +1928,22 @@
         <v>304</v>
       </c>
       <c r="D11" t="n">
-        <v>499</v>
+        <v>495</v>
       </c>
       <c r="E11" t="n">
         <v>395</v>
       </c>
       <c r="F11" t="n">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="G11" t="n">
-        <v>164.14</v>
+        <v>162.83</v>
       </c>
       <c r="H11" t="n">
         <v>129.93</v>
       </c>
       <c r="I11" t="n">
-        <v>34.21</v>
+        <v>32.89</v>
       </c>
     </row>
     <row r="12">
@@ -1959,22 +1959,22 @@
         <v>231</v>
       </c>
       <c r="D12" t="n">
-        <v>353</v>
+        <v>350</v>
       </c>
       <c r="E12" t="n">
         <v>208</v>
       </c>
       <c r="F12" t="n">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="G12" t="n">
-        <v>152.81</v>
+        <v>151.52</v>
       </c>
       <c r="H12" t="n">
         <v>90.04000000000001</v>
       </c>
       <c r="I12" t="n">
-        <v>62.77</v>
+        <v>61.47</v>
       </c>
     </row>
     <row r="13">
@@ -2083,84 +2083,84 @@
         <v>239</v>
       </c>
       <c r="D16" t="n">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="E16" t="n">
         <v>238</v>
       </c>
       <c r="F16" t="n">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G16" t="n">
-        <v>133.47</v>
+        <v>133.05</v>
       </c>
       <c r="H16" t="n">
         <v>99.58</v>
       </c>
       <c r="I16" t="n">
-        <v>33.89</v>
+        <v>33.47</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Irum Ikram</t>
+          <t>Sadia Rustum</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>373642</v>
+        <v>373649</v>
       </c>
       <c r="C17" t="n">
-        <v>239</v>
+        <v>152</v>
       </c>
       <c r="D17" t="n">
-        <v>307</v>
+        <v>192</v>
       </c>
       <c r="E17" t="n">
-        <v>238</v>
+        <v>182</v>
       </c>
       <c r="F17" t="n">
-        <v>69</v>
+        <v>10</v>
       </c>
       <c r="G17" t="n">
-        <v>128.45</v>
+        <v>126.32</v>
       </c>
       <c r="H17" t="n">
-        <v>99.58</v>
+        <v>119.74</v>
       </c>
       <c r="I17" t="n">
-        <v>28.87</v>
+        <v>6.58</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Sadia Rustum</t>
+          <t>Irum Ikram</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>373649</v>
+        <v>373642</v>
       </c>
       <c r="C18" t="n">
-        <v>152</v>
+        <v>239</v>
       </c>
       <c r="D18" t="n">
-        <v>192</v>
+        <v>301</v>
       </c>
       <c r="E18" t="n">
-        <v>182</v>
+        <v>238</v>
       </c>
       <c r="F18" t="n">
-        <v>10</v>
+        <v>63</v>
       </c>
       <c r="G18" t="n">
-        <v>126.32</v>
+        <v>125.94</v>
       </c>
       <c r="H18" t="n">
-        <v>119.74</v>
+        <v>99.58</v>
       </c>
       <c r="I18" t="n">
-        <v>6.58</v>
+        <v>26.36</v>
       </c>
     </row>
     <row r="19">
@@ -2207,22 +2207,22 @@
         <v>324</v>
       </c>
       <c r="D20" t="n">
-        <v>395</v>
+        <v>391</v>
       </c>
       <c r="E20" t="n">
         <v>284</v>
       </c>
       <c r="F20" t="n">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="G20" t="n">
-        <v>121.91</v>
+        <v>120.68</v>
       </c>
       <c r="H20" t="n">
         <v>87.65000000000001</v>
       </c>
       <c r="I20" t="n">
-        <v>34.26</v>
+        <v>33.02</v>
       </c>
     </row>
     <row r="21">
@@ -2238,22 +2238,22 @@
         <v>309</v>
       </c>
       <c r="D21" t="n">
-        <v>369</v>
+        <v>365</v>
       </c>
       <c r="E21" t="n">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="F21" t="n">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="G21" t="n">
-        <v>119.42</v>
+        <v>118.12</v>
       </c>
       <c r="H21" t="n">
-        <v>89.31999999999999</v>
+        <v>89.64</v>
       </c>
       <c r="I21" t="n">
-        <v>30.1</v>
+        <v>28.48</v>
       </c>
     </row>
     <row r="22">
@@ -2269,22 +2269,22 @@
         <v>169</v>
       </c>
       <c r="D22" t="n">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="E22" t="n">
         <v>149</v>
       </c>
       <c r="F22" t="n">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="G22" t="n">
-        <v>118.93</v>
+        <v>116.57</v>
       </c>
       <c r="H22" t="n">
         <v>88.17</v>
       </c>
       <c r="I22" t="n">
-        <v>30.77</v>
+        <v>28.4</v>
       </c>
     </row>
     <row r="23">
@@ -2297,25 +2297,25 @@
         <v>373705</v>
       </c>
       <c r="C23" t="n">
-        <v>217</v>
+        <v>224</v>
       </c>
       <c r="D23" t="n">
-        <v>255</v>
+        <v>249</v>
       </c>
       <c r="E23" t="n">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="F23" t="n">
-        <v>69</v>
+        <v>61</v>
       </c>
       <c r="G23" t="n">
-        <v>117.51</v>
+        <v>111.16</v>
       </c>
       <c r="H23" t="n">
-        <v>85.70999999999999</v>
+        <v>83.93000000000001</v>
       </c>
       <c r="I23" t="n">
-        <v>31.8</v>
+        <v>27.23</v>
       </c>
     </row>
     <row r="24">
@@ -2331,22 +2331,22 @@
         <v>111</v>
       </c>
       <c r="D24" t="n">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="E24" t="n">
         <v>57</v>
       </c>
       <c r="F24" t="n">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="G24" t="n">
-        <v>107.21</v>
+        <v>103.6</v>
       </c>
       <c r="H24" t="n">
         <v>51.35</v>
       </c>
       <c r="I24" t="n">
-        <v>55.86</v>
+        <v>52.25</v>
       </c>
     </row>
     <row r="25">
@@ -2476,125 +2476,125 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Laiba Shams</t>
+          <t>Muniba Shamim</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>373706</v>
+        <v>373659</v>
       </c>
       <c r="C29" t="n">
-        <v>212</v>
+        <v>72</v>
       </c>
       <c r="D29" t="n">
-        <v>172</v>
+        <v>58</v>
       </c>
       <c r="E29" t="n">
-        <v>127</v>
+        <v>49</v>
       </c>
       <c r="F29" t="n">
-        <v>45</v>
+        <v>9</v>
       </c>
       <c r="G29" t="n">
-        <v>81.13</v>
+        <v>80.56</v>
       </c>
       <c r="H29" t="n">
-        <v>59.91</v>
+        <v>68.06</v>
       </c>
       <c r="I29" t="n">
-        <v>21.23</v>
+        <v>12.5</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Muniba Shamim</t>
+          <t>Muhammad Yousaf</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>373659</v>
+        <v>373690</v>
       </c>
       <c r="C30" t="n">
-        <v>72</v>
+        <v>132</v>
       </c>
       <c r="D30" t="n">
-        <v>58</v>
+        <v>105</v>
       </c>
       <c r="E30" t="n">
-        <v>49</v>
+        <v>96</v>
       </c>
       <c r="F30" t="n">
         <v>9</v>
       </c>
       <c r="G30" t="n">
-        <v>80.56</v>
+        <v>79.55</v>
       </c>
       <c r="H30" t="n">
-        <v>68.06</v>
+        <v>72.73</v>
       </c>
       <c r="I30" t="n">
-        <v>12.5</v>
+        <v>6.82</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Muhammad Yousaf</t>
+          <t>Khalida Bibi</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>373690</v>
+        <v>373673</v>
       </c>
       <c r="C31" t="n">
-        <v>132</v>
+        <v>177</v>
       </c>
       <c r="D31" t="n">
-        <v>105</v>
+        <v>140</v>
       </c>
       <c r="E31" t="n">
-        <v>96</v>
+        <v>140</v>
       </c>
       <c r="F31" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="G31" t="n">
-        <v>79.55</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="H31" t="n">
-        <v>72.73</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="I31" t="n">
-        <v>6.82</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Khalida Bibi</t>
+          <t>Laiba Shams</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>373673</v>
+        <v>373706</v>
       </c>
       <c r="C32" t="n">
-        <v>177</v>
+        <v>212</v>
       </c>
       <c r="D32" t="n">
-        <v>140</v>
+        <v>166</v>
       </c>
       <c r="E32" t="n">
-        <v>140</v>
+        <v>126</v>
       </c>
       <c r="F32" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="G32" t="n">
-        <v>79.09999999999999</v>
+        <v>78.3</v>
       </c>
       <c r="H32" t="n">
-        <v>79.09999999999999</v>
+        <v>59.43</v>
       </c>
       <c r="I32" t="n">
-        <v>0</v>
+        <v>18.87</v>
       </c>
     </row>
     <row r="33">
@@ -2724,125 +2724,125 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Summiya Hayat</t>
+          <t>Shehla Noor</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>373710</v>
+        <v>373650</v>
       </c>
       <c r="C37" t="n">
-        <v>183</v>
+        <v>14</v>
       </c>
       <c r="D37" t="n">
-        <v>118</v>
+        <v>9</v>
       </c>
       <c r="E37" t="n">
-        <v>85</v>
+        <v>9</v>
       </c>
       <c r="F37" t="n">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="G37" t="n">
-        <v>64.48</v>
+        <v>64.29000000000001</v>
       </c>
       <c r="H37" t="n">
-        <v>46.45</v>
+        <v>64.29000000000001</v>
       </c>
       <c r="I37" t="n">
-        <v>18.03</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Shehla Noor</t>
+          <t>Furqan Ullah Khan</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>373650</v>
+        <v>373683</v>
       </c>
       <c r="C38" t="n">
-        <v>14</v>
+        <v>195</v>
       </c>
       <c r="D38" t="n">
-        <v>9</v>
+        <v>124</v>
       </c>
       <c r="E38" t="n">
-        <v>9</v>
+        <v>116</v>
       </c>
       <c r="F38" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="G38" t="n">
-        <v>64.29000000000001</v>
+        <v>63.59</v>
       </c>
       <c r="H38" t="n">
-        <v>64.29000000000001</v>
+        <v>59.49</v>
       </c>
       <c r="I38" t="n">
-        <v>0</v>
+        <v>4.1</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Furqan Ullah Khan</t>
+          <t>Usman Ali</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>373683</v>
+        <v>373687</v>
       </c>
       <c r="C39" t="n">
-        <v>195</v>
+        <v>8</v>
       </c>
       <c r="D39" t="n">
-        <v>124</v>
+        <v>5</v>
       </c>
       <c r="E39" t="n">
-        <v>116</v>
+        <v>5</v>
       </c>
       <c r="F39" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="G39" t="n">
-        <v>63.59</v>
+        <v>62.5</v>
       </c>
       <c r="H39" t="n">
-        <v>59.49</v>
+        <v>62.5</v>
       </c>
       <c r="I39" t="n">
-        <v>4.1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Usman Ali</t>
+          <t>Summiya Hayat</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>373687</v>
+        <v>373710</v>
       </c>
       <c r="C40" t="n">
-        <v>8</v>
+        <v>188</v>
       </c>
       <c r="D40" t="n">
-        <v>5</v>
+        <v>114</v>
       </c>
       <c r="E40" t="n">
-        <v>5</v>
+        <v>85</v>
       </c>
       <c r="F40" t="n">
-        <v>0</v>
+        <v>29</v>
       </c>
       <c r="G40" t="n">
-        <v>62.5</v>
+        <v>60.64</v>
       </c>
       <c r="H40" t="n">
-        <v>62.5</v>
+        <v>45.21</v>
       </c>
       <c r="I40" t="n">
-        <v>0</v>
+        <v>15.43</v>
       </c>
     </row>
     <row r="41">

</xml_diff>

<commit_message>
Refactor consent checks in girls.py and enhance duration validation in household.py; update error log and performance summary files
</commit_message>
<xml_diff>
--- a/Error_log/Enumerator_Performance.xlsx
+++ b/Error_log/Enumerator_Performance.xlsx
@@ -502,10 +502,10 @@
         <v>373646</v>
       </c>
       <c r="C4" t="n">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="D4" t="n">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="E4" t="n">
         <v>107</v>
@@ -552,39 +552,39 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Shazia begum</t>
+          <t>Irum Ikram</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>373696</v>
+        <v>373642</v>
       </c>
       <c r="C7" t="n">
-        <v>318</v>
+        <v>301</v>
       </c>
       <c r="D7" t="n">
         <v>238</v>
       </c>
       <c r="E7" t="n">
-        <v>80</v>
+        <v>63</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Irum Ikram</t>
+          <t>Shazia begum</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>373642</v>
+        <v>373696</v>
       </c>
       <c r="C8" t="n">
-        <v>301</v>
+        <v>317</v>
       </c>
       <c r="D8" t="n">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="E8" t="n">
-        <v>63</v>
+        <v>80</v>
       </c>
     </row>
     <row r="9">
@@ -597,10 +597,10 @@
         <v>373651</v>
       </c>
       <c r="C9" t="n">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="D9" t="n">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="E9" t="n">
         <v>142</v>
@@ -609,39 +609,39 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Mahnoor</t>
+          <t>Sadia Rustum</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>373705</v>
+        <v>373649</v>
       </c>
       <c r="C10" t="n">
-        <v>249</v>
+        <v>192</v>
       </c>
       <c r="D10" t="n">
-        <v>188</v>
+        <v>182</v>
       </c>
       <c r="E10" t="n">
-        <v>61</v>
+        <v>10</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Sadia Rustum</t>
+          <t>Mahnoor</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>373649</v>
+        <v>373705</v>
       </c>
       <c r="C11" t="n">
-        <v>192</v>
+        <v>231</v>
       </c>
       <c r="D11" t="n">
-        <v>182</v>
+        <v>170</v>
       </c>
       <c r="E11" t="n">
-        <v>10</v>
+        <v>61</v>
       </c>
     </row>
     <row r="12">
@@ -654,10 +654,10 @@
         <v>373716</v>
       </c>
       <c r="C12" t="n">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="D12" t="n">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="E12" t="n">
         <v>48</v>
@@ -704,39 +704,39 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Laiba Shams</t>
+          <t>Bushra Ayub</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>373706</v>
+        <v>373671</v>
       </c>
       <c r="C15" t="n">
-        <v>166</v>
+        <v>126</v>
       </c>
       <c r="D15" t="n">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="E15" t="n">
-        <v>40</v>
+        <v>4</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Bushra Ayub</t>
+          <t>Laiba Shams</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>373671</v>
+        <v>373706</v>
       </c>
       <c r="C16" t="n">
-        <v>126</v>
+        <v>159</v>
       </c>
       <c r="D16" t="n">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="E16" t="n">
-        <v>4</v>
+        <v>40</v>
       </c>
     </row>
     <row r="17">
@@ -787,10 +787,10 @@
         <v>373692</v>
       </c>
       <c r="C19" t="n">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="D19" t="n">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E19" t="n">
         <v>165</v>
@@ -825,10 +825,10 @@
         <v>373658</v>
       </c>
       <c r="C21" t="n">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="D21" t="n">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="E21" t="n">
         <v>177</v>
@@ -894,77 +894,77 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Summiya Hayat</t>
+          <t>Rehana Bibi</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>373710</v>
+        <v>373691</v>
       </c>
       <c r="C25" t="n">
-        <v>114</v>
+        <v>265</v>
       </c>
       <c r="D25" t="n">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="E25" t="n">
-        <v>29</v>
+        <v>181</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Rehana Bibi</t>
+          <t>Irum ikram</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>373691</v>
+        <v>541376</v>
       </c>
       <c r="C26" t="n">
-        <v>265</v>
+        <v>88</v>
       </c>
       <c r="D26" t="n">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E26" t="n">
-        <v>181</v>
+        <v>5</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Irum ikram</t>
+          <t>Lati Khan</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>541376</v>
+        <v>373665</v>
       </c>
       <c r="C27" t="n">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="D27" t="n">
         <v>83</v>
       </c>
       <c r="E27" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Lati Khan</t>
+          <t>Summiya Hayat</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>373665</v>
+        <v>373710</v>
       </c>
       <c r="C28" t="n">
-        <v>86</v>
+        <v>111</v>
       </c>
       <c r="D28" t="n">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E28" t="n">
-        <v>3</v>
+        <v>29</v>
       </c>
     </row>
     <row r="29">
@@ -1027,39 +1027,39 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Nadia bibi</t>
+          <t>Anum Gul</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>373669</v>
+        <v>373656</v>
       </c>
       <c r="C32" t="n">
-        <v>115</v>
+        <v>55</v>
       </c>
       <c r="D32" t="n">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="E32" t="n">
-        <v>58</v>
+        <v>4</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Anum Gul</t>
+          <t>Nadia bibi</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>373656</v>
+        <v>373669</v>
       </c>
       <c r="C33" t="n">
-        <v>55</v>
+        <v>108</v>
       </c>
       <c r="D33" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E33" t="n">
-        <v>4</v>
+        <v>58</v>
       </c>
     </row>
     <row r="34">
@@ -1804,19 +1804,19 @@
         <v>101</v>
       </c>
       <c r="D7" t="n">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="E7" t="n">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F7" t="n">
         <v>165</v>
       </c>
       <c r="G7" t="n">
-        <v>263.37</v>
+        <v>262.38</v>
       </c>
       <c r="H7" t="n">
-        <v>100</v>
+        <v>99.01000000000001</v>
       </c>
       <c r="I7" t="n">
         <v>163.37</v>
@@ -1866,19 +1866,19 @@
         <v>120</v>
       </c>
       <c r="D9" t="n">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="E9" t="n">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="F9" t="n">
         <v>177</v>
       </c>
       <c r="G9" t="n">
-        <v>230</v>
+        <v>228.33</v>
       </c>
       <c r="H9" t="n">
-        <v>82.5</v>
+        <v>80.83</v>
       </c>
       <c r="I9" t="n">
         <v>147.5</v>
@@ -1959,19 +1959,19 @@
         <v>231</v>
       </c>
       <c r="D12" t="n">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="E12" t="n">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="F12" t="n">
         <v>142</v>
       </c>
       <c r="G12" t="n">
-        <v>151.52</v>
+        <v>150.65</v>
       </c>
       <c r="H12" t="n">
-        <v>90.04000000000001</v>
+        <v>89.18000000000001</v>
       </c>
       <c r="I12" t="n">
         <v>61.47</v>
@@ -2083,19 +2083,19 @@
         <v>239</v>
       </c>
       <c r="D16" t="n">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="E16" t="n">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="F16" t="n">
         <v>80</v>
       </c>
       <c r="G16" t="n">
-        <v>133.05</v>
+        <v>132.64</v>
       </c>
       <c r="H16" t="n">
-        <v>99.58</v>
+        <v>99.16</v>
       </c>
       <c r="I16" t="n">
         <v>33.47</v>
@@ -2207,19 +2207,19 @@
         <v>324</v>
       </c>
       <c r="D20" t="n">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="E20" t="n">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F20" t="n">
         <v>107</v>
       </c>
       <c r="G20" t="n">
-        <v>120.68</v>
+        <v>120.37</v>
       </c>
       <c r="H20" t="n">
-        <v>87.65000000000001</v>
+        <v>87.34999999999999</v>
       </c>
       <c r="I20" t="n">
         <v>33.02</v>
@@ -2269,19 +2269,19 @@
         <v>169</v>
       </c>
       <c r="D22" t="n">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="E22" t="n">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="F22" t="n">
         <v>48</v>
       </c>
       <c r="G22" t="n">
-        <v>116.57</v>
+        <v>115.38</v>
       </c>
       <c r="H22" t="n">
-        <v>88.17</v>
+        <v>86.98</v>
       </c>
       <c r="I22" t="n">
         <v>28.4</v>
@@ -2300,19 +2300,19 @@
         <v>224</v>
       </c>
       <c r="D23" t="n">
-        <v>249</v>
+        <v>231</v>
       </c>
       <c r="E23" t="n">
-        <v>188</v>
+        <v>170</v>
       </c>
       <c r="F23" t="n">
         <v>61</v>
       </c>
       <c r="G23" t="n">
-        <v>111.16</v>
+        <v>103.12</v>
       </c>
       <c r="H23" t="n">
-        <v>83.93000000000001</v>
+        <v>75.89</v>
       </c>
       <c r="I23" t="n">
         <v>27.23</v>
@@ -2331,19 +2331,19 @@
         <v>111</v>
       </c>
       <c r="D24" t="n">
-        <v>115</v>
+        <v>108</v>
       </c>
       <c r="E24" t="n">
-        <v>57</v>
+        <v>50</v>
       </c>
       <c r="F24" t="n">
         <v>58</v>
       </c>
       <c r="G24" t="n">
-        <v>103.6</v>
+        <v>97.3</v>
       </c>
       <c r="H24" t="n">
-        <v>51.35</v>
+        <v>45.05</v>
       </c>
       <c r="I24" t="n">
         <v>52.25</v>
@@ -2569,63 +2569,63 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Laiba Shams</t>
+          <t>Asma Gull</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>373706</v>
+        <v>373672</v>
       </c>
       <c r="C32" t="n">
-        <v>212</v>
+        <v>144</v>
       </c>
       <c r="D32" t="n">
-        <v>166</v>
+        <v>109</v>
       </c>
       <c r="E32" t="n">
-        <v>126</v>
+        <v>105</v>
       </c>
       <c r="F32" t="n">
-        <v>40</v>
+        <v>4</v>
       </c>
       <c r="G32" t="n">
-        <v>78.3</v>
+        <v>75.69</v>
       </c>
       <c r="H32" t="n">
-        <v>59.43</v>
+        <v>72.92</v>
       </c>
       <c r="I32" t="n">
-        <v>18.87</v>
+        <v>2.78</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Asma Gull</t>
+          <t>Laiba Shams</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>373672</v>
+        <v>373706</v>
       </c>
       <c r="C33" t="n">
-        <v>144</v>
+        <v>212</v>
       </c>
       <c r="D33" t="n">
-        <v>109</v>
+        <v>159</v>
       </c>
       <c r="E33" t="n">
-        <v>105</v>
+        <v>119</v>
       </c>
       <c r="F33" t="n">
-        <v>4</v>
+        <v>40</v>
       </c>
       <c r="G33" t="n">
-        <v>75.69</v>
+        <v>75</v>
       </c>
       <c r="H33" t="n">
-        <v>72.92</v>
+        <v>56.13</v>
       </c>
       <c r="I33" t="n">
-        <v>2.78</v>
+        <v>18.87</v>
       </c>
     </row>
     <row r="34">
@@ -2817,63 +2817,63 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Summiya Hayat</t>
+          <t>Ishaq Khan</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>373710</v>
+        <v>373699</v>
       </c>
       <c r="C40" t="n">
-        <v>188</v>
+        <v>170</v>
       </c>
       <c r="D40" t="n">
-        <v>114</v>
+        <v>101</v>
       </c>
       <c r="E40" t="n">
-        <v>85</v>
+        <v>100</v>
       </c>
       <c r="F40" t="n">
-        <v>29</v>
+        <v>1</v>
       </c>
       <c r="G40" t="n">
-        <v>60.64</v>
+        <v>59.41</v>
       </c>
       <c r="H40" t="n">
-        <v>45.21</v>
+        <v>58.82</v>
       </c>
       <c r="I40" t="n">
-        <v>15.43</v>
+        <v>0.59</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Ishaq Khan</t>
+          <t>Summiya Hayat</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>373699</v>
+        <v>373710</v>
       </c>
       <c r="C41" t="n">
-        <v>170</v>
+        <v>188</v>
       </c>
       <c r="D41" t="n">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="E41" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="F41" t="n">
-        <v>1</v>
+        <v>29</v>
       </c>
       <c r="G41" t="n">
-        <v>59.41</v>
+        <v>59.04</v>
       </c>
       <c r="H41" t="n">
-        <v>58.82</v>
+        <v>43.62</v>
       </c>
       <c r="I41" t="n">
-        <v>0.59</v>
+        <v>15.43</v>
       </c>
     </row>
     <row r="42">

</xml_diff>

<commit_message>
Update survey data, quality logs, and session analysis documents
</commit_message>
<xml_diff>
--- a/Error_log/Enumerator_Performance.xlsx
+++ b/Error_log/Enumerator_Performance.xlsx
@@ -464,13 +464,13 @@
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="n">
-        <v>1526</v>
+        <v>1441</v>
       </c>
       <c r="D2" t="n">
-        <v>1487</v>
+        <v>1400</v>
       </c>
       <c r="E2" t="n">
-        <v>39</v>
+        <v>41</v>
       </c>
     </row>
     <row r="3">
@@ -483,13 +483,13 @@
         <v>373641</v>
       </c>
       <c r="C3" t="n">
-        <v>495</v>
+        <v>519</v>
       </c>
       <c r="D3" t="n">
-        <v>395</v>
+        <v>412</v>
       </c>
       <c r="E3" t="n">
-        <v>100</v>
+        <v>107</v>
       </c>
     </row>
     <row r="4">
@@ -502,13 +502,13 @@
         <v>373646</v>
       </c>
       <c r="C4" t="n">
-        <v>390</v>
+        <v>411</v>
       </c>
       <c r="D4" t="n">
-        <v>283</v>
+        <v>290</v>
       </c>
       <c r="E4" t="n">
-        <v>107</v>
+        <v>121</v>
       </c>
     </row>
     <row r="5">
@@ -521,13 +521,13 @@
         <v>373648</v>
       </c>
       <c r="C5" t="n">
-        <v>365</v>
+        <v>384</v>
       </c>
       <c r="D5" t="n">
-        <v>277</v>
+        <v>287</v>
       </c>
       <c r="E5" t="n">
-        <v>88</v>
+        <v>97</v>
       </c>
     </row>
     <row r="6">
@@ -559,13 +559,13 @@
         <v>373642</v>
       </c>
       <c r="C7" t="n">
-        <v>301</v>
+        <v>310</v>
       </c>
       <c r="D7" t="n">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="E7" t="n">
-        <v>63</v>
+        <v>70</v>
       </c>
     </row>
     <row r="8">
@@ -597,13 +597,13 @@
         <v>373651</v>
       </c>
       <c r="C9" t="n">
-        <v>348</v>
+        <v>360</v>
       </c>
       <c r="D9" t="n">
-        <v>206</v>
+        <v>213</v>
       </c>
       <c r="E9" t="n">
-        <v>142</v>
+        <v>147</v>
       </c>
     </row>
     <row r="10">
@@ -635,13 +635,13 @@
         <v>373705</v>
       </c>
       <c r="C11" t="n">
-        <v>231</v>
+        <v>237</v>
       </c>
       <c r="D11" t="n">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="E11" t="n">
-        <v>61</v>
+        <v>66</v>
       </c>
     </row>
     <row r="12">
@@ -654,13 +654,13 @@
         <v>373716</v>
       </c>
       <c r="C12" t="n">
-        <v>195</v>
+        <v>201</v>
       </c>
       <c r="D12" t="n">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="E12" t="n">
-        <v>48</v>
+        <v>51</v>
       </c>
     </row>
     <row r="13">
@@ -704,39 +704,39 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Bushra Ayub</t>
+          <t>Laiba Shams</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>373671</v>
+        <v>373706</v>
       </c>
       <c r="C15" t="n">
-        <v>126</v>
+        <v>169</v>
       </c>
       <c r="D15" t="n">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="E15" t="n">
-        <v>4</v>
+        <v>46</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Laiba Shams</t>
+          <t>Bushra Ayub</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>373706</v>
+        <v>373671</v>
       </c>
       <c r="C16" t="n">
-        <v>159</v>
+        <v>126</v>
       </c>
       <c r="D16" t="n">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="E16" t="n">
-        <v>40</v>
+        <v>4</v>
       </c>
     </row>
     <row r="17">
@@ -958,13 +958,13 @@
         <v>373710</v>
       </c>
       <c r="C28" t="n">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="D28" t="n">
         <v>82</v>
       </c>
       <c r="E28" t="n">
-        <v>29</v>
+        <v>32</v>
       </c>
     </row>
     <row r="29">
@@ -1103,58 +1103,58 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Alia Khan</t>
+          <t>aisha.aman</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>373681</v>
+        <v>752327</v>
       </c>
       <c r="C36" t="n">
-        <v>44</v>
+        <v>75</v>
       </c>
       <c r="D36" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E36" t="n">
-        <v>4</v>
+        <v>33</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Lati khan</t>
+          <t>Alia Khan</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>671211</v>
+        <v>373681</v>
       </c>
       <c r="C37" t="n">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="D37" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="E37" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>aisha.aman</t>
+          <t>Lati khan</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>752327</v>
+        <v>671211</v>
       </c>
       <c r="C38" t="n">
-        <v>59</v>
+        <v>38</v>
       </c>
       <c r="D38" t="n">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="E38" t="n">
-        <v>26</v>
+        <v>0</v>
       </c>
     </row>
     <row r="39">
@@ -1887,125 +1887,125 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>aisha.aman</t>
+          <t>Asma Bibi</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>752327</v>
+        <v>373641</v>
       </c>
       <c r="C10" t="n">
-        <v>36</v>
+        <v>326</v>
       </c>
       <c r="D10" t="n">
-        <v>59</v>
+        <v>519</v>
       </c>
       <c r="E10" t="n">
-        <v>33</v>
+        <v>412</v>
       </c>
       <c r="F10" t="n">
-        <v>26</v>
+        <v>107</v>
       </c>
       <c r="G10" t="n">
-        <v>163.89</v>
+        <v>159.2</v>
       </c>
       <c r="H10" t="n">
-        <v>91.67</v>
+        <v>126.38</v>
       </c>
       <c r="I10" t="n">
-        <v>72.22</v>
+        <v>32.82</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Asma Bibi</t>
+          <t>aisha.aman</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>373641</v>
+        <v>752327</v>
       </c>
       <c r="C11" t="n">
-        <v>304</v>
+        <v>51</v>
       </c>
       <c r="D11" t="n">
-        <v>495</v>
+        <v>75</v>
       </c>
       <c r="E11" t="n">
-        <v>395</v>
+        <v>42</v>
       </c>
       <c r="F11" t="n">
-        <v>100</v>
+        <v>33</v>
       </c>
       <c r="G11" t="n">
-        <v>162.83</v>
+        <v>147.06</v>
       </c>
       <c r="H11" t="n">
-        <v>129.93</v>
+        <v>82.34999999999999</v>
       </c>
       <c r="I11" t="n">
-        <v>32.89</v>
+        <v>64.70999999999999</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Javairia</t>
+          <t>Mehran Khan</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>373651</v>
+        <v>373684</v>
       </c>
       <c r="C12" t="n">
-        <v>231</v>
+        <v>200</v>
       </c>
       <c r="D12" t="n">
-        <v>348</v>
+        <v>293</v>
       </c>
       <c r="E12" t="n">
-        <v>206</v>
+        <v>265</v>
       </c>
       <c r="F12" t="n">
-        <v>142</v>
+        <v>28</v>
       </c>
       <c r="G12" t="n">
-        <v>150.65</v>
+        <v>146.5</v>
       </c>
       <c r="H12" t="n">
-        <v>89.18000000000001</v>
+        <v>132.5</v>
       </c>
       <c r="I12" t="n">
-        <v>61.47</v>
+        <v>14</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Mehran Khan</t>
+          <t>Javairia</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>373684</v>
+        <v>373651</v>
       </c>
       <c r="C13" t="n">
-        <v>200</v>
+        <v>247</v>
       </c>
       <c r="D13" t="n">
-        <v>293</v>
+        <v>360</v>
       </c>
       <c r="E13" t="n">
-        <v>265</v>
+        <v>213</v>
       </c>
       <c r="F13" t="n">
-        <v>28</v>
+        <v>147</v>
       </c>
       <c r="G13" t="n">
-        <v>146.5</v>
+        <v>145.75</v>
       </c>
       <c r="H13" t="n">
-        <v>132.5</v>
+        <v>86.23</v>
       </c>
       <c r="I13" t="n">
-        <v>14</v>
+        <v>59.51</v>
       </c>
     </row>
     <row r="14">
@@ -2142,25 +2142,25 @@
         <v>373642</v>
       </c>
       <c r="C18" t="n">
-        <v>239</v>
+        <v>250</v>
       </c>
       <c r="D18" t="n">
-        <v>301</v>
+        <v>310</v>
       </c>
       <c r="E18" t="n">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="F18" t="n">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="G18" t="n">
-        <v>125.94</v>
+        <v>124</v>
       </c>
       <c r="H18" t="n">
-        <v>99.58</v>
+        <v>96</v>
       </c>
       <c r="I18" t="n">
-        <v>26.36</v>
+        <v>28</v>
       </c>
     </row>
     <row r="19">
@@ -2204,25 +2204,25 @@
         <v>373646</v>
       </c>
       <c r="C20" t="n">
-        <v>324</v>
+        <v>348</v>
       </c>
       <c r="D20" t="n">
-        <v>390</v>
+        <v>411</v>
       </c>
       <c r="E20" t="n">
-        <v>283</v>
+        <v>290</v>
       </c>
       <c r="F20" t="n">
-        <v>107</v>
+        <v>121</v>
       </c>
       <c r="G20" t="n">
-        <v>120.37</v>
+        <v>118.1</v>
       </c>
       <c r="H20" t="n">
-        <v>87.34999999999999</v>
+        <v>83.33</v>
       </c>
       <c r="I20" t="n">
-        <v>33.02</v>
+        <v>34.77</v>
       </c>
     </row>
     <row r="21">
@@ -2235,25 +2235,25 @@
         <v>373648</v>
       </c>
       <c r="C21" t="n">
-        <v>309</v>
+        <v>335</v>
       </c>
       <c r="D21" t="n">
-        <v>365</v>
+        <v>384</v>
       </c>
       <c r="E21" t="n">
-        <v>277</v>
+        <v>287</v>
       </c>
       <c r="F21" t="n">
-        <v>88</v>
+        <v>97</v>
       </c>
       <c r="G21" t="n">
-        <v>118.12</v>
+        <v>114.63</v>
       </c>
       <c r="H21" t="n">
-        <v>89.64</v>
+        <v>85.67</v>
       </c>
       <c r="I21" t="n">
-        <v>28.48</v>
+        <v>28.96</v>
       </c>
     </row>
     <row r="22">
@@ -2266,25 +2266,25 @@
         <v>373716</v>
       </c>
       <c r="C22" t="n">
-        <v>169</v>
+        <v>183</v>
       </c>
       <c r="D22" t="n">
-        <v>195</v>
+        <v>201</v>
       </c>
       <c r="E22" t="n">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="F22" t="n">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="G22" t="n">
-        <v>115.38</v>
+        <v>109.84</v>
       </c>
       <c r="H22" t="n">
-        <v>86.98</v>
+        <v>81.97</v>
       </c>
       <c r="I22" t="n">
-        <v>28.4</v>
+        <v>27.87</v>
       </c>
     </row>
     <row r="23">
@@ -2297,25 +2297,25 @@
         <v>373705</v>
       </c>
       <c r="C23" t="n">
-        <v>224</v>
+        <v>241</v>
       </c>
       <c r="D23" t="n">
-        <v>231</v>
+        <v>237</v>
       </c>
       <c r="E23" t="n">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F23" t="n">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="G23" t="n">
-        <v>103.12</v>
+        <v>98.34</v>
       </c>
       <c r="H23" t="n">
-        <v>75.89</v>
+        <v>70.95</v>
       </c>
       <c r="I23" t="n">
-        <v>27.23</v>
+        <v>27.39</v>
       </c>
     </row>
     <row r="24">
@@ -2600,63 +2600,63 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Laiba Shams</t>
+          <t>Rahila Naaz</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>373706</v>
+        <v>373715</v>
       </c>
       <c r="C33" t="n">
-        <v>212</v>
+        <v>4</v>
       </c>
       <c r="D33" t="n">
-        <v>159</v>
+        <v>3</v>
       </c>
       <c r="E33" t="n">
-        <v>119</v>
+        <v>2</v>
       </c>
       <c r="F33" t="n">
-        <v>40</v>
+        <v>1</v>
       </c>
       <c r="G33" t="n">
         <v>75</v>
       </c>
       <c r="H33" t="n">
-        <v>56.13</v>
+        <v>50</v>
       </c>
       <c r="I33" t="n">
-        <v>18.87</v>
+        <v>25</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Rahila Naaz</t>
+          <t>Laiba Shams</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>373715</v>
+        <v>373706</v>
       </c>
       <c r="C34" t="n">
-        <v>4</v>
+        <v>229</v>
       </c>
       <c r="D34" t="n">
-        <v>3</v>
+        <v>169</v>
       </c>
       <c r="E34" t="n">
-        <v>2</v>
+        <v>123</v>
       </c>
       <c r="F34" t="n">
-        <v>1</v>
+        <v>46</v>
       </c>
       <c r="G34" t="n">
-        <v>75</v>
+        <v>73.8</v>
       </c>
       <c r="H34" t="n">
-        <v>50</v>
+        <v>53.71</v>
       </c>
       <c r="I34" t="n">
-        <v>25</v>
+        <v>20.09</v>
       </c>
     </row>
     <row r="35">
@@ -2855,25 +2855,25 @@
         <v>373710</v>
       </c>
       <c r="C41" t="n">
-        <v>188</v>
+        <v>202</v>
       </c>
       <c r="D41" t="n">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="E41" t="n">
         <v>82</v>
       </c>
       <c r="F41" t="n">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="G41" t="n">
-        <v>59.04</v>
+        <v>56.44</v>
       </c>
       <c r="H41" t="n">
-        <v>43.62</v>
+        <v>40.59</v>
       </c>
       <c r="I41" t="n">
-        <v>15.43</v>
+        <v>15.84</v>
       </c>
     </row>
     <row r="42">

</xml_diff>

<commit_message>
Remove guidance for GPS out of district from household and girls interviews
</commit_message>
<xml_diff>
--- a/Error_log/Enumerator_Performance.xlsx
+++ b/Error_log/Enumerator_Performance.xlsx
@@ -483,108 +483,108 @@
         <v>373641</v>
       </c>
       <c r="C3" t="n">
-        <v>549</v>
+        <v>546</v>
       </c>
       <c r="D3" t="n">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="E3" t="n">
-        <v>116</v>
+        <v>112</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Shafaq Zahra</t>
+          <t>Shazia Bibi</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>373646</v>
+        <v>373648</v>
       </c>
       <c r="C4" t="n">
-        <v>449</v>
+        <v>402</v>
       </c>
       <c r="D4" t="n">
-        <v>306</v>
+        <v>343</v>
       </c>
       <c r="E4" t="n">
-        <v>143</v>
+        <v>59</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Shazia Bibi</t>
+          <t>Shafaq Zahra</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>373648</v>
+        <v>373646</v>
       </c>
       <c r="C5" t="n">
-        <v>402</v>
+        <v>449</v>
       </c>
       <c r="D5" t="n">
-        <v>301</v>
+        <v>342</v>
       </c>
       <c r="E5" t="n">
-        <v>101</v>
+        <v>107</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Mehran Khan</t>
+          <t>Irum Ikram</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>373684</v>
+        <v>373642</v>
       </c>
       <c r="C6" t="n">
-        <v>293</v>
+        <v>332</v>
       </c>
       <c r="D6" t="n">
-        <v>265</v>
+        <v>276</v>
       </c>
       <c r="E6" t="n">
-        <v>28</v>
+        <v>56</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Irum Ikram</t>
+          <t>Shazia begum</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>373642</v>
+        <v>373696</v>
       </c>
       <c r="C7" t="n">
-        <v>332</v>
+        <v>317</v>
       </c>
       <c r="D7" t="n">
-        <v>247</v>
+        <v>274</v>
       </c>
       <c r="E7" t="n">
-        <v>85</v>
+        <v>43</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Shazia begum</t>
+          <t>Mehran Khan</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>373696</v>
+        <v>373684</v>
       </c>
       <c r="C8" t="n">
-        <v>317</v>
+        <v>293</v>
       </c>
       <c r="D8" t="n">
-        <v>237</v>
+        <v>265</v>
       </c>
       <c r="E8" t="n">
-        <v>80</v>
+        <v>28</v>
       </c>
     </row>
     <row r="9">
@@ -600,29 +600,29 @@
         <v>386</v>
       </c>
       <c r="D9" t="n">
-        <v>232</v>
+        <v>253</v>
       </c>
       <c r="E9" t="n">
-        <v>154</v>
+        <v>133</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Sadia Rustum</t>
+          <t>Kainat</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>373649</v>
+        <v>373712</v>
       </c>
       <c r="C10" t="n">
-        <v>192</v>
+        <v>308</v>
       </c>
       <c r="D10" t="n">
-        <v>182</v>
+        <v>207</v>
       </c>
       <c r="E10" t="n">
-        <v>10</v>
+        <v>101</v>
       </c>
     </row>
     <row r="11">
@@ -635,298 +635,298 @@
         <v>373705</v>
       </c>
       <c r="C11" t="n">
-        <v>255</v>
+        <v>246</v>
       </c>
       <c r="D11" t="n">
-        <v>181</v>
+        <v>200</v>
       </c>
       <c r="E11" t="n">
-        <v>74</v>
+        <v>46</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Naureen Khan</t>
+          <t>Sadia Rustum</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>373716</v>
+        <v>373649</v>
       </c>
       <c r="C12" t="n">
-        <v>202</v>
+        <v>192</v>
       </c>
       <c r="D12" t="n">
-        <v>150</v>
+        <v>182</v>
       </c>
       <c r="E12" t="n">
-        <v>52</v>
+        <v>10</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Khalida Bibi</t>
+          <t>Samara</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>373673</v>
+        <v>373658</v>
       </c>
       <c r="C13" t="n">
-        <v>140</v>
+        <v>274</v>
       </c>
       <c r="D13" t="n">
-        <v>140</v>
+        <v>179</v>
       </c>
       <c r="E13" t="n">
-        <v>0</v>
+        <v>95</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Laiba Shams</t>
+          <t>Naureen Khan</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>373706</v>
+        <v>373716</v>
       </c>
       <c r="C14" t="n">
-        <v>184</v>
+        <v>202</v>
       </c>
       <c r="D14" t="n">
-        <v>135</v>
+        <v>173</v>
       </c>
       <c r="E14" t="n">
-        <v>49</v>
+        <v>29</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Kainat</t>
+          <t>Laiba Shams</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>373712</v>
+        <v>373706</v>
       </c>
       <c r="C15" t="n">
-        <v>308</v>
+        <v>174</v>
       </c>
       <c r="D15" t="n">
-        <v>126</v>
+        <v>144</v>
       </c>
       <c r="E15" t="n">
-        <v>182</v>
+        <v>30</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Bushra Ayub</t>
+          <t>Khalida Bibi</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>373671</v>
+        <v>373673</v>
       </c>
       <c r="C16" t="n">
-        <v>126</v>
+        <v>140</v>
       </c>
       <c r="D16" t="n">
-        <v>122</v>
+        <v>140</v>
       </c>
       <c r="E16" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Furqan Ullah Khan</t>
+          <t>Rehana Bibi</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>373683</v>
+        <v>373691</v>
       </c>
       <c r="C17" t="n">
-        <v>124</v>
+        <v>265</v>
       </c>
       <c r="D17" t="n">
-        <v>116</v>
+        <v>139</v>
       </c>
       <c r="E17" t="n">
-        <v>8</v>
+        <v>126</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Asma Gull</t>
+          <t>Zohra</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>373672</v>
+        <v>373692</v>
       </c>
       <c r="C18" t="n">
-        <v>109</v>
+        <v>257</v>
       </c>
       <c r="D18" t="n">
-        <v>105</v>
+        <v>126</v>
       </c>
       <c r="E18" t="n">
-        <v>4</v>
+        <v>131</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Zohra</t>
+          <t>Bushra Ayub</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>373692</v>
+        <v>373671</v>
       </c>
       <c r="C19" t="n">
-        <v>265</v>
+        <v>126</v>
       </c>
       <c r="D19" t="n">
-        <v>100</v>
+        <v>122</v>
       </c>
       <c r="E19" t="n">
-        <v>165</v>
+        <v>4</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Ishaq Khan</t>
+          <t>Furqan Ullah Khan</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>373699</v>
+        <v>373683</v>
       </c>
       <c r="C20" t="n">
-        <v>101</v>
+        <v>124</v>
       </c>
       <c r="D20" t="n">
-        <v>100</v>
+        <v>116</v>
       </c>
       <c r="E20" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Samara</t>
+          <t>Asma Gull</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>373658</v>
+        <v>373672</v>
       </c>
       <c r="C21" t="n">
-        <v>274</v>
+        <v>109</v>
       </c>
       <c r="D21" t="n">
-        <v>97</v>
+        <v>105</v>
       </c>
       <c r="E21" t="n">
-        <v>177</v>
+        <v>4</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Muhammad Yousaf</t>
+          <t>Ishaq Khan</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>373690</v>
+        <v>373699</v>
       </c>
       <c r="C22" t="n">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="D22" t="n">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="E22" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Lati Khan</t>
+          <t>Muhammad Yousaf</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>564273</v>
+        <v>373690</v>
       </c>
       <c r="C23" t="n">
-        <v>97</v>
+        <v>105</v>
       </c>
       <c r="D23" t="n">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="E23" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Naureen khan</t>
+          <t>Lati Khan</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>453925</v>
+        <v>564273</v>
       </c>
       <c r="C24" t="n">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="D24" t="n">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="E24" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Summiya Hayat</t>
+          <t>Naureen khan</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>373710</v>
+        <v>453925</v>
       </c>
       <c r="C25" t="n">
-        <v>121</v>
+        <v>91</v>
       </c>
       <c r="D25" t="n">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="E25" t="n">
-        <v>34</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Rehana Bibi</t>
+          <t>Summiya Hayat</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>373691</v>
+        <v>373710</v>
       </c>
       <c r="C26" t="n">
-        <v>265</v>
+        <v>116</v>
       </c>
       <c r="D26" t="n">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="E26" t="n">
-        <v>181</v>
+        <v>30</v>
       </c>
     </row>
     <row r="27">
@@ -1008,77 +1008,77 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>aisha.aman</t>
+          <t>Nadia bibi</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>752327</v>
+        <v>373669</v>
       </c>
       <c r="C31" t="n">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D31" t="n">
-        <v>64</v>
+        <v>73</v>
       </c>
       <c r="E31" t="n">
-        <v>45</v>
+        <v>35</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Nillum Bibi</t>
+          <t>aisha.aman</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>373652</v>
+        <v>752327</v>
       </c>
       <c r="C32" t="n">
-        <v>64</v>
+        <v>109</v>
       </c>
       <c r="D32" t="n">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="E32" t="n">
-        <v>3</v>
+        <v>42</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Anum Gul</t>
+          <t>Nillum Bibi</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>373656</v>
+        <v>373652</v>
       </c>
       <c r="C33" t="n">
-        <v>55</v>
+        <v>64</v>
       </c>
       <c r="D33" t="n">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="E33" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Nadia bibi</t>
+          <t>Anum Gul</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>373669</v>
+        <v>373656</v>
       </c>
       <c r="C34" t="n">
-        <v>108</v>
+        <v>55</v>
       </c>
       <c r="D34" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E34" t="n">
-        <v>58</v>
+        <v>4</v>
       </c>
     </row>
     <row r="35">
@@ -1312,17 +1312,17 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Summiya Hayat 123</t>
+          <t>Sadia rustum</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>51020</v>
+        <v>852541</v>
       </c>
       <c r="C47" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D47" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E47" t="n">
         <v>0</v>
@@ -1331,11 +1331,11 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Sadia rustum</t>
+          <t>Usman Ali</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>852541</v>
+        <v>373687</v>
       </c>
       <c r="C48" t="n">
         <v>5</v>
@@ -1350,49 +1350,49 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Usman Ali</t>
+          <t>Muhammad Noor</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>373687</v>
+        <v>373701</v>
       </c>
       <c r="C49" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D49" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E49" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Muhammad Noor</t>
+          <t>Muhammad Naeem</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>373701</v>
+        <v>373694</v>
       </c>
       <c r="C50" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D50" t="n">
         <v>3</v>
       </c>
       <c r="E50" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Muhammad Naeem</t>
+          <t>Muhammad Shahid Khan</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>373694</v>
+        <v>373662</v>
       </c>
       <c r="C51" t="n">
         <v>3</v>
@@ -1407,11 +1407,11 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Muhammad Shahid Khan</t>
+          <t>Sajjad Khan</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>373662</v>
+        <v>373700</v>
       </c>
       <c r="C52" t="n">
         <v>3</v>
@@ -1426,30 +1426,30 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Sajjad Khan</t>
+          <t>Aisha Aman</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>373700</v>
+        <v>373704</v>
       </c>
       <c r="C53" t="n">
         <v>3</v>
       </c>
       <c r="D53" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E53" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Aisha Aman</t>
+          <t>Rahila Naaz</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>373704</v>
+        <v>373715</v>
       </c>
       <c r="C54" t="n">
         <v>3</v>
@@ -1464,11 +1464,11 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Rahila Naaz</t>
+          <t>Robina Shaheen</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>373715</v>
+        <v>373639</v>
       </c>
       <c r="C55" t="n">
         <v>3</v>
@@ -1483,68 +1483,68 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Robina Shaheen</t>
+          <t>Iqra Bibi</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>373639</v>
+        <v>373708</v>
       </c>
       <c r="C56" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D56" t="n">
         <v>2</v>
       </c>
       <c r="E56" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Iqra Bibi</t>
+          <t>Mahnoorr</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>373708</v>
+        <v>373670</v>
       </c>
       <c r="C57" t="n">
         <v>2</v>
       </c>
       <c r="D57" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E57" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Mahnoorr</t>
+          <t>Gul Rukh</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>373670</v>
+        <v>373644</v>
       </c>
       <c r="C58" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D58" t="n">
         <v>1</v>
       </c>
       <c r="E58" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Gul Rukh</t>
+          <t>Hijab Zahra</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>373644</v>
+        <v>373637</v>
       </c>
       <c r="C59" t="n">
         <v>1</v>
@@ -1559,11 +1559,11 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Hijab Zahra</t>
+          <t>Sidra Khan</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>373637</v>
+        <v>373645</v>
       </c>
       <c r="C60" t="n">
         <v>1</v>
@@ -1578,11 +1578,11 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Sidra Khan</t>
+          <t>Summiya Hayat 123</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>373645</v>
+        <v>51020</v>
       </c>
       <c r="C61" t="n">
         <v>1</v>
@@ -1671,19 +1671,19 @@
         <v>91</v>
       </c>
       <c r="E2" t="n">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="F2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G2" t="n">
         <v>4550</v>
       </c>
       <c r="H2" t="n">
-        <v>4450</v>
+        <v>4550</v>
       </c>
       <c r="I2" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -1795,19 +1795,19 @@
         <v>308</v>
       </c>
       <c r="E6" t="n">
-        <v>126</v>
+        <v>207</v>
       </c>
       <c r="F6" t="n">
-        <v>182</v>
+        <v>101</v>
       </c>
       <c r="G6" t="n">
         <v>296.15</v>
       </c>
       <c r="H6" t="n">
-        <v>121.15</v>
+        <v>199.04</v>
       </c>
       <c r="I6" t="n">
-        <v>175</v>
+        <v>97.12</v>
       </c>
     </row>
     <row r="7">
@@ -1823,22 +1823,22 @@
         <v>101</v>
       </c>
       <c r="D7" t="n">
-        <v>265</v>
+        <v>257</v>
       </c>
       <c r="E7" t="n">
-        <v>100</v>
+        <v>126</v>
       </c>
       <c r="F7" t="n">
-        <v>165</v>
+        <v>131</v>
       </c>
       <c r="G7" t="n">
-        <v>262.38</v>
+        <v>254.46</v>
       </c>
       <c r="H7" t="n">
-        <v>99.01000000000001</v>
+        <v>124.75</v>
       </c>
       <c r="I7" t="n">
-        <v>163.37</v>
+        <v>129.7</v>
       </c>
     </row>
     <row r="8">
@@ -1857,19 +1857,19 @@
         <v>265</v>
       </c>
       <c r="E8" t="n">
-        <v>84</v>
+        <v>139</v>
       </c>
       <c r="F8" t="n">
-        <v>181</v>
+        <v>126</v>
       </c>
       <c r="G8" t="n">
         <v>238.74</v>
       </c>
       <c r="H8" t="n">
-        <v>75.68000000000001</v>
+        <v>125.23</v>
       </c>
       <c r="I8" t="n">
-        <v>163.06</v>
+        <v>113.51</v>
       </c>
     </row>
     <row r="9">
@@ -1888,19 +1888,19 @@
         <v>274</v>
       </c>
       <c r="E9" t="n">
-        <v>97</v>
+        <v>179</v>
       </c>
       <c r="F9" t="n">
-        <v>177</v>
+        <v>95</v>
       </c>
       <c r="G9" t="n">
         <v>228.33</v>
       </c>
       <c r="H9" t="n">
-        <v>80.83</v>
+        <v>149.17</v>
       </c>
       <c r="I9" t="n">
-        <v>147.5</v>
+        <v>79.17</v>
       </c>
     </row>
     <row r="10">
@@ -1916,22 +1916,22 @@
         <v>359</v>
       </c>
       <c r="D10" t="n">
-        <v>549</v>
+        <v>546</v>
       </c>
       <c r="E10" t="n">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="F10" t="n">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="G10" t="n">
-        <v>152.92</v>
+        <v>152.09</v>
       </c>
       <c r="H10" t="n">
-        <v>120.61</v>
+        <v>120.89</v>
       </c>
       <c r="I10" t="n">
-        <v>32.31</v>
+        <v>31.2</v>
       </c>
     </row>
     <row r="11">
@@ -2043,19 +2043,19 @@
         <v>386</v>
       </c>
       <c r="E14" t="n">
-        <v>232</v>
+        <v>253</v>
       </c>
       <c r="F14" t="n">
-        <v>154</v>
+        <v>133</v>
       </c>
       <c r="G14" t="n">
         <v>137.86</v>
       </c>
       <c r="H14" t="n">
-        <v>82.86</v>
+        <v>90.36</v>
       </c>
       <c r="I14" t="n">
-        <v>55</v>
+        <v>47.5</v>
       </c>
     </row>
     <row r="15">
@@ -2074,19 +2074,19 @@
         <v>317</v>
       </c>
       <c r="E15" t="n">
-        <v>237</v>
+        <v>274</v>
       </c>
       <c r="F15" t="n">
-        <v>80</v>
+        <v>43</v>
       </c>
       <c r="G15" t="n">
         <v>132.64</v>
       </c>
       <c r="H15" t="n">
-        <v>99.16</v>
+        <v>114.64</v>
       </c>
       <c r="I15" t="n">
-        <v>33.47</v>
+        <v>17.99</v>
       </c>
     </row>
     <row r="16">
@@ -2136,19 +2136,19 @@
         <v>332</v>
       </c>
       <c r="E17" t="n">
-        <v>247</v>
+        <v>276</v>
       </c>
       <c r="F17" t="n">
-        <v>85</v>
+        <v>56</v>
       </c>
       <c r="G17" t="n">
         <v>122.06</v>
       </c>
       <c r="H17" t="n">
-        <v>90.81</v>
+        <v>101.47</v>
       </c>
       <c r="I17" t="n">
-        <v>31.25</v>
+        <v>20.59</v>
       </c>
     </row>
     <row r="18">
@@ -2185,156 +2185,156 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Summiya Hayat 123</t>
+          <t>Shafaq Zahra</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>51020</v>
+        <v>373646</v>
       </c>
       <c r="C19" t="n">
-        <v>5</v>
+        <v>381</v>
       </c>
       <c r="D19" t="n">
-        <v>6</v>
+        <v>449</v>
       </c>
       <c r="E19" t="n">
-        <v>6</v>
+        <v>342</v>
       </c>
       <c r="F19" t="n">
-        <v>0</v>
+        <v>107</v>
       </c>
       <c r="G19" t="n">
-        <v>120</v>
+        <v>117.85</v>
       </c>
       <c r="H19" t="n">
-        <v>120</v>
+        <v>89.76000000000001</v>
       </c>
       <c r="I19" t="n">
-        <v>0</v>
+        <v>28.08</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Shafaq Zahra</t>
+          <t>aisha.aman</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>373646</v>
+        <v>752327</v>
       </c>
       <c r="C20" t="n">
-        <v>381</v>
+        <v>94</v>
       </c>
       <c r="D20" t="n">
-        <v>449</v>
+        <v>109</v>
       </c>
       <c r="E20" t="n">
-        <v>306</v>
+        <v>67</v>
       </c>
       <c r="F20" t="n">
-        <v>143</v>
+        <v>42</v>
       </c>
       <c r="G20" t="n">
-        <v>117.85</v>
+        <v>115.96</v>
       </c>
       <c r="H20" t="n">
-        <v>80.31</v>
+        <v>71.28</v>
       </c>
       <c r="I20" t="n">
-        <v>37.53</v>
+        <v>44.68</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>aisha.aman</t>
+          <t>Shazia Bibi</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>752327</v>
+        <v>373648</v>
       </c>
       <c r="C21" t="n">
-        <v>94</v>
+        <v>363</v>
       </c>
       <c r="D21" t="n">
-        <v>109</v>
+        <v>402</v>
       </c>
       <c r="E21" t="n">
-        <v>64</v>
+        <v>343</v>
       </c>
       <c r="F21" t="n">
-        <v>45</v>
+        <v>59</v>
       </c>
       <c r="G21" t="n">
-        <v>115.96</v>
+        <v>110.74</v>
       </c>
       <c r="H21" t="n">
-        <v>68.09</v>
+        <v>94.48999999999999</v>
       </c>
       <c r="I21" t="n">
-        <v>47.87</v>
+        <v>16.25</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Shazia Bibi</t>
+          <t>Naureen Khan</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>373648</v>
+        <v>373716</v>
       </c>
       <c r="C22" t="n">
-        <v>363</v>
+        <v>190</v>
       </c>
       <c r="D22" t="n">
-        <v>402</v>
+        <v>202</v>
       </c>
       <c r="E22" t="n">
-        <v>301</v>
+        <v>173</v>
       </c>
       <c r="F22" t="n">
-        <v>101</v>
+        <v>29</v>
       </c>
       <c r="G22" t="n">
-        <v>110.74</v>
+        <v>106.32</v>
       </c>
       <c r="H22" t="n">
-        <v>82.92</v>
+        <v>91.05</v>
       </c>
       <c r="I22" t="n">
-        <v>27.82</v>
+        <v>15.26</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Naureen Khan</t>
+          <t>Nadia bibi</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>373716</v>
+        <v>373669</v>
       </c>
       <c r="C23" t="n">
-        <v>190</v>
+        <v>111</v>
       </c>
       <c r="D23" t="n">
-        <v>202</v>
+        <v>108</v>
       </c>
       <c r="E23" t="n">
-        <v>150</v>
+        <v>73</v>
       </c>
       <c r="F23" t="n">
-        <v>52</v>
+        <v>35</v>
       </c>
       <c r="G23" t="n">
-        <v>106.32</v>
+        <v>97.3</v>
       </c>
       <c r="H23" t="n">
-        <v>78.95</v>
+        <v>65.77</v>
       </c>
       <c r="I23" t="n">
-        <v>27.37</v>
+        <v>31.53</v>
       </c>
     </row>
     <row r="24">
@@ -2350,332 +2350,332 @@
         <v>262</v>
       </c>
       <c r="D24" t="n">
-        <v>255</v>
+        <v>246</v>
       </c>
       <c r="E24" t="n">
-        <v>181</v>
+        <v>200</v>
       </c>
       <c r="F24" t="n">
-        <v>74</v>
+        <v>46</v>
       </c>
       <c r="G24" t="n">
-        <v>97.33</v>
+        <v>93.89</v>
       </c>
       <c r="H24" t="n">
-        <v>69.08</v>
+        <v>76.34</v>
       </c>
       <c r="I24" t="n">
-        <v>28.24</v>
+        <v>17.56</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Nadia bibi</t>
+          <t>Zain Ul Abideen</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>373669</v>
+        <v>373667</v>
       </c>
       <c r="C25" t="n">
-        <v>111</v>
+        <v>13</v>
       </c>
       <c r="D25" t="n">
-        <v>108</v>
+        <v>12</v>
       </c>
       <c r="E25" t="n">
-        <v>50</v>
+        <v>12</v>
       </c>
       <c r="F25" t="n">
-        <v>58</v>
+        <v>0</v>
       </c>
       <c r="G25" t="n">
-        <v>97.3</v>
+        <v>92.31</v>
       </c>
       <c r="H25" t="n">
-        <v>45.05</v>
+        <v>92.31</v>
       </c>
       <c r="I25" t="n">
-        <v>52.25</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Zain Ul Abideen</t>
+          <t>Bushra Ayub</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>373667</v>
+        <v>373671</v>
       </c>
       <c r="C26" t="n">
-        <v>13</v>
+        <v>138</v>
       </c>
       <c r="D26" t="n">
-        <v>12</v>
+        <v>126</v>
       </c>
       <c r="E26" t="n">
-        <v>12</v>
+        <v>122</v>
       </c>
       <c r="F26" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G26" t="n">
-        <v>92.31</v>
+        <v>91.3</v>
       </c>
       <c r="H26" t="n">
-        <v>92.31</v>
+        <v>88.41</v>
       </c>
       <c r="I26" t="n">
-        <v>0</v>
+        <v>2.9</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Bushra Ayub</t>
+          <t>Lati khan</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>373671</v>
+        <v>652938</v>
       </c>
       <c r="C27" t="n">
-        <v>138</v>
+        <v>11</v>
       </c>
       <c r="D27" t="n">
-        <v>126</v>
+        <v>10</v>
       </c>
       <c r="E27" t="n">
-        <v>122</v>
+        <v>10</v>
       </c>
       <c r="F27" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G27" t="n">
-        <v>91.3</v>
+        <v>90.91</v>
       </c>
       <c r="H27" t="n">
-        <v>88.41</v>
+        <v>90.91</v>
       </c>
       <c r="I27" t="n">
-        <v>2.9</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Lati khan</t>
+          <t>Chashm Gul</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>652938</v>
+        <v>373695</v>
       </c>
       <c r="C28" t="n">
-        <v>11</v>
+        <v>31</v>
       </c>
       <c r="D28" t="n">
-        <v>10</v>
+        <v>27</v>
       </c>
       <c r="E28" t="n">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="F28" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="G28" t="n">
-        <v>90.91</v>
+        <v>87.09999999999999</v>
       </c>
       <c r="H28" t="n">
-        <v>90.91</v>
+        <v>58.06</v>
       </c>
       <c r="I28" t="n">
-        <v>0</v>
+        <v>29.03</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Chashm Gul</t>
+          <t>Muniba Shamim</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>373695</v>
+        <v>373659</v>
       </c>
       <c r="C29" t="n">
-        <v>31</v>
+        <v>72</v>
       </c>
       <c r="D29" t="n">
-        <v>27</v>
+        <v>58</v>
       </c>
       <c r="E29" t="n">
-        <v>18</v>
+        <v>49</v>
       </c>
       <c r="F29" t="n">
         <v>9</v>
       </c>
       <c r="G29" t="n">
-        <v>87.09999999999999</v>
+        <v>80.56</v>
       </c>
       <c r="H29" t="n">
-        <v>58.06</v>
+        <v>68.06</v>
       </c>
       <c r="I29" t="n">
-        <v>29.03</v>
+        <v>12.5</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Muniba Shamim</t>
+          <t>Muhammad Yousaf</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>373659</v>
+        <v>373690</v>
       </c>
       <c r="C30" t="n">
-        <v>72</v>
+        <v>132</v>
       </c>
       <c r="D30" t="n">
-        <v>58</v>
+        <v>105</v>
       </c>
       <c r="E30" t="n">
-        <v>49</v>
+        <v>96</v>
       </c>
       <c r="F30" t="n">
         <v>9</v>
       </c>
       <c r="G30" t="n">
-        <v>80.56</v>
+        <v>79.55</v>
       </c>
       <c r="H30" t="n">
-        <v>68.06</v>
+        <v>72.73</v>
       </c>
       <c r="I30" t="n">
-        <v>12.5</v>
+        <v>6.82</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Muhammad Yousaf</t>
+          <t>Khalida Bibi</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>373690</v>
+        <v>373673</v>
       </c>
       <c r="C31" t="n">
-        <v>132</v>
+        <v>177</v>
       </c>
       <c r="D31" t="n">
-        <v>105</v>
+        <v>140</v>
       </c>
       <c r="E31" t="n">
-        <v>96</v>
+        <v>140</v>
       </c>
       <c r="F31" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="G31" t="n">
-        <v>79.55</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="H31" t="n">
-        <v>72.73</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="I31" t="n">
-        <v>6.82</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Khalida Bibi</t>
+          <t>Asma Gull</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>373673</v>
+        <v>373672</v>
       </c>
       <c r="C32" t="n">
-        <v>177</v>
+        <v>144</v>
       </c>
       <c r="D32" t="n">
-        <v>140</v>
+        <v>109</v>
       </c>
       <c r="E32" t="n">
-        <v>140</v>
+        <v>105</v>
       </c>
       <c r="F32" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G32" t="n">
-        <v>79.09999999999999</v>
+        <v>75.69</v>
       </c>
       <c r="H32" t="n">
-        <v>79.09999999999999</v>
+        <v>72.92</v>
       </c>
       <c r="I32" t="n">
-        <v>0</v>
+        <v>2.78</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Asma Gull</t>
+          <t>Rahila Naaz</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>373672</v>
+        <v>373715</v>
       </c>
       <c r="C33" t="n">
-        <v>144</v>
+        <v>4</v>
       </c>
       <c r="D33" t="n">
-        <v>109</v>
+        <v>3</v>
       </c>
       <c r="E33" t="n">
-        <v>105</v>
+        <v>2</v>
       </c>
       <c r="F33" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G33" t="n">
-        <v>75.69</v>
+        <v>75</v>
       </c>
       <c r="H33" t="n">
-        <v>72.92</v>
+        <v>50</v>
       </c>
       <c r="I33" t="n">
-        <v>2.78</v>
+        <v>25</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Rahila Naaz</t>
+          <t>Sadia rustum</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>373715</v>
+        <v>852541</v>
       </c>
       <c r="C34" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="D34" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E34" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F34" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G34" t="n">
-        <v>75</v>
+        <v>71.43000000000001</v>
       </c>
       <c r="H34" t="n">
-        <v>50</v>
+        <v>71.43000000000001</v>
       </c>
       <c r="I34" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35">
@@ -2691,50 +2691,50 @@
         <v>249</v>
       </c>
       <c r="D35" t="n">
-        <v>184</v>
+        <v>174</v>
       </c>
       <c r="E35" t="n">
-        <v>135</v>
+        <v>144</v>
       </c>
       <c r="F35" t="n">
-        <v>49</v>
+        <v>30</v>
       </c>
       <c r="G35" t="n">
-        <v>73.90000000000001</v>
+        <v>69.88</v>
       </c>
       <c r="H35" t="n">
-        <v>54.22</v>
+        <v>57.83</v>
       </c>
       <c r="I35" t="n">
-        <v>19.68</v>
+        <v>12.05</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Sadia rustum</t>
+          <t>Saba Ramzan</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>852541</v>
+        <v>373703</v>
       </c>
       <c r="C36" t="n">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="D36" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="E36" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="F36" t="n">
         <v>0</v>
       </c>
       <c r="G36" t="n">
-        <v>71.43000000000001</v>
+        <v>69.23</v>
       </c>
       <c r="H36" t="n">
-        <v>71.43000000000001</v>
+        <v>69.23</v>
       </c>
       <c r="I36" t="n">
         <v>0</v>
@@ -2743,14 +2743,14 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Saba Ramzan</t>
+          <t>Shehla Noor</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>373703</v>
+        <v>373650</v>
       </c>
       <c r="C37" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D37" t="n">
         <v>9</v>
@@ -2762,10 +2762,10 @@
         <v>0</v>
       </c>
       <c r="G37" t="n">
-        <v>69.23</v>
+        <v>64.29000000000001</v>
       </c>
       <c r="H37" t="n">
-        <v>69.23</v>
+        <v>64.29000000000001</v>
       </c>
       <c r="I37" t="n">
         <v>0</v>
@@ -2774,259 +2774,259 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Shehla Noor</t>
+          <t>Furqan Ullah Khan</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>373650</v>
+        <v>373683</v>
       </c>
       <c r="C38" t="n">
-        <v>14</v>
+        <v>195</v>
       </c>
       <c r="D38" t="n">
-        <v>9</v>
+        <v>124</v>
       </c>
       <c r="E38" t="n">
-        <v>9</v>
+        <v>116</v>
       </c>
       <c r="F38" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="G38" t="n">
-        <v>64.29000000000001</v>
+        <v>63.59</v>
       </c>
       <c r="H38" t="n">
-        <v>64.29000000000001</v>
+        <v>59.49</v>
       </c>
       <c r="I38" t="n">
-        <v>0</v>
+        <v>4.1</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Furqan Ullah Khan</t>
+          <t>Usman Ali</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>373683</v>
+        <v>373687</v>
       </c>
       <c r="C39" t="n">
-        <v>195</v>
+        <v>8</v>
       </c>
       <c r="D39" t="n">
-        <v>124</v>
+        <v>5</v>
       </c>
       <c r="E39" t="n">
-        <v>116</v>
+        <v>5</v>
       </c>
       <c r="F39" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="G39" t="n">
-        <v>63.59</v>
+        <v>62.5</v>
       </c>
       <c r="H39" t="n">
-        <v>59.49</v>
+        <v>62.5</v>
       </c>
       <c r="I39" t="n">
-        <v>4.1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Usman Ali</t>
+          <t>Ishaq Khan</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>373687</v>
+        <v>373699</v>
       </c>
       <c r="C40" t="n">
-        <v>8</v>
+        <v>170</v>
       </c>
       <c r="D40" t="n">
-        <v>5</v>
+        <v>101</v>
       </c>
       <c r="E40" t="n">
-        <v>5</v>
+        <v>100</v>
       </c>
       <c r="F40" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G40" t="n">
-        <v>62.5</v>
+        <v>59.41</v>
       </c>
       <c r="H40" t="n">
-        <v>62.5</v>
+        <v>58.82</v>
       </c>
       <c r="I40" t="n">
-        <v>0</v>
+        <v>0.59</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Ishaq Khan</t>
+          <t>Summiya Hayat</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>373699</v>
+        <v>373710</v>
       </c>
       <c r="C41" t="n">
-        <v>170</v>
+        <v>217</v>
       </c>
       <c r="D41" t="n">
-        <v>101</v>
+        <v>116</v>
       </c>
       <c r="E41" t="n">
-        <v>100</v>
+        <v>86</v>
       </c>
       <c r="F41" t="n">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="G41" t="n">
-        <v>59.41</v>
+        <v>53.46</v>
       </c>
       <c r="H41" t="n">
-        <v>58.82</v>
+        <v>39.63</v>
       </c>
       <c r="I41" t="n">
-        <v>0.59</v>
+        <v>13.82</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Summiya Hayat</t>
+          <t>Anum Gul</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>373710</v>
+        <v>373656</v>
       </c>
       <c r="C42" t="n">
-        <v>217</v>
+        <v>103</v>
       </c>
       <c r="D42" t="n">
-        <v>121</v>
+        <v>55</v>
       </c>
       <c r="E42" t="n">
-        <v>87</v>
+        <v>51</v>
       </c>
       <c r="F42" t="n">
-        <v>34</v>
+        <v>4</v>
       </c>
       <c r="G42" t="n">
-        <v>55.76</v>
+        <v>53.4</v>
       </c>
       <c r="H42" t="n">
-        <v>40.09</v>
+        <v>49.51</v>
       </c>
       <c r="I42" t="n">
-        <v>15.67</v>
+        <v>3.88</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Anum Gul</t>
+          <t>Munawar Khan</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>373656</v>
+        <v>373668</v>
       </c>
       <c r="C43" t="n">
-        <v>103</v>
+        <v>73</v>
       </c>
       <c r="D43" t="n">
-        <v>55</v>
+        <v>38</v>
       </c>
       <c r="E43" t="n">
-        <v>51</v>
+        <v>32</v>
       </c>
       <c r="F43" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G43" t="n">
-        <v>53.4</v>
+        <v>52.05</v>
       </c>
       <c r="H43" t="n">
-        <v>49.51</v>
+        <v>43.84</v>
       </c>
       <c r="I43" t="n">
-        <v>3.88</v>
+        <v>8.220000000000001</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Munawar Khan</t>
+          <t>Muhammad Noor</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>373668</v>
+        <v>373701</v>
       </c>
       <c r="C44" t="n">
-        <v>73</v>
+        <v>8</v>
       </c>
       <c r="D44" t="n">
-        <v>38</v>
+        <v>4</v>
       </c>
       <c r="E44" t="n">
-        <v>32</v>
+        <v>3</v>
       </c>
       <c r="F44" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="G44" t="n">
-        <v>52.05</v>
+        <v>50</v>
       </c>
       <c r="H44" t="n">
-        <v>43.84</v>
+        <v>37.5</v>
       </c>
       <c r="I44" t="n">
-        <v>8.220000000000001</v>
+        <v>12.5</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Muhammad Noor</t>
+          <t>Muhammad Naeem</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>373701</v>
+        <v>373694</v>
       </c>
       <c r="C45" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D45" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E45" t="n">
         <v>3</v>
       </c>
       <c r="F45" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G45" t="n">
         <v>50</v>
       </c>
       <c r="H45" t="n">
-        <v>37.5</v>
+        <v>50</v>
       </c>
       <c r="I45" t="n">
-        <v>12.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Muhammad Naeem</t>
+          <t>Muhammad Shahid Khan</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>373694</v>
+        <v>373662</v>
       </c>
       <c r="C46" t="n">
         <v>6</v>
@@ -3053,73 +3053,73 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Muhammad Shahid Khan</t>
+          <t>Nillum Bibi</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>373662</v>
+        <v>373652</v>
       </c>
       <c r="C47" t="n">
-        <v>6</v>
+        <v>169</v>
       </c>
       <c r="D47" t="n">
+        <v>64</v>
+      </c>
+      <c r="E47" t="n">
+        <v>61</v>
+      </c>
+      <c r="F47" t="n">
         <v>3</v>
       </c>
-      <c r="E47" t="n">
-        <v>3</v>
-      </c>
-      <c r="F47" t="n">
-        <v>0</v>
-      </c>
       <c r="G47" t="n">
-        <v>50</v>
+        <v>37.87</v>
       </c>
       <c r="H47" t="n">
-        <v>50</v>
+        <v>36.09</v>
       </c>
       <c r="I47" t="n">
-        <v>0</v>
+        <v>1.78</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Nillum Bibi</t>
+          <t>Robina Shaheen</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>373652</v>
+        <v>373639</v>
       </c>
       <c r="C48" t="n">
-        <v>169</v>
+        <v>8</v>
       </c>
       <c r="D48" t="n">
-        <v>64</v>
+        <v>3</v>
       </c>
       <c r="E48" t="n">
-        <v>61</v>
+        <v>2</v>
       </c>
       <c r="F48" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G48" t="n">
-        <v>37.87</v>
+        <v>37.5</v>
       </c>
       <c r="H48" t="n">
-        <v>36.09</v>
+        <v>25</v>
       </c>
       <c r="I48" t="n">
-        <v>1.78</v>
+        <v>12.5</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Robina Shaheen</t>
+          <t>Sajjad Khan</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>373639</v>
+        <v>373700</v>
       </c>
       <c r="C49" t="n">
         <v>8</v>
@@ -3128,162 +3128,162 @@
         <v>3</v>
       </c>
       <c r="E49" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F49" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G49" t="n">
         <v>37.5</v>
       </c>
       <c r="H49" t="n">
-        <v>25</v>
+        <v>37.5</v>
       </c>
       <c r="I49" t="n">
-        <v>12.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Sajjad Khan</t>
+          <t>Nazia</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>373700</v>
+        <v>373657</v>
       </c>
       <c r="C50" t="n">
-        <v>8</v>
+        <v>144</v>
       </c>
       <c r="D50" t="n">
-        <v>3</v>
+        <v>51</v>
       </c>
       <c r="E50" t="n">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="F50" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G50" t="n">
-        <v>37.5</v>
+        <v>35.42</v>
       </c>
       <c r="H50" t="n">
-        <v>37.5</v>
+        <v>34.03</v>
       </c>
       <c r="I50" t="n">
-        <v>0</v>
+        <v>1.39</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Nazia</t>
+          <t>Alia Khan</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>373657</v>
+        <v>373681</v>
       </c>
       <c r="C51" t="n">
-        <v>144</v>
+        <v>129</v>
       </c>
       <c r="D51" t="n">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="E51" t="n">
-        <v>49</v>
+        <v>40</v>
       </c>
       <c r="F51" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G51" t="n">
-        <v>35.42</v>
+        <v>34.11</v>
       </c>
       <c r="H51" t="n">
-        <v>34.03</v>
+        <v>31.01</v>
       </c>
       <c r="I51" t="n">
-        <v>1.39</v>
+        <v>3.1</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Alia Khan</t>
+          <t>Aisha Aman</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>373681</v>
+        <v>373704</v>
       </c>
       <c r="C52" t="n">
-        <v>129</v>
+        <v>11</v>
       </c>
       <c r="D52" t="n">
-        <v>44</v>
+        <v>3</v>
       </c>
       <c r="E52" t="n">
-        <v>40</v>
+        <v>2</v>
       </c>
       <c r="F52" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G52" t="n">
-        <v>34.11</v>
+        <v>27.27</v>
       </c>
       <c r="H52" t="n">
-        <v>31.01</v>
+        <v>18.18</v>
       </c>
       <c r="I52" t="n">
-        <v>3.1</v>
+        <v>9.09</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Aisha Aman</t>
+          <t>Iqra Bibi</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>373704</v>
+        <v>373708</v>
       </c>
       <c r="C53" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D53" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E53" t="n">
         <v>2</v>
       </c>
       <c r="F53" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G53" t="n">
-        <v>27.27</v>
+        <v>25</v>
       </c>
       <c r="H53" t="n">
-        <v>18.18</v>
+        <v>25</v>
       </c>
       <c r="I53" t="n">
-        <v>9.09</v>
+        <v>0</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Iqra Bibi</t>
+          <t>Hijab Zahra</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>373708</v>
+        <v>373637</v>
       </c>
       <c r="C54" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="D54" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E54" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F54" t="n">
         <v>0</v>
@@ -3301,63 +3301,63 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Hijab Zahra</t>
+          <t>Laiba Khan</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>373637</v>
+        <v>373653</v>
       </c>
       <c r="C55" t="n">
+        <v>121</v>
+      </c>
+      <c r="D55" t="n">
+        <v>26</v>
+      </c>
+      <c r="E55" t="n">
+        <v>22</v>
+      </c>
+      <c r="F55" t="n">
         <v>4</v>
       </c>
-      <c r="D55" t="n">
-        <v>1</v>
-      </c>
-      <c r="E55" t="n">
-        <v>1</v>
-      </c>
-      <c r="F55" t="n">
-        <v>0</v>
-      </c>
       <c r="G55" t="n">
-        <v>25</v>
+        <v>21.49</v>
       </c>
       <c r="H55" t="n">
-        <v>25</v>
+        <v>18.18</v>
       </c>
       <c r="I55" t="n">
-        <v>0</v>
+        <v>3.31</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Laiba Khan</t>
+          <t>Summiya Hayat 123</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>373653</v>
+        <v>51020</v>
       </c>
       <c r="C56" t="n">
-        <v>121</v>
+        <v>5</v>
       </c>
       <c r="D56" t="n">
-        <v>26</v>
+        <v>1</v>
       </c>
       <c r="E56" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="F56" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G56" t="n">
-        <v>21.49</v>
+        <v>20</v>
       </c>
       <c r="H56" t="n">
-        <v>18.18</v>
+        <v>20</v>
       </c>
       <c r="I56" t="n">
-        <v>3.31</v>
+        <v>0</v>
       </c>
     </row>
     <row r="57">

</xml_diff>

<commit_message>
Update error log and performance summary files with latest data
</commit_message>
<xml_diff>
--- a/Error_log/Enumerator_Performance.xlsx
+++ b/Error_log/Enumerator_Performance.xlsx
@@ -464,13 +464,13 @@
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="n">
-        <v>1211</v>
+        <v>1147</v>
       </c>
       <c r="D2" t="n">
-        <v>1157</v>
+        <v>1090</v>
       </c>
       <c r="E2" t="n">
-        <v>54</v>
+        <v>57</v>
       </c>
     </row>
     <row r="3">
@@ -483,13 +483,13 @@
         <v>373641</v>
       </c>
       <c r="C3" t="n">
-        <v>571</v>
+        <v>581</v>
       </c>
       <c r="D3" t="n">
-        <v>450</v>
+        <v>456</v>
       </c>
       <c r="E3" t="n">
-        <v>121</v>
+        <v>125</v>
       </c>
     </row>
     <row r="4">
@@ -502,13 +502,13 @@
         <v>373648</v>
       </c>
       <c r="C4" t="n">
-        <v>427</v>
+        <v>434</v>
       </c>
       <c r="D4" t="n">
-        <v>355</v>
+        <v>360</v>
       </c>
       <c r="E4" t="n">
-        <v>72</v>
+        <v>74</v>
       </c>
     </row>
     <row r="5">
@@ -521,13 +521,13 @@
         <v>373646</v>
       </c>
       <c r="C5" t="n">
-        <v>474</v>
+        <v>482</v>
       </c>
       <c r="D5" t="n">
-        <v>354</v>
+        <v>358</v>
       </c>
       <c r="E5" t="n">
-        <v>120</v>
+        <v>124</v>
       </c>
     </row>
     <row r="6">
@@ -540,10 +540,10 @@
         <v>373642</v>
       </c>
       <c r="C6" t="n">
-        <v>349</v>
+        <v>354</v>
       </c>
       <c r="D6" t="n">
-        <v>281</v>
+        <v>286</v>
       </c>
       <c r="E6" t="n">
         <v>68</v>
@@ -559,13 +559,13 @@
         <v>373696</v>
       </c>
       <c r="C7" t="n">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="D7" t="n">
         <v>274</v>
       </c>
       <c r="E7" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="8">
@@ -597,13 +597,13 @@
         <v>373651</v>
       </c>
       <c r="C9" t="n">
-        <v>400</v>
+        <v>407</v>
       </c>
       <c r="D9" t="n">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="E9" t="n">
-        <v>140</v>
+        <v>145</v>
       </c>
     </row>
     <row r="10">
@@ -635,13 +635,13 @@
         <v>373705</v>
       </c>
       <c r="C11" t="n">
-        <v>261</v>
+        <v>255</v>
       </c>
       <c r="D11" t="n">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="E11" t="n">
-        <v>59</v>
+        <v>50</v>
       </c>
     </row>
     <row r="12">
@@ -654,13 +654,13 @@
         <v>373716</v>
       </c>
       <c r="C12" t="n">
-        <v>218</v>
+        <v>214</v>
       </c>
       <c r="D12" t="n">
         <v>183</v>
       </c>
       <c r="E12" t="n">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
     <row r="13">
@@ -711,13 +711,13 @@
         <v>373706</v>
       </c>
       <c r="C15" t="n">
-        <v>186</v>
+        <v>181</v>
       </c>
       <c r="D15" t="n">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="E15" t="n">
-        <v>38</v>
+        <v>34</v>
       </c>
     </row>
     <row r="16">
@@ -768,13 +768,13 @@
         <v>373692</v>
       </c>
       <c r="C18" t="n">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="D18" t="n">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="E18" t="n">
-        <v>134</v>
+        <v>131</v>
       </c>
     </row>
     <row r="19">
@@ -901,10 +901,10 @@
         <v>453925</v>
       </c>
       <c r="C25" t="n">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="D25" t="n">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="E25" t="n">
         <v>0</v>
@@ -920,13 +920,13 @@
         <v>373710</v>
       </c>
       <c r="C26" t="n">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="D26" t="n">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="E26" t="n">
-        <v>34</v>
+        <v>30</v>
       </c>
     </row>
     <row r="27">
@@ -989,39 +989,39 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Naureen</t>
+          <t>aisha.aman</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>884887</v>
+        <v>752327</v>
       </c>
       <c r="C30" t="n">
-        <v>86</v>
+        <v>151</v>
       </c>
       <c r="D30" t="n">
         <v>82</v>
       </c>
       <c r="E30" t="n">
-        <v>4</v>
+        <v>69</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>aisha.aman</t>
+          <t>Naureen</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>752327</v>
+        <v>884887</v>
       </c>
       <c r="C31" t="n">
-        <v>151</v>
+        <v>86</v>
       </c>
       <c r="D31" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="E31" t="n">
-        <v>70</v>
+        <v>4</v>
       </c>
     </row>
     <row r="32">
@@ -1034,13 +1034,13 @@
         <v>373669</v>
       </c>
       <c r="C32" t="n">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="D32" t="n">
         <v>73</v>
       </c>
       <c r="E32" t="n">
-        <v>39</v>
+        <v>35</v>
       </c>
     </row>
     <row r="33">
@@ -1668,19 +1668,19 @@
         <v>2</v>
       </c>
       <c r="D2" t="n">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="E2" t="n">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="F2" t="n">
         <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>4550</v>
+        <v>4650</v>
       </c>
       <c r="H2" t="n">
-        <v>4550</v>
+        <v>4650</v>
       </c>
       <c r="I2" t="n">
         <v>0</v>
@@ -1823,22 +1823,22 @@
         <v>101</v>
       </c>
       <c r="D7" t="n">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="E7" t="n">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="F7" t="n">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="G7" t="n">
-        <v>253.47</v>
+        <v>254.46</v>
       </c>
       <c r="H7" t="n">
-        <v>120.79</v>
+        <v>124.75</v>
       </c>
       <c r="I7" t="n">
-        <v>132.67</v>
+        <v>129.7</v>
       </c>
     </row>
     <row r="8">
@@ -1913,25 +1913,25 @@
         <v>373641</v>
       </c>
       <c r="C10" t="n">
-        <v>376</v>
+        <v>389</v>
       </c>
       <c r="D10" t="n">
-        <v>571</v>
+        <v>581</v>
       </c>
       <c r="E10" t="n">
-        <v>450</v>
+        <v>456</v>
       </c>
       <c r="F10" t="n">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="G10" t="n">
-        <v>151.86</v>
+        <v>149.36</v>
       </c>
       <c r="H10" t="n">
-        <v>119.68</v>
+        <v>117.22</v>
       </c>
       <c r="I10" t="n">
-        <v>32.18</v>
+        <v>32.13</v>
       </c>
     </row>
     <row r="11">
@@ -2037,25 +2037,25 @@
         <v>373651</v>
       </c>
       <c r="C14" t="n">
-        <v>286</v>
+        <v>298</v>
       </c>
       <c r="D14" t="n">
-        <v>400</v>
+        <v>407</v>
       </c>
       <c r="E14" t="n">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="F14" t="n">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="G14" t="n">
-        <v>139.86</v>
+        <v>136.58</v>
       </c>
       <c r="H14" t="n">
-        <v>90.91</v>
+        <v>87.92</v>
       </c>
       <c r="I14" t="n">
-        <v>48.95</v>
+        <v>48.66</v>
       </c>
     </row>
     <row r="15">
@@ -2071,22 +2071,22 @@
         <v>239</v>
       </c>
       <c r="D15" t="n">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="E15" t="n">
         <v>274</v>
       </c>
       <c r="F15" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="G15" t="n">
-        <v>133.05</v>
+        <v>132.64</v>
       </c>
       <c r="H15" t="n">
         <v>114.64</v>
       </c>
       <c r="I15" t="n">
-        <v>18.41</v>
+        <v>17.99</v>
       </c>
     </row>
     <row r="16">
@@ -2136,81 +2136,81 @@
         <v>151</v>
       </c>
       <c r="E17" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F17" t="n">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G17" t="n">
         <v>125.83</v>
       </c>
       <c r="H17" t="n">
-        <v>67.5</v>
+        <v>68.33</v>
       </c>
       <c r="I17" t="n">
-        <v>58.33</v>
+        <v>57.5</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Irum Ikram</t>
+          <t>Jaweria</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>373642</v>
+        <v>163495</v>
       </c>
       <c r="C18" t="n">
-        <v>283</v>
+        <v>74</v>
       </c>
       <c r="D18" t="n">
-        <v>349</v>
+        <v>90</v>
       </c>
       <c r="E18" t="n">
-        <v>281</v>
+        <v>87</v>
       </c>
       <c r="F18" t="n">
-        <v>68</v>
+        <v>3</v>
       </c>
       <c r="G18" t="n">
-        <v>123.32</v>
+        <v>121.62</v>
       </c>
       <c r="H18" t="n">
-        <v>99.29000000000001</v>
+        <v>117.57</v>
       </c>
       <c r="I18" t="n">
-        <v>24.03</v>
+        <v>4.05</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Jaweria</t>
+          <t>Irum Ikram</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>163495</v>
+        <v>373642</v>
       </c>
       <c r="C19" t="n">
-        <v>74</v>
+        <v>292</v>
       </c>
       <c r="D19" t="n">
-        <v>90</v>
+        <v>354</v>
       </c>
       <c r="E19" t="n">
-        <v>87</v>
+        <v>286</v>
       </c>
       <c r="F19" t="n">
-        <v>3</v>
+        <v>68</v>
       </c>
       <c r="G19" t="n">
-        <v>121.62</v>
+        <v>121.23</v>
       </c>
       <c r="H19" t="n">
-        <v>117.57</v>
+        <v>97.95</v>
       </c>
       <c r="I19" t="n">
-        <v>4.05</v>
+        <v>23.29</v>
       </c>
     </row>
     <row r="20">
@@ -2223,25 +2223,25 @@
         <v>373646</v>
       </c>
       <c r="C20" t="n">
-        <v>396</v>
+        <v>411</v>
       </c>
       <c r="D20" t="n">
-        <v>474</v>
+        <v>482</v>
       </c>
       <c r="E20" t="n">
-        <v>354</v>
+        <v>358</v>
       </c>
       <c r="F20" t="n">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="G20" t="n">
-        <v>119.7</v>
+        <v>117.27</v>
       </c>
       <c r="H20" t="n">
-        <v>89.39</v>
+        <v>87.09999999999999</v>
       </c>
       <c r="I20" t="n">
-        <v>30.3</v>
+        <v>30.17</v>
       </c>
     </row>
     <row r="21">
@@ -2254,25 +2254,25 @@
         <v>373648</v>
       </c>
       <c r="C21" t="n">
-        <v>385</v>
+        <v>398</v>
       </c>
       <c r="D21" t="n">
-        <v>427</v>
+        <v>434</v>
       </c>
       <c r="E21" t="n">
-        <v>355</v>
+        <v>360</v>
       </c>
       <c r="F21" t="n">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="G21" t="n">
-        <v>110.91</v>
+        <v>109.05</v>
       </c>
       <c r="H21" t="n">
-        <v>92.20999999999999</v>
+        <v>90.45</v>
       </c>
       <c r="I21" t="n">
-        <v>18.7</v>
+        <v>18.59</v>
       </c>
     </row>
     <row r="22">
@@ -2288,22 +2288,22 @@
         <v>211</v>
       </c>
       <c r="D22" t="n">
-        <v>218</v>
+        <v>214</v>
       </c>
       <c r="E22" t="n">
         <v>183</v>
       </c>
       <c r="F22" t="n">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="G22" t="n">
-        <v>103.32</v>
+        <v>101.42</v>
       </c>
       <c r="H22" t="n">
         <v>86.73</v>
       </c>
       <c r="I22" t="n">
-        <v>16.59</v>
+        <v>14.69</v>
       </c>
     </row>
     <row r="23">
@@ -2319,177 +2319,177 @@
         <v>111</v>
       </c>
       <c r="D23" t="n">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="E23" t="n">
         <v>73</v>
       </c>
       <c r="F23" t="n">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="G23" t="n">
-        <v>100.9</v>
+        <v>97.3</v>
       </c>
       <c r="H23" t="n">
         <v>65.77</v>
       </c>
       <c r="I23" t="n">
-        <v>35.14</v>
+        <v>31.53</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Mahnoor</t>
+          <t>Zain Ul Abideen</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>373705</v>
+        <v>373667</v>
       </c>
       <c r="C24" t="n">
-        <v>281</v>
+        <v>13</v>
       </c>
       <c r="D24" t="n">
-        <v>261</v>
+        <v>12</v>
       </c>
       <c r="E24" t="n">
-        <v>202</v>
+        <v>12</v>
       </c>
       <c r="F24" t="n">
-        <v>59</v>
+        <v>0</v>
       </c>
       <c r="G24" t="n">
-        <v>92.88</v>
+        <v>92.31</v>
       </c>
       <c r="H24" t="n">
-        <v>71.89</v>
+        <v>92.31</v>
       </c>
       <c r="I24" t="n">
-        <v>21</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Zain Ul Abideen</t>
+          <t>Bushra Ayub</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>373667</v>
+        <v>373671</v>
       </c>
       <c r="C25" t="n">
-        <v>13</v>
+        <v>138</v>
       </c>
       <c r="D25" t="n">
-        <v>12</v>
+        <v>126</v>
       </c>
       <c r="E25" t="n">
-        <v>12</v>
+        <v>122</v>
       </c>
       <c r="F25" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G25" t="n">
-        <v>92.31</v>
+        <v>91.3</v>
       </c>
       <c r="H25" t="n">
-        <v>92.31</v>
+        <v>88.41</v>
       </c>
       <c r="I25" t="n">
-        <v>0</v>
+        <v>2.9</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Bushra Ayub</t>
+          <t>Lati khan</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>373671</v>
+        <v>652938</v>
       </c>
       <c r="C26" t="n">
-        <v>138</v>
+        <v>11</v>
       </c>
       <c r="D26" t="n">
-        <v>126</v>
+        <v>10</v>
       </c>
       <c r="E26" t="n">
-        <v>122</v>
+        <v>10</v>
       </c>
       <c r="F26" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G26" t="n">
-        <v>91.3</v>
+        <v>90.91</v>
       </c>
       <c r="H26" t="n">
-        <v>88.41</v>
+        <v>90.91</v>
       </c>
       <c r="I26" t="n">
-        <v>2.9</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Lati khan</t>
+          <t>Chashm Gul</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>652938</v>
+        <v>373695</v>
       </c>
       <c r="C27" t="n">
-        <v>11</v>
+        <v>31</v>
       </c>
       <c r="D27" t="n">
-        <v>10</v>
+        <v>27</v>
       </c>
       <c r="E27" t="n">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="F27" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="G27" t="n">
-        <v>90.91</v>
+        <v>87.09999999999999</v>
       </c>
       <c r="H27" t="n">
-        <v>90.91</v>
+        <v>58.06</v>
       </c>
       <c r="I27" t="n">
-        <v>0</v>
+        <v>29.03</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Chashm Gul</t>
+          <t>Mahnoor</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>373695</v>
+        <v>373705</v>
       </c>
       <c r="C28" t="n">
-        <v>31</v>
+        <v>294</v>
       </c>
       <c r="D28" t="n">
-        <v>27</v>
+        <v>255</v>
       </c>
       <c r="E28" t="n">
-        <v>18</v>
+        <v>205</v>
       </c>
       <c r="F28" t="n">
-        <v>9</v>
+        <v>50</v>
       </c>
       <c r="G28" t="n">
-        <v>87.09999999999999</v>
+        <v>86.73</v>
       </c>
       <c r="H28" t="n">
-        <v>58.06</v>
+        <v>69.73</v>
       </c>
       <c r="I28" t="n">
-        <v>29.03</v>
+        <v>17.01</v>
       </c>
     </row>
     <row r="29">
@@ -2681,63 +2681,63 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Laiba Shams</t>
+          <t>Saba Ramzan</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>373706</v>
+        <v>373703</v>
       </c>
       <c r="C35" t="n">
-        <v>266</v>
+        <v>13</v>
       </c>
       <c r="D35" t="n">
-        <v>186</v>
+        <v>9</v>
       </c>
       <c r="E35" t="n">
-        <v>148</v>
+        <v>9</v>
       </c>
       <c r="F35" t="n">
-        <v>38</v>
+        <v>0</v>
       </c>
       <c r="G35" t="n">
-        <v>69.92</v>
+        <v>69.23</v>
       </c>
       <c r="H35" t="n">
-        <v>55.64</v>
+        <v>69.23</v>
       </c>
       <c r="I35" t="n">
-        <v>14.29</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Saba Ramzan</t>
+          <t>Laiba Shams</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>373703</v>
+        <v>373706</v>
       </c>
       <c r="C36" t="n">
-        <v>13</v>
+        <v>279</v>
       </c>
       <c r="D36" t="n">
-        <v>9</v>
+        <v>181</v>
       </c>
       <c r="E36" t="n">
-        <v>9</v>
+        <v>147</v>
       </c>
       <c r="F36" t="n">
-        <v>0</v>
+        <v>34</v>
       </c>
       <c r="G36" t="n">
-        <v>69.23</v>
+        <v>64.87</v>
       </c>
       <c r="H36" t="n">
-        <v>69.23</v>
+        <v>52.69</v>
       </c>
       <c r="I36" t="n">
-        <v>0</v>
+        <v>12.19</v>
       </c>
     </row>
     <row r="37">
@@ -2898,104 +2898,104 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Summiya Hayat</t>
+          <t>Munawar Khan</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>373710</v>
+        <v>373668</v>
       </c>
       <c r="C42" t="n">
-        <v>229</v>
+        <v>73</v>
       </c>
       <c r="D42" t="n">
-        <v>122</v>
+        <v>38</v>
       </c>
       <c r="E42" t="n">
-        <v>88</v>
+        <v>32</v>
       </c>
       <c r="F42" t="n">
-        <v>34</v>
+        <v>6</v>
       </c>
       <c r="G42" t="n">
-        <v>53.28</v>
+        <v>52.05</v>
       </c>
       <c r="H42" t="n">
-        <v>38.43</v>
+        <v>43.84</v>
       </c>
       <c r="I42" t="n">
-        <v>14.85</v>
+        <v>8.220000000000001</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Munawar Khan</t>
+          <t>Muhammad Noor</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>373668</v>
+        <v>373701</v>
       </c>
       <c r="C43" t="n">
-        <v>73</v>
+        <v>8</v>
       </c>
       <c r="D43" t="n">
-        <v>38</v>
+        <v>4</v>
       </c>
       <c r="E43" t="n">
-        <v>32</v>
+        <v>3</v>
       </c>
       <c r="F43" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="G43" t="n">
-        <v>52.05</v>
+        <v>50</v>
       </c>
       <c r="H43" t="n">
-        <v>43.84</v>
+        <v>37.5</v>
       </c>
       <c r="I43" t="n">
-        <v>8.220000000000001</v>
+        <v>12.5</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Muhammad Noor</t>
+          <t>Muhammad Naeem</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>373701</v>
+        <v>373694</v>
       </c>
       <c r="C44" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D44" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E44" t="n">
         <v>3</v>
       </c>
       <c r="F44" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G44" t="n">
         <v>50</v>
       </c>
       <c r="H44" t="n">
-        <v>37.5</v>
+        <v>50</v>
       </c>
       <c r="I44" t="n">
-        <v>12.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Muhammad Naeem</t>
+          <t>Muhammad Shahid Khan</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>373694</v>
+        <v>373662</v>
       </c>
       <c r="C45" t="n">
         <v>6</v>
@@ -3022,32 +3022,32 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Muhammad Shahid Khan</t>
+          <t>Summiya Hayat</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>373662</v>
+        <v>373710</v>
       </c>
       <c r="C46" t="n">
-        <v>6</v>
+        <v>242</v>
       </c>
       <c r="D46" t="n">
-        <v>3</v>
+        <v>119</v>
       </c>
       <c r="E46" t="n">
-        <v>3</v>
+        <v>89</v>
       </c>
       <c r="F46" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="G46" t="n">
-        <v>50</v>
+        <v>49.17</v>
       </c>
       <c r="H46" t="n">
-        <v>50</v>
+        <v>36.78</v>
       </c>
       <c r="I46" t="n">
-        <v>0</v>
+        <v>12.4</v>
       </c>
     </row>
     <row r="47">
@@ -3649,7 +3649,7 @@
         <v>453925</v>
       </c>
       <c r="C66" t="n">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="D66" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Remove outdated Annex B Duration Cases file and add new Fast Surveys Duration Cases file for updated data analysis.
</commit_message>
<xml_diff>
--- a/Error_log/Enumerator_Performance.xlsx
+++ b/Error_log/Enumerator_Performance.xlsx
@@ -464,13 +464,13 @@
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="n">
-        <v>1107</v>
+        <v>1096</v>
       </c>
       <c r="D2" t="n">
-        <v>1038</v>
+        <v>1025</v>
       </c>
       <c r="E2" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
     </row>
     <row r="3">
@@ -483,51 +483,51 @@
         <v>373641</v>
       </c>
       <c r="C3" t="n">
-        <v>601</v>
+        <v>619</v>
       </c>
       <c r="D3" t="n">
-        <v>470</v>
+        <v>484</v>
       </c>
       <c r="E3" t="n">
-        <v>131</v>
+        <v>135</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Shazia Bibi</t>
+          <t>Shafaq Zahra</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>373648</v>
+        <v>373646</v>
       </c>
       <c r="C4" t="n">
-        <v>448</v>
+        <v>519</v>
       </c>
       <c r="D4" t="n">
-        <v>367</v>
+        <v>380</v>
       </c>
       <c r="E4" t="n">
-        <v>81</v>
+        <v>139</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Shafaq Zahra</t>
+          <t>Shazia Bibi</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>373646</v>
+        <v>373648</v>
       </c>
       <c r="C5" t="n">
-        <v>499</v>
+        <v>452</v>
       </c>
       <c r="D5" t="n">
-        <v>366</v>
+        <v>371</v>
       </c>
       <c r="E5" t="n">
-        <v>133</v>
+        <v>81</v>
       </c>
     </row>
     <row r="6">
@@ -540,51 +540,51 @@
         <v>373642</v>
       </c>
       <c r="C6" t="n">
-        <v>364</v>
+        <v>370</v>
       </c>
       <c r="D6" t="n">
-        <v>290</v>
+        <v>294</v>
       </c>
       <c r="E6" t="n">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Shazia begum</t>
+          <t>Javairia</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>373696</v>
+        <v>373651</v>
       </c>
       <c r="C7" t="n">
-        <v>317</v>
+        <v>429</v>
       </c>
       <c r="D7" t="n">
-        <v>274</v>
+        <v>281</v>
       </c>
       <c r="E7" t="n">
-        <v>43</v>
+        <v>148</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Javairia</t>
+          <t>Shazia begum</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>373651</v>
+        <v>373696</v>
       </c>
       <c r="C8" t="n">
-        <v>416</v>
+        <v>324</v>
       </c>
       <c r="D8" t="n">
-        <v>268</v>
+        <v>281</v>
       </c>
       <c r="E8" t="n">
-        <v>148</v>
+        <v>43</v>
       </c>
     </row>
     <row r="9">
@@ -616,10 +616,10 @@
         <v>373705</v>
       </c>
       <c r="C10" t="n">
-        <v>264</v>
+        <v>279</v>
       </c>
       <c r="D10" t="n">
-        <v>213</v>
+        <v>228</v>
       </c>
       <c r="E10" t="n">
         <v>51</v>
@@ -635,10 +635,10 @@
         <v>373712</v>
       </c>
       <c r="C11" t="n">
-        <v>308</v>
+        <v>317</v>
       </c>
       <c r="D11" t="n">
-        <v>207</v>
+        <v>216</v>
       </c>
       <c r="E11" t="n">
         <v>101</v>
@@ -647,58 +647,58 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Naureen Khan</t>
+          <t>Samara</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>373716</v>
+        <v>373658</v>
       </c>
       <c r="C12" t="n">
-        <v>214</v>
+        <v>281</v>
       </c>
       <c r="D12" t="n">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="E12" t="n">
-        <v>31</v>
+        <v>95</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Sadia Rustum</t>
+          <t>Naureen Khan</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>373649</v>
+        <v>373716</v>
       </c>
       <c r="C13" t="n">
-        <v>192</v>
+        <v>214</v>
       </c>
       <c r="D13" t="n">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="E13" t="n">
-        <v>10</v>
+        <v>31</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Samara</t>
+          <t>Sadia Rustum</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>373658</v>
+        <v>373649</v>
       </c>
       <c r="C14" t="n">
-        <v>274</v>
+        <v>192</v>
       </c>
       <c r="D14" t="n">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="E14" t="n">
-        <v>95</v>
+        <v>10</v>
       </c>
     </row>
     <row r="15">
@@ -711,51 +711,51 @@
         <v>373706</v>
       </c>
       <c r="C15" t="n">
-        <v>188</v>
+        <v>194</v>
       </c>
       <c r="D15" t="n">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="E15" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Khalida Bibi</t>
+          <t>Rehana Bibi</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>373673</v>
+        <v>373691</v>
       </c>
       <c r="C16" t="n">
-        <v>140</v>
+        <v>275</v>
       </c>
       <c r="D16" t="n">
-        <v>140</v>
+        <v>149</v>
       </c>
       <c r="E16" t="n">
-        <v>0</v>
+        <v>126</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Rehana Bibi</t>
+          <t>Khalida Bibi</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>373691</v>
+        <v>373673</v>
       </c>
       <c r="C17" t="n">
-        <v>265</v>
+        <v>140</v>
       </c>
       <c r="D17" t="n">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="E17" t="n">
-        <v>126</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
@@ -768,10 +768,10 @@
         <v>373692</v>
       </c>
       <c r="C18" t="n">
-        <v>257</v>
+        <v>261</v>
       </c>
       <c r="D18" t="n">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="E18" t="n">
         <v>131</v>
@@ -818,134 +818,134 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Asma Gull</t>
+          <t>Naureen khan</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>373672</v>
+        <v>453925</v>
       </c>
       <c r="C21" t="n">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="D21" t="n">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="E21" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Naureen khan</t>
+          <t>Summiya Hayat</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>453925</v>
+        <v>373710</v>
       </c>
       <c r="C22" t="n">
-        <v>104</v>
+        <v>136</v>
       </c>
       <c r="D22" t="n">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="E22" t="n">
-        <v>2</v>
+        <v>30</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Ishaq Khan</t>
+          <t>Asma Gull</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>373699</v>
+        <v>373672</v>
       </c>
       <c r="C23" t="n">
-        <v>101</v>
+        <v>109</v>
       </c>
       <c r="D23" t="n">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="E23" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Summiya Hayat</t>
+          <t>Ishaq Khan</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>373710</v>
+        <v>373699</v>
       </c>
       <c r="C24" t="n">
-        <v>128</v>
+        <v>101</v>
       </c>
       <c r="D24" t="n">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="E24" t="n">
-        <v>30</v>
+        <v>1</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Muhammad Yousaf</t>
+          <t>aisha.aman</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>373690</v>
+        <v>752327</v>
       </c>
       <c r="C25" t="n">
-        <v>105</v>
+        <v>173</v>
       </c>
       <c r="D25" t="n">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="E25" t="n">
-        <v>9</v>
+        <v>74</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Lati Khan</t>
+          <t>Muhammad Yousaf</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>564273</v>
+        <v>373690</v>
       </c>
       <c r="C26" t="n">
-        <v>97</v>
+        <v>105</v>
       </c>
       <c r="D26" t="n">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="E26" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>aisha.aman</t>
+          <t>Lati Khan</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>752327</v>
+        <v>564273</v>
       </c>
       <c r="C27" t="n">
-        <v>160</v>
+        <v>97</v>
       </c>
       <c r="D27" t="n">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="E27" t="n">
-        <v>72</v>
+        <v>4</v>
       </c>
     </row>
     <row r="28">
@@ -1034,10 +1034,10 @@
         <v>373669</v>
       </c>
       <c r="C32" t="n">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="D32" t="n">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="E32" t="n">
         <v>35</v>
@@ -1685,22 +1685,22 @@
         <v>2</v>
       </c>
       <c r="D2" t="n">
-        <v>104</v>
+        <v>114</v>
       </c>
       <c r="E2" t="n">
-        <v>102</v>
+        <v>111</v>
       </c>
       <c r="F2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G2" t="n">
-        <v>5200</v>
+        <v>5700</v>
       </c>
       <c r="H2" t="n">
-        <v>5100</v>
+        <v>5550</v>
       </c>
       <c r="I2" t="n">
-        <v>100</v>
+        <v>150</v>
       </c>
     </row>
     <row r="3">
@@ -1809,19 +1809,19 @@
         <v>104</v>
       </c>
       <c r="D6" t="n">
-        <v>308</v>
+        <v>317</v>
       </c>
       <c r="E6" t="n">
-        <v>207</v>
+        <v>216</v>
       </c>
       <c r="F6" t="n">
         <v>101</v>
       </c>
       <c r="G6" t="n">
-        <v>296.15</v>
+        <v>304.81</v>
       </c>
       <c r="H6" t="n">
-        <v>199.04</v>
+        <v>207.69</v>
       </c>
       <c r="I6" t="n">
         <v>97.12</v>
@@ -1840,19 +1840,19 @@
         <v>101</v>
       </c>
       <c r="D7" t="n">
-        <v>257</v>
+        <v>261</v>
       </c>
       <c r="E7" t="n">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="F7" t="n">
         <v>131</v>
       </c>
       <c r="G7" t="n">
-        <v>254.46</v>
+        <v>258.42</v>
       </c>
       <c r="H7" t="n">
-        <v>124.75</v>
+        <v>128.71</v>
       </c>
       <c r="I7" t="n">
         <v>129.7</v>
@@ -1871,19 +1871,19 @@
         <v>111</v>
       </c>
       <c r="D8" t="n">
-        <v>265</v>
+        <v>275</v>
       </c>
       <c r="E8" t="n">
-        <v>139</v>
+        <v>149</v>
       </c>
       <c r="F8" t="n">
         <v>126</v>
       </c>
       <c r="G8" t="n">
-        <v>238.74</v>
+        <v>247.75</v>
       </c>
       <c r="H8" t="n">
-        <v>125.23</v>
+        <v>134.23</v>
       </c>
       <c r="I8" t="n">
         <v>113.51</v>
@@ -1902,19 +1902,19 @@
         <v>120</v>
       </c>
       <c r="D9" t="n">
-        <v>274</v>
+        <v>281</v>
       </c>
       <c r="E9" t="n">
-        <v>179</v>
+        <v>186</v>
       </c>
       <c r="F9" t="n">
         <v>95</v>
       </c>
       <c r="G9" t="n">
-        <v>228.33</v>
+        <v>234.17</v>
       </c>
       <c r="H9" t="n">
-        <v>149.17</v>
+        <v>155</v>
       </c>
       <c r="I9" t="n">
         <v>79.17</v>
@@ -1959,25 +1959,25 @@
         <v>373641</v>
       </c>
       <c r="C11" t="n">
-        <v>408</v>
+        <v>417</v>
       </c>
       <c r="D11" t="n">
-        <v>601</v>
+        <v>619</v>
       </c>
       <c r="E11" t="n">
-        <v>470</v>
+        <v>484</v>
       </c>
       <c r="F11" t="n">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="G11" t="n">
-        <v>147.3</v>
+        <v>148.44</v>
       </c>
       <c r="H11" t="n">
-        <v>115.2</v>
+        <v>116.07</v>
       </c>
       <c r="I11" t="n">
-        <v>32.11</v>
+        <v>32.37</v>
       </c>
     </row>
     <row r="12">
@@ -2083,25 +2083,25 @@
         <v>373651</v>
       </c>
       <c r="C15" t="n">
-        <v>307</v>
+        <v>315</v>
       </c>
       <c r="D15" t="n">
-        <v>416</v>
+        <v>429</v>
       </c>
       <c r="E15" t="n">
-        <v>268</v>
+        <v>281</v>
       </c>
       <c r="F15" t="n">
         <v>148</v>
       </c>
       <c r="G15" t="n">
-        <v>135.5</v>
+        <v>136.19</v>
       </c>
       <c r="H15" t="n">
-        <v>87.3</v>
+        <v>89.20999999999999</v>
       </c>
       <c r="I15" t="n">
-        <v>48.21</v>
+        <v>46.98</v>
       </c>
     </row>
     <row r="16">
@@ -2117,19 +2117,19 @@
         <v>239</v>
       </c>
       <c r="D16" t="n">
-        <v>317</v>
+        <v>324</v>
       </c>
       <c r="E16" t="n">
-        <v>274</v>
+        <v>281</v>
       </c>
       <c r="F16" t="n">
         <v>43</v>
       </c>
       <c r="G16" t="n">
-        <v>132.64</v>
+        <v>135.56</v>
       </c>
       <c r="H16" t="n">
-        <v>114.64</v>
+        <v>117.57</v>
       </c>
       <c r="I16" t="n">
         <v>17.99</v>
@@ -2176,25 +2176,25 @@
         <v>752327</v>
       </c>
       <c r="C18" t="n">
-        <v>130</v>
+        <v>140</v>
       </c>
       <c r="D18" t="n">
-        <v>160</v>
+        <v>173</v>
       </c>
       <c r="E18" t="n">
-        <v>88</v>
+        <v>99</v>
       </c>
       <c r="F18" t="n">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="G18" t="n">
-        <v>123.08</v>
+        <v>123.57</v>
       </c>
       <c r="H18" t="n">
-        <v>67.69</v>
+        <v>70.70999999999999</v>
       </c>
       <c r="I18" t="n">
-        <v>55.38</v>
+        <v>52.86</v>
       </c>
     </row>
     <row r="19">
@@ -2231,63 +2231,63 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Irum Ikram</t>
+          <t>Shafaq Zahra</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>373642</v>
+        <v>373646</v>
       </c>
       <c r="C20" t="n">
-        <v>307</v>
+        <v>434</v>
       </c>
       <c r="D20" t="n">
-        <v>364</v>
+        <v>519</v>
       </c>
       <c r="E20" t="n">
-        <v>290</v>
+        <v>380</v>
       </c>
       <c r="F20" t="n">
-        <v>74</v>
+        <v>139</v>
       </c>
       <c r="G20" t="n">
-        <v>118.57</v>
+        <v>119.59</v>
       </c>
       <c r="H20" t="n">
-        <v>94.45999999999999</v>
+        <v>87.56</v>
       </c>
       <c r="I20" t="n">
-        <v>24.1</v>
+        <v>32.03</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Shafaq Zahra</t>
+          <t>Irum Ikram</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>373646</v>
+        <v>373642</v>
       </c>
       <c r="C21" t="n">
-        <v>425</v>
+        <v>312</v>
       </c>
       <c r="D21" t="n">
-        <v>499</v>
+        <v>370</v>
       </c>
       <c r="E21" t="n">
-        <v>366</v>
+        <v>294</v>
       </c>
       <c r="F21" t="n">
-        <v>133</v>
+        <v>76</v>
       </c>
       <c r="G21" t="n">
-        <v>117.41</v>
+        <v>118.59</v>
       </c>
       <c r="H21" t="n">
-        <v>86.12</v>
+        <v>94.23</v>
       </c>
       <c r="I21" t="n">
-        <v>31.29</v>
+        <v>24.36</v>
       </c>
     </row>
     <row r="22">
@@ -2303,19 +2303,19 @@
         <v>417</v>
       </c>
       <c r="D22" t="n">
-        <v>448</v>
+        <v>452</v>
       </c>
       <c r="E22" t="n">
-        <v>367</v>
+        <v>371</v>
       </c>
       <c r="F22" t="n">
         <v>81</v>
       </c>
       <c r="G22" t="n">
-        <v>107.43</v>
+        <v>108.39</v>
       </c>
       <c r="H22" t="n">
-        <v>88.01000000000001</v>
+        <v>88.97</v>
       </c>
       <c r="I22" t="n">
         <v>19.42</v>
@@ -2324,63 +2324,63 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Naureen Khan</t>
+          <t>Nadia bibi</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>373716</v>
+        <v>373669</v>
       </c>
       <c r="C23" t="n">
-        <v>211</v>
+        <v>111</v>
       </c>
       <c r="D23" t="n">
-        <v>214</v>
+        <v>113</v>
       </c>
       <c r="E23" t="n">
-        <v>183</v>
+        <v>78</v>
       </c>
       <c r="F23" t="n">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="G23" t="n">
-        <v>101.42</v>
+        <v>101.8</v>
       </c>
       <c r="H23" t="n">
-        <v>86.73</v>
+        <v>70.27</v>
       </c>
       <c r="I23" t="n">
-        <v>14.69</v>
+        <v>31.53</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Nadia bibi</t>
+          <t>Naureen Khan</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>373669</v>
+        <v>373716</v>
       </c>
       <c r="C24" t="n">
-        <v>111</v>
+        <v>211</v>
       </c>
       <c r="D24" t="n">
-        <v>108</v>
+        <v>214</v>
       </c>
       <c r="E24" t="n">
-        <v>73</v>
+        <v>183</v>
       </c>
       <c r="F24" t="n">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="G24" t="n">
-        <v>97.3</v>
+        <v>101.42</v>
       </c>
       <c r="H24" t="n">
-        <v>65.77</v>
+        <v>86.73</v>
       </c>
       <c r="I24" t="n">
-        <v>31.53</v>
+        <v>14.69</v>
       </c>
     </row>
     <row r="25">
@@ -2479,63 +2479,63 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Chashm Gul</t>
+          <t>Mahnoor</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>373695</v>
+        <v>373705</v>
       </c>
       <c r="C28" t="n">
-        <v>31</v>
+        <v>320</v>
       </c>
       <c r="D28" t="n">
-        <v>27</v>
+        <v>279</v>
       </c>
       <c r="E28" t="n">
-        <v>18</v>
+        <v>228</v>
       </c>
       <c r="F28" t="n">
-        <v>9</v>
+        <v>51</v>
       </c>
       <c r="G28" t="n">
-        <v>87.09999999999999</v>
+        <v>87.19</v>
       </c>
       <c r="H28" t="n">
-        <v>58.06</v>
+        <v>71.25</v>
       </c>
       <c r="I28" t="n">
-        <v>29.03</v>
+        <v>15.94</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Mahnoor</t>
+          <t>Chashm Gul</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>373705</v>
+        <v>373695</v>
       </c>
       <c r="C29" t="n">
-        <v>311</v>
+        <v>31</v>
       </c>
       <c r="D29" t="n">
-        <v>264</v>
+        <v>27</v>
       </c>
       <c r="E29" t="n">
-        <v>213</v>
+        <v>18</v>
       </c>
       <c r="F29" t="n">
-        <v>51</v>
+        <v>9</v>
       </c>
       <c r="G29" t="n">
-        <v>84.89</v>
+        <v>87.09999999999999</v>
       </c>
       <c r="H29" t="n">
-        <v>68.48999999999999</v>
+        <v>58.06</v>
       </c>
       <c r="I29" t="n">
-        <v>16.4</v>
+        <v>29.03</v>
       </c>
     </row>
     <row r="30">
@@ -2789,63 +2789,63 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Furqan Ullah Khan</t>
+          <t>Laiba Shams</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>373683</v>
+        <v>373706</v>
       </c>
       <c r="C38" t="n">
-        <v>195</v>
+        <v>302</v>
       </c>
       <c r="D38" t="n">
-        <v>124</v>
+        <v>194</v>
       </c>
       <c r="E38" t="n">
-        <v>116</v>
+        <v>156</v>
       </c>
       <c r="F38" t="n">
-        <v>8</v>
+        <v>38</v>
       </c>
       <c r="G38" t="n">
-        <v>63.59</v>
+        <v>64.23999999999999</v>
       </c>
       <c r="H38" t="n">
-        <v>59.49</v>
+        <v>51.66</v>
       </c>
       <c r="I38" t="n">
-        <v>4.1</v>
+        <v>12.58</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Laiba Shams</t>
+          <t>Furqan Ullah Khan</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>373706</v>
+        <v>373683</v>
       </c>
       <c r="C39" t="n">
-        <v>297</v>
+        <v>195</v>
       </c>
       <c r="D39" t="n">
-        <v>188</v>
+        <v>124</v>
       </c>
       <c r="E39" t="n">
-        <v>152</v>
+        <v>116</v>
       </c>
       <c r="F39" t="n">
-        <v>36</v>
+        <v>8</v>
       </c>
       <c r="G39" t="n">
-        <v>63.3</v>
+        <v>63.59</v>
       </c>
       <c r="H39" t="n">
-        <v>51.18</v>
+        <v>59.49</v>
       </c>
       <c r="I39" t="n">
-        <v>12.12</v>
+        <v>4.1</v>
       </c>
     </row>
     <row r="40">
@@ -2975,73 +2975,73 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Muhammad Noor</t>
+          <t>Summiya Hayat</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>373701</v>
+        <v>373710</v>
       </c>
       <c r="C44" t="n">
-        <v>8</v>
+        <v>265</v>
       </c>
       <c r="D44" t="n">
-        <v>4</v>
+        <v>136</v>
       </c>
       <c r="E44" t="n">
-        <v>3</v>
+        <v>106</v>
       </c>
       <c r="F44" t="n">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="G44" t="n">
-        <v>50</v>
+        <v>51.32</v>
       </c>
       <c r="H44" t="n">
-        <v>37.5</v>
+        <v>40</v>
       </c>
       <c r="I44" t="n">
-        <v>12.5</v>
+        <v>11.32</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Muhammad Naeem</t>
+          <t>Muhammad Noor</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>373694</v>
+        <v>373701</v>
       </c>
       <c r="C45" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D45" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E45" t="n">
         <v>3</v>
       </c>
       <c r="F45" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G45" t="n">
         <v>50</v>
       </c>
       <c r="H45" t="n">
-        <v>50</v>
+        <v>37.5</v>
       </c>
       <c r="I45" t="n">
-        <v>0</v>
+        <v>12.5</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Muhammad Shahid Khan</t>
+          <t>Muhammad Naeem</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>373662</v>
+        <v>373694</v>
       </c>
       <c r="C46" t="n">
         <v>6</v>
@@ -3068,32 +3068,32 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Summiya Hayat</t>
+          <t>Muhammad Shahid Khan</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>373710</v>
+        <v>373662</v>
       </c>
       <c r="C47" t="n">
-        <v>260</v>
+        <v>6</v>
       </c>
       <c r="D47" t="n">
-        <v>128</v>
+        <v>3</v>
       </c>
       <c r="E47" t="n">
-        <v>98</v>
+        <v>3</v>
       </c>
       <c r="F47" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="G47" t="n">
-        <v>49.23</v>
+        <v>50</v>
       </c>
       <c r="H47" t="n">
-        <v>37.69</v>
+        <v>50</v>
       </c>
       <c r="I47" t="n">
-        <v>11.54</v>
+        <v>0</v>
       </c>
     </row>
     <row r="48">
@@ -3695,7 +3695,7 @@
         <v>453925</v>
       </c>
       <c r="C67" t="n">
-        <v>79</v>
+        <v>91</v>
       </c>
       <c r="D67" t="n">
         <v>0</v>

</xml_diff>